<commit_message>
Add sentiment + stance analysis and update datasets
</commit_message>
<xml_diff>
--- a/data/raw_extracted_data.xlsx
+++ b/data/raw_extracted_data.xlsx
@@ -476,6 +476,19 @@
           <t>Guidance on safe and responsible use of Gen AI tools The aim of this guidance is to help you use GenAI tools safely and responsibly, so you feel confident about exploring different ways of using this technology to support your learning. Generative Artificial Intelligence (GenAI) is a fast-evolving technology and, during your time at Oxford, the University wants to enable and support the safe and productive use of these tools that will be important in your future. Ethical use GenAI tools must be used responsibly and ethically, in accordance with the academic standards of rigour and integrity that are expected of you as a student at Oxford. You should always use AI tools with integrity, honesty, and transparency, and maintain a critical approach to using any output generated by these tools. This document contains some useful tips for using GenAI to support your studies at Oxford. You should always follow the advice and guidance of your tutors and/or supervisors, and consult your department or faculty in relation to ethical use. Assessment For each specific assessment you will be given prior written notice of whether or not the use of AI is permitted. You are fully responsible for the accuracy, originality, and quality of work you submit for assessment, and you must follow the rules on AI use for each specific assessment you are taking. You must make a formal declaration of any permitted AI-use in the format prescribed by your assessment setter. Any unauthorised use of AI in work submitted for assessment constitutes cheating and plagiarism under University rules, penalties for which include failing the relevant assessment and, in appropriate cases, expulsion. Any use of AI in work submitted for assessment is unauthorised unless you are specifically told differently in writing, in advance of the assessment, in instructions from your faculty’s or department for the specific assessment in question. Even if a type of AI use has been authorised for a previous assessment, or for formative work, it is your responsibility to ensure that you comply with the rules on AI use for the specific assessment you are taking, in the knowledge that all types of AI use are unauthorised unless specifically listed in assessment instructions. Cases of suspected unauthorised use of AI in assessment are covered by the University’s student conduct regulations. You should make yourself familiar with these regulations, as any actions that are found potentially to be in breach of them will be reviewed in line with the University’s Code of Discipline and Academic Disciplinary procedure. You should always follow the guidance of your tutors and/or supervisors, and of your department or faculty. Use in research All research undertaken by academic staff and students, including by postgraduate students, must meet the expectations in the Policy for using Generative AI in Research: guidelines for researchers and professional staff. Substantive use of GenAI should be declared whenever a stand-alone AI tool is used (such as ChatGPT Edu), but not where GenAI functionality is embedded within existing software. Substantive use of GenAI by students who are conducting research as part of a graduate research programme is defined as: - interpreting and analysing data (including audio and image files) and texts, - undertaking a literature review or translation, - identifying research gaps, - formulating research aims, - developing hypotheses, - assisting with generating ideas or to develop one’s own thinking, - generating code and synthetic data, - undertaking transcription of interviews, meetings etc. to save time and effort rather than overcoming barriers (see exclusions below) - producing documents using other people’s work or from transcripts or recordings. Substantive use may exclude using GenAI for tasks such as assisting you with translation if you are a non-native speaker, transforming transcribed spoken language into written language if you face barriers to writing, formatting documents, or improving the standard of your English or of a foreign language. As with assessment, you should always follow the guidance of your tutors, supervisors, and of your department or faculty. Use of GenAI in research falls within the scope of research conduct and the permitted use of AI as outlined abov. Actions that are found to be in potential breach will be reviewed in line with the University's Code of practice and procedure on academic integrity in research. Your health and wellbeing Because of the way that GenAI tools work, they are not a replacement for human interaction and are not equipped to offer therapy or mental health support. You should be aware that GenAI tools lack emotional nuance and clinical awareness. They can sometimes give inaccurate and potentially dangerous advice. At times of heightened distress or mental health crisis, AI chatbots may reinforce harmful thoughts through feedback loops. The University’s Student Welfare and Support Services offer a range of support with welfare and wellbeing. This includes access to Togetherall, a free and anonymous online platform where for connecting with others about what’s going on in life - big or small. Togetherall also offers free courses, resources, and anonymous chats to support your wellbeing, 24 hours a day. The SWSS also provide a free counselling service and a wealth of resources on the Oxford Students website and MyOxford app. In addition, support and advice are available from your college, department, fellow students and the Students' Union. There are contacts for emergency (including out of hours) and non-emergency services for health, welfare and academic support. All student welfare services remain open throughout the vacations (except Bank Holiday Mondays and the Christmas closure period), with some adjusted opening hours (listed on each service's page) and vacation welfare support page. Using GenAI to support your studies Part of what a university education teaches is academic skills such as assimilating information, constructing an evidence-based argument, and expressing your thoughts in clear, coherent prose. AI tools cannot replace human critical thinking or the development of scholarly, evidence-based arguments and the subject knowledge that form the basis of your university education. You should always cross-check AI generated outputs against established sources to verify accuracy and identify erroneous information. You may make use of University-supported generative AI tools (e.g. ChatGPT Edu, Google Gemini, Notebook LM and Copilot Chat) to develop your academic skills and to support your studies. This should be done in consultation with your tutors, faculty, or department, and you should always follow their advice in relation to how they expect AI tools to be used (or not used) for different tasks. These tools are accessed via your University Single Sign-On (SSO) account. Your ongoing critical appraisal of GenAI outputs, by reviewing them critically for accuracy and relevance, will maximise their potential to support you in your studies. Academic writing and presentation skills Depending on your academic discipline, GenAI tools can be useful in developing your academic writing skills and providing initial feedback on them, translating between different styles, and critiquing your own writing. They cannot replace the need for you to develop such skills through tutorials or supervisions, and independent learning, however. Depending on your academic discipline, GenAI tools also may be used to support your academic reading, but there is a risk that they could undermine the development of critical academic skills (e.g. if you use a GenAI tool to summarise an article for you, rather than fully engaging with the literature or undertaking the task yourself). You should always remain alert to the limitations of AI-generated outputs. Here, again, the subject-specific guidance of your tutors, supervisors, and faculty or department is crucial, because appropriate use of AI to support academic reading varies across different academic disciplines. Appropriate use of GenAI tools to support your academic writing and presentation skills varies across academic disciplines. Always follow any advice and guidance of your tutors or supervisors, department/faculty, or college, on what is appropriate in your subject area. Supporting the learning process Generative AI tools may be useful in supporting your academic studies, but be sure to discuss AI outputs with academic staff to confirm your understanding and to help verify them against established sources, to ensure their accuracy. Appropriate use of GenAI tools to support the learning process varies across different academic disciplines. Always follow any advice and guidance of your tutors or supervisors, and of your department or faculty, and/or college, on what is appropriate in your subject area. Tips for using GenAI tools effectively The University provides you with access to secure, enterprise-level ChatGPT Edu, Google Gemini, Notebook LM and Copilot Chat tools. Different GenAI tools can be used for different purposes. Here are some examples of key uses for some of the secure tools the University supports: - ChatGPT Edu – Advanced content generation, summarising information and complex reasoning - Microsoft Copilot Chat – Web-grounded chat, summarising information, drafting content and web-based information retrieval - Google Gemini – AI assistance that is integrated with Google Workspace, or can be used as a standalone chat tool - Notebook LM – An AI assistant that can interact with and summarise lecture notes, papers and other uploaded sources to aid research and study. You may find it useful to try a few different GenAI tools and you should be aware that different tools will give different outputs to one another, from the same prompts. Within a single tool you may also get different outputs in response to the same prompt. It is important to be aware that: - You will get different responses using the same prompts from the same GenAI tool. AI outputs are not repeatable, and all tools can generate outputs that contain inaccuracies and fabrications. - You could spend a lot of time trying out different AI tools. Be careful to balance your exploration of GenAI with managing your time effectively. - GenAI tools may draw on data that can be months or years out of date and, whilst outputs seem plausible, they may contain errors and/or reflect biases from the original data the tool was trained on. For example, Western perspectives are overly represented. - GenAI tools do not replace the need for you to develop your own knowledge, skills, and critical awareness, as an independent learner. - Take care when inputting material into any third-party tools that are not provided by the University. These may not meet the University’s standards of information security and data protection. Never upload confidential, sensitive, or unpublished material into third-party AI tools. Help and technical support with GenAI tools If you need help or technical support with using University-supported GenAI tools: - Consider first seeking support from the company whose product you're using: - ChatGPT Edu: For access and activation queries, please use the OpenAI help portal. You can use the chat at the bottom of the page to ask questions and connect with support by clicking on the Message tab. If you are unable to resolve your issue through the help portal, then you should contact OpenAI support directly by email at [email protected]. - Microsoft Copilot: The Microsoft Support site can be searched to assist with queries on Copilot. - Google Gemini: Google's Gemini Apps Help page offers various pieces of advice and support for using Gemini. - NotebookLM: Google’s NotebookLM Help page covers help topics from getting started to troubleshooting NotebookLM. - If your query is about whether an outage is affecting your connection to a particular tool, try the relevant status pages: - OpenAI Status page for ChatGPT Edu - Microsoft Status page for Microsoft Copilot - Google Status page for Google Gemini and NotebookLM - For simple queries regarding University-supported GenAI tools and support, use the AI Competency Centre chatbot to be directed to relevant information. - Contact the University's IT Service Desk if you need more support - they can help you with ChatGPT Edu, Microsoft Copilot, or the GenAI tools in the University's Google workspace (Gemini and Notebook LM). If your query needs escalating, the IT Service Desk will involve our GenAI specialists at the AI Competency Centre or signpost you to tailored support from elsewhere in the University, as needed. Find out more To find out more about using GenAI tools at Oxford, please visit the Generative AI at Oxford webpage. This guidance is under continuous review and will be updated to reflect the evolving landscape of AI use across the University. Content last updated on 22 September 2025.</t>
         </is>
       </c>
+      <c r="D2" t="n">
+        <v>2045</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -490,7 +503,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AI guidance Guidance for University of Cambridge Staff on the Administrative Use of Generative AI This page provides guidance on the use of Generative Artificial Intelligence (GenAI) for administrative tasks in support of University activities, and links to sources of further information. - Scope - Structure and overview of this guidance - Benefits - Risks - Best practice: practical examples - Copilot: Useful Facts - Further reading on best practice with use of GenAI This guidance was published in February 2025 and is accurate as of that date. Due to the fast pace of change in this area, in particular with regard to the range of licensed GenAI tools being made available to staff and students, it will be reviewed and updated during autumn 2025. A summary of key points is also available here. Scope Please be aware this guidance only applies in limited circumstances, as described below. Scope of this guidance: technology This guidance exclusively concerns the use of GenAI. GenAI typically describes any type of AI which can be instructed to produce content. Large Language Models (LLMs), such as Copilot, OpenAI ChatGPT, Google Bard and Gemini, are part of this category of AI. They produce text-based outputs based on written or verbal instructions from human users. These are sometimes referred to as natural language text prompts. There are also GenAI tools such as DALL.E, Midjourney and Stable Diffusion that produce digital imagery based on written or verbal instructions. In addition to the standalone GenAI tools described above, GenAI is increasingly incorporated into software and systems to enhance their capabilities. This guidance applies to both use of standalone GenAI tools and GenAI features in software and systems. It does not apply to use of systems or software that may include GenAI features where those features are not being utilised. This guidance does not apply to other forms of AI that may be conceived, developed or utilised across the University. Nevertheless, some of the broad principles for good practice outlined below may be relevant in other contexts. Scope of this guidance: audience and context This guidance is aimed at members of staff (or equivalents such as casual workers, interns, volunteers or visiting staff) considering the use of GenAI for administrative tasks in support of University activities. This guidance applies to routine tasks such as the production of content for an email to a student or colleague. It also applies to more complex tasks such as the production of content for formal policies or strategic reports. Ultimately, staff are responsible for ensuring any use of GenAI is conducted reasonably, lawfully, and in conjunction with relevant University policies and procedures. Scope of this guidance: where this guidance does not apply This guidance does not apply to use of GenAI in other contexts. In particular, this guidance does not apply to: - Education - This guidance does not apply to any task or content creation undertaken in the direct provision of teaching, student learning and/or academic assessment. - It does not apply to the appropriate use of GenAI by students to support their learning. - It does not apply to inappropriate use of GenAI by students in regard to plagiarism or any other perceived form of academic misconduct. - It does not apply to programmes of study, courses or lectures where GenAI is the subject matter. - Research - This guidance does not apply to GenAI as a topic of research – it does not apply to research regarding any dimension of GenAI as a technology, its application, nor the impact of its application in any given scenario. - It does not apply to any research undertaken with the assistance of any form of GenAI. The ethics and appropriateness of its use in those circumstances will be assessed by other established means (e.g. research ethics processes). - Colleges and other non-University legal entities - This guidance does not apply to use of GenAI tools by College employees for any College business, or to the Students’ Union, student societies, or Cambridge University Press &amp; Assessment. Please see the ‘Further reading on best practice with use of GenAI’ section for other University resources on use of GenAI that may be relevant to the matters identified above. Structure and overview of this guidance Given the diverse range of work the University undertakes, it is not possible for the University to provide comprehensive instruction on circumstances in which it would or would not be appropriate to use GenAI tools. It is up to departments, faculties and individual members of staff to balance the benefits and risks of the use of GenAI, to make an informed decision about whether its use is appropriate or desirable – before it is initiated. In the limited circumstances where a formal risk assessment is required, the University Data Protection Impact Assessment (DPIA) and Information Security Risk Assessment (ISRA) processes remain the relevant risk assessments processes to follow. To help guide staff in their decision making we have provided the following: - a brief outline of some of the benefits of the use of GenAI - guidance on the risks associated with use of GenAI tools - practical examples of good and bad practice - useful facts about Copilot Regardless of the work being undertaken, it is recommended that staff avoid inputting confidential, sensitive or personal information into GenAI tools unless warranted and only in accordance with this guidance. Please see the UIS guidance on different data types: https://help.uis.cam.ac.uk/service/security/data-sec-classes. Where the use of GenAI will not encompass the use of confidential, sensitive, or personal information, the risk to the University is reduced. However, it is still important to consider whether its use constitutes the best available means of completing a task. Any use of AI must be appropriately transparent and accountable. If it is necessary and beneficial to use GenAI tools, it is recommended that wherever practicable the University’s licensed AI tools, Microsoft Copilot and Copilot for Microsoft 365 are utilised, regardless of the type of data that may be input. Use of other licenced GenAI tools is not prohibited, but such tools must be procured in accordance with any applicable procurement policy or process, including but not limited to the completion of any requisite risk assessments such as DPIAs and/or ISRAs. Any risk associated with their deployment rests with the relevant department. Any use of such GenAI tools should also be accordance with this guidance. Copilot is already available to staff. Microsoft Copilot is the basic licensed version and is available via a staff login and Copilot for Microsoft 365 is the more comprehensive version, which is available via an additional purchased licence. The public free version, available via a web browser, must not be used for University activities and purposes as it does not guarantee a sufficient level of information security or confidentiality. More information on Microsoft Copilot and Copilot for Microsoft 365 is available on the UIS website: https://help.uis.cam.ac.uk/service/collaboration/365/copilot. Please remember the Acceptable Use Policy (AUP) continues to apply, including its compliance monitoring and enforcement provisions, when using GenAI tools and staff are reminded of their obligation to abide by its terms. In all circumstances, staff are expected to exercise caution and use their judgement in their use of GenAI. Benefits Many potential benefits of using GenAI tools are already apparent, and the University encourages all its staff to make the best use of the information services made available to them. Here is a brief list of potential benefits in supporting University activities. Efficiency and productivity GenAI tools can quickly process a lot of information to produce a large amount of output, saving time that can be spent on other tasks, and boosting efficiency and productivity. Flexibility GenAI can create content in various formats, styles and languages, making it useful in a wide range of circumstances. For example, it could be used to generate drafts of meeting minutes, letters, press releases, social media posts, and other forms of documentation produced in the course of University business. That flexibility also allows the University to engage with different audiences across various platforms. In some circumstances, it may be appropriate and beneficial to use it to produce personalised content. Creativity GenAI can produce novel or unusual content from existing source material, making it a useful tool for the initial part of some creative tasks. For example, it could be used to draft materials that could form part of a marketing campaign. Understanding GenAI doesn’t just have to be used for content production and creation. It could be used to discover and summarise vast amounts of information in more digestible formats, and so it can be a valuable tool in the early stages of research undertaken to support administrative tasks. Risks There are, however, significant legal and reputational risks associated with use of GenAI tools, which can be broadly categorised as follows: - Bias, misinformation and inaccuracy - Data protection law non-compliance - Intellectual property and copyright law non-compliance - AI legislation non-compliance - Reputational damage and other risks This list is not exhaustive, given the overlapping nature of risk categories and the pace of AI development. Staff must consider relevant risks, and whether they are applicable to the circumstances in which they are considering use of GenAI, before any use of GenAI is initiated. Risk: Bias, misinformation and inaccuracy Much GenAI is trained to produce outputs based on information and patterns extracted from data in the public domain. Consequently, outputs will sometimes reflect the biases and prejudices of individuals and groups in society. GenAI can also be manipulated to deliberately produce biased or inaccurate outputs, presented as fact. Unlike human intelligence, AI does not have the capacity to apply judgement or understand context. It cannot apply moral or critical perspectives. Additionally, there is an inherent risk that the ongoing use of GenAI tools will create and sustain feedback loops, whereby GenAI tools will be trained on text outputs generated by other GenAI tools, further reinforcing existing biases and inaccuracies. In practical terms, that means some outputs will be inaccurate or unbalanced regardless of the phrasing of the text prompt, because the source material is inaccurate or unbalanced. Some output may also be inaccurate because the GenAI tool is ‘hallucinating’ – creating nonsensical or inaccurate outputs that are not directly attributable to the source material. For those reasons, it is important that any GenAI output is thoroughly evaluated by a human being before it is utilised for any purpose. This is especially important where there is the risk of an adverse impact on a group or individual, or the potential for infringement of a person’s rights (e.g. as defined under the Equality Act 2010, the Human Rights Act 1998 or any other relevant legislation). Risk mitigation(s): Ensure that all GenAI outputs are thoroughly evaluated by a human being before they are used. Ensure use of GenAI is acknowledged if it is used to make a significant and unrevised contribution to a substantive or impactful piece of work such as the production of content for formal policies or strategic reports. Risk: data protection law non-compliance GenAI tools and their use are subject to existing laws and regulations and any University policy relevant to their use. This includes data protection laws such as the UK GDPR, the Data Protection Act 2018 and the University Data Protection Policy. As with the use of other information tools and services, it is important to use licensed versions of tools paid for from a University budget and procured through any applicable procurement process. (Free, unlicensed information tools and services often rely upon intrusive data processing and/or selling as part of their business model.) The University’s standard licensed AI tools are Microsoft Copilot and Copilot for Microsoft 365, and this is the tool that should be used to process personal data, where necessary, for which the University is responsible. This ensures that technical, operational and legal safeguards are in place, which protect any personal data that the University controls or otherwise processes. By contrast, inputting data into a free or unlicensed GenAI tool could be considered equivalent to putting it into the public domain – signifying a potential personal data breach. Information input into GenAI tools is also often used to train those tools, which may not be a lawful use of personal data – especially if that data cannot be retrieved or deleted, for example from an AI neural network. Data input into the University’s licensed version of Microsoft Copilot and Copilot for Microsoft 365 is not used to train those tools. It is particularly important to be cautious about inputting sensitive personal information (special category data) such as medical information into GenAI tools. Processing of such information is subject to additional safeguards, and misuse could represent a serious breach of data protection law and/or a breach of confidentiality. Regardless of the type of information you wish to input into a GenAI, you must consider the task you are using it to support. Data must be collected, held and used for only that purpose – for example, as part of a governance process – and any use of AI must be compatible with that reason. With some exceptions (e.g. for academic research), it is not appropriate to use personal data that was collected for a different purpose to do something else with a GenAI tool. It is also important to be mindful of ‘automated decision making’. Automated decision making involves: - making a decision that will affect a person solely by automated means without any human involvement; or - profiling someone – automated processing of personal data to evaluate certain things about an individual that could be used as part of a decision-making process. A common example of automated decision making is a credit check conducted exclusively using AI to decide whether to provide someone with a personal loan. While the use of GenAI to produce text or digital imagery would not necessarily result in a decision being made about an individual, it is not inconceivable that the use of such technology could be used as part of an evaluation process. For example, to review an application for a parking permit to ensure the person applying meets the eligibility criteria. In such circumstances, it is imperative that a human being is ultimately involved in the decision-making process. If after careful consideration you decide to use a GenAI tool, you must tell the affected people that you’re going to do that. That doesn’t mean you must seek consent on a case-by-case basis, but it will mean that relevant privacy notices should be provided or updated. Risk mitigation(s): Be cautious about inputting personal data into GenAI tools, especially sensitive personal data, and only do so where warranted. Do not use free GenAI tools. Use the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. Deploy relevant privacy notices. Risk: intellectual property and copyright non-compliance It has been argued by some affected parties that the entire basis for training GenAI tools through publicly available data is a violation of intellectual property rights and copyright law. There are a series of ongoing and well-publicised copyright cases where high profile individuals and organisations have sued companies that own and operate GenAI. Bearing that in mind, it is important to consider the nature of the content being input into any GenAI tool and to consider whether the University has the right to input that information into that GenAI tool. It is also important that GenAI outputs are thoroughly checked by a human being and cited where appropriate. Risk mitigation(s): Consider whether it is appropriate to input material into GenAI tools. Cite outputs where appropriate. Use the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. Risk: AI legislation non-compliance In March 2024, the European Union (EU) introduced new laws that will require organisations using AI in the EU to employ a risk-based approach to their use of AI, especially with regard to the use of personal information. It will incrementally start to take effect from February 2025, and non-compliance with the legislation could result in penalties from European regulators. It will affect the University where it is processing EU citizens’ data using AI. Risk mitigation(s): Exercise caution and judgement regarding deployment of GenAI on EU citizens’ data. Document any use of GenAI tools in these circumstances. Risk: Reputational damage and other risks As outlined above, there are various legal risks posed by the use of GenAI, all of which could result in reputational damage to the University. There is also an environmental cost associated to use of GenAI: training GenAI tools requires vast amounts of power and indirectly generates enormous amounts of carbon, meaning there is a sustainability consideration to its use. In the development of some GenAI tools, outputs are checked and refined in a process known as Reinforcement Learning from Human Feedback (RLHF). That process includes human reviewers, often working in countries in the global south for very low wages, routinely viewing objectionable and distasteful materials, and has been reported to have a profoundly negative impact on the health and well-being of many of those workers. University staff will also be expected to provide human oversight of GenAI outputs. Whilst they would not ordinarily be exposed to objectionable nor distasteful materials in the course of administrative work, it is important to consider the risk to University staff wellbeing that could be posed by increased workloads and unrealistic expectations of what can be reasonably achieved using GenAI tools. Risk mitigation(s): Consider the wider impact on the University’s reputation before using GenAI. Consider any other relevant risks. Best practice: practical examples Here are a series of practical examples intended to show both best practice and scenarios in which the use of AI should be considered carefully. It remains important to bear in mind the general risks and benefits associated with use of GenAI in these different contexts. Example 1: Using GenAI for background research Capability: GenAI can be used as a research tool to help gather background information on a topic relating to something you are unfamiliar with. Example scenario: Using GenAI to provide an overview of a new piece of legislation that may affect your work at the University. Good practice: Using the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. Not inputting any personal or confidential information into Microsoft Copilot or Copilot for Microsoft 365, because it is not required to understand the new legislation. Bad practice: Using an unlicensed GenAI tool. Inputting confidential data into that unlicensed AI tool with the aim of further understanding the legislation, thus committing a personal data breach and/or breach of confidentiality. Example 2: Using GenAI to summarise information Capability: GenAI can be used to summarise information. Example scenario: Using GenAI to prepare a briefing on a University project for a meeting with a commercial partner. Good practice: Using the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. Treating the output as a draft and amending it as appropriate. Thoroughly checking the output to ensure it is factually accurate and unbiased, does not reveal anything confidential to the commercial partner and is reflective of the source material. Acknowledging GenAI has been used to help create the briefing if it has not been materially altered as part of the fact-checking or drafting process. Bad practice: Using an unlicensed GenAI tool. Treating the output as a final draft. Accepting the output as factually accurate and suitable for sharing with a third party and not bothering to check it before presenting it to the commercial partner. Failing to mention it has been created using a GenAI tool. Example 3: Using GenAI to draft a document Capability: GenAI has the ability to produce written outputs in various styles and formats. Example scenario: Using GenAI to create meeting minutes. Good practice: Considering whether use of GenAI is appropriate in these circumstances – this will depend on what the meeting is about. Considering whether the document is likely to contain sensitive information. If the document is likely to contain sensitive information, considering the type of sensitive information, and whether use of GenAI is warranted. If it is appropriate to use a GenAI tool, using the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365, and ensuring unauthorised AI note-taking bots are prevented from joining the meeting. Using the output as a draft and amending it as appropriate. Bad practice: Using an unlicensed GenAI tool. Inputting confidential or sensitive data into that unlicensed GenAI tool thus committing a personal data breach and/or breach of confidentiality. Failing to follow UIS advice on preventing unauthorised AI note-taking bots from joining your Teams meeting. Example 4: Using GenAI for numerical analysis Capability: GenAI can perform numerical analysis. Example scenario: Using GenAI to analyse the statistical results of a staff survey. Good practice: Considering whether the raw survey data contains personal or sensitive information. If it is appropriate to deploy a GenAI tool, using the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. Telling staff that AI will be used to analyse responses when they are choosing whether they wish to participate. Treating the output as a draft and verifying and amending it as appropriate. Bad practice: Using an unlicensed GenAI tool. Not telling staff that GenAI will be used to analyse their responses. Accepting the output as factually accurate and making an unquestioning decision based on the analysis. Failing to follow UIS advice on preventing unauthorised AI note-taking bots from joining your Teams meeting. Copilot: Useful Facts This section contains a few useful facts that may assist staff in using the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. The version of Copilot accessible to most University MS365 users is called “Microsoft Copilot”. A more comprehensive version of Copilot is available called “Copilot for Microsoft 365”, and a licence for its use can be purchased by contacting UIS. This table compares the functionality available in Microsoft Copilot against the functionality available in Copilot for Microsoft 365. (Please be aware that GenAI tools are being constantly updated, so the information tabulated below may be out of date). | Functionality Questions | Microsoft Copilot | Copilot for Microsoft 365 | |---|---|---| | Is it available to University MS365 users? | Yes, through their standard login. | No, an additional licence must be purchased from UIS. | | Does it integrate with Microsoft Apps? | No. | Yes. | | Can it draft emails? | Yes, but text output must be copied into Outlook. | Yes, it will draft emails in Outlook. | | Can it draft documents? | Yes, but text must be copied into Word. | Yes, it will draft documents in Word. | | Can it be used with spreadsheets? | Yes, spreadsheets can be attached to chats. | Yes, but it will sometimes fail to produce outputs from Excel files with complex formatting | | Can it be used to create PowerPoint presentations? | No, but it can be used to create the content for a presentation via the chat function. | Yes. | | Can it summarise documents? | Yes, documents can be attached to chats. | Yes, documents can be attached to chats and it will summarise Microsoft documents in those apps. | | Will it summarise PDFs and other documents in standard formats? | Yes, via a chat. | Yes, via a chat. | | Is there a word limit for documents attached to a chat? | There is no known limit. | There is no known limit. | | What is the character limit for chat instructions? | 8,000 | 16,000 | | Is there a limit on the number of questions I can ask? | There is conversation limit of 30 questions, but you can start as many new chats as necessary. | There is conversation limit of 30 questions, but you can start as many new chats as necessary. | | What is the word limit on chat text outputs? | There is no known limit. | There is no known limit. | Here are some potentially useful tips for using Copilot: - When accessing Microsoft Copilot, you can check whether you are logged into your University MS365 account by viewing the top right-hand corner of your window – you will be able to see your initials (and your name if you click on the initials) if you are logged in. - When attaching documents, these will be automatically saved in a folder called ‘Microsoft Copilot Chat Files’ in your University MS365 account OneDrive. - Delete chat files that are no longer required. - Delete files uploaded into OneDrive as part of the chat process when no longer required. - There is more information regarding OneDrive on the UIS website: https://help.uis.cam.ac.uk/service/collaboration/365/onedrive. Further reading on best practice with use of GenAI University resources: - Applications: AI and undergraduate applications - Communications: OEAC staff please see the relevant pages of the OEAC website for further guidance on using GenAI in the production of content for communications. - Education: Blended Learning Service – AI and Education - UIS: Copilot - UIS: Guidance on information security (including policies and data classification) - UIS: LinkedIn Learning at the University of Cambridge (type in ‘GenAI’ when logged in) External resources: - ICO guidance resources on data protection and AI - An introduction to copyright law and practice in education, and the concerns arising in the context of GenerativeAI - Artificial intelligence (jiscinvolve.org) - Generative AI Framework for HM Government - Organisation for Economic Co-operation and Development (OECD) AI principles Authorship This guidance was composed without the use of AI.</t>
+          <t>AI guidance Guidance for University of Cambridge Staff on the Administrative Use of Generative AI This page provides guidance on the use of Generative Artificial Intelligence (GenAI) for administrative tasks in support of University activities, and links to sources of further information. - Scope - Structure and overview of this guidance - Benefits - Risks - Best practice: practical examples - Copilot, Gemini and NotebookLM: Useful Facts - Further reading on best practice with use of GenAI This guidance was first published in February 2025 and last updated in December 2025. It is accurate as of the latter date. Due to the fast pace of change in this area, in particular with regard to the range of licensed GenAI tools being made available to staff and students, it will be reviewed and updated again during summer 2026. A summary of key points is also available here. Scope Please be aware this guidance only applies in limited circumstances, as described below. Scope of this guidance: technology This guidance exclusively concerns the use of GenAI. GenAI typically describes any type of AI which can be instructed to produce content. Large Language Models (LLMs), such as Copilot, OpenAI ChatGPT, Google Gemini and Claude are part of this category of AI. Their primary function is to produce text-based outputs based on written or verbal instructions from human users. These are sometimes referred to as natural language text prompts. There are also GenAI tools such as DALL.E, Midjourney, Stable Diffusion, Adobe Firefly and Google Imagen that produce digital imagery based on written or verbal instructions. In addition to the standalone GenAI tools described above, GenAI is increasingly incorporated into software and systems to enhance their capabilities. This guidance applies to both use of standalone GenAI tools and GenAI features in software and systems. It does not apply to use of systems or software that may include GenAI features where those features are not being utilised. This guidance does not apply to other forms of AI that may be conceived, developed or utilised across the University. Nevertheless, some of the broad principles for good practice outlined below may be relevant in other contexts. Scope of this guidance: audience and context This guidance is aimed at members of staff (or equivalents such as casual workers, interns, volunteers or visiting staff) considering the use of GenAI for administrative tasks in support of University activities. This guidance applies to routine tasks such as the production of content for an email to a student or colleague. It also applies to more complex tasks such as the production of content for formal policies or strategic reports. Ultimately, staff are responsible for ensuring any use of GenAI is conducted reasonably, lawfully and in conjunction with relevant University policies and procedures. Scope of this guidance: where this guidance does not apply This guidance does not apply to use of GenAI in other contexts. In particular, this guidance does not apply to: - Education - This guidance does not apply to any task or content creation undertaken in the direct provision of teaching, student learning and/or academic assessment. - It does not apply to the appropriate use of GenAI by students to support their learning. - It does not apply to inappropriate use of GenAI by students in regard to plagiarism or any other perceived form of academic misconduct. - It does not apply to programmes of study, courses or lectures where GenAI is the subject matter. - Research - This guidance does not apply to GenAI as a topic of research – it does not apply to research regarding any dimension of GenAI as a technology, its application, nor the impact of its application in any given scenario. - It does not apply to any research undertaken with the assistance of any form of GenAI. The ethics and appropriateness of its use in those circumstances will be assessed by other established means (e.g. research ethics processes). - Colleges and other non-University legal entities - This guidance does not apply to use of GenAI tools by College employees for any College business, or to the Students’ Union, student societies, or Cambridge University Press &amp; Assessment. Please see the ‘Further reading on best practice with use of GenAI’ section for other University resources on use of GenAI that may be relevant to the matters identified above. Structure and overview of this guidance Given the diverse range of work the University undertakes, it is not possible for the University to provide comprehensive instruction on circumstances in which it would or would not be appropriate to use GenAI tools. It is up to departments, faculties and individual members of staff to balance the benefits and risks of the use of GenAI, to make an informed decision about whether its use is appropriate or desirable – before it is initiated. In the limited circumstances where a formal risk assessment is required, the University Data Protection Impact Assessment (DPIA) and Information Security Risk Assessment (ISRA) processes remain the relevant risk assessments processes to follow. To help guide staff in their decision making we have provided the following: - a brief outline of some of the benefits of the use of GenAI - guidance on the risks associated with use of GenAI tools - practical examples of good and bad practice - useful facts about Copilot, Gemini and NotebookLM Regardless of the work being undertaken, it is recommended that staff avoid inputting confidential, sensitive or personal information into GenAI tools unless warranted and only in accordance with this guidance. Please see the UIS guidance on different data types. Where the use of GenAI will not encompass the use of confidential, sensitive, or personal information, the risk to the University is reduced. However, it is still important to consider whether its use constitutes the best available means of completing a task. Any use of AI must be appropriately transparent and accountable. If it is necessary and beneficial to use GenAI tools, it is recommended that wherever practicable the University’s licensed GenAI tools, Copilot, Gemini and NotebookLM are utilised, regardless of the type of data that may be input. Use of other licenced GenAI tools is not prohibited, but such tools must be procured in accordance with any applicable procurement policy or process, including but not limited to the completion of any requisite risk assessments such as DPIAs and/or ISRAs. Any risk associated with their deployment rests with the relevant department. Any use of such GenAI tools should also be accordance with this guidance. Copilot, Gemini and NotebookLM are already available to staff. Microsoft 365 Copilot is the basic licensed version of Copilot and is available via a staff login, and Copilot for Microsoft 365 is the more comprehensive version, which is available via an additional purchased licence. More information on Microsoft 365 Copilot and Copilot for Microsoft 365 is available on the UIS website. Gemini and NotebookLM are available to all University members through Google Workspace. More information on Gemini is available here, and more information on NotebookLM is available here. The public, free versions of Copilot, Gemini and NotebookLM, available via a web browser, must not be used for University activities and purposes as they do not guarantee a sufficient level of information security or confidentiality. Please remember the Acceptable Use Policy (AUP) continues to apply, including its compliance monitoring and enforcement provisions, when using GenAI tools and staff are reminded of their obligation to abide by its terms. In all circumstances, staff are expected to exercise caution and use their judgement in their use of GenAI. Benefits Many potential benefits of using GenAI tools are already apparent, and the University encourages all its staff to make the best use of the information services made available to them. Here is a brief list of the potential benefits of using GenAI tools in support of University administrative activities. Efficiency and productivity GenAI tools can quickly process a lot of information to produce a large amount of output, saving time that can be spent on other tasks, thus boosting efficiency and productivity. Flexibility GenAI can create content in various formats, styles and languages, making it useful in a wide range of circumstances. For example, it could be used to generate drafts of meeting minutes, letters, press releases, social media posts, and other forms of documentation produced in the course of University business. That flexibility also allows the University to engage with different audiences across various platforms. In some circumstances, it may be appropriate and beneficial to use it to produce personalised content. Creativity GenAI can produce novel or unusual content from existing source material, making it a useful tool for the initial part of some creative tasks. For example, it could be used to draft materials that could form part of a marketing campaign. Understanding GenAI doesn’t just have to be used for content production and creation. It could be used to discover and summarise vast amounts of information in more digestible formats, and so it can be a valuable tool in the early stages of research undertaken to support administrative tasks. Risks There are, however, significant legal and reputational risks associated with use of GenAI tools, which can be broadly categorised as follows: - Bias, misinformation and inaccuracy - Data protection law non-compliance - Intellectual property and copyright law non-compliance - AI legislation non-compliance - Reputational damage and other risks This list is not exhaustive, given the overlapping nature of risk categories and the pace of AI development. Staff must consider relevant risks, and whether they are applicable to the circumstances in which they are considering use of GenAI, before any use of GenAI is initiated. Risk: Bias, misinformation and inaccuracy Much GenAI is trained to produce outputs based on information and patterns extracted from data in the public domain. Some of that data will be inaccurate because it is erroneous or obsolete, and some of it will be opinion. Consequently, outputs will sometimes be factually inaccurate or reflect the ignorance, biases or prejudices of individuals or groups in society. GenAI can also be manipulated to deliberately produce biased or inaccurate outputs, presented as fact. Unlike human intelligence, AI does not have the capacity to apply judgement or understand context. It cannot apply moral or critical perspectives. Additionally, there is an inherent risk that the ongoing use of GenAI tools will create and sustain feedback loops, whereby GenAI tools will be trained on text outputs generated by other GenAI tools, further reinforcing existing biases and inaccuracies. In practical terms, that means some outputs will be inaccurate or unbalanced regardless of the phrasing of the text prompt, because the source material is inaccurate or unbalanced. Some output may also be inaccurate because the GenAI tool is ‘hallucinating’ – creating nonsensical or inaccurate outputs that are not directly attributable to the source material. For those reasons, it is important that any GenAI output is thoroughly evaluated by a human being before it is utilised for any purpose. This is especially important where there is the risk of an adverse impact on a group or individual, or the potential for infringement of a person’s rights (e.g. as defined under the Equality Act 2010, the Human Rights Act 1998 or any other relevant legislation). Risk mitigation(s): Ensure that all GenAI outputs are thoroughly evaluated by a human being before they are used. Ensure use of GenAI is acknowledged if it is used to make a significant and unrevised contribution to a substantive or impactful piece of work such as the production of content for formal policies or strategic reports. Risk: data protection law non-compliance GenAI tools and their use are subject to existing laws and regulations and any University policy relevant to their use. This includes data protection laws such as the UK GDPR, the Data Protection Act 2018, the Data (Use and Access) Act 2025 and the University Data Protection Policy. As with the use of other information tools and services, it is important to use licensed versions of tools paid for from a University budget and procured through any applicable procurement process. (Free, unlicensed information tools and services often rely upon intrusive data processing and/or selling as part of their business model.) The University’s standard licensed GenAI tools are Copilot, Gemini and NotebookLM, and these are the tools that should be used to process personal data, where necessary, for which the University is responsible. This ensures that technical, operational and legal safeguards are in place, which protect any personal data that the University controls or otherwise processes. By contrast, inputting data into a free or unlicensed GenAI tool could be considered equivalent to putting it into the public domain – signifying a potential personal data breach. Information input into GenAI tools is also often used to train those tools, which may not be a lawful use of personal data – especially if that data cannot be retrieved or deleted, for example from an AI neural network. Data input into the University’s licensed versions of Copilot, Gemini and NotebookLM is not used to train those tools. It is particularly important to be cautious about inputting sensitive personal information (special category data) such as medical information into GenAI tools. Processing of such information is subject to additional safeguards, and misuse could represent a serious breach of data protection law and/or a breach of confidentiality. Regardless of the type of information you wish to input into a GenAI, you must consider the task you are using it to support. Data must be collected, held and used for only that purpose – for example, as part of a governance process – and any use of AI must be compatible with that reason. With some exceptions (e.g. for academic research), it is not appropriate to use personal data that was collected for a different purpose to do something else with a GenAI tool. It is also important to be mindful of ‘automated decision making’. Automated decision making involves: - making a decision that will affect a person solely by automated means without any human involvement; or - profiling someone – automated processing of personal data to evaluate certain things about an individual that could be used as part of a decision-making process. A common example of automated decision making is a credit check conducted exclusively using AI to decide whether to provide someone with a personal loan. While the use of GenAI to produce text or digital imagery would not necessarily result in a decision being made about an individual, it is not inconceivable that the use of such technology could be used as part of an evaluation process. For example, to review an application for a parking permit to ensure the person applying meets the eligibility criteria. In such circumstances, it is imperative that a human being is ultimately involved in the decision-making process. If after careful consideration you decide to use a GenAI tool, you must tell the affected people that you’re going to do that. That doesn’t mean you must seek consent on a case-by-case basis, but it will mean that relevant privacy notices should be provided or updated. Risk mitigation(s): Be cautious about inputting personal data into GenAI tools, especially sensitive personal data, and only do so where warranted. Do not use free GenAI tools. Use the University’s licensed versions of Copilot, Gemini or NotebookLM. Deploy relevant privacy notices. Risk: intellectual property and copyright non-compliance It has been argued by some affected parties that the entire basis for training GenAI tools through publicly available data is a violation of intellectual property rights and copyright law. There are a series of ongoing and well-publicised copyright cases where high profile individuals and organisations have sued companies that own and operate GenAI. Bearing that in mind, it is important to consider the nature of the content being input into any GenAI tool and whether the University has the right to input that information into that GenAI tool. It is also important that GenAI outputs are thoroughly checked by a human being and cited where appropriate. Risk mitigation(s): Consider whether it is appropriate to input material into GenAI tools. Cite outputs where appropriate. Use the University’s licensed versions of Copilot, Gemini or NotebookLM. Risk: AI legislation non-compliance In March 2024, the European Union (EU) introduced new laws that require organisations using AI in the EU to employ a risk-based approach to their use of AI, especially with regard to the use of personal information. It incrementally started to take effect from February 2025, and non-compliance with the legislation could result in penalties from European regulators. It affects the University where it is processing EU citizens’ data using AI. Risk mitigation(s): Exercise caution and judgement regarding deployment of GenAI to process EU citizens’ data. Document any use of GenAI tools in these circumstances. Risk: Reputational damage and other risks As outlined above, there are various legal risks posed by the use of GenAI, all of which could result in reputational damage to the University. There is also an environmental cost associated to use of GenAI: training GenAI tools requires vast amounts of power and indirectly generates enormous amounts of carbon, meaning there is a sustainability consideration to its use. In the development of some GenAI tools, outputs are checked and refined in a process known as Reinforcement Learning from Human Feedback (RLHF). That process includes human reviewers, often working in countries in the global south for very low wages, routinely viewing objectionable and distasteful materials, and has been reported to have a profoundly negative impact on the health and well-being of many of those workers. University staff will also be expected to provide human oversight of GenAI outputs. Whilst they would not ordinarily be exposed to objectionable nor distasteful materials in the course of administrative work, it is important to consider the risk to University staff wellbeing that could be posed by increased workloads and unrealistic expectations of what can be reasonably achieved using GenAI tools. Risk mitigation(s): Consider the wider impact on the University’s reputation before using GenAI. Consider any other relevant risks. Best practice: practical examples Here are a series of practical examples intended to show both best practice and scenarios in which the use of AI should be considered carefully. It remains important to bear in mind the general risks and benefits associated with use of GenAI in these different contexts. Example 1: Using GenAI for background research Capability: GenAI can be used as a research tool to help gather background information on a topic relating to something you are unfamiliar with. Example scenario: Using GenAI to provide an overview of a new piece of legislation that may affect your work at the University. Good practice: Using the University’s licensed versions of Copilot, Gemini or NotebookLM. Not inputting any personal or confidential information into Mthe University’s licensed versions of Copilot, Gemini or NotebookLM, because it is not required to understand the new legislation. Bad practice: Using an unlicensed GenAI tool. Inputting confidential data into that unlicensed AI tool with the aim of further understanding the legislation, thus committing a personal data breach and/or breach of confidentiality. Example 2: Using GenAI to summarise information Capability: GenAI can be used to summarise information. Example scenario: Using GenAI to prepare a briefing on a University project for a meeting with a commercial partner. Good practice: Using the University’s licensed versions of Copilot, Gemini or NotebookLM. Treating the output as a draft and amending it as appropriate. Thoroughly checking the output to ensure it is factually accurate and unbiased, does not reveal anything confidential to the commercial partner and is reflective of the source material. Acknowledging GenAI has been used to help create the briefing if it has not been materially altered as part of the fact-checking or drafting process. Bad practice: Using an unlicensed GenAI tool. Treating the output as a final draft. Accepting the output as factually accurate and suitable for sharing with a third party and not bothering to check it before presenting it to the commercial partner. Failing to mention it has been created using a GenAI tool. Example 3: Using GenAI to draft a document Capability: GenAI has the ability to produce written outputs in various styles and formats. Example scenario: Using GenAI to create meeting minutes. Good practice: Considering whether use of GenAI is appropriate in these circumstances – this will depend on what the meeting is about. Considering whether the document is likely to contain sensitive information. If the document is likely to contain sensitive information, considering the type of sensitive information, and whether use of GenAI is warranted. If it is appropriate to use a GenAI tool, uusing the University’s licensed versions of Copilot, Gemini or NotebookLM, and ensuring unauthorised AI note-taking bots are prevented from joining the meeting. Using the output as a draft and amending it as appropriate. Bad practice: Using an unlicensed GenAI tool. Inputting confidential or sensitive data into that unlicensed GenAI tool thus committing a personal data breach and/or breach of confidentiality. Failing to follow UIS advice on preventing unauthorised AI note-taking bots from joining your Teams meeting. Example 4: Using GenAI for numerical analysis Capability: GenAI can perform numerical analysis. Example scenario: Using GenAI to analyse the statistical results of a staff survey. Good practice: Considering whether the raw survey data contains personal or sensitive information. If it is appropriate to deploy a GenAI tool, using the University’s licensed versions of Copilot, Gemini or NotebookLM. Telling staff that AI will be used to analyse responses when they are choosing whether they wish to participate. Treating the output as a draft and verifying and amending it as appropriate. Bad practice: Using an unlicensed GenAI tool. Not telling staff that GenAI will be used to analyse their responses. Accepting the output as factually accurate and making an unquestioning decision based on the analysis. Copilot, Gemini and NotebookLM: Useful Facts This section contains a few useful facts that may assist staff in using the University’s licensed GenAI tools. Copilot Here are some tips for using Copilot: - The version of Copilot accessible to most University MS365 users is called “Microsoft 365 Copilot”. A more comprehensive version of Copilot is available called “Copilot for Microsoft 365”, and a licence for its use can be purchased by contacting UIS. - When accessing Microsoft 365 Copilot, you can check whether you are logged into your University MS365 account by viewing the top right-hand corner of your window – you will be able to see your initials (and your name if you click on the initials) if you are logged in. - When attaching documents, these will be automatically saved in a folder called ‘Microsoft Copilot Chat Files’ in your University MS365 account OneDrive. - Delete chat files that are no longer required. - Delete files uploaded into OneDrive as part of the chat process when no longer required. - There is more information regarding OneDrive on the UIS website. Gemini Here are some tips for using Gemini: - When accessing Google Gemini, you can check whether you are logged into your University account by viewing the top right-hand corner of your window – you will be able to see the University of Cambridge logo and one of your initials. - Standard users cannot delete conversations. These can only be deleted by UIS administrators. Consider whether using Copilot would be more appropriate in circumstances where you need or wish to delete any conversations with Gemini. NotebookLM Here are some tips for using NotebookLM: - When accessing Google NotebookLM, you can check whether you are logged into your University account by viewing the top right-hand corner of your window – you will be able to see one of your initials. - Delete notebooks that are no longer required. Further reading on best practice with use of GenAI University resources: - Admissions: AI and undergraduate applications - Communications: Generative AI tools guidelines - Education: Blended Learning Service – AI and Education - Education: Resources for use of AI in education and operations - UIS: Copilot - UIS: Google Gemini - UIS: Google NotebookLM - UIS: Guidance on information security (including policies and data classification) - UIS: LinkedIn Learning at the University of Cambridge (type in ‘GenAI’ when logged in) External resources: - ICO: Guidance and resources on data protection and AI - ISO: ISO - Artificial intelligence - JISC: An introduction to copyright law and practice in education, and the concerns arising in the context of GenerativeAI - GOV.UK: AI Playbook for the UK Government - National Cyber Security Centre: AI and cyber security: what you need to know - OECD: AI Principles Overview Authorship This guidance was composed without the use of AI.</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4109</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
         </is>
       </c>
     </row>
@@ -510,6 +536,19 @@
           <t>Guidance on how you might engage with Generative AI (GenAI) in your assessments effectively and ethically. GenAI is a technique in artificial intelligence in which outputs such as text, images, code, music, and video are generated by software. GenAI is potentially transformative as well as disruptive, and GenAI tools will feature in many academic and professional workplaces. Rather than seek to prohibit your use of them, we will support you in using them effectively, ethically and transparently. However, it may not always be appropriate to use GenAI. Whilst they are attractively powerful and easy to use, GenAI tools can provide misleading or incorrect information. They can also negatively impact your learning by reducing the need for critical engagement that is key to deep and meaningful learning. Additionally, you need to be aware of the difference between reasonable use of such tools, and at what point their use might be regarded as giving you an unfair advantage. Visit the Generative AI Hub For more details on how GenAI works, the ethical implications and limitations of the tools and the ways in which you can use them, please visit the Generative AI Hub. The Generative AI and Academic Skills Moodle course provides a more in-depth look at GenAI in an academic context. GenAI and academic integrity Academic misconduct is strictly prohibited, including the use of essay mills, homework help sites, plagiarism, collusion, falsification, impersonation or any other action which might give me an unfair advantage. An unfair advantage is: • when you hide something and aren't transparent about your approach. • when you take something directly from someone (or something) else and don't reference or acknowledge it. • when you don't follow the assessment guidance. It is not acceptable to use GenAI tools to write your entire assessment and present this as your own work. Words and ideas from GenAI tools are making use of other human authors' ideas without referencing them, which is considered by many to be a form of plagiarism. Using GenAI tools to check your grammar or spelling is usually appropriate if the tool is not rewriting a large proportion of your work. Similarly, tasks such as ideas generation or planning may be an appropriate use. For all assessments, your context and the nature of the assessment must be considered. Your teachers will give guidance on: • what ways (if at all) you are permitted to use GenAI. • which aspects of your work it is appropriate (or even expected) that you use GenAI for. If you are unsure about what constitutes acceptable use of GenAI in an assessment, ask for clarification from the module leader. If no explicit instructions are given, the default for assessments should be that you use GenAI in an assistive role while making sure that the final submission is still substantially your own work. Staff resources on how to guide students on the use of GenAI in assessments can be found on the Generative AI Hub. Category 2 describes in more detail how GenAI might be used in an assistive role. UCL does not use GenAI detectors when marking. Instead, if a marker has any concerns about your work, they may speak to you to get more information. You should not automatically assume this means that they suspect you of academic misconduct. Inappropriate use of GenAI is viewed as plagiarism. This is defined as the representation of other people’s work or ideas as your own without appropriate referencing or acknowledgement. This includes the use of GenAI tools that exceeds that permitted in the assessment brief. If teaching staff suspect that you are trying to pass off GenAI output as your own work then the regulations in the Academic Manual (9.2.5 a), 9.2.5 e) iii, and 9.2.6 c) may apply. You may be invited to an investigatory viva to probe the authorship of your work. How to acknowledge GenAI use in your work You should acknowledge GenAI use where it has been used to assist in the process of creating your work. The Library Skills pages share guidance on how and when to acknowledge GenAI in your work.</t>
         </is>
       </c>
+      <c r="D4" t="n">
+        <v>684</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -527,6 +566,19 @@
           <t>About Generative AI Generative AI tools automatically create content, including text, code, images, and more, based on user prompts. Examples include ChatGPT, Google Gemini, and Microsoft Copilot. Imperial has also launched the dAIsy platform. Text-focused tools are known as Large Language Models (LLMs) and use collections of existing data to predict outputs. They offer rapid content generation but can produce unreliable outputs, making them unsuitable for unverified academic use. Appropriate academic use of generative AI - Consider use of AI outputs as a starting point for research only and rely on academic sources such as databases and peer-reviewed sources. Developing critical thinking and evaluation skills is a key aspect of your education at Imperial. - If you use generative AI as a search tool, be sure to verify all information and cite any material you use for academic purposes. - Guard against AI “hallucinations” by fact-checking every statement before use. - Preserve your own voice in written work - uncritical AI use often yields generic, superficial text lacking true insight and will not demonstrate learning or substantial communication. - For support in developing your academic and scientific writing, consult Imperial’s Centre for Academic English guidance on GenAI and access the support they provide. Imperial guidance and support - Review your department’s current policy on using and disclosing generative AI in academic work. - Consult your Subject Librarian and library resources for advice on evaluating and selecting scholarly sources. - Refer to the guidance below as well as the library’s reference management pages for acknowledgement and referencing guidance. - Unless explicitly authorised, using AI to create assessed work may be treated as an offence such as contract cheating under Imperial’s Plagiarism, Academic Integrity &amp; Exam Offences regulations. - Familiarise yourself with Imperial’s Academic Misconduct Policy for rules on appropriate AI usage. Acknowledging and referencing use of generative AI tools Acknowledging A statement of acknowledgment shows the reader which AI tool you used and for what specific purpose. You should include a statement to acknowledge your use of generative AI tools for all assessed work, in accordance with guidelines from your department or course team. This statement should be written in complete sentences and include the following information: - Name and version of the generative AI tool e.g. Copilot, ChatGPT-5 - Publisher (name of company that provides the AI system) e.g. Microsoft, OpenAI - URL of the AI tool - Brief description (single sentence) of the way in which the tool was used (e.g. summarising notes, generating outlines) - Confirmation that the work is your own Example: I acknowledge the use of ChatGPT-5 (OpenAI, https://chatgpt.com) to generate an outline for background study. I confirm that no content generated by AI has been presented as my own work. Further requirements may be stipulated for a particular piece of assessed work where AI tools are allowed or required. This must be made clear to students when it is set. If unclear, please clarify with your module leader. Additional requirements may include expanded description in the ‘Acknowledgements’ or ‘Methods’ section, such as: - If relevant, the prompt(s) used to generate a response in the AI system. - The date the output was generated. - The output obtained (e.g. a ‘link to chat’ if ChatGPT, or a compilation of all output generated as an appendix). - How the output was changed for use or incorporation into a piece of work (e.g. a tracked-changes document or a descriptive paragraph). Referencing Referencing guidance is provided for Harvard and Vancouver referencing styles on the following pages: Your reference list and bibliography – Harvard Your reference list and bibliography – Vancouver</t>
         </is>
       </c>
+      <c r="D5" t="n">
+        <v>601</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -544,6 +596,19 @@
           <t>General guidance for all students on using generative AI tools in your studies. The University trusts you to act with integrity in your use of generative AI for your studies.It does not ban the use of generative AI, though its use is restricted for assessment. Some of your courses may also restrict its use in other ways. Always check your course level guidance.These top-level guidelines provide clarity on which uses of generative AI are strictly prohibited and constitute academic misconductThey also explain why you should be cautious about over-reliance on generative AI for your learning.This guidance is general and sets out the basics of the University’s position – it is essential that you also check the detailed information provided for each of your courses.Generative AI at EdinburghThe University recognises that developing skills in the responsible use of generative AI is important and will likely be significant for your future life and work. It also recognises that there are times when you may want – or be asked – to use it in your current studies. We want to ensure that you have the knowledge and skills to thrive in a changing world, and we recognise that generative AI can be used creatively, critically and with integrity.These guidelines are general to the whole University. It is important that you are aware that each course will have its own, more detailed, guidance. You should always check your course documentation on this, and speak to your Course Organiser if you are unsure.The University trusts you as students to act responsibly in relation to the use of generative AI. It also recognises that you need clarity on when its use breaches the University’s rules on academic misconduct. These guidelines provide you with this clarity. Unacceptable uses of generative AI for assessmentPassing off someone – or something’s – work as your own for an assessment is academic misconduct. This could be failing to cite a source you have used in piece of assessed work, getting someone else to complete an assessment for you, claiming authorship of machine-generated content or presenting machine-translated work as your own.If you submit a piece of work for assessment that is not your own original work you risk being investigated according to the university’s academic misconduct investigation procedures. This could have serious implications for you and your studies.The following uses of generative AI are not acceptable and constitute misconduct: if you use them you risk investigation and penalties.Presenting AI outputs as your own, original work.Use of an AI translator to convert assessments to English before submission: English is the language of teaching and assessment at Edinburgh – machine translation is treated as false authorship and is not acceptable.Submitting an assessment which includes elements of AI-generated text without acknowledgment.Submitting an assessment which includes AI-generated images, audio or video without acknowledgment.Submitting an assessment which includes AI-generated mathematical formulae or reasoning, or computer code, without acknowledgment.Citing AI-found sources without reading and verifying them.For more detailed information about the restrictions around using AI-supported online proofing tools, please see the University’s Guidance on Proofreading of Student Assessments. Using generative AI to support your learningWhile we have these clear restrictions around the use of generative AI in your assessed work, the University understands that there are ways in which you may wish to use it to support your studies. This might include using it to:brainstorm ideasget quick definitions of conceptsovercome writer’s block through dialoguecheck your grammarorganise or summarise informationre-format your referencesSome courses may encourage or even require you to use it in certain ways, while others may ask you not to use it at all. Again, it is important that you check your course-level guidance on this. Reasons to be cautious about your use of generative AIYou should be aware that there are risks and disadvantages associated with over-use of generative AI to support learning. Cognitive offloadingThere is growing research evidence that over-use of generative AI can negatively affect your learning. You may want to look at studies which raise concern over how ‘cognitive offloading’, ‘metacognitive laziness’ and reduction in capacity for critical thinking may be associated with over-reliance on this technology. If you routinely use generative AI for breaking down and summarising long texts, for example, you will not be developing your own critical skills in the analysis of complex documents. You will also not be practicing and learning how to bring together complex ideas using the power of your own intelligence. Similarly, if you are using it to regularly assist with mathematical reasoning or coding, you are undermining your own ability to learn and become expert at doing this yourself. To make the most of your time at university, embracing the hard work of learning is a better approach than looking for short-cuts. Bias and inaccuracyGenerative AI models are not ‘intelligent’ in the way that humans are intelligent. They have been trained on more text than a human could ever read, but have different capabilities and make different mistakes. While their output often appears convincing and reliable, their behaviour is strongly influenced by the data they are trained on, so they can perpetuate harmful biases, fabricate information and make errors. You will be held accountable for these errors and biases if you include them in assessed work. Higher education should help you develop advanced knowledge which is creative and rigorous, not generic and unreliable. It is best to use your time at university to develop high-level skills that are going to help you throughout life – original thought, engaging writing, critical use of evidence, creative risk-taking and innovation. Using the University’s own generative AI platform (ELM)All University of Edinburgh students have free access to ELM, which offers you a secure gateway to a range of generative AI models. The university encourages you to use ELM over other platforms such as GPT, DeepSeek, Grok etc for the following reasons:In ELM your data is secure – it will not be retained by third party services to train their models or for any other purpose.It is free to use for all staff and students, providing the same access for all and saving you money.ELM provides access to a range of language models including a locally-hosted instance of Llama. This has an optimized architecture that can achieve faster response times and reduced power consumption. You can also choose other models such as GPT within ELM if necessary for your task.Your lecturers do not have access to your chat history in ELM for the purposes of 'checking' your work - like your email account, it is private to you.You can access ELM and find out about training opportunities here. Acknowledging your use of AIIf you choose to use generative AI for aspects of an assessment, it is important to be transparent about how you have done so. You should include a brief acknowledgment at the end of your piece of work, for example:I used OpenAI o4 Mini via ELM to check grammar and spelling throughout my assignment. I also used the Create Image function in ChatGPT to generate the image on page 2.Again – check the detail in your course guidance if you are unsure what is required, as there may be specific things your Course Organiser would like you to cover in your acknowledgment. Citing your use of generative AIIf you use content generated by AI within your work, for example an AI-generated image or text from an AI chatbot, you will need to reference it. This means including an in-text citation or footnote in the body of your work, and a corresponding reference in your reference list. The Library’s guide to using generative AI gives very useful guidance on this. Environmental and social impact of generative AIMany in our community are concerned about the negative impacts of generative AI in areas such as:Energy and resource useExploitative labour practicesIntellectual propertyYou may wish to read more about these via the links above. While there are ongoing efforts to reduce the environmental impact of the datacentres that make AI models work, it is clear that use of generative AI has a higher impact than, for example, a simple web search. If you are concerned about this, consider using the locally-hosted instance of Llama in ELM (see above). It is more efficient in terms of resource use, and provides a more transparent alternative to OpenAI, meaning that it is easier for the university to measure and manage its power consumption.You might also try to limit use of generative AI to purposeful rather than casual use. Links to other sourcesPrinciplesEdinburgh Student Assembly principles on the use of generative AIRussell Group principles on generative AI use in education Further guidanceGenerative AI use for Postgraduate Research studentsLibrary guide to using generative AI in academic work TrainingUniversity of Edinburgh Digital Skills Programme Academic misconduct guidanceFurther guidance on academic misconduct (including plagiarism) and how to avoid itUniversity of Edinburgh Academic Misconduct Procedures Return to ELM main page This article was published on 2025-07-23</t>
         </is>
       </c>
+      <c r="D6" t="n">
+        <v>1486</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -561,6 +626,19 @@
           <t>University of Glasgow - MyGlasgow - not found Skip to main content Cookies We use cookies to improve user experience and allow for personalised advertising via third parties. You can find out more about cookies and how we use them on our privacy policy page . Analytics I'm happy with analytics data being recorded I do not want analytics data recorded Please choose your analytics preference Personalised advertising I’m happy to get personalised ads I do not want personalised ads Please choose your personalised ads preference save choices accept all privacy settings accept We use cookies Necessary cookies Necessary cookies enable core functionality. The website cannot function properly without these cookies, and can only be disabled by changing your browser preferences. Analytics cookies Analytical cookies help us improve our website. We use Google Analytics. All data is anonymised. Switch analytics ON OFF Clarity Clarity helps us to understand our users’ behaviour by visually representing their clicks, taps and scrolling. All data is anonymised. Switch clarity ON OFF Privacy policy close search Staff login Student login Staff a-z MyGlasgow MyGlasgow not found MyGlasgow Students MyGlasgow Staff IT Sport Not found The web page or resource you requested could not be found. Check that you have the right address, or: Go to MyGlasgow Students homepage Go to MyGlasgow Staff homepage Try searching MyGlasgow Search MyGlasgow search</t>
         </is>
       </c>
+      <c r="D7" t="n">
+        <v>224</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -578,6 +656,19 @@
           <t>Artificial Intelligence (AI) Guidance - Key Information for Students (1) Our approach to Artificial Intelligence (AI) Warwick Law School is committed to developing a holistic approach to AI in all aspects of our education. We seek to develop AI literacy among our students to instil good practice regarding the responsible use of AI as a tool to assist (but not replace) their learning and skills development. This includes promoting awareness about the ethical use of AI as well as about the concerns over the robustness and bias of many AI systems. We will monitor the use of AI by students to ensure that this is done responsibly and ethically. This includes monitoring the impact the use of AI has on development of essential academic skills by our students. Academic integrity must be ensured in all activities involving the use of AI. We are committed to understanding the implications of AI for our own subjects as well as the ethical issues raised in all aspects of AI and to ensurin that what we teach includes consideration of the legal and ethical challenges brought about by the use of AI. (2) Artificial Intelligence (AI) (a) AI Technologies Artificial Intelligence is an umbrella term covering a wide range of algorithmic and data-driven software systems. There are different types of algorithms (and combinations of different approaches) with varying capabilities, either of a deterministic or adaptive machine-learning type. AI performs a wide variety of tasks, not always clearly identified as “AI” in people’s minds (e.g., spell-checkers, auto-complete, recommendations on shopping websites or streaming services, etc). The Organisation for Economic Co-operation and Development (OECD) defines an AI system as “a machine-based system that, for explicit or implicit objectives, infers, from the input it receives, how to generate outputs such as predictions, content, recommendations, or decisions that can influence physical or virtual environments. Different AI systems vary in their levels of autonomy and adaptiveness after deployment”.[1] All AI systems have in common that they offer varying degrees of automation for particular tasks, often more efficiently and quicker than humans. A particular sub-category of AI is Generative AI Systems (“GenAI”). They can be useful for some academic tasks, but can also be misused in a way that violates our standards and expectations as to academic integrity. GenAI, such as ChatGPT or Claude, is based on deep-learning neutral networks utilising “transformer” technology. They are trained on vast amounts of data and produces outputs based on that data. The robustness and reliability of outputs can vary dramatically, and there are many caveats to the use of generative AI systems. (b) Limitations of GenAI Importantly, AI does not process information in the way humans do. It does not develop knowledge. It lacks common sense and the ability to locate information in a wider context/experience. Its outputs are generally based on the data on which it was trained, and, in the case of “self-learning” (adaptive) algorithms, data acquired during deployment; it therefore lacks the ability to produce truly original and creative outputs. It does not have the ability for critical thinking – one of the key academic skills we seek to instil and develop in our students. AI can be a very useful tool to help with certain tasks. It can uncover connections in data that might not be apparent to humans (although it is at risk of overfitting, or “hallucinating”, such connections) and can structure data better and faster than humans. Recent advances in the performance and capability of certain AI systems, particularly generative AI systems, have renewed interest in this technology, and have led to an explosion in academic, policy and legislative work. A lot of unsubstantiated or exaggerated claims are made about AI, and it is sometimes difficult to get a clear sense of what the technology is capable of and what its limitations are. There are also concerns about the quality of the data on which AI systems are trained, particularly regarding its robustness and accuracy, and biases. Furthermore, the degree of energy use and the resulting environmental impact of the infrastructure (e.g., data centres) required for some AI systems is starting to attract more attention and concern. (3) Permitted and prohibited uses of GenAI and other AI tools in the classroom (4) Academic Integrity With regard to academic integrity, our policy builds on the University’s Institutional Approach to Artificial Intelligence and Academic Integrity. Any changes to the University’s Institutional Approach, or any new University policies on the use of AI take precedence over this policy whenever there is a conflict between them. In accordance with both the University’s and the Law School’s academic integrity policy, the Law School prohibits copying/paraphrasing either whole outputs or elements of outputs generated by a GenAI system and submitted by students as their own work. Similarly, the use of AI to complete certain parts of an assessment, such as analysis or evaluation, is not permitted. However, even where the use of GenAI systems is not prohibited, the Law School discourages the use of such outputs even with correct and complete attribution. Assessments should be used by students to demonstrate their knowledge of the subject (i.e., what has been taught, including set readings) and their understanding and ability to utilise this in responding to specific questions. The use of GenAI in this process might make it more difficult for markers to establish how well a student has demonstrated this. The way in which such outputs are used as part of an assessment will be considered in grading the assessment against our marking criteria. The use of an AI system for any aspect of completing an assessment must be disclosed by a student. A failure to do so constitutes an academic misconduct. Such a disclosure must cover the following points: - Why was a GenAI system used (help in understanding the question; help in structuring work based on arguments developed; assist with initial summary of readings etc)? - Which GenAI system or systems was/were used (e.g., ChatGPT, Claude etc)? - How has the AI output been used in preparing the assessment? (as a research tool, to test arguments etc; see table below for acceptable uses). The way AI generated outputs are used by you in drafting your assessments will be taken into account when grading the assessment against the generic grade descriptors and assessment-specific marking criteria. (5) Permitted and prohibited uses of GenAI – Guidance to Students Unless expressly required for a specific assessment task, Warwick Law School does not encourage the use of GenAI tools for assessments. Students should be aware that GenAI tools can weaken the quality of your work – particularly if you rely on GenAI for accuracy, relevance and rigour. You should be particularly mindful of the tendency of GenAI tools to cite non-existent resources or information (“hallucinations”). GenAI may generate inaccurate or otherwise poorly constructed arguments. GenAI does not have the ability to demonstrate critical thinking, nor the ability to be genuinely creative. Most importantly, assessments are there for you to demonstrate to us (and to yourself!) how well you have understood what you have studied. Nevertheless, WLS acknowledges that some students may use GenAI technology when preparing for assessments and writing essays, and may want to gain experience of utilising it for their future legal careers. Below, we provide a clear rule and interpretative guidance on what would constitute tolerated and prohibited use of GenAI. This is always subject to specific instructions given for each assessment. Rule and Guidance The key overarching rule is: GenAI can act as a personal assistant for you (e.g. assistance in understanding key issues, help with research, proof-reading your work etc.). However, it must never be used to create the work, or certain parts of the work, for you. You must not submit any AI-generated output as your own work. The table below summarises what is acceptable and what is prohibited in a bit more detail. Note that any use of GenAI may be prohibited for specific assessment tasks. This might be the case e.g., where the assessment tests your key legal or academic skills.Here, your own unaided work would be essential. Always check the assessment instructions before you use any GenAI tool! | YOU CAN | YOU MUST NOT | o Example prompt:“Is the following question asking for a discussion on topic X?” o Careful here! Do not simply ask GenAI to prepare an outline for you. Do your preliminary research and have your points ready. Even slight variations in the prompt can produce vastly different results as can repeating the same prompt twice or more. o Example prompt: “Suggest an outline for the essay I am going to write on the topic X. I will argue for/against Y and the points I will make in my essay are A, B and C. My supporting evidence/examples are D and E.” or “What would be the best order to argue for/against Y with the points A, B and C, and examples D and E?” o Example prompt: “Check the tone and style of this essay and highlight the parts that need to be rewritten, but do not rewrite them!” ·Use GenAI as a search engine/database to find further sources. o Careful here! GenAI tools may sometimes generate sources that do not exist. Always remember to check that the source exists; that the reference/citation is accurate ( check books and journals though the library pages; check case databases for cases); verify that any quotations were taken from the indicated source etc. o Example prompt: “Provide some feedback on the consistency of the arguments made in the project, without rewriting it for me.” o Please remember that GenAI feedback may not reflect the assessment criteria. It’s important to refer to the module's assessment criteria to fully understand the expectations. | o Example prompt:“I need to write an essay, but I could not understand the question. Can you write me an essay on the following essay question: [the essay question].” o Example prompt: “I need to write an essay on the topic X, what should I argue, what should my stance be? Can you suggest some arguments I could use?” o You can only ask GenAI to provide guidance on the accuracy or validity of your arguments or improve the ideas you already have. Asking GenAI to generate ideas and arguments do not result in accurate or original supervised projects. Therefore, you must always double check what the GenAI tools suggest to you and never substitute them for your own voice. o Example prompt:“Provide some feedback on the following essay and rewrite the parts that need improvement.” or “Can you provide some feedback on the following essay?” (Careful here!GenAI tools usually tend to rewrite/revise the text you provide them, unless you clearly restrict them and/or prohibit them from rewriting the whole text in accordance with the feedback they provide. Therefore, even when you ask for feedback, you must ensure that it is you who makes the necessary changes depending on that feedback, not AI.) o Example prompt: “Check the tone and style of the following essay and make the necessary changes/improvements to make it sound more formal.” (You should only ask for suggestions or for some emphasis to be made on the parts that need improvement, you should never ask any GenAI tool to change the sentences you have written. Remember, it should entirely be your own work, GenAI should not and cannot be a contributing author!) |</t>
         </is>
       </c>
+      <c r="D8" t="n">
+        <v>1902</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -595,6 +686,19 @@
           <t>Using generative AI Understand where to use generative artificial intelligence (AI) appropriately for your studies and in preparation for your future. Go to: What is generative AI? | Generative AI and your studies | University of Nottingham policy | Further information Always check expectations for generative AI use and acknowledgement for any given module or assessment. What is generative AI? “Artificial intelligence, or AI, is technology that enables computers and machines to simulate human intelligence and problem-solving capabilities.” (IBM, 2024) Generative artificial intelligence is a form of AI technology that can produce text, images, and other media in response to user prompts. These tools (including ChatGPT and Microsoft Copilot) are not sentient - they only mimic intelligence, through algorithmic prediction and pattern recognition. Drawing on large quantities of data, these tools create outputs based on probability. It is important to remember that the responses provided by generative AI tools do not express meaning, understanding, or intentionality. As a result, responses generated by these tools cannot be relied upon to be accurate and always need to be fact-checked. Back to the top Generative AI and your studies The use of AI tools is becoming common practice across a variety of industries, which means that understanding how to use generative AI effectively and responsibly will likely be a key skill for employment. You might at times be asked to use AI within your studies, to help you develop skills relating to its effective, responsible, and professional use. For other assessments, use of generative AI may be prohibited, as the assessment is designed to develop your academic and transferable skills. Back to the top University of Nottingham policy Key points to remember Content created or significantly modified by generative AI, whether text, code, images, or video, should only be used if this is clearly stated to be essential or optional for an assessment task, and should always be fully evidenced and acknowledged. - Always consult your tutor or assessment documents on expectations for AI use - Always fact-check any information generated using AI - Always be transparent in acknowledging your use of generative AI, - Always keep records of your interactions with AI tools Back to the top Back to the top Continue your journey You may also be interested in: Further support Disability support service Language and communication skills</t>
         </is>
       </c>
+      <c r="D9" t="n">
+        <v>387</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -612,6 +716,19 @@
           <t>This is the current version of this document. You can provide feedback on this document to the document author - refer to the Status and Details on the document's navigation bar. Section 1 - Purpose (1) This Policy outlines the principles that support the responsible and ethical use of Artificial Intelligence (AI) at Macquarie University (the University), in alignment with the University’s purpose, values and strategic priorities. (2) This Policy ensures the consistent application of the eight principles that guide the responsible and ethical use of AI. Scope (3) This Policy applies to all Staff, Students and Affiliates of the University, encompassing all uses of Artificial Intelligence (AI) by these groups. Top of PageSection 2 - Policy (4) Artificial Intelligence (AI) has the potential to enhance teaching and learning, research, innovation and social impact at the University. However, AI also poses significant ethical, legal and social challenges that need to be addressed with care and responsibility. (5) The following eight principles outline the University’s expectations for the design and the responsible and ethical use of AI, which are informed by Australia’s AI Ethics Principles and the NSW Mandatory Ethical Principles for the use of AI: - Positive Impact: - AI should deliver positive results across research, education, and operations, supporting informed decision-making. Its use should align with the goal of delivering meaningful benefits compared to other available tools. - AI Literacy and Confidence: - The University will encourage AI literacy among Staff and Students, ensuring they can use AI tools responsibly and understand their broader implications in various contexts. - Academic and research integrity: - The University will build awareness among Students and Staff of their responsibilities around the use of AI tools. - The University will manage integrity-related risks posed by AI tools in accordance with the Academic Integrity Policy, the Assessment Policy and the Macquarie University Code for the Responsible Conduct of Research. - Fairness and Inclusivity: - AI tools and systems made available and authorised by the University for Students and Staff will be evaluated carefully before deployment to ensure that these do not unfairly discriminate against individuals or groups. - Diverse perspectives should be encouraged and included in AI development teams to ensure that systems are designed and deployed with a comprehensive understanding of potential impacts on different groups. - Engagement with Students, Staff and Affiliates should occur in order to understand needs and concerns relating to AI systems and to allow for feedback to be considered in the AI development process. - Privacy and Security: - The University will undertake regular assessments to ensure that the use of AI systems and tools does not compromise data security or intellectual property rights and complies with University policy, including the Privacy Policy, the Cyber Security Policy, the Data Breach Policy, the Intellectual Property Policy, and the AI Reference Architecture. - Accessibility and Equity: - The University will work to eliminate barriers and aim to ensure that appropriate AI systems and tools are available regardless of financial or personal circumstances. - Human Oversight and Responsibility: - The University is responsible for those AI tools and systems made available and authorised by the University to Staff, Students and Affiliates (Users). - For AI tools and systems supporting staff decision-making, the final decision-making authority resides with qualified staff who can validate or override AI outputs, particularly in high-risk contexts. - Users of AI systems and tools are responsible for any generated output used for work, research or study purposes. - The University will establish clear reporting processes for concerns about AI tools and systems provided by the University. - Users of AI tools and systems provided by the University must use these for their intended purpose and in accordance with the Acceptable Use of IT Resources Policy. - A risk assessment will be conducted by the Head of AI prior to the implementation of an AI system to identify potential risks and measures to mitigate these risks in accordance with the Risk Management Policy, and in compliance with the AI Reference Architecture. - Continuous Review and Improvement: - The University will regularly review its AI Policy (and any related procedures) and update as necessary to meet evolving needs and maintain ethical standards. (6) If a Student or Staff member is alleged to have used Generative AI in a manner that is inconsistent with the principles of this Policy, the University may investigate the allegation in accordance the relevant policy (i.e. Academic Integrity Policy, Staff Code of Conduct, Macquarie University Code for the Responsible Conduct of Research, Acceptable Use of IT Resources Policy). Top of PageSection 3 - Procedures (7) Nil. Top of PageSection 4 - Guidelines (8) Nil. Top of PageSection 5 - Definitions (9) The following definitions apply for the purpose of this Policy: - Affiliates refers to contractors, agents, honorary, clinical or adjunct appointees and consultants of the University. - AI has the meaning provided in the NSW AI Assurance Framework, being “intelligent technology, programs and the use of advanced computing Algorithms that can augment decision-making by identifying meaningful patterns in data”. - Deep Learning is a subset of machine learning that uses advanced neural networks to simulate human cognitive processes, enabling the handling of complex tasks. - Generative Artificial Intelligence (Gen AI) is subset of Deep Learning and a wide-ranging term that refers to any form of artificial intelligence capable of generating new content, such as text, images, video, audio or code (New South Wales Government’s Generative AI: Basic Guidance). - Machine Learning refers to systems that use advanced algorithms to learn from historical data and improve performance over time. - Staff means all persons employed by the University, including continuing, fixed term and casual Staff members. - Student means a person currently enrolled in a unit of study or program at the University.</t>
         </is>
       </c>
+      <c r="D10" t="n">
+        <v>967</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -629,6 +746,19 @@
           <t>Students will be equipped to use generative AI responsibly in their education and future careers under the sector-leading new assessment policy at the University of Sydney. From Semester 1 2025, the University will change its default to allow the use of AI for assessments, except for exams and in-semester tests or if teaching staff choose not to. From Semester 2, the University will move to a realistic and forward-looking ‘two-lane approach’ to assessments comprising: Students will be required to apply critical thinking and analysis to produce original work aided by appropriate learning tools, including acknowledging how they use AI. Professor Joanne Wright, Deputy Vice-Chancellor (Education), said the University of Sydney is leading the way in integrating modern AI technologies within education. “This is a substantial change to our teaching, assessment and program design, and it is absolutely necessary to ensure our graduates are equipped with the tools they need for the modern workforce. “Generative AI has already had a profound impact on workplaces and our graduates are expected to demonstrate skilled use of the relevant tools in job interviews. The changes we’re making to teaching and assessments ensures we are preparing students for their careers, without compromising their learning or the integrity of our world-class education.” Two academics from the University of Sydney were recently asked by TEQSA, the national quality assurance and regulatory agency, to show the risks and opportunities of AI in assessment. The resulting videos reveal just how easy it is for a novice to complete many traditional assessments, and equally how helpful AI can be to accelerate learning and enhance productivity. Professor Adam Bridgeman, Pro Vice-Chancellor (Educational Innovation), said universities have needed to adapt rapidly to the significant advancement in the capability of generative AI tools over the past two years. “It’s no secret that any take-home assessment can be completed to a high level by AI, and it’s not practical, enforceable or desirable to implement a blanket ban on these tools, or even to restrict their use. “We have worked closely with the regulator, educators and students to chart a way forward in a world where AI is ubiquitous and that satisfies the principles and purposes of higher education.” Training has been developed for staff to support the transition alongside workshops, resources and ongoing communications for students and staff. The changes are the latest in a range of University initiatives helping students and staff use generative AI equitably, effectively and ethically. These include a partnership with Microsoft to make the generative AI tool Copilot for Web available to students and staff for free, with regular training sessions. The University’s AI in Education Working Group of staff and students recently co-designed and launched a publicly available online guide AI in Education showing how generative AI can be used productively and responsibly in assessment and learning. The University has also developed an AI assistant for students called Cogniti, which allows teachers to create customised AI agents that can be steered with instructions and subject-specific information, answer students’ questions about content and syllabus, and provide instant personalised feedback, guidance and support, 24 hours a day. At Sydney, over 1000 Cogniti agents have been developed. Cogniti has won many awards and has been adopted by many other institutions in Australia and beyond. The University was named AI University of the Year in the 2024 Future Campus Awards, in recognition of its leadership in the field.</t>
         </is>
       </c>
+      <c r="D11" t="n">
+        <v>566</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -646,6 +776,19 @@
           <t>Using Artificial Intelligence (AI) in university Learn about our stance on Artificial Intelligence (AI) UNSW recognises there are ethical and responsible uses of AI and generative AI (GenAI) tools that can support student learning. AI can be a helpful tool for tasks, such as initial research, summarising information, data analysis and more. However, when it comes to completing independent research, coursework and assessments, it's important to ensure the work you produce is your own. The university adopts a firm approach to ensuring you complete the work that is expected and that this demonstrates you have met learning outcomes assigned within your courses. The degree to which you can use AI varies between faculties, programs and courses. Reach out to your course convenor, lecturer or tutor to understand the rules and expectations. Unsure about using AI in your work? When using AI in your assessment, a simple principle to remember is: If you are given permission and wish to use AI in the process of planning, designing, or writing your assessment, you should always clearly acknowledge this. Responsible use of Generative AI tools As an early adopter, UNSW supports and nurtures the ethical and responsible use of AI in research, learning, teaching, administration, and thought leadership. See our principles below on the ethical and responsible use of Artificial Intelligence at UNSW: - The use of AI systems at UNSW benefits UNSW, individuals, society, and the environment. - The use of AI systems at UNSW is equitable, and respectful of human rights, diversity, inclusivity, and accessibility. - AI systems and their lifecycle at UNSW are trustworthy and are used responsibly, safely, and reliably in accordance with their intended purpose. - The use of AI systems is transparent, and people understand when the AI system is engaging with or impacting them, the environment, and/or society. - AI systems and their lifecycle used at UNSW are identifiable, explainable, interpretable, accountable, and contestable. - AI systems and their lifecycle used at UNSW are secure and resilient. See also When using AI, remember to: - Check your course guidelines to see if the use of AI is permitted, including its usage as a translation tool. See the levels of AI assistance and what they entail - Maintain your academic integrity. Do not copy and paste AI-generated materials and claim them as your own. Learn how to reference AI in your assessments - Protect personal information. Do not include any personal or sensitive information in prompts, your own or other people's (i.e. addresses, name, emails, zID or intellectual property). For data privacy and protection, use Microsoft Copilot using your UNSW account - Verify accuracy of AI outputs. GenAI tools could produce invalid or unreliable information ('fabrications' or 'hallucinations'). Book an appointment with the Academic Skills team if you need guidance. Levels of AI assistance The Levels of AI Assistance framework is designed to help convenors communicate to students how much, or how little AI can be used in the process of planning, creating and producing an assignment. To ensure clarity in UNSW AI policy, and how to use AI responsibly in your assessments, we've created this resource for further guidance. Download the framework or read below. - This assessment is designed for you to complete without the use of any generative AI. You are not permitted to use any generative AI tools, software or service to search for or generate information or answers. - In completing this assessment, you are permitted to use standard editing and referencing functions in the software you use to complete your assessment (for example Microsoft Word, Mendeley, Zotero). You are not allowed to use any generative AI tools including prompts or features that generate text. Using functions that generate or paraphrase passages of text or other media, whether based on your own work or not, can be grounds for academic misconduct. - This category permits the use of generative AI as ‘inspiration’ for assessment. For example, generating initial ideas, structures, or outlines. Beyond that, the use of generative AI is prohibited. You are permitted to use generative AI tools, software or services to generate initial ideas, structures, or outlines only. After you've used generative AI for inspiration you must develop those ideas to produce your own work. - This category permits the use of generative AI as a 'coach'. Learning usually takes effort. In recognition of this, this category requires you to make a first attempt at the task yourself. Once this is done you can use generative AI to improve your submission. The focus is on your thoughts and creation with the AI helping you edit your work. The AI-based edit must be attributed, and this reinforces the responsible use of generative AI in a scholarly context. The degree of referencing or attribution may vary on the nature of the task – from general acknowledgement to full attribution of all editing suggestions. Your Convenor will specify the types of attribution required, as well as when generative AI tools can be used throughout the assessment. Keep copies of your drafts as your convenor may also request them as part of the submission If outputs of generative AI tools, software or services form part of your submission and are not appropriately attributed, your Convenor may ask you to explain your work. If you are unable to satisfactorily demonstrate your understanding of your submission and how you have done it you may be referred to UNSW Conduct &amp; Integrity Office for investigation for academic misconduct and possible penalties. - This assessment is designed for you to use generative AI as part of the assessed learning outcomes. Please refer to the assessment instructions for more details. This category expects a wide range of use of generative AI in assessment. Your convenor will specify what they want you to do with generative AI. This may include assessments where a first draft is generated by generative AI and you are asked to critique that draft; it may be an assessment where a particular generative AI tool is required to be used; or it may be an assessment where you have options to use or not use those tools. - This assessment would not likely require or benefit from the use of AI. However, if you do use it, it must be properly referenced. Frequently Asked Questions (FAQs) - Read your assessment instructions carefully to understand what level of AI use is permitted, and note that what is permitted will vary across different assessments. - At some points in your learning, it will be important to assess your understanding without the use of AI tools. - At other points, you may be assessed on how well you have learnt to use the tools. Your convenors will set the level of acceptable use of AI for each assessment based on course learning outcomes. - The unauthorised or unacknowledged use of AI in assessments is a form of cheating and is considered to be student misconduct at UNSW under the current Code of Conduct and Values. If you have been found to use AI in a manner that does not meet the course instructions, penalties may occur which would include a fail, a mark of zero for the course, suspension or permanent exclusion. - All academics marking assessments submitted through either Moodle Turnitin Assignment or Inspera now have access to Turnitin’s new AI detection tool. This provides academics with an estimated percentage of text that has similarities to AI-generated or AI-paraphrased text (text that was originally written by AI but then rewritten to avoid detection). The document will include highlights of the relevant passages that the detector has flagged. This is not always conclusive evidence that a student has inappropriately used generative AI, however, this will be a flag for a marker to further review a student’s submission. It’s important that students are aware of what tools use generative AI and may be inappropriate in an assessment. For example, Grammarly, Quillbot and translation tools such as Google Translate, DeepL and Baidu Translate are forms of generative AI. - When using AI tools, such as ChatGPT or Copilot, it's important to properly cite and credit use. Acknowledging the use of AI when you have used it helps ensure the honesty and integrity of your work. In cases where the use of AI has been prohibited, please respect this and be aware that where unauthorised use is detected, penalties may apply. - If you need help with your assessments, there are alternatives to unauthorised AI use. You can: - Seek support from your teacher if you’re under too much pressure or apply for Special Consideration if you’re eligible, or - Seek help from the Academic Skills Team by booking a consultation, attending a Study Hacks session, or exploring our toolkit to see our available resources. - Translation tools automatically convert text or speech from one language to another. Some popular tools include ChatGPT, Copilot, Google Translate and DeepL Translator. Acceptable use varies by course, so check assessment guidelines or consult teaching staff if you’re unsure. It is essential to create and express your own ideas in assessments. Misusing tools, such as copying outputs from ChatGPT and claiming them as your own, undermines your ability to demonstrate a genuine understanding of course material. Spelling and grammar checks, like those in Microsoft Word, are generally acceptable as they don’t alter the meaning of your work. However, verify suggested changes, as editing tools can unintentionally distort your understanding. Some programs, like Google Docs, include AI editing features that may generate or refine text. If AI tools such as ChatGPT or Grammarly are used where permitted, you must reference or acknowledge them. Keep draft versions of your work to show your process if concerns about validity arise. - UNSW acknowledges that these tools can sometimes support learning but warns that inappropriate use may hinder English language development. Many multilingual students note that translating writing into English can negatively affect learning and reduce originality. For example, dictating in one language and translating into English often results in AI-generated text that lacks nuance or fails to convey the intended meaning. Additionally, relying on translation tools may pose challenges if your work is flagged as AI-generated, requiring you to explain ideas that may not fully reflect your understanding. Always check assessment guidelines to confirm whether AI translation tools are permitted in your course. - If your Convenor has concerns that your submission contains passages of AI-generated text or media, you may be asked to have a conversation about your work. If you are unable to satisfactorily demonstrate your understanding of your submission, you may be referred to UNSW Conduct &amp; Integrity Office for investigation for academic misconduct and possible penalties. Have a question? If you have any questions about UNSW AI policy or referencing AI in university, we’re here to help.</t>
         </is>
       </c>
+      <c r="D12" t="n">
+        <v>1802</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -663,6 +806,19 @@
           <t>Page not found | Australian National University Skip to main content Page not found The requested page could not be found. We use cookies to improve your experience with ANU. For an optimal experience, we recommend enabling all cookies. The ANU Privacy Policy outlines how we handle your personal information - Read more Cookie settings Accept all Cookie Settings We recommend enabling all cookies to provide you with the optimal experience while visiting our website. Essential Cookies Always Active These cookies are required for basic site functionality and are always enabled. Analytics cookies are used to record anonymous site usage data. No personally identifiable data is collected. Marketing Cookies Marketing Cookies These cookies are set by a range of social media services that we have added to the site to enable you to share our content with your friends and networks. They are capable of tracking your browser across other sites and building up a profile of your interests. This may impact the content and messages you see on other websites you visit. If you do not allow these cookies you may not be able to use or see these sharing tools. Back Button Cookie List Search Icon Filter Icon Clear checkbox label label Apply Cancel Consent Leg.Interest checkbox label label checkbox label label checkbox label label Confirm my choices Your Privacy [`dialog closed`]</t>
         </is>
       </c>
+      <c r="D13" t="n">
+        <v>224</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -680,6 +836,19 @@
           <t>Page not found - my.UQ - University of Queensland Skip to menu Skip to content Skip to footer my.UQ Menu Page not found The requested page could not be found. We're sorry, but there is no web page that matches your entry. It is possible you typed the address incorrectly, or the page may no longer exist. You may wish to try another entry or choose from the links below, which we hope will help you find what you’re looking for. If you are certain that this URL is valid, please send us feedback about the broken link. You may wish to try one of the following links: my.UQ homepage UQ Search page UQ Homepage</t>
         </is>
       </c>
+      <c r="D14" t="n">
+        <v>115</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -694,7 +863,20 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>On this page AI Statement of Intent | Purpose | Scope | Principles | Policy statements | Roles and responsibilities | Definitions | Approval information | Version history | References AI Statement of Intent UTS is a recognised global leader in Artificial Intelligence (AI). Our thought leadership and innovation extend across: - The creation of new AI models, tools and technology through our research and research collaborations - The implementation of AI in real-world applications through our innovations and partnerships with business, civil society, and government - The education of our students to be skilful, responsible users of AI in their studies and future employment, and - Our work to ensure that ethical, legal and other societal impacts are considered in the development and use of AI. As a progressive organisation, UTS also evaluates and leverages AI models and tools in our business operations where it is appropriate to do so. 1. Purpose 1.1 The Artificial Intelligence Operations Policy (the policy) guides the use, procurement, development and management of artificial intelligence (AI) at UTS for the purposes of teaching, learning and operations. 2. Scope 2.1 This policy applies to staff and affiliates (hereafter staff) who are responsible for AI at UTS for teaching, learning and operational functions. 2.2 This policy applies to the: - development, approval, use and management of AI software, systems or platforms developed or created for use by UTS, and - approval, use and management of AI software, systems or platforms procured for use by UTS. 2.3 This policy does not apply to research projects and outputs (including university consulting). Information on the use of AI in research, as well as required research approvals and ethics clearances, is provided in the Research Policy and the Use of AI in Research Guidelines. 3. Principles 3.1 AI at UTS may be used for administrative and operational functions, teaching and learning activities and to improve user experiences as part of the delivery of the university’s object and functions (refer University of Technology Sydney Act 1989 (NSW)). 3.2 To ensure confidence in UTS processes, and alignment with the UTS 2030 strategy, AI must be ethical, reliable, transparent, secure and comply with applicable laws and regulations. 3.3 UTS acknowledges that: - there are legitimate concerns about the use and reliability of AI and will seek to identify the balance between opportunity for improvement and automation, while managing and mitigating risks to the university and its community at all times - algorithmic bias may result in erroneous or unjustified differential treatment which could have unintended or serious consequences for groups of individuals and/or for their human rights - the use of AI will be increasingly regulated and, as such, this policy and any associated procedure must be maintained to ensure compliance with current and emerging regulatory standards and government advice. 3.4 Use of AI systems must comply with the Privacy Policy, the Procurement Policy, the Information Security Policy and the Acceptable Use of Information Technology Resources Policy as appropriate. 4. Policy statements How is AI used at UTS? 4.1 At UTS, AI may be used to support teaching, learning and operational functions and activities, including but not limited to: - making operations more efficient (increasing consistency, speed, agility and scalability) - improving competitiveness to quickly adapt to changing conditions - improving speed and agility to identify issues, risks and opportunities or improve controls - protecting UTS physical and digital resources - verifying identity and highlighting potential cheating - providing feedback to students - identifying at-risk and high-achieving students (to improve learning outcomes and provide additional support) - engaging in student support activities - improving student and staff experiences and/or capabilities - recommending study pathways towards identified career goals - recommending optimal allocation of campus facilities, and - marketing activities including ranking prospects and personalisation. AI risks and opportunities 4.2 All AI systems exist on a spectrum of risk, ranging from low-risk (not automated, often non-operational, does not contain personal or sensitive data and does not have direct impacts on individuals) to high-risk automations (highly autonomous, normally operational AI systems with minimal controls that could impact individual and institutional safety and wellbeing). 4.3 Guided by the NSW Government’s AI Assessment Framework (the NSW framework) operational and non-operational AI will be assessed for risks and opportunities as outlined in the Artificial Intelligence Operations Procedure (the procedure) and the Risk Management Policy. 4.4 UTS will: - assess and manage the use of AI to understand and effectively manage these risks (refer the procedure), and - balance risks and opportunities to protect UTS and individuals and their human rights (refer also Risk Management Policy). AI endorsement, approval and oversight 4.5 Business owners must submit proposed AI systems to the Head of Data Analytics and Artificial Intelligence for feedback before commencement of any development or procurement activities as outlined in the procedure. 4.6 The Artificial Intelligence Operations Board (the board) will develop institutional knowledge and insights about the use, management and control of AI for the purposes of teaching, learning and operations at UTS. 4.7 The board’s terms of reference and membership are approved by the Chief Operating Officer (COO) and are available to staff (refer the procedure). The board will provide an annual report to the University Leadership Team. 4.8 The board is responsible for endorsing the use of AI as part of an identified business activity or solution before the procurement and/or development of AI systems. Where the board considers a system to be high risk, further advice (internal or external) may be sought before submission to the COO for endorsement. 4.9 Following the board’s or the COO’s endorsement of an AI system, the final approval for expenditure of funds will apply as follows: - For projects that require funding: refer to the financial delegations for project approval authority (refer Delegations). - For IT Capital Management Plan (ITCMP): follow standard ITCMP processes (available at ITCMP project governance and delivery framework (Staff Connect)). - For projects that result in the acquisition or procurement of an IT resource: refer to the Procurement Policy and the Acceptable Use of Information Technology Resources Policy for approval process and authority. 4.10 AI system owners must work with AI business owners in the ongoing management, governance and monitoring of AI in systems once procured or implemented, including liaising with information system stewards (refer Data Governance Policy and Transparency and reliability) or the Information Technology Unit as appropriate. Ethical principles for the use of AI 4.11 UTS follows the NSW Government’s Mandatory Ethical Principles for the Use of AI, summarised as follows: - Community benefit: AI should deliver the best outcome for human users, in this case, the UTS community, and provide key insights into decision-making. AI must be the most appropriate solution for a service delivery or a policy problem, considered against other analysis and policy tools. - Fairness: Use of AI will include safeguards to manage data bias or data quality risks. The best use of AI will depend on data quality and relevant data as well as careful data management to ensure potential data biases are identified and appropriately managed (refer also Data Governance Policy). - Privacy and security: AI will include the highest levels of assurance. The UTS community must have confidence that data is used safely and securely in a manner that is consistent with privacy, data sharing and information access requirements (refer also the Privacy Policy and the Records Management Policy). - Transparency: Review mechanisms will ensure that the UTS community can challenge and question AI-based outcomes and will have access to an efficient and transparent review mechanism if there are questions about the use of data or AI-informed outcomes (refer Policy breaches and complaints). - Accountability: While AI is recognised for analysing and looking for patterns in large quantities of data, undertaking high-volume routine process work, or making recommendations based on complex information, AI-based functions and decisions must always be subject to human review and intervention. AI system owners and business owners are responsible for the management of their AI systems. 4.12 The ethical principles for the use of AI are applied at each phase of the AI system lifecycle. The lifecycle stages include: - problem identification and requirements analysis - planning, design, data collection and modelling - development and validation (including training and testing stages) - deployment and implementation - monitoring, review and refinement (including when fixing any problems that occur) or destruction (removal of the system from use). Transparency and reliability 4.13 AI systems must only operate in accordance with their primary purpose or objective as outlined as part of the approval process. Where a change to the primary purpose is needed, this requires a separate risk assessment and endorsement. 4.14 Where AI is used by UTS to automate a function, process or decision that may impact staff, students or others, this must be specifically identified in the relevant privacy and/or AI use disclosure notice, which must include a review or enquiry mechanism. Privacy and records management 4.15 Where personal information is captured, used or stored by an AI system the business owner must complete a privacy impact assessment (refer Privacy hub: Privacy impact assessments (SharePoint)). This must be approved and managed in line with the Privacy Policy and information security classifications. 4.16 Use of biometric identification must be treated as processing sensitive personal information (refer Privacy Policy). 4.17 Data used to develop algorithms or AI systems, and any data generated, shared, managed and/or recorded as part of an AI system’s operation or algorithm, is considered corporate data and must be managed in line with the Data Governance Policy and the Privacy Policy. This requirement applies to the full system lifecycle and to the lifetime of the data (whichever is the longer). Policy breaches and complaints 4.18 Breaches of this policy or any associated procedures must be reported to the Chief Data Officer (CDO) and managed in line with the Code of Conduct and the relevant Enterprise agreement as appropriate. 4.19 Any data breaches or suspected data breaches will be managed in line with the Data Breach Policy. 4.20 Complaints in relation to the use or outcomes of UTS AI systems will be managed in line with the Staff Complaints Policy or the Student Complaints Policy. 5. Roles and responsibilities 5.1 Policy owner: The Chief Data Officer (CDO) is responsible for policy enforcement and compliance, ensuring that its principles and statements are observed. The CDO is also responsible for the approval of any associated university level procedure. 5.2 Policy contact: The Head of Data Analytics and Artificial Intelligence (Data Analytics and Insights Unit) is responsible for the day-to-day implementation of the policy and acts as a primary point of contact for advice on fulfilling its provisions. The Head of Data Analytics and Artificial Intelligence is also responsible for providing guidance and advice on the application of this policy and the procedure and for recommending appropriate training for staff who have responsibility for AI. 5.3 Implementation and governance roles: The Chief Operating Officer (COO) is responsible for the establishment of the Artificial Intelligence Operations Board as outlined in this policy and the procedure. The COO is responsible for endorsing high-risk AI systems before normal approval processes in line with this policy. The Deputy Vice-Chancellor (Research) is responsible for the management of all research activities, including guidance on AI in research (refer the Research Policy and the Use of AI in Research Guidelines). AI system owners and AI business owners are responsible for the approval, management and oversight of AI systems within their remit. 6. Definitions The following definitions apply for this policy and all associated procedures. These are in addition to the definitions outlined in Schedule 1, Student Rules. Definitions in the singular also include the plural meaning of the word. Algorithm means a series of specific directions or instructions built into computer software or systems to solve a defined problem or automate decision-making. Algorithms may use AI to produce improved outcomes. Algorithmic bias means an error or prejudice built into an algorithm (intentionally or unintentionally) that creates outcomes that are unfair, erroneous or favour one group of people over another and may impact an individual’s human rights. Artificial intelligence (AI) UTS uses the NSW Government’s AI Assessment Framework definition, which states that AI is ‘intelligent technology, programs and the use of advanced computing algorithms that can augment decision-making by identifying meaningful patterns in data’. AI is used to solve problems autonomously, and perform tasks to achieve defined objectives, in some cases without explicit human guidance. AI system (also system) means any software system, technology or program at UTS that uses AI as part of its decision-making processes, in part or in whole. AI systems include capabilities, analytics and algorithms on new or existing IT resources. AI system lifecycle means the time from inception through to review and renewal or destruction of an AI system. AI system owner means appropriate staff identified as responsible for the technical implementation of the AI system and its review and monitoring as outlined in the approved project. Where there are multiple AI system owners, a primary owner (normally the most senior staff member) must be identified. AI system owners must have a working relationship with any relevant information system steward (refer Data Governance Policy). Business owner (of AI systems) means staff with overall accountability for the AI system. Business owners have responsibility for establishing the business case for the system, implementing the system (including identifying users, user training and risk management), monitoring its activities (including reporting and review, ensuring benefits and outcomes are realised in line with the purpose), AI ethics and providing support to the AI system owner(s). Business owners may be self-identified (during an approval or initial scoping exercise) or appointed in line with their position description. Normally business owners will be a dean, director, senior manager or equivalent. Corporate data is defined in the Data Governance Policy. Information system steward is defined in the Data Governance Policy. IT resource is defined in the Acceptable Use of Information Technology Resources Policy. Non-operational AI system means AI systems that do not use a live environment for their source data, rather, provide analysis and insight from historical data. While, normally, non-operational AI represents a lower level of risk, the risk level needs to be carefully assessed, particularly where the outputs may be used to influence decision-making or action. Operational AI system means to either produce an act or decision, or to prompt a human to act. Normally these systems work in real time using a live environment for their source data. These systems generally present more risks than non-operational AI systems as they tend to have a real-world effect. However, not all operational AI systems are high risk (for example, digital information boards or apps that show the time of arrival of the next bus). Personal information (which includes health information for the purposes of this policy) is defined in the Privacy Policy. Research project is defined in the Research Policy. Research output is defined in the Research Policy. Approval information | Policy contact | Head of Data Analytics and Artificial Intelligence | |---|---| | Approval authority | Vice-Chancellor | | Review date | 2026 | | File number | UR23/685 | | Superseded documents | New policy | Version history | Version | Approved by | Approval date | Effective date | Sections modified | |---|---|---|---|---| | 1.0 | Vice-Chancellor | 18/05/2023 | 09/06/2023 | New policy. | | 1.1 | Vice-Chancellor | 24/05/2024 | 29/05/2024 | Updated to include the AI Statement of Intent. | | 1.2 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 20/06/2024 | 08/07/2024 | Updates to reflect the review of the Acceptable Use of Information Technology Resources Policy and the Information Security Policy. | | 1.3 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 24/04/2025 | 30/04/2025 | Update to refer to new Use of AI in Research Guidelines. | | 1.4 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 09/05/2025 | 04/06/2025 | Update to reflect new UTS 2030 strategy. |</t>
+          <t>On this page AI Statement of Intent | Purpose | Scope | Principles | Policy statements | Roles and responsibilities | Definitions | Approval information | Version history | References AI Statement of Intent UTS is a recognised global leader in Artificial Intelligence (AI). Our thought leadership and innovation extend across: - The creation of new AI models, tools and technology through our research and research collaborations - The implementation of AI in real-world applications through our innovations and partnerships with business, civil society, and government - The education of our students to be skilful, responsible users of AI in their studies and future employment, and - Our work to ensure that ethical, legal and other societal impacts are considered in the development and use of AI. As a progressive organisation, UTS also evaluates and leverages AI models and tools in our business operations where it is appropriate to do so. 1. Purpose 1.1 The Artificial Intelligence Operations Policy (the policy) guides the use, procurement, development and management of artificial intelligence (AI) at UTS for the purposes of teaching, learning and operations. 2. Scope 2.1 This policy applies to staff and affiliates (hereafter staff) who are responsible for AI at UTS for teaching, learning and operational functions. 2.2 This policy applies to the: - development, approval, use and management of AI software, systems or platforms developed or created for use by UTS, and - approval, use and management of AI software, systems or platforms procured for use by UTS. 2.3 This policy does not apply to research projects and outputs (including university consulting). Information on the use of AI in research, as well as required research approvals and ethics clearances, is provided in the Research Policy and the Use of AI in Research Guidelines. 3. Principles 3.1 AI at UTS may be used for administrative and operational functions, teaching and learning activities and to improve user experiences as part of the delivery of the university’s object and functions (refer University of Technology Sydney Act 1989 (NSW)). 3.2 To ensure confidence in UTS processes, and alignment with the UTS 2030 strategy, AI must be ethical, reliable, transparent, secure and comply with applicable laws and regulations. 3.3 UTS acknowledges that: - there are legitimate concerns about the use and reliability of AI and will seek to identify the balance between opportunity for improvement and automation, while managing and mitigating risks to the university and its community at all times - algorithmic bias may result in erroneous or unjustified differential treatment which could have unintended or serious consequences for groups of individuals and/or for their human rights - the use of AI will be increasingly regulated and, as such, this policy and any associated procedure must be maintained to ensure compliance with current and emerging regulatory standards and government advice. 3.4 Use of AI systems must comply with the Privacy Policy, the Procurement Policy, the Information Security Policy and the Acceptable Use of Information Technology Resources Policy as appropriate. 4. Policy statements How is AI used at UTS? 4.1 At UTS, AI may be used to support teaching, learning and operational functions and activities, including but not limited to: - making operations more efficient (increasing consistency, speed, agility and scalability) - improving competitiveness to quickly adapt to changing conditions - improving speed and agility to identify issues, risks and opportunities or improve controls - protecting UTS physical and digital resources - verifying identity and highlighting potential cheating - providing feedback to students - identifying at-risk and high-achieving students (to improve learning outcomes and provide additional support) - engaging in student support activities - improving student and staff experiences and/or capabilities - recommending study pathways towards identified career goals - recommending optimal allocation of campus facilities, and - marketing activities including ranking prospects and personalisation. AI risks and opportunities 4.2 All AI systems exist on a spectrum of risk, ranging from low-risk (not automated, often non-operational AI systems, do not contain personal or sensitive data and do not have direct impacts on individuals) to high-risk automations (highly autonomous, normally operational AI systems with minimal controls that could impact individual and institutional safety and wellbeing). 4.3 Guided by the NSW Government’s AI Assessment Framework (the NSW framework), UTS will: - assess operational and non-operational AI systems for risks and opportunities as outlined in the Artificial Intelligence Operations Procedure (the procedure) and the Risk Management Policy. - assess the use of AI to understand and effectively manage any risks through appropriate controls (refer the procedure), and - balance risks and opportunities to protect UTS and individuals and their human rights (refer also Risk Management Policy). 4.4 AI systems assessed as high-risk are unsanctioned and may be blocked or restricted. Unsanctioned AI systems must not be used on UTS devices or on personal devices that are used to undertake UTS activities (refer Acceptable Use of Information Technology Resources Policy and ThinkSecurely: High-risk GenAI monitoring on managed devices (SharePoint)). AI endorsement, approval and oversight 4.5 Business owners must submit proposed AI systems to the Head of Data Analytics and Artificial Intelligence for feedback before commencement of any development or procurement activities as outlined in the procedure. 4.6 The Artificial Intelligence Operations Board (the board) will develop institutional knowledge and insights about the use, management and control of AI for the purposes of teaching, learning and operations at UTS. 4.7 The board’s terms of reference and membership are approved by the Chief Operating Officer (COO) and are available to staff (refer the procedure). The board will provide an annual report to the University Leadership Team. 4.8 The board is responsible for endorsing the use of AI as part of an identified business activity or solution before the procurement and/or development of AI systems. Where the board considers a system to be high risk, further advice (internal or external) may be sought before submission to the COO for endorsement. 4.9 Following the board’s or the COO’s endorsement of an AI system, the final approval for expenditure of funds will apply as follows: - For projects that require funding: refer to the financial delegations for project approval authority (refer Delegations). - For IT Capital Management Plan (ITCMP): follow standard ITCMP processes (available at ITCMP project governance and delivery framework (Staff Connect)). - For projects that result in the acquisition or procurement of an IT resource: refer to the Procurement Policy and the Acceptable Use of Information Technology Resources Policy for approval process and authority. 4.10 AI system owners must work with AI business owners in the ongoing management, governance and monitoring of AI in systems once procured or implemented, including liaising with information system stewards (refer Data Governance Policy and Transparency and reliability) or the Information Technology Unit as appropriate. Ethical principles for the use of AI 4.11 UTS follows the NSW Government’s Mandatory Ethical Principles for the Use of AI, summarised as follows: - Community benefit: AI should deliver the best outcome for human users, in this case, the UTS community, and provide key insights into decision-making. AI must be the most appropriate solution for a service delivery or a policy problem, considered against other analysis and policy tools. - Fairness: Use of AI will include safeguards to manage data bias or data quality risks. The best use of AI will depend on data quality and relevant data as well as careful data management to ensure potential data biases are identified and appropriately managed (refer also Data Governance Policy). - Privacy and security: AI will include the highest levels of assurance. The UTS community must have confidence that data is used safely and securely in a manner that is consistent with privacy, data sharing and information access requirements (refer also the Privacy Policy and the Records Management Policy). - Transparency: Review mechanisms will ensure that the UTS community can challenge and question AI-based outcomes and will have access to an efficient and transparent review mechanism if there are questions about the use of data or AI-informed outcomes (refer Policy breaches and complaints). - Accountability: While AI is recognised for analysing and looking for patterns in large quantities of data, undertaking high-volume routine process work, or making recommendations based on complex information, AI-based functions and decisions must always be subject to human review and intervention. AI system owners and business owners are responsible for the management of their AI systems. 4.12 The ethical principles for the use of AI are applied at each phase of the AI system lifecycle. The lifecycle stages include: - problem identification and requirements analysis - planning, design, data collection and modelling - development and validation (including training and testing stages) - deployment and implementation - monitoring, review and refinement (including when fixing any problems that occur) or destruction (removal of the system from use). Transparency and reliability 4.13 AI systems must only operate in accordance with their primary purpose or objective as outlined as part of the approval process. Where a change to the primary purpose is needed, this requires a separate risk assessment and endorsement. 4.14 Where AI is used by UTS to automate a function, process or decision that may impact staff, students or others, this must be specifically identified in the relevant privacy and/or AI use disclosure notice, which must include a review or enquiry mechanism. Privacy and records management 4.15 Where personal information is captured, used or stored by an AI system the business owner must complete a privacy impact assessment (refer Privacy hub: Privacy impact assessments (SharePoint)). This must be approved and managed in line with the Privacy Policy and information security classifications. 4.16 Use of biometric identification must be treated as processing sensitive personal information (refer Privacy Policy). 4.17 Data used to develop algorithms or AI systems, and any data generated, shared, managed and/or recorded as part of an AI system’s operation or algorithm, is considered corporate data and must be managed in line with the Data Governance Policy and the Privacy Policy. This requirement applies to the full system lifecycle and to the lifetime of the data (whichever is the longer). Policy breaches and complaints 4.18 Breaches of this policy or any associated procedures must be reported to the Chief Data Officer (CDO) and managed in line with the Code of Conduct and the relevant Enterprise agreement as appropriate. 4.19 Any data breaches or suspected data breaches will be managed in line with the Data Breach Policy. 4.20 Complaints in relation to the use or outcomes of UTS AI systems will be managed in line with the Staff Complaints Policy or the Student Complaints Policy. 5. Roles and responsibilities 5.1 Policy owner: The Chief Data Officer (CDO) is responsible for policy enforcement and compliance, ensuring that its principles and statements are observed. The CDO is also responsible for the approval of any associated university level procedure. 5.2 Policy contact: The Head of Data Analytics and Artificial Intelligence (Data Analytics and Insights Unit) is responsible for the day-to-day implementation of the policy and acts as a primary point of contact for advice on fulfilling its provisions. The Head of Data Analytics and Artificial Intelligence is also responsible for providing guidance and advice on the application of this policy and the procedure and for recommending appropriate training for staff who have responsibility for AI. 5.3 Implementation and governance roles: The Chief Operating Officer (COO) is responsible for the establishment of the Artificial Intelligence Operations Board as outlined in this policy and the procedure. The COO is responsible for endorsing high-risk AI systems before normal approval processes in line with this policy. The Deputy Vice-Chancellor (Research) is responsible for the management of all research activities, including guidance on AI in research (refer the Research Policy and the Use of AI in Research Guidelines). AI system owners and AI business owners are responsible for the approval, management and oversight of AI systems within their remit. 6. Definitions The following definitions apply for this policy and all associated procedures. These are in addition to the definitions outlined in Schedule 1, Student Rules. Definitions in the singular also include the plural meaning of the word. Algorithm means a series of specific directions or instructions built into computer software or systems to solve a defined problem or automate decision-making. Algorithms may use AI to produce improved outcomes. Algorithmic bias means an error or prejudice built into an algorithm (intentionally or unintentionally) that creates outcomes that are unfair, erroneous or favour one group of people over another and may impact an individual’s human rights. Artificial intelligence (AI) UTS uses the NSW Government’s AI Assessment Framework definition, which states that AI is ‘intelligent technology, programs and the use of advanced computing algorithms that can augment decision-making by identifying meaningful patterns in data’. AI is used to solve problems autonomously, and perform tasks to achieve defined objectives, in some cases without explicit human guidance. AI system (also system) means any software system, technology, application or program at UTS that uses AI as part of its decision-making processes, in part or in whole. AI systems include capabilities, analytics and algorithms on new or existing IT resources. AI system lifecycle means the time from inception through to review and renewal or destruction of an AI system. AI system owner means appropriate staff identified as responsible for the technical implementation of the AI system and its review and monitoring as outlined in the approved project. Where there are multiple AI system owners, a primary owner (normally the most senior staff member) must be identified. AI system owners must have a working relationship with any relevant information system steward (refer Data Governance Policy). Business owner (of AI systems) means staff with overall accountability for the AI system. Business owners have responsibility for establishing the business case for the system, implementing the system (including identifying users, user training and risk management), monitoring its activities (including reporting and review, ensuring benefits and outcomes are realised in line with the purpose), AI ethics and providing support to the AI system owner(s). Business owners may be self-identified (during an approval or initial scoping exercise) or appointed in line with their position description. Normally business owners will be a dean, director, senior manager or equivalent. Corporate data is defined in the Data Governance Policy. Information system steward is defined in the Data Governance Policy. IT resource is defined in the Acceptable Use of Information Technology Resources Policy. Non-operational AI system means AI systems that do not use a live environment for their source data, rather, provide analysis and insight from historical data. While, normally, non-operational AI represents a lower level of risk, the risk level needs to be carefully assessed, particularly where the outputs may be used to influence decision-making or action. Operational AI system means to either produce an act or decision, or to prompt a human to act. Normally these systems work in real time using a live environment for their source data. These systems generally present more risks than non-operational AI systems as they tend to have a real-world effect. However, not all operational AI systems are high risk (for example, digital information boards or apps that show the time of arrival of the next bus). Personal information (which includes health information for the purposes of this policy) is defined in the Privacy Policy. Research project is defined in the Research Policy. Research output is defined in the Research Policy. Approval information | Policy contact | Head of Data Analytics and Artificial Intelligence | |---|---| | Approval authority | Vice-Chancellor | | Review date | 2026 | | File number | UR23/685 | | Superseded documents | New policy | Version history | Version | Approved by | Approval date | Effective date | Sections modified | |---|---|---|---|---| | 1.0 | Vice-Chancellor | 18/05/2023 | 09/06/2023 | New policy. | | 1.1 | Vice-Chancellor | 24/05/2024 | 29/05/2024 | Updated to include the AI Statement of Intent. | | 1.2 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 20/06/2024 | 08/07/2024 | Updates to reflect the review of the Acceptable Use of Information Technology Resources Policy and the Information Security Policy. | | 1.3 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 24/04/2025 | 30/04/2025 | Update to refer to new Use of AI in Research Guidelines. | | 1.4 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 09/05/2025 | 04/06/2025 | Update to reflect new UTS 2030 strategy. | | 1.5 | Director, Governance Support Unit (Delegation 3.14.1) | 17/12/2025 | 22/12/2025 | Update to address use of high-risk GenAI. Minor update to definition of AI system. | References Acceptable Use of Information Technology Resources Policy Artificial Intelligence Operations Procedure NSW Government AI Assessment Framework NSW Government Mandatory Ethical Principles for the use of AI ThinkSecurely: High-risk GenAI monitoring on managed devices (SharePoint) Use of AI in Research Guidelines</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2795</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
         </is>
       </c>
     </row>
@@ -714,6 +896,19 @@
           <t>Key points: Gen AI isn’t going away, so learn to use it wisely and within the bounds of Curtin’s Gen AI guidelines. • Get permission before using Gen AI in your assessments • Declare any use of Gen AI • Use Curtin’s version of Grammarly for safe editing support • Double-check AI-generated content for accuracy • Never submit AI-written text as your own Generative AI tools like ChatGPT, Claude, or Google Gemini are everywhere. From writing help to meal plans, they’re reshaping how we learn and live. At Curtin, students are allowed to use Gen AI tools, but not without boundaries. Here’s how to navigate Gen AI tools at Curtin while keeping your academic integrity intact. Rule 1: You need permission Let’s start with the big one: if you want to use Gen AI to help with an assignment, you must get permission from your Unit Coordinator. That means before using AI to brainstorm ideas, generate outlines, get feedback on your writing or help with sentence structure or clarity, you need to check your unit’s specific rules or contact your tutor directly. Some units allow limited use of Gen AI, while others don’t allow it at all. Rule 2: If you use it, declare it If you get permission to use Gen AI, you also need to be transparent about how you used it. Curtin has provided a clear format for this: a declaration you include in your assignment submission that outlines what tools you used and how. You can find a declaration template and example on the Library website. If you use AI and don’t declare it? That could be seen as misconduct, even if you didn’t mean to cheat. Rule 3: Check your outputs for accuracy Gen AI tools are impressive, but they’re not perfect. They can ‘hallucinate’ false facts, give outdated advice or suggest biased responses. Always check anything it tells you against real sources, and don’t assume it’s right just because it sounds confident. You are responsible for all information submitted for assessments, so if the information from the Gen AI tool was incorrect and still used, this may affect your marks. What tools are available? All students have free access to Curtin’s version of Grammarly through Blackboard. This version has the generative AI features disabled, meaning it checks grammar and clarity but won’t rewrite your text or suggest full sentences. That makes it safe to use across all units. Microsoft Copilot, Adobe Express Premium and Microsoft Teams are other tools you can use at Curtin using your student log-in details. For more information, visit our website. Tools you should be cautious of While popular AI platforms like ChatGPT can be useful, don’t assume they’re always allowed. If you use them to generate parts of your assignment without permission or proper referencing, it’s likely to trigger Turnitin and raise red flags. When in doubt, ask Every unit at Curtin has different expectations. If you’re unsure whether GenAI use is okay in a particular assignment, don’t guess. Instead, ask your tutor or Unit Coordinator directly. Using Gen AI responsibly at Curtin is about being honest, informed and clear about your process. To learn more about using Gen AI at Curtin, familiarise yourself with the information available on our website.</t>
         </is>
       </c>
+      <c r="D16" t="n">
+        <v>542</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -728,7 +923,20 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ERROR: The request could not be satisfied 403 ERROR The request could not be satisfied. Request blocked. We can't connect to the server for this app or website at this time. There might be too much traffic or a configuration error. Try again later, or contact the app or website owner. If you provide content to customers through CloudFront, you can find steps to troubleshoot and help prevent this error by reviewing the CloudFront documentation. Generated by cloudfront (CloudFront) Request ID: hZs_xS4yJF8V9ACHH6f69YxrhQDybs2ZM5Qhc-Fob230l2WyR-otGg==</t>
+          <t>ERROR: The request could not be satisfied 403 ERROR The request could not be satisfied. Request blocked. We can't connect to the server for this app or website at this time. There might be too much traffic or a configuration error. Try again later, or contact the app or website owner. If you provide content to customers through CloudFront, you can find steps to troubleshoot and help prevent this error by reviewing the CloudFront documentation. Generated by cloudfront (CloudFront) Request ID: t2-yWNkESFrwS1kYo-F1lhIoOXMaMcGscuLDIpqEzsqxyAhxX3K5pQ==</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>82</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
         </is>
       </c>
     </row>
@@ -745,7 +953,20 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Using generative AI in teaching and learning Explore the new myCourses self-paced module: Generative AI for Teaching and Learning What is generative AI? Generative AI is a type of artificial intelligence that uses machine learning to create new types of media, including text, images, sound, and video. Many tools exist that use generative AI to create new content. Some examples include: Media | Example tools | |---|---| Text | Copilot (Secure version approved at McGill) | Images | Copilot (Secure version approved at McGill) Adobe Firefly, Midjourney, DALL-E3 (not approved for use at McGill) | Sound | Copilot (Secure version approved at McGill) Voiceify (not approved for use at McGill) | Video | D-ID (not approved for use at McGill) | A secure version of Microsoft Copilot has been approved at McGill. Copilot is an AI chatbot tool integrated into Microsoft Edge and accessible from other browsers. Read more about using Copilot at McGill. Generative AI tools are built upon large language models (LLM) that have been trained on enormous corpora of information and are designed to respond to input prompts with well-structured output. They are focused on predictive text (i.e., the most likely word to follow a previous word), as well as generated media based on patterns or styles in existing datasets. While the outputs can often demonstrate seemingly sophisticated language interaction, there may be situations where they provide inaccurate information in that interaction (e.g., fictional sources). These tools are constantly improving; however, it is important to examine any generative AI output with a critical lens. The McGill Library has a page on artificial intelligence with a section on AI Literacy that discusses the importance of critically approaching AI. Ethical use of generative AI The development of generative AI has brought many ethical considerations that must be addressed with its use. The 2018 Montreal Declaration for a Responsible Development of Artificial Intelligence and the 2021 UNESCO Recommendation on the Ethics of Artificial Intelligence provide a number of principles important to the adoption of these new technologies. Both documents offer an excellent framework for how organizations need to consider these new technologies. The emergence of generative AI is leading to a process of reflection on the evolution of the concept of academic integrity. For any questions related to disciplinary procedures, contact the Office of the Dean of Students. Learn more: AI in academia: The end of the essay? (Maple League of Universities - YouTube video) Infographic: Generative AI explained by AI (Visual Capitalist) Teaching AI literacy: How to begin (Inside Higher Education) What is generative AI? (McKinsey) How can generative AI be used in teaching and learning? In May 2023, the Senate Subcommittee on Teaching and Learning (STL) created a working group to address the use of generative AI at McGill. The working group drafted a report with key recommendations for the use of generative AI at McGill. The report also presents principles for the use of generative AI in teaching and learning. Many different strategies exist for using generative AI tools in course teaching. For example, instructors can use them to create sample texts for students to analyze; create images for presentations; design entire presentation materials; and generate sample practice questions. Strategies also exist for students to use generative AI tools to support their learning. For example, they can be used to brainstorm ideas; create images to support assignments such as presentations; and summarize documents. These resources offer more ideas for creating instructional materials and supporting student learning: How could AI be used for learning and teaching? and How AI can be used meaningfully by teachers and students in 2023. It is important to note that students need AI literacy skills to responsibly use generative AI tools. These potentially new literacy skills could include elements such as fact-checking and prompt engineering. Avoid AI detection tools AI detection tools are tools designed to identify content that is partially or wholly generated by AI. These tools (specifically regarding generated text) are unreliable and often inaccurate, a statement corroborated by OpenAI, the creators of ChatGPT. OpenAI states that their false positive rate is 9%, which is a similar rate found in other AI detection tools. A false positive is when the tool identifies text as being generated by AI when it was actually created by a student. False positive results misguide instructors and can create situations where students are wrongly accused of a violation that they did not commit, forcing them to defend work that is rightfully theirs. Such situations can result in a negative classroom climate and create unnecessary stress and anxiety for all involved. McGill therefore discourages the use of AI detection tools. Course outline statements There should be no default assumption as to the use of generative AI tools. Therefore, McGill recommends that instructors explain to students in their course outline what the appropriate use or non-use is of generative AI tools in the context of that course. The use or non-use of these tools should align with the learning outcomes associated with the course. For this reason, instructors will need to write their own context-appropriate course outline statements. Below are four external examples to draw on: Monash University policy and practice guidance around acceptable and responsible use of AI technologies: See the Actions box and the section entitled Specify conditions for the use of generative AI in assessment. University of Florida has an excellent AI resource page that shows concise examples of course outline statements and multiple categories of suggestions on how to either neutralize or capitalize on using AI in courses. University of Toronto syllabus language: This document provides suggestions for clarifying whether students can use generative AI tools; can use generative AI tools in certain instances; or cannot use them at all in the course. Update your course syllabus for ChatGPT (Medium): See the section entitled Before editing your syllabus and the one entitled Update your syllabus. If you allow students to use generative AI tools in your course, provide guidance in your course outline for how students should acknowledge the use. Monash University provides useful examples, as well as links to APA and MLA citation guidelines. See the section entitled How students acknowledge the use of generative AI. AI and assessment of student learning Generative AI tools can be used to support many different types of assessment. As with the planning of any assessment of student learning, it is important to be intentional about the strategy. In this case, be intentional about either designing AI into your assessments or designing AI out of your assessments. This reflective process will encourage you to think through your assessments and determine if the integration of AI is appropriate (or not) for allowing students to demonstrate their learning. Designing AI into an assessment could involve having students generate the assignment with an AI tool, then critique the output, and reflect on the process. Designing AI out of the assessment could involve in-class writing exercises, where students create and share their ideas with other students in class during class time. Either way, the decision should align with students’ achievement of the desired learning outcomes. Monash University provides excellent considerations for assessment design. Learn more: 6 Tenets of postplagiarism: Writing in the age of artificial intelligence (Teaching and Leadership) AI-generated content in the classroom: Considerations for course design (Illinois State University) Artificial Intelligence (UNESCO) Beyond Grading: Assessment in the age of AI (McGill, video, 50 minutes) Bloom’s taxonomy revisited with AI (Oregon State University) Bowen, J. A., &amp; Watson, C. E. (2024). Teaching with AI: A practical guide to a new era of human learning. Johns Hopkins University Press How do I Consider the Options for a Generative AI Course Policy? (Center for Teaching and Learning, University of Massachusetts Amherst) McGill Library guide on artificial intelligence (McGill Library) The Artificial Intelligence Assessment Scale (AIAS): A Framework for Ethical Integration of Generative AI in Educational Assessment. (2024). Journal of University Teaching and Learning Practice, 21(06). Resources: Have a question that was not answered in this article? Visit our FAQs. McGill University is on land which has served and continues to serve as a site of meeting and exchange amongst Indigenous peoples, including the Haudenosaunee and Anishinabeg nations. Teaching and Academic Programs acknowledges and thanks the diverse Indigenous peoples whose footsteps mark this territory on which peoples of the world now gather. This land acknowledgment is shared as a starting point to provide context for further learning and action. McLennan Library Building 3415 McTavish Street Suite MS-12 (ground level), Montreal, Quebec H3A 0C8 | mcgill.ca/tap</t>
+          <t>Using generative AI in teaching and learning Explore the new myCourses self-paced module: Generative AI for Teaching and Learning What is generative AI? Generative AI (gen AI) is a type of artificial intelligence that uses machine learning to create new types of media, including text, images, sound, and video. Many tools exist that use generative AI to create new content. Some examples include: Media | Example tools | |---|---| Text | Copilot (Secure version approved at McGill) | Images | Copilot (Secure version approved at McGill) Adobe Firefly, Midjourney, DALL-E3 (not approved for use at McGill) | Sound | Copilot (Secure version approved at McGill) Voiceify (not approved for use at McGill) | Video | D-ID (not approved for use at McGill) | A secure version of Microsoft Copilot has been approved at McGill. Copilot is an AI chatbot tool integrated into Microsoft Edge and accessible from other browsers. Read more about using Copilot at McGill. Generative AI tools are built upon large language models (LLM) that have been trained on enormous corpora of information and are designed to respond to input prompts with well-structured output. They are focused on predictive text (i.e., the most likely word to follow a previous word), as well as generated media based on patterns or styles in existing datasets. While the outputs can often demonstrate seemingly sophisticated language interaction, there may be situations where they provide inaccurate information in that interaction (e.g., fictional sources). These tools are constantly improving, however, it is important to examine any generative AI output with a critical lens. The McGill Library has a page on artificial intelligence with a section on AI Literacy that discusses the importance of critically approaching AI. Ethical use of generative AI The development of generative AI has brought many ethical considerations that must be addressed with its use. The 2018 Montreal Declaration for a Responsible Development of Artificial Intelligence and the 2021 UNESCO Recommendation on the Ethics of Artificial Intelligence provide a number of principles important to the adoption of these new technologies. Both documents offer an excellent framework for how organizations need to consider these new technologies. The emergence of generative AI is leading to a process of reflection on the evolution of the concept of academic integrity. For any questions related to disciplinary procedures, contact the Office of the Dean of Students. McGill instructors should follow the same disciplinary procedures as for any other instance where there are concerns about academic integrity. To note: the Code of Student Conduct was updated last month and it now includes specific reference to generative AI with respect to academic offenses (see Articles 25-b and 26-f). For further information, such as the quantity of cases McGill is dealing with, the Office of the Dean of Students might be able to provide information. Instructors might be able to mitigate such cases by providing students with guidance about whether and how gen AI use is permitted in their courses. McGill strongly recommends that all instructors include in their course outlines a statement about gen AI use. Learn more: AI in academia: The end of the essay? (Maple League of Universities - YouTube video) Infographic: Generative AI explained by AI (Visual Capitalist) Teaching AI literacy: How to begin (Inside Higher Education) What is generative AI? (McKinsey) How can generative AI be used in teaching and learning? In May 2023, the Senate Subcommittee on Teaching and Learning (STL) created a working group to address the use of generative AI at McGill. The working group drafted a report with key recommendations for the use of generative AI at McGill. The report also presents principles for the use of generative AI in teaching and learning. Many different strategies exist for using generative AI tools in course teaching. For example, instructors can use them to create sample texts for students to analyze, create images for presentations, design entire presentation materials, and generate sample practice questions. Strategies also exist for students to use generative AI tools to support their learning. For example, they can be used to brainstorm ideas, create images to support assignments such as presentations, and summarize documents. These resources offer more ideas for creating instructional materials and supporting student learning: How could AI be used for learning and teaching? and How AI can be used meaningfully by teachers and students in 2023. Assessment is one facet of course design. The course design approach we promote at McGill suggests beginning with learning outcomes – what knowledge/skills/values would we like students to leave a course with? From there, we can consider what types of assessments align with the desired outcomes. The advent of gen AI might mean rethinking what those learning outcomes are before considering how to redesign assessment. Rethinking learning outcomes – this is an important consideration with implications for higher ed/society. Specifically in online education, McGill promotes experiential learning activities that require students to apply skills, make decisions, and produce work similar to what they would encounter in professional practice. These activities may take the form of interactive simulations, scenario-based assessments, authentic tasks linked to real-world contexts, and reflective activities that help students connect their experiences with course concepts. In some cases, gen AI use is intentionally integrated into the learning activities and requires that any use of gen AI tools be properly cited. It is important to note that students need AI literacy skills to responsibly use generative AI tools. These potentially new literacy skills could include elements such as fact-checking and prompt engineering. All McGill instructors and students can explore the new myCourses self-paced module Generative AI for Teaching and Learning. Avoid AI detection tools AI detection tools are tools designed to identify content that is partially or wholly generated by AI. These tools (specifically regarding generated text) are unreliable and often inaccurate, a statement corroborated by OpenAI, the creators of ChatGPT. OpenAI states that their false positive rate is 9%, which is a similar rate found in other AI detection tools. A false positive is when the tool identifies text as being generated by AI when it was actually created by a student. False positive results misguide instructors and can create situations where students are wrongly accused of a violation that they did not commit, forcing them to defend work that is rightfully theirs. Such situations can result in a negative classroom climate and create unnecessary stress and anxiety for all involved. McGill therefore discourages the use of AI detection tools. Note: McGill also does not recommend online proctoring. Course outline statements There should be no default assumption as to the use of generative AI tools. Therefore, McGill recommends that instructors explain to students in their course outline what the appropriate use or non-use is of generative AI tools in the context of that course. The use or non-use of these tools should align with the learning outcomes associated with the course. For this reason, instructors will need to write their own context-appropriate course outline statements. Below are four external examples to draw on: Monash University policy and practice guidance around acceptable and responsible use of AI technologies: See the Actions box and the section entitled Specify conditions for the use of generative AI in assessment. University of Florida has an excellent AI resource page that shows concise examples of course outline statements and multiple categories of suggestions on how to either neutralize or capitalize on using AI in courses. University of Toronto syllabus language: This document provides suggestions for clarifying whether students can use generative AI tools; can use generative AI tools in certain instances; or cannot use them at all in the course. Update your course syllabus for ChatGPT (Medium): See the section entitled Before editing your syllabus and the one entitled Update your syllabus. If you allow students to use generative AI tools in your course, provide guidance in your course outline for how students should acknowledge the use. Monash University provides useful examples, as well as links to APA and MLA citation guidelines. See the section entitled How students acknowledge the use of generative AI. AI and assessment of student learning Generative AI tools can be used to support many different types of assessment. As with the planning of any assessment of student learning, it is important to be intentional about the strategy. In this case, be intentional about either designing AI into your assessments or designing AI out of your assessments. This reflective process will encourage you to think through your assessments and determine if the integration of AI is appropriate (or not) for allowing students to demonstrate their learning. Designing AI into an assessment could involve having students generate the assignment with an AI tool, then critique the output, and reflect on the process. Designing AI out of the assessment could involve in-class writing exercises, where students create and share their ideas with other students in class during class time. Either way, the decision should align with students’ achievement of the desired learning outcomes. Monash University provides excellent considerations for assessment design. Learn more: 6 Tenets of postplagiarism: Writing in the age of artificial intelligence (Teaching and Leadership) AI-generated content in the classroom: Considerations for course design (Illinois State University) Artificial Intelligence (UNESCO) Beyond Grading: Assessment in the age of AI (McGill, video, 50 minutes) Bloom’s taxonomy revisited with AI (Oregon State University) Bowen, J. A., &amp; Watson, C. E. (2024). Teaching with AI: A practical guide to a new era of human learning. Johns Hopkins University Press How do I Consider the Options for a Generative AI Course Policy? (Center for Teaching and Learning, University of Massachusetts Amherst) McGill Library guide on artificial intelligence (McGill Library) The Artificial Intelligence Assessment Scale (AIAS): A Framework for Ethical Integration of Generative AI in Educational Assessment. (2024). Journal of University Teaching and Learning Practice, 21(06). Resources: Generative AI for teaching and learning (myCourses module for instructors and students) Generative AI perspectives and practices from McGill instructors across disciplines (podcast series) (Re)designing assessments in the age of generative AI - slides (Re)designing assessment tasks in the age of generative AI - activity sheet Sharing experiences with generative AI in teaching and learning - slides Sharing experiences with generative AI (teaching and learning community) Teaching consultations (one-on-one meeting with a TAP staff member) Have a question that was not answered in this article? Visit our FAQs. McGill University is on land which has served and continues to serve as a site of meeting and exchange amongst Indigenous peoples, including the Haudenosaunee and Anishinabeg nations. Teaching and Academic Programs acknowledges and thanks the diverse Indigenous peoples whose footsteps mark this territory on which peoples of the world now gather. This land acknowledgment is shared as a starting point to provide context for further learning and action. McLennan Library Building 3415 McTavish Street Suite MS-12 (ground level), Montreal, Quebec H3A 0C8 | mcgill.ca/tap</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1805</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
         </is>
       </c>
     </row>
@@ -765,6 +986,19 @@
           <t>Policy on use of generative artificial intelligence (AI) in Major Research Papers (MRP) The MRP is an opportunity for the student to demonstrate knowledge and understanding of the research conducted on their topic, and show their ability to perform independent, graduate-level work. Researching and writing the MRP contribute to student learning, including the development and enrichment of critical thinking and critical analysis. For these reasons, it is important to understand when and how AI should and should not be used when developing and writing the MRP. Before using AI as part of writing an MRP, students should be aware that AI poses certain risks, including: • Academic integrity issues when AI-generated material is passed off as the student’s own work • Jeopardizing intellectual property of any materials or data that students input into AI – and many other free apps Jeopardizing confidentiality in the case of primary sources of data • • Environmental costs, including electricity consumption. While generative AI can be an effective tool to help with specific parts of the research process (see below), it is essential to consider whether it supports critical thinking and critical analysis and the building of skills in those domains (appropriate) or whether it offloads these skills to a generative AI tool (not appropriate).1 Before using AI generated output in your MRP, you must verify that it is accurate, avoids (unacknowledged) biases, and correctly acknowledges contributions from others. It is never acceptable to use AI generated text in your MRP. The following is a non-exhaustive list of permitted and prohibited uses.2 If you have questions, please ask your MRP supervisor and/or the professor responsible for the MA in Public and International Affairs. Permitted uses: Identifying preliminary sources • Brainstorming your topic or preliminary research questions • • Generating synonyms of keywords for database searches • Translating a text3 • (Re)formatting citations and references • Checking grammar, spelling and clarity Use with caution: • Clarifying concepts • Overcoming writer’s block • Assisting with data visualization • Summarizing source documents Prohibited uses: • Using verbatim or slightly modified AI-generated content to write any or all sections of the MRP • Creating a full bibliography, including the inclusion of fabricated references • Generating false data • Analyzing data instead of student-led verification and interpretation 1 Professor Jim Davies (Carleton University) shared this insight during the development of this policy. 2 These examples are inspired by the flyer developed by Majela Guzman, https://infograph.venngage.com/pl/LkF6MMgU3FA 3 Translating data or parts or the entirety of your MRP may result in losing intellectual property on this material. Policy on use of generative artificial intelligence (AI) in Major Research Papers (MRP) You must include a statement indicating how you used AI in your MRP research and writing. Any student suspected of prohibited use of AI will be referred to the disciplinary approach under Academic Regulation A-44. 4 https://www.uottawa.ca/about-us/leadership-governance/policies-regulations/a-4-academic-integrity-academic-misconduct</t>
         </is>
       </c>
+      <c r="D19" t="n">
+        <v>476</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -782,6 +1016,19 @@
           <t>Quick Links Artificial intelligence is everywhere and with it comes new opportunities and challenges. As these new platforms evolve so must the way instructors, TAs and students use them. Given the rapid pace of change and growth in artificial intelligence - this issue will be ongoing for the foreseeable future. The Associate Vice-President, Academic's website has more information about artificial intelligence in teaching and learning at University of Waterloo. At present, it's important for instructors to be explicit about whether artificial intelligence or tools like ChatGPT are allowed to be used to complete assignments, tests or exams, and if so, the extent to which it is allowed, and if it should be cited and how to cite it. A student who does not comply with the instructor's rules about the use of such tools will be subject to Policy 71 and an investigation into academic misconduct. *Note: Effective September 2025, AI detection functionality in Turnitin will no longer be available. We recommend that instructors focus on evidence of learning rather than focusing on finding misuse of artificial intelligence. Instructors, students and staff should use GenAI transparently. The Library has resources for citing the use of GenAI. Dr. Kari Weaver (UW Library) has also developed an Artificial Intelligence Disclosure (AID) Framework. Microsoft Copilot should be used through your UWaterloo account in order to protect the privacy and security of the data that you enter. Be sure not to share any personal, institutional or research data in a GenAI tool that saves and uses your prompt data!</t>
         </is>
       </c>
+      <c r="D20" t="n">
+        <v>255</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -799,6 +1046,19 @@
           <t>Guidelines: The Use of Generative Artificial Intelligence (AI) in Teaching and Learning at McMaster University – August, 2024 by McMaster University is licensed under a Creative Commons Attribution-NonCommercial 4.0 International License Introduction and Context In June 2023 McMaster launched an initial set of Provisional Guidelines on the Use of Generative AI in Teaching and Learning. These Provisional Guidelines were updated further in August 2024 and then used throughout the academic year. After a further year of teaching and learning with generative AI, these Provisional Guidelines require some revision. These revisions were informed by feedback from faculty, students and staff and were written and endorsed by the Expert Panel on AI in Teaching and Learning and the AI Advisory Committee. They are intended to guide both educators and students in understanding and interacting with generative AI in teaching and learning contexts. Staff may wish to consult the Provisional Guidelines on the Use of Generative AI in Operational Excellence. In this update we move from “Provisional” to “Guidelines” recognizing that the Guidelines are not a policy but do intersect with existing McMaster policies and that the Guidelines will need further updating. Questions, comments or suggestions about these Guidelines may be directed to the Vice-Provost, Teaching and Learning or to the Special Advisor to the Provost on Generative AI at macgenai@mcmaster.ca Learning requires active engagement: building mental models and habits of mind, then communicating, applying, evaluating, and reflecting on those mental models and habits of mind. Learning requires work – often slow and challenging work. Generative artificial intelligence offers a promise of efficiency and speed, a promise that can be at odds with the deliberate effort of learning. At McMaster, we suggest that generative artificial intelligence tools should be used for learning only when the educator judges that their use will aid in active, critical, and reflective engagement. In most disciplines, university-level learning focuses on process, rather than the end-product. In other words, it is more important that students learn the how (e.g. how to find a solution, how to evaluate sources, how to construct an argument, how to perform a lab task, etc.), as opposed to the what (i.e. specific content). Generative AI poses a significant risk to the process of learning by bypassing or obscuring the how. While generative AI poses these risks to learning, at McMaster we remain open to generative AI use for teaching and learning, as well as experimentation with new tools and techniques when they advance a course or program’s goals. Educators experimenting with generative AI for its benefits for learning will want to be clear on pedagogical goals and how generative AI will advance those goals. Beyond learning, generative AI introduces a range of concerns, including environmental impacts, disinformation, impacts on labour, questions of copyright and ownership, lack of transparency in model design and function, privacy and data collection and use. Educators and students can learn more about these issues and should discuss them in courses where appropriate. Educators can get support in talking with their students about generative AI through the MacPherson Institute, the Privacy Office, or through these resources. Generative artificial intelligence systems are trained to produce outputs that are plausible in each context. The models learn to associate inputs to outputs by processing massive amounts of text and image data from the open web and other sources. Despite their ability to produce human-like outputs, there is no proven correspondence between the way that human beings think and learn and the way that generative AI models learn, process, and generate text, images, sounds, and other media. Because of the way they process training data and produce their outputs, generative AI systems are prone to producing ‘hallucinations’ (false statements, impossible images, false citations and attributions and other errors). Likewise, these systems produce outputs that are biased by their training data; these biases are often subtle and thus hold the risk of being uncritically reproduced. There is no current solution for the hallucination and bias problems. As generative AI models produce output that cannot be guaranteed to be accurate and unbiased, university-educated domain experts will continue to be required, both to produce original work and to verify the accuracy of the work that generative models produce. McMaster must continue to train students in the core competencies of any domain of study, regardless of the ability of generative AI models to answer undergraduate-level questions in that domain. Deciding as a learner and educator whether, when, and how to use generative artificial intelligence requires careful thought and evaluation of the benefits and risks to learning. It is ever more essential for educators to carefully consider what skills they need students to learn – that is, what process of learning – for the course and program. Educational developers at the MacPherson Institute can support this planning. Guidelines on the Use of Generative AI in Teaching and Learning - 1. Undergraduate and graduate course outlines should include a statement on the acceptable and unacceptable use of generative artificial intelligence in the course, with attention to the use of generative artificial intelligence for studying/learning and/or assessment. For instance, students may or may not use generative AI tools for idea generation, structuring, editing assistance, translation, summarizing/paraphrasing information, etc. (refer to the Use of Translation and Editing Tools guide for information about how to use these tools responsibly in the context of academic integrity). - If no syllabus statement is included, students should ask the educator for clarification on expectations, and if generative AI use is permitted, receive written confirmation before using generative AI in the course. - Educators should review expectations on the use of generative AI with their students in class [see: sample slide deck]. - 2. Educators incorporating generative AI into courses should consider how the course and its goals align with those of the program and with program learning outcomes. Educators should consult with the Departmental chair for the program learning outcomes and any program or departmental norms and expectations related to the use of generative AI at the program level. Programs may wish to establish norms and expectations of generative AI use at the program level. Support for this work is available by contacting macgenai@mcmaster.ca - 3. Use of generative artificial intelligence by students in ways not described in the course outline may be cause for a violation of the academic integrity policy. Likewise, the submission for course credit of uncited or unacknowledged work not created by the student(s) who submitted it violates academic integrity (See McMaster Policy on Academic Integrity). Reach out to the Office of Academic Integrity with any questions on process or for support. Reach out to the MacPherson Institute at mi@mcmaster.ca for support with redesigning assessments. - 4. Automatic AI detection systems are not reliable and are therefore not recommended for separating student- from AI-produced work. Educators who suspect work may have been inappropriately generated by artificial intelligence should follow the academic integrity process. This conversation guide may be useful for talking with students. - 5. If using generative artificial intelligence in courses or for teaching and learning activities, educators and students should use institutionally supported tools that have a completed Privacy and Algorithmic Impact Assessment. McMaster has an enterprise license with Microsoft Copilot. Educators and students who use generative AI should use their McMaster single-sign on credentials to login to Microsoft’s Copilot. - 6. In selecting third-party technology tools educators must avoid those that sell student data to companies building large language models, as well as companies that use student data to train AI models or to improve services and products; educators should review user agreements and consult with the Office of Legal Services or the Privacy Office if unsure. - 7. Legal questions of intellectual property (such as copyright and privacy) continue to be evaluated by provincial and federal courts. Until such questions are resolved, employees should not use generative AI created content for proprietary work and all McMaster policies continue to remain in effect. - 8. Students in co-op and experiential learning environments that use generative AI as directed by or approved by the co-op/experiential learning employer should initiate a discussion with the course instructor on how to document and reflect on this use with respect to the course learning. - 9. Students and educators who use generative AI should complete this module to help them review and reflect on broader societal implications of the use of generative AI, including labour, copyright, bias, and environmental impact. - 10. Students and educators who use generative AI in any context within a course should cite or acknowledge its use drawing on McMaster Libraries’ LibGuide and follow any course specific instructions. - 11. Generative AI tools should not be used to provide grades (letter or numeric) for student work. Generative AI tools may be used to provide feedback on student work, provided the following conditions are met: - When generative AI tools are used to provide feedback of student work this use must be explicitly included in the course syllabus. - Students should have the ability to opt-out of AI generated feedback. - AI generated feedback must be checked for accuracy and bias before being returned to the student. - Documentation of the AI tool used for feedback is required. - Instructors, or teaching assistants when directed, are responsible for feedback, however it is produced, to ensure appropriateness and accuracy. If you would like to discuss options for feedback and evaluation, please reach out to the MacPherson Institute at mi@mcmaster.ca - 12. If instructors use generative AI in their teaching materials, they should explain in the course outline the extent to which generative AI has been, or will be, used and should clearly cite or label such uses in their course materials. Instructors should fact-check any generative AI produced materials and evaluate these materials for bias. - 13. Course instructors have three options for directing teaching assistant use of generative AI. These directions should be given to teaching assistants in writing. - Permitting teaching assistants to use generative AI for any aspect of teaching assistant work, with the exception of evaluations that include a numeric or letter grade (see #11). TAs must inform the instructor of the intended use of generative AI, and receive approval, before implementation. - Requiring teaching assistants to use generative AI for specified teaching tasks as outlined in the hours of work form and with training provided.?In the instance of required use: As directed by the course instructor explicitly in the hours of work form, teaching assistants will use generative AI for the specific teaching tasks. Teaching assistant may create role-based accounts for such use. Course instructors will provide teaching assistants with the necessary training to use generative AI for the specified teaching purpose(s) with this training included in the hours of work. Teaching assistants will evaluate all teaching materials/formative feedback developed with generative AI for accuracy before use with students. Any planned use of generative AI by teaching assistants will be shared with students in the course outline.? - Prohibiting teaching assistants from using generative AI for teaching tasks. Over the fall and winter of 2024 the AI Expert Panel on Teaching and Learning will continue to work. Some of the activities of the Expert Panel include: - Additional course outline language to differentiate uses of generative AI and recommendations for consideration in policies related to course outlines - Engaging educators and students in discussion about the use of generative AI for evaluating student work - Developing resources to support departmental chairs - Additional resources for educators to talk with students about generative AI - Suggested language for acknowledgement of generative AI use (in addition to language for citation) If you have suggestions for additional resources or discussions the AI Expert Panel on Teaching and Learning could support, please reach out to macgenai@mcmaster.ca Sample Syllabus Statements These sample syllabus statements may be included on a course syllabus to communicate with students the expectations around generative AI in a course. Instructors may adapt or modify these statements according to their individual teaching goals and course learning outcomes. Students are not permitted to use generative AI in this course. In alignment with McMaster academic integrity policy, it “shall be an offence knowingly to … submit academic work for assessment that was purchased or acquired from another source”. This includes work created by generative AI tools. Also state in the policy is the following, “Contract Cheating is the act of “outsourcing of student work to third parties” (Lancaster &amp; Clarke, 2016, p. 639) with or without payment.” Using Generative AI tools is a form of contract cheating. Charges of academic dishonesty will be brought forward to the Office of Academic Integrity. Example One Students may use generative AI in this course in accordance with the guidelines outlined for each assessment, and so long as the use of generative AI is referenced and cited following citation instructions given in the syllabus. Use of generative AI outside assessment guidelines or without citation will constitute academic dishonesty. It is the student’s responsibility to be clear on the limitations for use for each assessment and to be clear on the expectations for citation and reference and to do so appropriately. Example Two Students may use generative AI for [editing/translating/outlining/brainstorming/revising/etc] their work throughout the course so long as the use of generative AI is referenced and cited following citation instructions given in the syllabus. Use of generative AI outside the stated use of [editing/translating/outling/brainstorming/revising/etc] without citation will constitute academic dishonesty. It is the student’s responsibility to be clear on the limitations for use and to be clear on the expectations for citation and reference and to do so appropriately. Example Three Students may freely use generative AI in this course so long as the use of generative AI is referenced and cited following citation instructions given in the syllabus. Use of generative AI outside assessment guidelines or without citation will constitute academic dishonesty. It is the student’s responsibility to be clear on the expectations for citation and reference and to do so appropriately. Students may use generative AI throughout this course in whatever way enhances their learning; no special documentation or citation is required. Honour Pledges Honour pledges are formal, student-led commitments to uphold the principles of academic honesty and integrity. These pledges represent students’ personal assurance to maintain and respect academic standards, abstaining from any form of plagiarism, cheating, or other academic misconduct. They often form part of the assessment submission process, where students attach a pre-defined pledge to their work as a statement of authenticity. Several studies have investigated the use of honour codes and academic integrity and found them effective in reducing academic dishonesty. Instructors might consider developing honour pledges together with their students, or adapting this McMaster honour pledge to their purposes. “I understand and believe the main purpose of McMaster and of a university to be the pursuit of knowledge and scholarship. This pursuit requires my academic integrity; I do not take credit that I have not earned. I believe that academic dishonesty, in whatever form, is ultimately destructive to the values of McMaster, and unfair to those students who pursue their studies honestly. I pledge that I completed this assessment following the guidelines of McMaster’s academic integrity policy.”</t>
         </is>
       </c>
+      <c r="D21" t="n">
+        <v>2537</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -816,6 +1076,19 @@
           <t>As generative AI (GenAI) tools and platforms continue to expand and evolve, it is important to provide the UBC community with guidance and advice related to their opportunities as well as risks and challenges. Download: Principles and Guidelines for Generative Artificial Intelligence (GenAI) in Teaching and Learning GenAI tools are artificial intelligence systems that can generate content – such as texts, images, audio, and video – in response to prompts by a user, after being trained on an earlier set of data (from Glossary of GenAI terms). Some GenAI tools are accessed through standalone platforms (e.g., ChatGPT), while others may be embedded in other applications or platforms (e.g., Grammarly). GenAI has the potential to enrich teaching and learning activities, and some may also support inclusion and enhance accessibility, depending on how they are used. Learning how to responsibly use GenAI is important for all members of the UBC community given its growing presence in many academic and work environments. However, such tools can and have been used in ways that are harmful to individuals and communities, and careful attention must be paid to topics such as academic integrity, accessibility, equity, Indigenous data sovereignty, and privacy and intellectual property. The following principles and guidelines have been developed through discussions with a Generative AI in Teaching and Learning Advisory Committee during the 2023-2024 academic year, and through multiple consultations with various individuals and groups at UBC. They provide guidance on responsible and ethical use of GenAI in teaching and learning at UBC, balancing both opportunities and risks. These guidelines are designed to adhere to and support UBC’s strategic plans and commitments, and to align with existing UBC policies, procedures, and legal requirements (linked where relevant below). They also support and build upon the UBC Principles for Use of Generative AI. This is meant to be a living document, evolving as needed in a rapidly-changing landscape around GenAI in teaching and learning. For feedback or questions, please contact provost.vptl@ubc.ca. Principles The following broad principles around GenAI in teaching and learning at UBC serve as a foundation for the more specific guidelines that follow. Download: Principles For GenAI in Teaching &amp; Learning Alignment to Our Values and Priorities UBC strategic plans and commitments Use of GenAI in teaching and learning should be aligned with and support UBC strategic plans and commitments, including those related to decolonization and Indigenous human rights, equity, accessibility, sustainability, and wellness. Opportunities to enhance education GenAI can provide significant value in both teaching and learning activities through informed, responsible, and ethical use that mitigates risks and potential harms. Value for students’ future endeavours It is important for students to learn how to use GenAI effectively and responsibly, to prepare them for further work or studies when they leave UBC. Indigenous data sovereignty Use of GenAI should respect Indigenous data sovereignty and community protocols for use and sharing of Indigenous knowledges, intellectual properties, and data. Harm from false information about Indigenous communities, cultures, knowledges, histories, and contexts should be avoided. Academic integrity All uses of GenAI at UBC must uphold academic integrity and adhere to the academic misconduct regulations in the UBC Okanagan and Vancouver calendars. Building Capacity and Literacy GenAI literacy UBC will continue to provide opportunities to learn about capabilities and limitations of GenAI tools. Faculty, staff, and students should use those opportunities to develop basic GenAI literacy skills over time. Faculty and staff use of GenAI Faculty and staff may use GenAI in teaching and learning so long as this is within the bounds of legal, university, Faculty, or program-level policies and requirements, and the guidelines below. Student use of GenAI Students may use GenAI in work submitted for courses or other academic requirements only if expressly permitted within their courses or programs. They may choose to use GenAI to support their learning in other ways, within the bounds of legal and university policies and requirements, and the guidelines below. Considerations Accessibility Some GenAI tools can enhance accessibility for learners with a range of disabilities. It is important to also recognize, however, that there may be varying levels of accessibility to GenAI tools, whether related to cost, inaccessible infrastructure (such as websites or applications), or for other reasons. Those using GenAI in teaching and learning should ensure equitable access to the best of their ability. Intellectual property &amp; copyright Those using GenAI in teaching and learning should respect intellectual property rights in material they input into the tools, and in how they use outputs. Privacy &amp; confidentiality Use of GenAI in teaching and learning should protect privacy and confidentiality of personal and other sensitive information. Personal Responsibility Equity Biased training data and inputs can produce biased, discriminatory, inaccurate, or otherwise harmful outputs, with the potential to perpetuate systemic inequities. Those using GenAI in academic work should assess the risks and mitigate, to the best of their ability, the harmful effects of such bias. Human oversight and critical thinking All outputs of GenAI for teaching and learning purposes should undergo human review before sharing. Users should think critically about outputs from GenAI, including their potential for producing false or misleading information, especially if sources of information in the outputs cannot be identified and/or verified. Transparency Use of GenAI to produce text, images, videos, or other materials shared with others for teaching or learning purposes should be acknowledged by attributing the source of those materials. Responsibility Users of GenAI are accountable for the consequences of sharing the outputs generated with these tools, and have a responsibility to review them for inaccuracy and potential harm to the best of their ability. The university will provide resources to help individuals develop requisite skills.</t>
         </is>
       </c>
+      <c r="D22" t="n">
+        <v>941</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -833,6 +1106,19 @@
           <t>Page not found | Office of Teaching and Learning Page not found The requested page "/teaching-assessment-resources/teaching-context-ai/provisional-recommendations-use-generative-ai%20https://www.uregina.ca/policy/browse-policy/policy-ops-080-050.html" could not be found.</t>
         </is>
       </c>
+      <c r="D23" t="n">
+        <v>20</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -845,6 +1131,24 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Provisional Guidelines on the Use of Generative Artificial Intelligence (GenAI) in Teaching and Learning for Instructors at the University of Prince Edward Island – December 2023 Provisional Guidelines: The Use of Generative Artificial Intelligence (GenAI) in Teaching and Learning at the University of Prince Edward Island was adapted from Provisional Guidelines: The Use of Generative Artificial Intelligence (AI) in Teaching and Learning at McMaster University – June 2023 by McMaster University which is licensed under a Creative Commons Attribution-NonCommercial 4.0 International License. Preamble The Teaching and Learning Centre at UPEI has been engaging in conversations around the use of generative artificial intelligence and identified a need for institutional guidance for instructors prior to the start of the fall semester at the University of Prince Edward Island. The original version of these guidelines was developed by the Task Force on Generative AI in Teaching and Learning at McMaster University. The guidelines developed for UPEI were shared with a small group of instructors and administrators in August 2023 to adapt them to the UPEI context. We gratefully acknowledge the feedback these individuals provided. Over the fall 2023 semester the Generative Artificial Intelligence Taskforce (GAIT) was created and tasked with reviewing these guidelines as well as the exploration of challenges, risks and opportunities associated with Gen AI in teaching and learning at UPEI. These guidelines will continue to be updated as UPEI explores additional topics and as technology rapidly changes. Members of the Generative Artificial Intelligence Taskforce (GAIT) invite feedback and suggestions on these guidelines through this form. Feedback collected this semester on experiences, questions and concerns about using generative AI in teaching and learning will inform further updates as developments surrounding generative AI are dynamic. It is expected these guidelines will be updated again in time for spring course preparation. This current version was updated in December 2023. Potential policy changes implied by these guidelines will be addressed by the relevant governance bodies. Institutional policies take precedence over these recommendations. UPEI acknowledges the costs of generative AI arising from significant ethical issues related to academic integrity, labour, intellectual and artistic property rights in the data sets, and the environmental impacts of training large AI models (Lawton, 2023; Li, et al., 2023; Trust, n.d.). One goal of the Generative AI Task Force (GAIT) is to educate users regarding these costs and explore ways of mitigating their impact. 1 What is GenAI? Generative artificial intelligence uses models that learn the patterns and structure of their input training data and then generate new outputs (text, images, or other media) that have similar characteristics. Provisional Principles These overarching provisional principles have guided the development of these recommendations and will continue to be updated through conversations with our campus community. • Students want to learn, and instructors want to support their learning. • Participatory learning – learning which happens in relationships and community – continues to be a valuable and vital way for students to learn. • Assessments that require students to document the process of learning continue to be meaningful for student learning. • Generative AI poses risks, as well as opportunities. Individuals will have different reactions and different expectations for the technology. • Disciplinary differences and departmental cultures will vary around the use of generative AI. Provisional Guidelines 1. UPEI’s existing academic integrity regulations apply when using generative AI. Read Regulation 20 from the Undergraduate Academic Regulations on the UPEI website. For Graduate students it is Regulation 6 from the Graduate Academic Regulations. 2. Instructors have the freedom to choose whether or not to use generative AI tools for the teaching and learning processes, and to determine if generative AI will be used in course design, activities, and assessments. If an instructor chooses to implement generative AI, the decision should be based on course learning outcomes, instructors’ individual interests, and conventions and expectations of the discipline. As with any pedagogical tool or approach, instructors should weigh the benefits of incorporating generative AI into their courses against any risks inherent to the tool or approach. Instructors should also take into account the rapidly evolving nature of generative AI technology and reassess the opportunities and risks of any tool or approach on a regular basis. 3. Instructors with courses that incorporate generative AI should: • Build their own AI literacy. • Ensure the incorporation of generative AI will support core learning outcomes and offer meaningful learning. 2 • Describe or discuss with students the strengths, limitations, and ethical considerations of the technology, including factual inaccuracies and gaps, societal biases present in the training data, and the rationale for using generative AI in the course. • Recommendations for instructors to consider when incorporating generative AI into courses for student use. 4. 5. Individual instructors should clearly communicate to students if and to what extent generative AI is acceptable in the course as well as how it should be acknowledged or cited. It's recommended that instructors be very clear about their expectations regarding generative AI, and explicit when providing assignment instructions. To help reduce confusion, ensure these expectations are communicated in various ways, such as including them in course syllabi, on Moodle, instruction guidelines and repeated in class. Explain how different instructors can have different expectations for AI tools, and if use is permitted by one instructor, this does not mean AI tools will be permitted by others. Instructors should ensure that all students have a fair opportunity to gain access to the same set of features for any tools required in the course, which could mean choosing free tools or pursuing enterprise licensing. Any required subscriptions should be disclosed at the beginning of the course. Alternatives should be provided for Generative AI tools that are restricted to users 18+ (e.g., ChatGPT) and for situations where students have concerns about privacy or other terms and conditions. 6. Instructors who include assessments that incorporate generative AI should: • Consider including reflective components that invite students to comment on the use of/experience with generative AI in the assessment. • Explicitly review criteria and/or rubrics in ways that demonstrate how the use of generative AI is being assessed (see the TLC Instructional Resources Hub for examples). • Foster a learning environment that promotes academic integrity in all course learning activities. 7. Students may opt-out of assessments that require the use of generative AI in exceptional circumstances as approved by the course instructor. In these cases, students will not face academic penalty, but will be required to provide alternative and equivalent evidence of their learning as proposed to, and agreed to by, the course instructor. 8. Assessment alternatives that may be less susceptible to the use of generative AI include: oral exams, presentations followed by a Q and A, invigilated/in-class assessments, practical tests, assessments that incorporate class discussion/activities, and process-based work. 3 9. If instructors use generative AI in their course and teaching materials, they should explain in the course outline and/or materials the extent to which generative AI has been used. Instructors are responsible for the quality, ethics, and relevance of all of their course and teaching materials, including those produced by generative AI tools. Instructors using generative AI should take reasonable efforts (e.g., updating associated digital literacies) to mitigate adverse impacts to quality and ethical instruction. 10. Instructors incorporating generative AI should be aware of the privacy policies and user agreements of each generative AI tool and alert students to these policies. 11. Third-party tools designed to detect AI-generative text should not be used to check student work, as current evidence demonstrates that third-party AI-detection tools do not reliably work to detect text generated by artificial intelligence. 12. If you suspect student work may have violated the academic integrity policy, please review the steps to take and refer to the undergraduate and graduate calendars. You may want to use check out this educator resource on conducting a discovery interview with a student to understand the situation. 13. Consider risks before submitting student work to generative AI tools. Submitting a student’s work to AI tools is a breach of the student’s privacy and intellectual property rights and requires the consent of the student. More guidance on this is forthcoming. GAIT intends to continue dialogues with various units and Faculties across campuses, as well as between post-secondary institutions to refine and expand these guidelines as new information and technology emerges, and as we learn to work with these technologies. One example includes ongoing work to explore privacy impact assessments and security evaluations on recommended generative AI tools. GAIT recognizes that the Gen Ai landscape can change rapidly. These guidelines will be updated accordingly, and changes communicated with the campus community. The Teaching and Learning Centre (TLC) will continue to provide training and resources for instructors on how to use generative AI effectively. Instructors can email TLC@upei.ca for support or book an appointment with an Instructional Designer. Additional options for • Find responses to several FAQs around Gen AI the Instructional Resources Hub on the TLC website. • Refer to resources for faculty to talk with students about generative AI available through the Instructional Resources Hub on the TLC website. • See the TLC Newsletters delivered to your email inbox (also available on the TLC website). • Watch Campus Notices or check the TLC learning events calendar on the website for current • workshops. Request a 1-1 consultation and connect with members of the TLC team by emailing TLC@upei.ca. 4</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1566</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -857,6 +1161,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>The Sedona Conference Journal Volume 26 Forthcoming 2025 Navigating AI in the Judiciary: New Guidelines for Judges and Their Chambers Hon. Herbert B. Dixon Jr., Hon. Allison H. Goddard, Maura R. Grossman, Hon. Xavier Rodriguez, Hon. Scott U. Schlegel &amp; Hon. Samuel A. Thumma February 2025 Recommended Citation: Hon. Herbert B. Dixon Jr. et al., Navigating AI in the Judiciary: New Guidelines for Judges and Their Chambers, 26 SEDONA CONF. J. 1 (forthcoming 2025), https://thesedonaconference.org/sites/default/files/publications/Navigating% 20AI%20in%20the%20Judiciary_PDF_021925.pdf. Copyright 2025, The Sedona Conference For this and additional publications see: https://thesedonaconference.org/publications. THE SEDONA CONFERENCE JOURNAL 2/24/2025 11:17 AM NAVIGATING AI IN THE JUDICIARY: NEW GUIDELINES FOR JUDGES AND THEIR CHAMBERS Hon. Herbert B. Dixon, Jr., Hon. Allison H. Goddard, Prof. Maura R. Grossman, Hon. Xavier Rodriguez, Hon. Scott U. Schlegel, and Hon. Samuel A. Thumma Five judges and a lawyer/computer science professor walked into a bar . . . well, not exactly. But they did collaborate as members of the Working Group on AI and the Courts as part of the ABA’s Task Force on Law and Artificial Intelligence to develop the following guidelines for responsible use of AI by judicial officers. The guidelines reflect the consensus view of these Working Group members only, and not the views of the ABA, its Law and AI Task Force, The Sedona Conference, or any other organizations with which the authors may be affiliated. The authors include: • Dr. Maura R. Grossman, a Research Professor in the Cheriton School of Computer Science at the University of Waterloo and an Adjunct Profes- sor at Osgoode Hall Law School of York Univer- sity, who serves as a special master in both U.S. state and federal court; • Hon. Herbert B. Dixon, Jr., Senior Judge of the Superior Court of the District of Columbia; • Hon. Allison H. Goddard, U.S. Magistrate Judge of the U.S. District Court for the Southern Dis- trict of California; • Hon. Xavier Rodriguez, U.S. District Judge of the U.S. District Court for the Western District of Texas; NAVIGATING AI IN THE JUDICIARY: NEW GUIDELINES 2/24/2025 11:59 AM 2 THE SEDONA CONFERENCE JOURNAL [Vol. 26 • Hon. Scott U. Schlegel, Judge of the Louisiana Fifth Circuit Court of Appeal; and • Hon. Samuel A. Thumma, Judge of the Arizona Court of Appeal, Division One. We hope you will find these guidelines useful in your work as judges. They provide a framework for how you can use AI and Generative AI responsibly as judicial officers. THE SEDONA CONFERENCE JOURNAL 2/24/2025 11:17 AM 2025] NAVIGATING AI IN THE JUDICIARY 3 Guidelines for U.S. Judicial Officers Regarding the Responsible Use of Artificial Intelligence These Guidelines are intended to provide general, non-tech- nical advice about the use of artificial intelligence (AI) and gen- erative artificial intelligence (GenAI) by judicial officers and those with whom they work in state and federal courts in the United States. As used here, AI describes computer systems that perform tasks normally requiring human intelligence, often us- ing machine-learning techniques for classification or prediction. GenAI is a subset of AI that, in response to a prompt (i.e., query), generates new content, which can include text, images, sound, or video. While the primary impetus and focus of these Guide- lines is GenAI, many of the use cases that are described below may involve either AI or GenAI, or both. These Guidelines are neither intended to be exhaustive nor the final word on this sub- ject. I. FUNDAMENTAL PRINCIPLES An independent, competent, impartial, and ethical judiciary is indispensable to justice in our society. This foundational prin- ciple recognizes that judicial authority is vested solely in judicial officers, not in AI systems. While technological advances offer new tools to assist the judiciary, judicial officers must remain faithful to their core obligations of maintaining professional competence, upholding the rule of law, promoting justice, and adhering to applicable Canons of Judicial Conduct. In this rapidly evolving landscape, judicial officers and those with whom they work must ensure that any use of AI strength- ens rather than compromises the independence, integrity, and impartiality of the judiciary. Judicial officers must maintain im- partiality and an open mind to ensure public confidence in the justice system. The use of AI or GenAI tools must enhance, not diminish, this essential obligation. NAVIGATING AI IN THE JUDICIARY: NEW GUIDELINES 2/24/2025 11:59 AM 4 THE SEDONA CONFERENCE JOURNAL [Vol. 26 Although AI and GenAI can serve as valuable aids in per- forming certain judicial functions, judges remain solely respon- sible for their decisions and must maintain proficiency in under- standing and appropriately using these tools. This includes recognizing that when judicial officers obtain information, anal- ysis, or advice from AI or GenAI tools, they risk relying on ex- trajudicial information and influences that the parties have not had an opportunity to address or rebut. The promise of GenAI to increase productivity and advance the administration of justice must be balanced against these core principles. An overreliance on AI or GenAI undermines the es- sential human judgment that lies at the heart of judicial deci- sion-making. As technology continues to advance, judicial offic- ers must remain vigilant in ensuring that AI serves as a tool to enhance, not replace, their fundamental judicial responsibilities. Judicial officers and those with whom they work should be aware that GenAI tools do not generate responses like tradi- tional search engines. GenAI tools generate content using com- plex algorithms, based on the prompt they receive and the data on which the GenAI tool was trained. The response may not be the most correct or accurate answer. Further, GenAI tools do not engage in the traditional reasoning process used by judicial of- ficers. And, GenAI does not exercise judgment or discretion, which are two core components of judicial decision-making. Us- ers of GenAI tools should be cognizant of such limitations. Users must exercise vigilance to avoid becoming “anchored” to the AI’s response, sometimes called “automation bias,” where humans trust AI responses as correct without validating their results. Similarly, users of AI need to account for confirmation bias, where a human accepts the AI results because they appear to be consistent with the beliefs and opinions the user already has. Users also need to be aware that, under local rules, they THE SEDONA CONFERENCE JOURNAL 2/24/2025 11:17 AM 2025] NAVIGATING AI IN THE JUDICIARY 5 may be obligated to disclose the use of AI or GenAI tools, con- sistent with their obligation to avoid ex parte communication. Ultimately, judicial officers are responsible for any orders, opinions, or other materials which are produced in their name. Accordingly, any such work product must always be verified for accuracy when AI or GenAI is used. II. JUDICIAL OFFICERS SHOULD REMAIN COGNIZANT OF THE CAPABILITIES AND LIMITATIONS OF AI AND GENAI GenAI tools may use prompts and information provided to them to further train their model, and their developers may sell or otherwise disclose information to third parties. Accordingly, confidential or personally identifiable information (PII), health data, or other privileged or confidential information should not be used in any prompts or queries unless the user is reasonably confident that the GenAI tool being employed ensures that in- formation will be treated in a privileged or confidential manner. For all GenAI tools, users should pay attention to the tools’ set- tings, considering whether there may be good reason to retain, or to disable or delete, the prompt history after each session. Particularly when used as an aid to determine pretrial re- lease decisions, consequences following a criminal conviction, and other significant events, how the AI or GenAI tool has been trained and tested for validity, reliability, and potential bias is critically important. Users of AI or GenAI tools for these forego- ing purposes should exercise great caution. Other limitations or concerns include: • The quality of a GenAI response will often de- pend on the quality of the prompt provided. Even responses to the same prompt can vary on different occasions. • GenAI tools may be trained on information gathered from the Internet generally, or NAVIGATING AI IN THE JUDICIARY: NEW GUIDELINES 2/24/2025 11:59 AM 6 THE SEDONA CONFERENCE JOURNAL [Vol. 26 proprietary databases, and are not always trained on non-copyrighted or authoritative le- gal sources. • The terms of service for any GenAI tool used should always be reviewed for confidentiality, privacy, and security considerations. GenAI tools may provide incorrect or misleading infor- mation (commonly referred to as “hallucinations”). Accord- ingly, the accuracy of any responses must always be verified by a human. III. POTENTIAL JUDICIAL USES FOR AI OR GENAI Subject to the considerations set forth above: • AI and GenAI tools may be used to conduct le- gal research, provided that the tool was trained on a comprehensive collection of reputable le- gal authorities and the user bears in mind that GenAI tools can make errors; • GenAI tools may be used to assist in drafting routine administrative orders; • GenAI tools may be used to search and sum- marize depositions, exhibits, briefs, motions, and pleadings; • GenAI tools may be used to create timelines of relevant events; • AI and GenAI tools may be used for editing, proofreading, or checking spelling and gram- mar in draft opinions; • GenAI tools may be used to assist in determin- ing whether filings submitted by the parties have misstated the law or omitted relevant le- gal authority; THE SEDONA CONFERENCE JOURNAL 2/24/2025 11:17 AM 2025] NAVIGATING AI IN THE JUDICIARY 7 • GenAI tools may be used to generate standard court notices and communications; • AI and GenAI tools may be used for court scheduling and calendar management; • AI and GenAI tools may be used for time and workload studies; • GenAI tools may be used to create unoffi- cial/preliminary, real-time transcriptions; • GenAI tools may be used for unofficial/prelim- inary translation of foreign-language docu- ments; • AI tools may be used to analyze court opera- tional data, routine administrative workflows, and to identify efficiency improvements; • AI tools may be used for document organiza- tion and management; • AI and Gen AI tools may be used to enhance court accessibility services, including assisting self-represented litigants. IV. IMPLEMENTATION These Guidelines should be reviewed and updated regularly to reflect technological advances, emerging best practices in AI and GenAI usage within the judiciary, and improvements in AI and GenAI validity and reliability. As of February 2025, no known GenAI tools have fully resolved the hallucination prob- lem, i.e., the tendency to generate plausible-sounding but false or inaccurate information. While some tools perform better than others, human verification of all AI and GenAI outputs remains essential for all judicial use cases.</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1771</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -869,6 +1191,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>The University supports the responsible use of generative AI (GenAI) when helpful to further its mission, the preservation, advancement, and dissemination of knowledge. These guidelines provide general advice for the UW community and can help you use GenAI responsibly by aligning with UW’s values and privacy principles. Additional GenAI resources based on use case: - Research: Review the Effective and Responsible Use of AI in Research page. - Teaching: Refer to guidance on integrating GenAI while maintaining academic standards. - Health care and medical research: Review UW Medicine’s GenAI guidelines. (Net ID required) Key Takeaways - Only UW-approved services and applications may be used with University data. The use of unapproved services, applications, and the unauthorized release of university data could result in violations of policy or law for which you or the University may be liable. UW-IT can review tools and use cases to help inform unit decisions about whether to approve a service or application. - All use of GenAI must comply with all relevant UW policies and standards. - Complimentary training, tool review, architectural guidance, and security assessments are available via the UW-IT AI website. - You are ultimately responsible and accountable for your use of GenAI and all outcomes derived from it. - UW’s Appropriate Use Policy and related security and privacy policies apply to the use of all technologies, including GenAI. - Students must adhere to policies and rules applicable to their course or project. Course instructors have the discretion to allow, prohibit, or put parameters around the use of GenAI. - You must review GenAI output before using or publishing it and are responsible for any harm caused by your use of GenAI. - GenAI may enhance, but does not replace, human judgment, particularly in decision-making affecting individuals or communities. - Avoid GenAI use that may reinforce inappropriate biases or create barriers for underrepresented groups. - Disclosing GenAI use is often advisable and may be mandatory; failure to do so may have serious consequences, particularly in published research or coursework. - Maintain detailed records of GenAI use, especially when personal data is involved. Document relevant processes in the TrustArc personal data inventory. - Ensure compliance with records protection and preservation laws, including Records Management Services AI Guidance. - Data intended for public consumption (classification Level 1: All Audiences) can be used with GenAI.. - Do not use data that is restricted (classification Level 2: Limited Audience through Level 4: Special Handling Requirements), unless appropriate security and privacy controls, including contractual protections when working with other parties are in place. - If you want to use GenAI for high-risk processes like hiring, admissions, or performance evaluations, contact uwprivacy@uw.edu for a privacy impact assessment. - UW-IT AI Resources - AI@UW - UW AI Community of Practice - UW AI Task Force, Town Halls, and AI Perspectives Speaker Series - UW Health Sciences Library AI Overview - Artificial Intelligence at the Allen School of Computer Science and Engineering - University of Washington Bothell &amp; Cascadia College AI Guide for Students - Internet2 NET+ AI Updates - EDUCAUSE Artificial Intelligence Library - Interim Guidelines for Purposeful and Responsible Use of Generative Artificial Intelligence (AI) in Washington State Government - Washington State Attorney General Artificial Intelligence Task Force and Report - City of Seattle Generative Artificial Intelligence Policy - City of Seattle Responsible Artificial Intelligence Program - City of Tacoma Generative Artificial Intelligence Guidelines Report suspected security and privacy incidents immediately: - Urgent issues: Call 206-221-5000. - Other incidents: Email uwprivacy@uw.edu. - General questions: Email help@uw.edu.</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>587</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -881,6 +1221,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Addressing the Limitations of Using Generative AI for Learning Within the academic technology ecosystem, generative AI is increasingly everywhere. The Office of Academic Technology (OAT) is the central authority for evaluating learning technologies on campus, including generative AI. OAT supports the responsible adoption of generative AI for academic use, including for teaching and learning. Responsible AI Use in Teaching and Learning UT Austin defines responsible use of AI in teaching and learning as using AI in ways that foster the achievement of learning outcomes. That means using generative AI in ways that advance what students should know, be able to do and the attitudes they should develop as a result of a learning experience. At the same time, responsible AI use on the Forty Acres means not using generative AI in ways that would negate or inhibit the realization of those outcomes. UT encourages faculty, students and staff to be both AI-Forward and AI-Responsible. On the forward side, UT Austin provides access to a variety of tools and resources that foster the adoption of AI to achieve learning outcomes. On the responsible side, it emphasizes the critical importance of AI literacy and awareness of “the Big 6” limitations of using AI for learning (see below). Engaging in AI Forward – AI Responsible Learning Part of responsible adoption involves creating opportunities for the Longhorn community to gain literacy on the benefits and limitations of generative AI use in education. This starts with having a clear definition of what generative AI is and what it is not. What is generative AI? Generative AI refers to models that generate or create new or original output (text, code, images, videos, music, etc.) using pre-existing data the model has been trained on. The purpose of generative AI is to create brand-new content. Synthetic content can lead to wonderful, creative output — and that same output is often rife with limitations. Being AI-forward requires being aware of and taking action to mitigate the limitations below. The Big 6: Six Key Limitations of Using AI for Learning 1.0 Privacy and Security UT Austin supports data that is publicly available or defined as Published University information. When learning with AI, protect yourself and others by only using trusted vendors who allow you to disable chat history or model training easily. All students, faculty and staff must always follow the University’s generative AI acceptable use policy, which notes that inputting confidential or controlled university data is not allowed unless there is a University contract in place that protects such data. 2.0 Hallucinations and Deception Hallucinations are common and occur when generative AI produces content that is untrue or factually inaccurate. For example, bots such as ChatGPT might report that you have only 37 rows of data in a data set when there are 72. AI can also be deceptive in a variety of ways, including agreeing with users’ input or opinions even when they are incorrect or problematic, wrapping feedback in convincing, authoritative language that makes it appear credible. Such interactions can implicitly discourage critical analysis and discernment, leading learners to have more confidence in their knowledge or skills than they should. Always use more traditional approaches to research to confirm and verify facts. 3.0 Misalignment Misalignment occurs when a user prompts generative AI applications to produce a specific output, and the AI ends up producing an unexpected or undesired result. For example, when asking a bot to give you the Excel formula for merging two missing cells, it may give you the formula for splitting two cells instead. Misalignment is particularly problematic with image generation but also occurs within synthetic or AI-generated text. Careful prompt engineering helps address misalignment in text-based AI, but you will not be able to avoid it completely. Humans should always evaluate the output of generative AI with critical thinking skills. 4.0 Bias Because humans train them, generative AI output has both explicit and implicit biases baked into it, including stereotypes. It won’t be possible to entirely avoid bias in generative AI, just as it is not possible to avoid it in the real world, but a few small tips can help you engage with greater awareness. Educate yourself on the nature of implicit bias. Be aware that because humans train the models, they will reproduce our biases. Be skeptical and avoid over reliance on the models for any project. When you observe output from AI that is clearly biased or laced with stereotypes, report it to the vendor of the app you are using. 5.0 Ethics Al models have several ethical considerations, including digesting intellectual property, spreading misinformation, and using gen Al to produce new works or results without contribution. Other ethical considerations relate to the labor used to generate the models, the environmental impacts of generative Al, and the business ethics of releasing Al models for revenue generation without a clear understanding of the impact on society. Similar to bias, it is essential to be aware of the ethical concerns of using Al so that you can engage in a transparent manner. 6.0 Cognitive Offloading Cognitive offloading is the process of humans using external tools to reduce the demand or “cognitive load” of completing tasks (Risko and Gilbert, 2016). Technologies such as generative AI chatbots can help increase productivity through cognitive offloading; however, if you do not employ those freed-up resources for other tasks, the overuse of generative AI could potentially “diminish specific cognitive skills” (León-Dominguez, 2024). Engaging in human activities such as actively critiquing and evaluating output from generative AI can help protect problem-solving and creative and critical thinking skills. Other things you can do to avoid the downsides of cognitive offloading include engaging in transformation of gen Al output to make it your own. For example, evaluate the output for hallucinations, misalignment, bias, or ethics and then transform that output to make it authentically yours with your original thoughts, opinions, knowledge; or work. Have you adopted AI Forward - AI Responsible practices? The Office of Academic Technology is interested in learning from you. Please share your examples with the OAT using the form linked below. If you have questions or comments about generative AI for learning, please email us at oat@utexas.edu. Share Your ExamplesFebruary 21, 2024</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1036</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -893,6 +1251,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Page not found - Artificial Intelligence (AI) at Purdue University Purdue Virtual Assistant Hi! I'm the Purdue Virtual Assistant. I can help answer your questions about IT Services. How can I help you? Skip to content 404 ERROR We’re sorry you were not able to find the page you were looking for. Search Search Major Tuition &amp; Costs Schedule a Visit Boilermakers’ Stories Apply</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>64</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -905,6 +1281,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CU Boulder Guidelines Implementation of AI is subject to all applicable CU Boulder policies, standards and guidelines. If you have any questions about how to assess the implications of AI for your use case, please email security@colorado.edu. As the uses and ramifications of AI as a technology tool continue to evolve and be better understood, so too are the effects it will have on data security in higher education. This page is intended to guide our community as you consider using AI on the CU Boulder campus. Below are some guidelines for limiting data security risk while using generative AI tools: - Use AI tools available and recommended for use on the CU Boulder campus found on the Office of Vice Chancellor for IT and Chief Information Officer website. If you have any questions about access to these tools, please email oithelp@colorado.edu. - AI tool use is only approved for data classified as Public (see CU's Data Classification Standard for more information). The standard CU Boulder IT security contractual provisions may not be in place by default. If you intend to share Confidential or Highly Confidential information with an AI-based service (or any service for that matter), the service needs to be reviewed for compliance with CU’s data security requirements via ICT Review. Information shared with Generative AI tools using default settings is not private and could expose proprietary or sensitive information to unauthorized parties. - Review AI tool output to verify integrity: the output should be accurate and not incomplete, incorrect, or biased. - AI-generated computer code should NOT be used for institutional IT systems and services unless it has been reviewed by a human for accuracy, security (ensuring no vulnerabilities are introduced), and efficiency. - Faculty, staff, and students using these tools must read and understand the AI tool vendor’s policies and become familiar with the limitations of use and how the vendor plans to store, process, or handle CU’s data. For example, if using ChatGPT, you will need to read and comply with OpenAI’s Policies because there are some limitations regarding how the product may be used. Additional Resources With any new technology, there are always risks when utilizing it. If you decide to utilize or explore AI tools, you will need to consider the potential positive and/or negative impacts it will have on the campus, your department, and your personal life. A great framework to help you determine whether an AI tool is reliable and/or truthful is the NIST AI Risk Management framework. Below is a high-level overview of the framework. | Valid &amp; Reliable | Trustworthy AI produces accurate results within expected timeframes. | |---|---| | Safe | Trustworthy AI produces results that conform to safety expectations for the environment in which the AI is used (e.g., healthcare, transportation, etc.). | | Fair &amp; Bias is Managed | Bias can manifest in many ways; standards and expectations for bias minimization should be defined prior to using AI. | | Secure &amp; Resilient | Security is judged according to the standard triad of confidentiality, integrity, and availability. Resilience is the degree to which the AI can withstand and recover from attack. | | Transparent &amp; Accountable | Transparency refers to the ability to understand information about the AI system itself, as well as understanding when one is working with AI-generated (rather than human-generated) information. Accountability is the shared responsibility of the creators/vendors of the AI as well as those who have chosen to implement AI for a particular purpose. | | Explainable &amp; Interpretable | These terms relate to the ability to explain how an output was generated, and how to understand the meaning of the output. | | Privacy Enhanced | This refers to privacy from both a legal and ethical standpoint. This may overlap with some of the previously listed attributes. | *Please Note: Appendix B of the NIST framework discusses risks unique to AI. It recommends you review these risks to understand how AI risk differentiates from other more familiar technological risks. To assist you in your consideration and implementation of these guidelines, reading material on the topic of AI concerns can be found on the following webpages:</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>695</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -917,6 +1311,24 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Working group aims to ensure trust in research Guidelines for the use of AI in science Science thrives on reproducibility, transparency, and accountability, and trust in research stems in particular from the fact that results are valid regardless of the institution where they were produced. Furthermore, the underlying data of a study must be published, and researchers must take responsibility for their publications. But what if AI is involved in the research? Experts have long used AI tools to design new molecules, evaluate complex data, and even generate research questions or prove a mathematical conjecture. AI is changing the face of research, and experts are debating whether the results can still be trusted. Recommendations published in the scientific journal PNAS Five principles should continue to ensure human responsibility in research, according to an interdisciplinary working group with members from politics, business, and academia published in the latest issue of the journal Proceedings of the National Academies of Sciences (PNAS). Urs Gasser, Professor for Public Policy, Governance and Innovative Technology at TUM, was one of the experts. The recommendations in brief: - Researchers should disclose the tools and algorithms they used and clearly identify the contributions of machines and humans. - Researchers remain responsible for the accuracy of the data and the conclusions they draw from it, even if they have used AI analysis tools. - AI-generated data must be labeled so that it cannot be confused with real-world data and observations. - Experts must ensure that their findings are scientifically sound and do no harm. For example, the risk of the AI being "biased" by the training data used must be kept to a minimum. - Finally, researchers, together with policymakers, civil society and business, should monitor the impact of AI and adapt methods and rules as necessary. "Signal effect for researchers" "Previous AI principles were primarily concerned with the development of AI. The principles that have now been developed focus on scientific applications and come at the right time. They have a signal effect for researchers across disciplines and sectors," explains Urs Gasser. The working group suggests that a new strategy council - based at the US National Academy of Sciences, Engineering and Medicine - should advise the scientific community. "I hope that science academies in other countries - especially here in Europe - will take this up to further intensify the discussion on the responsible use of AI in research," says Urs Gasser. - Blau, W. et al. PNAS 2024 Vol. 121 (22) e2407886121 Technical University of Munich Corporate Communications Center - Dr. Jeanne Rubner - jeanne.rubner @tum.de - +49 89 289 25283 - presse @tum.de - Teamwebsite Contacts to this article: Prof. Dr. Urs Gasser Technical Univeristy of Munich Chair of Public Policy, Governance and Innovative Technology School of Social Sciences and Technology (SOT) urs.gasser(at)tum.de</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>468</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -929,6 +1341,24 @@
           <t>Unknown</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Prof. Dr. Volker Markl Chair of Database Systems and Informa:on Management (DIMA) Technische Universität Berlin June 7, 2023 Policy Statement. 1. Effective immediately, as a general policy, we do not permit the use of ChatGPT or other large language models (LLMs) in DIMA for the preparation of research papers, technical reports, theses, PhD dissertations, or any other original work. 2. The use of LLMs shall be strictly prohibited, as it on the one hand might prevent a fair grading of student performance, and on the other hand present the very serious risk of plagiarism. Similar to copying code from Stack Overflow, there is a spectrum with respect to when plagiarism occurs. However, in the scientific world one should be particularly aware and be careful with respect to this. 3. Every DIMA member should be aware of this policy and also point this out to your students and mentees. For course/project reports and theses, we will require students to sign a form that they confirm that they did not use any LLM tools, such as ChatGPT for the writing of their theses. Of course, this also applies to research papers and PhD dissertations. 4. Please be mindful of this matter and bring any violations of this policy to my attention, so that DIMA will be an environment free of the risk of plagiarism. Use of AI Tools for Course Assignments, Theses, Research Papers, and PhD Dissertations</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>235</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -941,6 +1371,24 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Policy on the Use of Generative AI in Research Status December 2024 In addition to the presentation on this website, you can also download the AI policy as a PDF. With this policy, the University of Freiburg would like to raise awareness for the conscious use of generative AI in the research context and provide recommendations on how to use the corresponding tools. The Central Data Facility supports all researchers of the University of Freiburg with the implementation of university policies. Contents - Preface - Introduction/Background - Recommendations for Researchers at the University of Freiburg - Further Information - List of Contributors - Contact Persons - References Preface The application of generative artificial intelligence (genAI) in research offers many opportunities, but these must be weighed against risks. The University of Freiburg developed this policy in accordance with its mission statement and the structural and development plan “Shaping Digital Transformation” (2023, 1.), based on the “Living guidelines on the responsible use of generative AI in research” of the EU Commission” (2024, 2.) and the Guidelines of the German Research Foundation (2023, 3.) for dealing with generative models for text and image generation. This document is based on the issues discussed during the event “ChatGPT – AI Tools in Research” (2023, 4.). A responsible and informed approach to genAI aims to prevent misuse and to ensure a sensible use of AI in all research processes. With this policy, we aim to raise awareness for a conscious use of genAI in research contexts and provide recommendations for the use of corresponding tools. Guidelines for the use of AI-based tools in study and teaching, as well as in administration, are currently in development. This policy must be understood as a snapshot since the development of AI is currently difficult to assess and changes will likely become necessary. Therefore, this document will be updated regularly. Introduction/Background What is “generative artificial intelligence”? The term “generative AI” describes AI systems that can autonomously create novel content in response to prompts. These systems learn from data received during their training phase and use this information to generate outputs. The basis for this are so-called Large Language Models (LLMs), which are created using very large datasets and highly complex calculations. Opportunities and Risks of AI The use of genAI in text and data processing provides the ability to quickly and conveniently create texts, images, videos, and code. Chatbots based on generative language models, such as ChatGPT or You.com, excel at generating texts with a wide range of applications from literature reviews to generating programming code or debugging it. AI-based annotation of audio/video recordings or simultaneous translations are already widely used. Extracting data from (multiple) publications and summarizing them is very easy and quick with LLMs. As a translation tool, LLMs potentially provide equal opportunities for researchers who are less proficient in the language used. However, risks exist as genAI is not neutral and may contain (derogatory) discrimination based on training data (so-called “biases”) or provide plausible but incorrect answers that do not correspond to facts (so-called “hallucinations”). This can promote the creation and dissemination of misinformation. Moreover, scientific misconduct, such as failing to disclose the use of genAI, poses a risk of misuse, as does the potential infringement of intellectual property. The linguistic quality of the generated results is often so good that the outcomes are hardly distinguishable from those created by humans. Additional risks for research may arise from the lack of transparency of tools, fees for accessing services, the use of unknown input data, or the concentration on a few providers. Recommendations for Researchers at the University of Freiburg Transparency Researchers should disclose which AI systems they have used and clearly label their contributions. Responsibility and Accountability Researchers remain responsible for the accuracy of the generated data, texts, and results, even if they are AI-generated or AI-based. Labelling and Documentation It must be indicated whether data and the results derived from them are AI-generated. The origin and use of the utilized methods, AI systems, and data sources must be fully documented, ideally in a way that the results can be reproduced. Yet, for solutions that are only accessible via API (Application Programming Interface) (such as ChatGPT), reproducibility is not always guaranteed, as the service changes over time, and the stochastic nature of LLMs can lead to differing outputs. Avoiding Bias Researchers must ensure that their results are scientifically grounded and must consider and, if necessary, avoid potential harm scenarios. The use of genAI also carries the risk of biases that can lead to discriminatory decisions. In relation to the training data used, systematic bias that stems from societal conditions, where certain prejudices are inherent in the data, must be avoided. Bias during the data collection or data annotation process, or in the choice of algorithm or system design, should be minimized. Authorship in Publications Related to AI The Committee on Publication Ethics (2023, 5.) states clearly that AI systems cannot be authors in scientific publications, among other reasons because they are not legal persons. The use of AI tools must be transparently listed in the methods section of publications. Only natural persons can appear as authors in scientific publications. They must ensure that the use of generative models does not infringe on anyone else’s intellectual property and that no scientific misconduct, such as plagiarism, occurs. Reference is made here to the regulations of the Albert Ludwig University for ensuring academic integrity (2022, 6.). The potential for generating texts, e.g., as templates for modifications by authors, can be used as long as this is documented and the authors take responsibility for the content, results (such as codes), and references. In publications, the rights of publishers or copyright holders must be respected, e.g., when data is provided to commercial vendors. It is critically important to assess whether the sharing of data can be free of charge if it involves a commercial provider. DFG Application Process, Review The use of generative models in applications to funding by the DFG is evaluated by the DFG itself as neither positive nor negative. However, when preparing reviews, the DFG (2023, 3.) prohibits the use of generative models with regard to the confidentiality of the review process. Documents submitted for review are confidential and must not be used as input for generative models. See also the section “Authorship in Publications Related to AI” in this policy. Promoting and Supporting the Responsible Use of genAI The responsible use and further development of generative AI should consider the limits of the technology, its environmental impact, and its societal effects. Based on liberal democratic values, discrimination must be avoided in the development and use of genAI, diversity and fairness must be ensured, and harm to persons, lives, and the environment must be averted. Last but not least, considerations about energy consumption by the use of AI systems, which require significant computational resources particularly for training, should be taken into account (see examples here). Orientation on Ethical Issues Researchers should consider ethical principles when using genAI. They must be aware of the risk of abuse even when using or developing AI tools. This includes abuse scenarios for unlawful military use or use for criminal activities (Dual Use Research of Concern). In doubtful cases, especially in instances with a high risk of abuse, researchers should consult the Committee for Responsibility in Research (Kommission für Verantwortung in der Forschung, KVF), which can discuss such issues in an interdisciplinary setting and advise researchers. See also here: Information on Good Research Practice at the University of Freiburg. Compliance with Legal Requirements Compliance with data protection regulations and the protection of intellectual property rights through responsible and appropriate handling of personal data must be guaranteed. In addition, regulations on export control law must be adhered to when publishing or conducting research across borders, and relevant medical device regulations must be observed if applicable. Further Information AI Tools at the University of Freiburg (intranet access required) The University of Freiburg provides its members with GDPR-compliant access to genAI, see here. The page also contains examples of energy consumption related to genAI. Research and Innovation in the EU Regarding AI The Commission and the countries of the European Research Area and stakeholders have jointly presented a number of guidelines to support the European research community in the responsible use of generative artificial intelligence (AI) (2.). EU AI Act The “EU Artificial Intelligence Act” (EU AI Act, 2024, 7.) addresses the rapid technological development of all AI systems and incorporates this into its legal framework. The EU AI Act aims to create reliable conditions for the research and application of AI. International Conference on Machine Learning Five principles are intended to further secure human responsibility in research, as now called for by an interdisciplinary working group with members from politics, industry, and science in the Proceedings of the National Academies of Sciences (PNAS) (2024, 8.). List of Contributors - Prof. Dr. Stefan Rensing, Vice Rector for Research and Innovation - Prof. Dr. Stefan Günther, Chief Information Officer - Prof. Dr. Frank Hutter, Professorship for Machine Learning - Prof. Dr. Silja Vöneky, Professorship for Public Law, International Law, Legal Ethics and Comparative Law, and Chair of the Committee for Responsibility in Research - Dr. Marc Herbstritt, Chief Information Security Officer - Klaus Scharpf, Data Protection Officer As a basis for the section “Recommendations for Researchers at the University of Freiburg,” individual text blocks were generated on July 9, 2024, by ChatGPT (GPT-4o) Comments from Senate members were integrated into this version following the resolution on December 18, 2024. Contact Persons References - Jahresbericht der Universität Freiburg 2023, S. 7 https://uni-freiburg.de/wp-content/uploads/Jahresbericht_der_Universitaet_Freiburg_2023.pdf (aufgerufen am 5.11.2024) - Living guidelines on the responsible use of generative AI in research (März 2024) https://research-and-innovation.ec.europa.eu/document/2b6cf7e5-36ac-41cb-aab5-0d32050143dc_en (aufgerufen am 5.11.2024) - Stellungnahme des Präsidiums der Deutschen Forschungsgemeinschaft (DFG) zum Einfluss generativer Modelle für die Text- und Bilderstellung auf die Wissenschaften und das Förderhandeln der DFG (September 2023) https://www.dfg.de/resource/blob/289674/ff57cf46c5ca109cb18533b21fba49bd/230921-stellungnahme-praesidium-ki-ai-data.pdf (aufgerufen am 5.11.2024). - ChatGPT – KI-Tools in der Forschung (Oktober 2023) https://videoportal.uni-freiburg.de/video/chatgpt-ki-tools-in-der-forschung-englisch-untertitelt/b08e66cd4ec53fba503a7f4028825d1b (aufgerufen am 5.11.2024) - Committee on Publication Ethics (COPE) (2023) https://publicationethics.org/guidance/cope-position/authorship-and-ai-tools (aufgerufen am 5.11.2024) - Ordnung der Albert-Ludwigs-Universität zur Sicherung der Redlichkeit in der Wissenschaft, Amtliche Bekanntmachungen Jahrgang 53, Nr. 31, S. 148ff (1. Juni 2022) https://uni-freiburg.de/wp-content/uploads/Uni-Freiburg-Ordnung-Redlichkeit-in-der-Wissenschaft-1.pdf (aufgerufen am 5.11.2024) - KI-Gesetz der Europäischen Kommission (2024) https://www.europarl.europa.eu/topics/de/article/20230601STO93804/ki-gesetz-erste-regulierung-der-kunstlichen-intelligenz (aufgerufen am 5.11.2024) - Blau, Wolfgang. et al. (2024), Protecting scientific integrity in an age of generative AI, Vol. 121 (22) e2407886121, PNAS.</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1735</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -953,6 +1401,24 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Status: 29 January 2025 The use of AI in your studies offers many opportunities. Generative AI, a sub-area of machine learning, can create content such as texts and images. This can have far-reaching changes for academic work. If used correctly, generative AI can enrich your studies. However, its use should always be understood as a support and complement and not as a substitute for independent learning, reflection and argumentation. This handout is intended to help you understand generative AI better and use it in a more reflective way. Due to the rapid pace of development, the website will be updated regularly. Only the German version of this page is legally valid. Guidelines for students 1. Be informed about the rules The teacher should decide and communicate in the first two weeks of lectures whether and to what extent AI applications may be used in the course of an examination. If no specifications are made, you can currently assume that its use is permitted as long as it has not been expressly prohibited. However, if in doubt, please ask! 2. Use generative AI responsibly 3. What AI can help with Finding ideas, researching topics and literature: AI can provide inspiration and spark creativity. AI can help to research topics, explore fields of research and find literature. Structure and time management: AI can help to structure your own learning process, organise a piece of work or plan a project. Repetition and understanding: AI can help to summarise content or explain difficult concepts. You can use generative AI to ask questions of a text. However, please note: AI also makes mistakes. Support with writing: AI can help you get into writing, find ideas for structuring texts and improve your ability to express yourself. AI can help to check for grammar and spelling mistakes and make stylistic refinements. However, make sure that the linguistic correction does not change the meaning and check the adjustments made by AI! Consistency check: AI can help you to critically check your own text, e.g. for consistent use of terms and argumentative consistency. However, independent discussion and reflection remain essential. Arguments must be developed independently and information critically scrutinised. You alone are responsible for the content and style of your text. 4. Improve your ability to use AI sensibly Prompt learning: Experiment with different questions and instructions to achieve the best possible results. Expand your skills: Use workshops, online courses or tutorials to further your training in the application of generative AI. Here you will find further information and counselling services. 5. Take a critical approach to AI Quality control: Always check the information provided by AI for accuracy. Language models often provide inaccurate or even invented sources. Check whether the sources mentioned even exist and are useful for your argumentation. Work independently with the sources. Learn to assess the value of AI-generated answers: AI-generated answers are often very well formulated and appear linguistically convincing. But they are not always factually correct or scientifically sound. The programmes are designed to give an incomplete or incorrect answer rather than no answer at all. Always check what you are being offered by AI! Practise independent thinking: Use AI results as inspiration and support, but think for yourself. Formulate your own arguments. Empower your own thoughts. 6. Observe ethical and academic integrity Comply with data protection: Do not upload any sensitive or confidential information to AI tools. Risk of unintentional plagiarism: The direct and unchecked use of AI-generated texts can lead to unintentional plagiarism. Check the generated texts carefully and do not adopt excessive amounts of text. Document and reflect on how you have worked with AI and which text passages are characterised by it. Follow the teacher´ s instructions. Cultivate a scientific ethos: The fact that unauthorised AI use may not be detected or that plagiarism or other attempts at deception may not be proven does not absolve you from working in a scientifically honest manner. Scientific research is a matter of honesty and integrity. Basically, you are responsible for the scientific quality of your text. You confirm this with your declaration of academic integrity (sample declaration of academic integrity in docx format). 7. Contribute to overcoming inequalities in studying Promoting equal opportunities in studies: AI can help you to personalise learning processes and balance out inequalities in your studies. However, students with more experience in using digital tools or with better research skills could benefit more from AI. Therefore, take advantage of courses and exchanges with fellow students to learn from their experience. Through exchange and practice, you can help to ensure that everyone benefits from AI and that existing differences in prior knowledge or digital skills are not reinforced. Regulations at the University of Erfurt on the use of generative AI for examinations On 4 December 2024, the Senate of the University of Erfurt adopted the recommendations for teachers on dealing with generative AI in teaching and examinations. In essence, it recommends active engagement with and a critical approach to generative AI in teaching and examinations. There is no and cannot be a regulation that applies to the entire university as to whether AI tools can be used for examinations. The specific design of examinations is generally at the discretion of the lecturers/examiners. They should generally communicate examination formats and examination conditions in the first two weeks of lectures. The teacher decides - whether and which AI applications are permitted in the course of an examination, - what restrictions exist - and how permitted use is to be documented and reflected upon. The University of Erfurt provides a template for a declaration of academic integrity and for a declaration of consent (template)regarding the authorised resources. Both declarations can and should be adapted by the lecturer to the respective examination. In the specific requirements for the examination, teachers who authorise the use of AI can request a critical analysis (in the form of a reflection of approx. 1 page). The examination paper should then contain a section in which you as a student state which tools you have used and reflect on how the use of AI has changed the content, structure and linguistic aspects of your examination paper. Can I use AI tools in written work (seminar papers, bachelor's, master's and master's theses)? Whether and which aids, including AI tools, you are allowed to use, how you should document and, if necessary, reflect on this and which assessment standards apply to the examination should be determined by the teacher in the first two weeks of the lecture. The declaration of consent (template) can be used for this purpose. With your declaration of academic integrity you as a student expressly declare that you have written your text independently and in accordance with academic standards, have only used authorised resources and have labelled them in accordance with the specifications. You are responsible for the content and quality of your text. Important: Observe the examination regulations! Students who demonstrably do not adhere to the specifications and use AI tools without authorisation or do not/insufficiently label them may be accused of cheating or using unauthorised aids and will receive a failing grade (5.0). A second attempt to cheat in the degree programme can lead to the loss of the right to take the examination. Can I use AI tools for written/electronic (remote) exams? Whether and which aids, including AI tools, you are allowed to use during an exam is determined by the teacher. Teachers can prohibit all aids, including the use of generative AI, during written and electronic (remote) examinations. If the use of AI tools is expressly permitted, clear guidelines must be set and compliance must be ensured by means of control mechanisms. Important: Observe the examination regulations. Students who demonstrably do not adhere to the specifications and use AI tools without authorisation and/or do not or insufficiently label them may be accused of cheating or using unauthorised aids and will receive a failing grade (5.0). A second attempt to cheat in the degree programme can lead to the loss of the right to take the examination Is my lecturer allowed to conduct oral examinations as a supplement to the written work? Since summer 2024, the framework examination regulations of the University of Erfurt allow a supplementary oral examination to the defence of the written thesis. This checks the extent to which students have actually understood the topic and explored it independently. This examination relates to the same examination content as the written paper. "In all modules [...] the module examination "h) Written paper 70% in conjunction with oral/practical examination 30%" is also part of the defence of the written paper. It is also permitted as an additional module examination for the defence of the written paper. If one of the two partial examinations is assessed with 5.0, the combined examination is deemed to have been assessed as insufficient."[1] Whether this examination format is used will be determined by the examiners in the first two weeks of lectures. A subsequent addition of an oral defence to a purely written examination is not permitted. [1] § Section 9 (6) and (9) B-RPO-2019, Section 10 (6) and (9) M-RPO-2019, Section 10 (6) and (9) MEd-RPO-2019, Section 6 (6) and (9) Theol-PO-KaTh-2021, Section 7 (8) Theol-PO-KaTh-2009</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1541</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -965,6 +1431,24 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>This guide provides orientation for all students, staff, and external parties at the University of Jena regarding the responsible use of generative artificial intelligence (AI) as a tool in professional life as well as in studies, teaching, and research. In order to use AI tools safely as an aid to support one's own work, users should also be aware of the risks. You can also find the handout as a PDF document in the HanFRIEDThis link requires a loginde administration manual. - What do we mean by generative artificial intelligence? By “generative AI” we mean computer models capable of autonomously generating new content—such as images, texts, or music—based on human or machine input, after learning patterns and structures from a training dataset. - Under what requirements is it possible to work at the university? AI-based tools have immense potential to increase the efficiency and effectiveness of our work. Where generative AI can be used profitably and without risk, its use should be permitted. To guide and raise awareness for responsible, reflective, and legally compliant use, key points are compiled in the chapter "What must be considered when using generative AI tools?". We must always bear in mind that although a text-generating AI may produce well-formulated texts based on statistical probabilities, it does not actually recognise their meaning or evaluate their coherence or factual accuracy. Examples of the use of AI tools Creative work - Generating new ideas - Supporting the development of one's own ideas Research - Discovering new sources or issues on specific topics - Summarising sources to gain an initial overview Writing process (e.g. letters, emails, minutes, publications, proposals) - Assistance with phrasing and sentence structure - Feedback on grammar, style, and structure to improve one’s own texts - Overcoming writer’s block (AI as a sparring partner) Text analysis of materials, literature synthesis or data preparation - Summarising or merging your own documents or texts - Analysing texts or examining them for specific characteristics - Supporting data preparation processes, e.g. for transcriptions Translations - Translating sentences or sections for practice or understanding - Translating emails or other correspondence for communication purposes Teaching materials and exam tasks - Generating ideas, examples or templates for new examination tasks - Supporting the design of teaching materials - Supporting the customisation of materials Targeted use of an AI tool in teaching - Training in the use of AI, e.g. for writing prompts - Digital assistants for learning and exam preparation Image material - Generating images, e.g. for internal presentations, reports or talks Assessments and evaluations - Supporting the preparation of evaluations (e.g. criteria selection and phrasing) - Assistance with phrasing Administrative tasks - Assistance with phrasing, summaries, or correspondence Examples against the use of AI tools - Processing of personal data (unless the data protection requirements can be met) - Unverified adoption of a complete concept or its elaboration by AI - Unverified adoption of a summary or analysis in a report or publication - Complete and unverified use of translations (e.g. in exams or reports) (note: use for language learning after consultation with the lecturer) - Use in examinations without being named as an aid and without the examiner's permission (note: the decision to use AI in examinations is made by the examiner) - Use of an AI tool as an aid in a course without prior consultation with the lecturer - Assessment of examinations (term paper or other examinations) or assessment of another person's performance - Evaluation of applicants or other personnel-related decisions - Preparation of an employment reference or employee appraisal - Analysis of employee data (e.g. absences, sick leave, holidays) - Evaluation of applications or assessments General information on the use of AI in specific areas In study and teaching, the guidelines for the preparation of academic work de apply. The writing of an academic piece of work or completion of exams must reflect the student’s own work. Use of AI in this context may only occur as a supporting tool and only with the examiner's agreement. Lecturers are required to design examinations in such a way that they adequately reflect the intended learning objective and are meaningful. If AI use is to be excluded, this is best achieved through a suitable assessment format. Guidance is available via the University’s pages on digital assessments and the support services of Servicestelle LehreLernen. In academic work, the “Principles of Good Scientific Practice” must also be upheld when using generative AI. In particular, reference is made to the DFG statement on the Influence of Generative Models of Text and Image Creation on Science and the HumanitiesExternal link and the statutes for safeguarding good research practice at the University of Jena. Researchers must remain aware of their responsibility for the integrity of any content created with or by AI. The ERA Forum’s guideExternal link is also recommended. Access and accounts Use of AI tools often requires registration with an email address. In professional contexts, institutional email addresses and contact details should be used. For team or API access, the University Computing Centre (URZ) can provide accounts for functional purposesExternal link. If you use your work e-mail address, it is possible that the external provider will create a user profile based on the name contained therein and link it to the person. The „IT-Zentrum der Thüringer Hochschulen“ enables anonymous use of ChatGPT via a web portal. No personal data of the employees is transmitted to OpenAI, only the chat is sent to ChatGPT. Staff can access it via https://ai-chatbot.hs-itz.deExternal link after selecting University Jena as institution and logging in with their URZ account. On 10 June 2025, the HAWKI HS-ITZ service was updated to the HAWKI2 version. The new version can be tested under: https://ai-chatbot.tu-ilmenau.de/hawki2/External link. We would also like to draw attention to the Chat AI tool (https://chat-ai.academiccloud.de/External link) from AcademicCloud, which is provided by the Gesellschaft für wissenschaftliche Datenverarbeitung mbH Göttingen (GWDG). University members can register with this service using their university email address and use various AI models for a chat. Another option for free access (including ChatGPT) is provided by KI-Campus: https://www.unidigital.news/kostenfreier-zugang-vom-ki-campus-zu-chatgpt-und-offenen-sprachmodellen-ueber-hawki-gwdg/External link. - Procurement To obtain commercial AI tools, please contact the URZ software service via the service portalExternal link. - Billing The following procedure is established for the use of OpenAI products (ChatGPT Plus and API): The costs are charged by collective booking to the PSP element specified in the service portal. The costs are averaged across all users in the respective billing period in order to distribute exchange rate fluctuations and foreign currency fees fairly. The URZ must receive the billing information from the OpenAI web portal in order to be able to carry out billing. The exact procedure differs depending on the type of product used. - ChatGPT Plus ChatGPT Plus users will be charged a subscription of $20.00 per month plus transaction costs (exchange rate fluctuations and foreign currency fees of approximately $4.00). All users are obliged to download the billing documents provided by OpenAI in the web portal for their account on a monthly basis and make them available to the URZ (via the service portal in the same process in which access was requested). - ChatGPT API When using the API, the costs are variable depending on the actual usage. An estimate of the expected monthly or annual costs is helpful for financial accounting. In each API access (organisation), several members can be authorised (‘team’). To give the URZ access to the billing information, softwarebeschaffung@uni-jena.de must be added as a user and authorised as an owner. What must be considered when using generative AI tools? - 1. Check tool settings before use. Data or information that is processed in the context of work-related activities should not be included in the training of an AI. This applies in particular to work protected by copyright, e.g. academic assignments by students, and personal data. Please check the settings in the AI tool before using it. There is usually an option to refuse use for training purposes. If this is not the case, we advise against using the tool in a university context. If possible, the input history and, if available, the memory function should also be deselected in the settings. - 2. Be cautious with personal, sensitive, or confidential information. When entering data into an AI tool, please ensure that no data relating to a person or sensitive university information is entered or uploaded. This also applies to copyright-protected works and documents declared as confidential as well as information that may allow conclusions to be drawn about individuals via indirect channels. It is advisable to anonymise personal data before entering it (e.g. use a synonym instead of a name). When entering your own personal details in AI tools, it should also be borne in mind that user profiles with personal information may be created and made available to third parties. - 3. Do not use AI for decision-making. Generative AI tools should not be used as the basis or even the final decision for personal decisions (see Art. 22 General Data Protection Regulation). For example, AI should not be used for the selection of applicants, the assessment of students' examination results or third-party funding applications by researchers. The processing of data in an AI on the purposes of which certain personal aspects are ‘evaluated’ is not permitted. Please always bear in mind that AI does not recognise the meaning, significance or implications of the outcome it creates. - 4. Careful and conscientious checking of the results. The result of generative AI should be treated with caution and evaluated carefully. The information generated by the system may be incorrect and correlations may not be represented correctly (phenomenon of confabulation). Users should also check the accuracy of references. Discrimination and inequality in the AI-generated work should also be checked so that certain groups are not disadvantaged and existing social injustices are not reinforced, as AI can create or reinforce distortions or bias. Users are ultimately responsible for critically scrutinising the generated content and ensuring that it is correct and ethically acceptable. It is also important to ensure that protected works or parts thereof are not reproduced. The rights of the author continue to exist, even if the AI has generated the result. - 5. Making the use of AI transparent. Be open about the use of generative AI. Its use should be clearly labelled and its use and underlying purposes openly communicated. It is also advisable to keep documentation on the use, for example when working on larger texts. In addition, the AI tool should also be named as the source for AI-generated images. For example, in the multimedia area of our content management system for image documents, the value ‘AI-generated’ can also be selected in the ‘Author’ field. Overall, we recommend that the use of generative AI in the university context be carefully considered and critically reflected upon, considering ethical, social and educational considerations to ensure that it supports the objectives of the university's activities. These recommendations are regularly updated and adapted to current developments and legal practice.</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1842</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -977,6 +1461,24 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>The Guideline on the use of generative AI tools in teaching and research can be found here on the website in full as a text to read or as a PDF to download. This text outlines the university's position regarding generative AI tools. The download section is organized thematically and sorted by subpages. Download Dear University Members and Staff, Talk is everywhere about ChatGPT and other generative AI (GenAI) tools. The University of Tübingen believes it is its duty to address this debate so as to help shape developments and produce guidelines. To this end, the President’s Office has set up the Generative AI work group, consisting of members from every faculty, central administration and relevant institutions. The role of the work group will be to advise the President’s Office on the use of GenAI at the University of Tübingen. Its members take a critical yet optimistic attitude to the potential of GenAI. Together, the President’s Office and the work group have discussed principles, which will continue to be developed. Their aim is to achieve the critical, reflexive, transparent and responsible use of GenAI. The current status of the discussion is given below. As a forward-looking and progressive university, the University of Tübingen recognizes the transformative potential of GenAI. This potential currently encompasses many areas of society and is changing both university and non-university work environments. GenAI is already becoming incorporated in various professions at rapid speed. There will no longer be a world without AI. In future, many University of Tübingen students will work in professions where the use of GenAI will be an everyday part of work processes. Likewise, GenAI will increasingly change the day-to-day work of researchers in various disciplines, as well as that of administrative staff. The University of Tübingen sees this as a major challenge, but also a substantial opportunity. After all, the University can be the place where critical, reflexive, transparent and responsible ways of working with GenAI are negotiated, developed, and transmitted. For instance, it contributes to shaping social change in the context of AI in a way that is both sensitive to problems and at the same time constructive. The potential for GenAI in the field of text and data processing is extremely diverse. For the University of Tübingen it extends over every relevant area: GenAI has the potential to change how students learn and operate in a data-saturated scientific world. It can enable new didactic approaches in digital teaching, open up new ways for researchers to work with texts or images, contribute to the expansion of science communication and last but not least provide support at an administrative level. The variety of possibilities makes it especially difficult to determine potential, or to develop rules on how to proceed. What is clear is that – whether in studies, teaching, research or science communication – the potential of GenAI varies, and sweeping assessments have little to offer. At present the University is in an exploratory phase, where it has to investigate, test and discuss critically the potential in all of these fields. Given the speed of technical development and the technological hype, we need to evaluate the potential of GenAI realistically, in order to define a framework in which it can be used by a forward-looking university. Besides its wide potential, GenAI also has many problematic implications. These include the fact that there are still many unresolved copyright and data protection issues. Generated texts can produce erroneous, ambiguous or misleading results and ‘hallucinate’ sources. GenAI can reproduce any bias recorded in the system’s training data. Social, cultural and scientific prejudices can be incorporated in the system and the generated texts. Developers can sometimes deliberately manipulate the generated texts. In addition, extensive use of GenAI has a substantial ecological footprint, in particular through electricity consumption, CO2 emissions, consumption of minerals and water. Furthermore, different payment models for stronger and weaker AI systems can further increase economic inequalities (e.g. between students with different incomes). Therefore, a key objective of the University of Tübingen is to test the potential of GenAI and apply it productively in various areas of the University, while bearing in mind these problematic implications. This includes developing both basic and subject-specific study programs as well as the legal framework, e.g. for application in examinations. The University will also benefit from a critical discourse on the potential and the limits of GenAI in relation to research, science communication and administration. Achieving these objectives will demand a lot of work and attention. However, it is already clear that key guiding principles will be indispensable. Firstly, members of the University must tackle GenAI in a critical and reflexive way. Many of the problems with GenAI (including at a social level) arise from a naive attitude. A critical and reflexive attitude demands not only the development of a sophisticated awareness of the problems, but also the ability to realistically assess the potential and limitations of GenAI. Secondly, use of GenAI should be organized transparently. If GenAI is used (whether for research, studies, administration or science communication), the procedure must be documented and made visible/transparent in the relevant format. Thirdly, all members of the University are exhorted to use GenAI responsibly in line with good scientific practice. Among other things this means that when working with GenAI it is the individual responsibility of the authors to ensure that their texts do not contain any plagiarism and all sources are critically examined. It also means that each user must assume responsibility for how and to what end the data provided by AI systems are processed. The way in which these principles are applied must by their nature be applied differently depending on the field of work and culture of the discipline. Departments and institutions are called on to formulate and provide their own guidelines. The Generative AI work group and the President’s Office are currently working on basic solutions in order to respond to urgent procedural questions concerning examinations. These will form the basis for future development in the faculties and institutions. If we can provide the fundamental conditions for critical, reflexive, transparent and responsible use, GenAI can offer potential to enhance work processes both within the University and beyond. What precisely these enhancements will consist of and how a critical process of evaluation can assess them with regard to their problematic implications will be the subject of ongoing discussion at the University of Tübingen in coming years.</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1070</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -987,6 +1489,24 @@
       <c r="B36" t="inlineStr">
         <is>
           <t>Germany</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Der Einsatz generativer KI (GKI) wie ChatGPT hat das Potenzial, akademische Arbeits- und Bildungsprozesse umfänglich und nachhaltig zu verändern. Sie kann personalisiertes Lernen ermöglichen, die Lehre unterstützen und Forschung fördern. Aus diesem Grund befürwortet die Goethe-Universität grundsätzlich die Erprobung und Anwendung von GKI in Studium und Lehre. Bei der Nutzung von GKI sind jedoch sowohl ethische, rechtliche und natürlich auch didaktische Aspekte zu berücksichtigen, weshalb mit einer speziell zu dem Thema eingerichteten, interdisziplinären Arbeitsgruppe unterschiedlicher Statusgruppen zielgruppenspezifische Handlungsempfehlungen erarbeitet wurden, die Ihnen, ausgehend von dieser allgemeinen Einführung zum Thema GKI, zur Verfügung stehen. Mit sorgfältiger Planung und Vorbereitung sowie einem klaren Handlungsrahmen kann generative KI ein wertvolles Werkzeug in der Hochschullehre sein. Allgemeine Empfehlungen und Hinweise Bitte beachten Sie die folgenden grundsätzlichen Hinweise im Umgang mit Tools der generativen Künstlichen Intelligenz (GKI) und den nachfolgenden Handreichungen: Kritische Reflektion: Reflektieren Sie die Ergebnisse der KI grundsätzlich kritisch, da es sich bei generativen KIs um statistische Modelle handelt, die häufig vorkommende Aussagen und Einstellungen aus vorab verarbeiteten Trainingsdaten reproduzieren. Sind z.B. Biases in den Trainingsdaten enthalten (z.B. einseitige oder verzerrte Darstellungen), so werden diese auch in den generierten Ergebnissen reproduziert. Je nach Fachgebiet und Fragestellung können die Ergebnisse sehr nützlich und korrekt oder aber falsch und irreführend sein. Geistiges Eigentum: Bitte beachten Sie, dass generative KIs Inhalte erstellen können, die auf bestehenden Daten basieren und entsprechend geistiges Eigentum eine wichtige Rolle spielt. So können z.B. in den Trainingsdaten der KI urheberrechtlich geschützte Inhalte vorhanden sein, wodurch generierte Inhalte problematisch sein könnten. Auch Daten, die man z.B. zur Überprüfung an eine KI gibt, können urheberrechtlich geschützt sein. Stellen Sie sicher, dass die Informationen, die Sie eingeben, und die Ergebnisse, die Sie erhalten, keine Urheberrechtsverletzungen darstellen. Zum jetzigen Stand können KI-Programme selbst keine Urheberschaft innehaben. Je nachdem wie stark die Einflussnahme derdie Nutzerin an dem generierten Text war, ist entweder ersie derdie Urheber*in oder das Ergebnis ist nach dem Urheberrecht gemeinfrei. Persönliche Daten: Geben Sie keine persönlichen oder sensiblen Informationen ein, wenn Sie KI-Tools nutzen. In den meisten Fällen liegt der Sitz der Betreiber der Tools aktuell noch in den Vereinigten Staaten und es lässt sich nicht kontrollieren, was mit den eingegebenen Daten passiert (Schrems II-Urteil des EuGHs). Selbst mit einer Einwilligung der betroffenen Personen lassen sich Rechte wie den Abruf aller erfassten Daten oder deren Löschung nicht oder nur sehr eingeschränkt wahrnehmen. Dies ist mit der Datenschutz-Grundverordnung (DS-GVO) nicht vereinbar. Aktualität: Vieles rund um KI-Technologien befindet sich im Moment noch in einer Aushandlungsphase. Daher können sich die Möglichkeiten, Risiken und rechtlichen Rahmenbedingungen jederzeit ändern. Wir bemühen uns, die Informationen auf dieser Seite auf dem neuesten Stand zu halten, können jedoch keine Garantie für die Aktualität geben. Korrekturen und Hinweise nehmen wir gerne entgegen. Was ist generative Künstliche Intelligenz (GKI)? Der Begriff “Generative KI” beschreibt KI-Systeme, die in der Lage sind, auf Anfrage neuartige Inhalte selbstständig zu erstellen. Diese Systeme lernen aus Daten, die sie während ihrer Trainingsphase erhalten haben, und nutzen dieses Wissen, um Ausgaben z.B. in Textform zu erzeugen. Neben der Textgenerierung gibt es auch andere Beispiele für generative KI wie Bildgenerierung, Musikkomposition und die Erzeugung von Programmcode zur Entwicklung von Anwendungen. Language Models (LM) oder Sprachmodelle sind eine Unterklasse der generativen KI. Diese Modelle lernen die Wahrscheinlichkeit von Sequenzen von Wörtern in einer bestimmten Sprache. Large Language Models (LLM) sind sehr große Sprachmodelle, die auf enormen Mengen von Textdaten trainiert wurden. Dadurch sind sie in der Lage, menschenähnliche Texte zu generieren, und können für eine Vielzahl von Aufgaben eingesetzt werden. Mit dem richtigen Training können sie Aufgaben wie maschinelles Übersetzen, Frage-Antwort-Systeme, Textzusammenfassung und mehr bewältigen. So beeindruckend die Ergebnisse sind, die mit LLMs erzielt werden können, sollten sie nicht mit Wissensdatenbanken verwechselt werden. Die Texte, die beim Trainieren der Modelle verarbeitet werden, sind im Endprodukt nicht mehr wörtlich enthalten. Man darf sich Programme wie ChatGPT deshalb nicht als Suchmaschinen vorstellen, die in Textkorpora nach relevanten Stellen suchen und Antworten durch Copy &amp; Paste zusammenstellen. Stattdessen handelt es sich um rein statistische Modelle, die Aussagen und Einstellungen reproduzieren, die häufig in ihren Trainingsdaten vorkommen. Weiterführende Informationen Friedrich Wolf – Über, mit und von KI lernen? – Ein pädagogischer Rundgang (Video, 1:26 h) Welche Anwendungen und Dienste gibt es? Da sich die verfügbaren Tools aktuell sehr schnell weiterentwickeln, versuchen wir hier einen Überblick über bestehende Tool-Kategorien zu geben, die im weiteren Verlauf der Handreichung immer wieder aufgegriffen werden. | Kategorie | Beschreibung der Kategorie | |---|---| | Literaturrecherche | Tools dieser Kategorie bieten eine Vielzahl von Funktionen zur Unterstützung der Literaturrecherche in der Hochschullehre. Sie ermöglichen es den Studierenden, wissenschaftliche Literatur effizient zu finden, zu organisieren und relevante Artikel oder Autor*innen zu identifizieren. Mithilfe dieser Tools können Studierende Literaturdatenbanken durchsuchen, Literaturlisten erstellen oder sich einen Überblick über aktuelle Forschungsergebnisse zu bestimmten Themen verschaffen. Durch die Integration in Literaturverwaltungsprogramme wie Citavi oder Zotero können gefundene Artikel auch direkt in die persönliche Bibliothek importiert werden. Ein Beispiel für ein Tool dieser Kategorie ist Researchrabbit*. Die Universitätsbibliothek bietet eine Übersicht verschiedener Tools für die Literaturrecherche. | | Textproduktion | Tools dieser Kategorie unterstützen Studierende aktiv bei der Schreibpraxis in der Hochschullehre. Mit Funktionen wie KI-Autovervollständigung, automatische Zitation, Formatierung nach verschiedenen Schreibstilen und Plagiatsprüfung assistieren sie beim Verfassen von wissenschaftlichen Arbeiten. Diese Tools können den Schreibprozess beschleunigen, indem sie beim Formulieren komplexer Sätze oder beim Finden passender Referenzen helfen. Sie ermöglichen Studierenden, ihre Schreibkompetenzen weiterzuentwickeln und wissenschaftliche Standards einzuhalten. Ein Beispiel für ein Tool dieser Kategorie ist JenniAI*. | | Textverständnis | Tools dieser Kategorie unterstützen das Textverständnis von Studierenden, indem sie ihnen ermöglichen, Texte interaktiv zu erkunden und besser zu verstehen. Durch das Markieren von Begriffen, Passagen oder wichtigen Informationen in einem Text und der anschließenden Nutzung eines integrierten Chatbots können Studierende Erklärungen, Definitionen oder zusätzliche Informationen erhalten. Diese Tools können auch Fragen beantworten oder weiterführende Quellen empfehlen, um das Verständnis eines bestimmten Textes zu vertiefen. Diese Tools sind besonders nützlich, wenn Studierende komplexe wissenschaftliche Texte lesen und analysieren müssen. Sie können dazu beitragen, dass Studierende bedeutungsvolle Verbindungen und Zusammenhänge in einem Text erkennen und das Verständnis vertiefen. Durch die Interaktion mit einem Chatbot erhalten Studierende individuelle Unterstützung und können ihr Textverständnis weiterentwickeln. Ein Beispiel für ein solches Tool ist Explainpaper*. | | Plagiatserkennung | Tools dieser Kategorie sind speziell darauf ausgerichtet, Plagiate in wissenschaftlichen Arbeiten aufzudecken. Sie ermöglichen Dozierenden und Studierenden, alle eingereichten Texte auf potenzielle Ähnlichkeiten mit anderen Quellen oder bereits veröffentlichten Arbeiten zu überprüfen. Diese Tools durchsuchen umfangreiche Datenbanken und nutzen fortschrittliche Algorithmen, um verdächtige Übereinstimmungen zu identifizieren. Sie helfen dabei, die Integrität der akademischen Arbeit zu wahren und Studierende zu ermutigen, eigenständig zu arbeiten und ihre eigenen Ideen zu entwickeln. Ein Beispiel für ein Tool dieser Kategorie ist Turnitin*. | | Bildgenerierung | Tools dieser Kategorie nutzen Deep-Learning-Algorithmen, um aus Texteingaben Bilder zu generieren oder bestehende Bilder zu verändern. Sie ermöglichen es Studierenden, mithilfe von Beschreibungen oder Anweisungen hochqualitative, visuelle Inhalte zu erstellen. Diese Tools sind besonders nützlich für die Erstellung von Bildern oder Diagrammen für Präsentationen, Poster, Webseiten oder Berichte. Ein Einsatz solcher Tools kann Zeit und Ressourcen bei der Materialerstellung sparen sowie Studierende oder Lehrende, welche nicht über ausgeprägte künstlerische Fähigkeiten oder umfangreiche Designkenntnisse und Software verfügen, dazu befähigen, visuell ansprechendes Material zu erstellen. Ein Beispiel für ein Tool dieser Kategorie ist DreamStudio* welches das StableDiffusion Modell zur Bildgenerierung verwendet. | | Präsentationserstellung | Tools dieser Kategorie ermöglichen es Studierenden und Lehrenden, auf einfache Weise ansprechende Präsentationen zu erstellen. Sie basieren auf Texteingaben, die bereitgestellt werden müssen, und generieren daraus automatisch Folien mit relevanten Inhalten. Diese Tools bieten verschiedene Designvorlagen, Animationsmöglichkeiten und die Möglichkeit, multimediale Elemente wie Bilder oder Videos einzufügen. Sie erleichtern die Erstellung von visuell ansprechenden Präsentationen und sparen Zeit. Studierende und Lehrende müssen sich weniger mit dem Gestalten der Folien beschäftigen, sondern können sich mehr auf den Inhalt ihrer Präsentationen konzentrieren. Diese Tools ermöglichen es, professionell aussehende Präsentationen zu erstellen und ihre Informationen auf eine zugängliche und ansprechende Weise zu präsentieren. Ein Beispiel für ein Tool dieser Kategorie ist SlidesAI*. | Bestehende Sammlungen und Datenbanken zu KI-Tools - Sammlung von Tools mit dem Fokus auf Textverarbeitung: VK:KIWA - Umfassende Toolliste zu verschiedensten Kategorien: AI Tools Directory - Datenbank mit über 50 Kategorien und 3000 Tools: AI Tools Update - Umfangreiche Datenbank und Community zu KI-Tools: FUTUREPEDIA - Datenbank zu KI-Tools: Future Tools - Umfangreiche Sammlung von KI-Tools mit Erklärvideos: Miroboard von Jan Foelsing - sehr umfassende und aktuelle KI-Sammlung: The Generative AI Landscape - KI-Tools nach Erscheinungsdatum sortiert: There’s An AI For That Nutzung von generativer KI in Studium und Lehre Ergänzend zu dieser allgemeinen Einführung zum Thema generativer KI (inkl. Toolkategorien und -sammlung) gibt es zwei weitere Handlungsempfehlungen speziell für Lehrenden und Studierende. - Einsatz von KI in der Lehre (Zielgruppe Lehrende) - Einsatz von KI im Studium (Zielgruppe Studierende) Weitere Unterstützungsangebote zu dem Thema KI in der Lehre an der Goethe-Universität sind: - „Über, mit und von KI lernen? – Ein pädagogischer Rundgang“ (studiumdigitale) - „Einsatzmöglichkeiten von KI-Tools in der Lehre“ (studiumdigitale) - „Was machen wir mit KI und was macht KI mit uns? Ethische Aspekte im Umgang mit KI-Tools in der Hochschullehre“ (studiumdigitale) - „KI-Anwendungen wie ChatGPT in Lehre und Prüfungen“ (IKH) - „KI-gestütztes Schreiben vermitteln“ (IKH &amp; Schreibzentrum) - Online Lehrlabor „ChatGPT als Herausforderung und Chance. Was macht die KI mit dem Schreiben?„ (Schreibzentrum) - Tipps zur Nutzung von KI-Schreibtools in der Lehre (Schreibzentrum) - Impulsreihe im Rahmen des Verbundprojekts HessenHub Frequently Asked Questions (FAQ) Kontakt Die Handreichungen wurden von der AG: Generative KI mit dem Fokus auf Studium und Lehre erstellt. Hinweise und Feedback nehmen wir gerne über folgende Adresse entgegen: ag-gki@studiumdigitale.uni-frankfurt.de</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1590</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
replaced absolute path to relative path
</commit_message>
<xml_diff>
--- a/data/raw_extracted_data.xlsx
+++ b/data/raw_extracted_data.xlsx
@@ -476,6 +476,19 @@
           <t>Guidance on safe and responsible use of Gen AI tools The aim of this guidance is to help you use GenAI tools safely and responsibly, so you feel confident about exploring different ways of using this technology to support your learning. Generative Artificial Intelligence (GenAI) is a fast-evolving technology and, during your time at Oxford, the University wants to enable and support the safe and productive use of these tools that will be important in your future. Ethical use GenAI tools must be used responsibly and ethically, in accordance with the academic standards of rigour and integrity that are expected of you as a student at Oxford. You should always use AI tools with integrity, honesty, and transparency, and maintain a critical approach to using any output generated by these tools. This document contains some useful tips for using GenAI to support your studies at Oxford. You should always follow the advice and guidance of your tutors and/or supervisors, and consult your department or faculty in relation to ethical use. Assessment For each specific assessment you will be given prior written notice of whether or not the use of AI is permitted. You are fully responsible for the accuracy, originality, and quality of work you submit for assessment, and you must follow the rules on AI use for each specific assessment you are taking. You must make a formal declaration of any permitted AI-use in the format prescribed by your assessment setter. Any unauthorised use of AI in work submitted for assessment constitutes cheating and plagiarism under University rules, penalties for which include failing the relevant assessment and, in appropriate cases, expulsion. Any use of AI in work submitted for assessment is unauthorised unless you are specifically told differently in writing, in advance of the assessment, in instructions from your faculty’s or department for the specific assessment in question. Even if a type of AI use has been authorised for a previous assessment, or for formative work, it is your responsibility to ensure that you comply with the rules on AI use for the specific assessment you are taking, in the knowledge that all types of AI use are unauthorised unless specifically listed in assessment instructions. Cases of suspected unauthorised use of AI in assessment are covered by the University’s student conduct regulations. You should make yourself familiar with these regulations, as any actions that are found potentially to be in breach of them will be reviewed in line with the University’s Code of Discipline and Academic Disciplinary procedure. You should always follow the guidance of your tutors and/or supervisors, and of your department or faculty. Use in research All research undertaken by academic staff and students, including by postgraduate students, must meet the expectations in the Policy for using Generative AI in Research: guidelines for researchers and professional staff. Substantive use of GenAI should be declared whenever a stand-alone AI tool is used (such as ChatGPT Edu), but not where GenAI functionality is embedded within existing software. Substantive use of GenAI by students who are conducting research as part of a graduate research programme is defined as: - interpreting and analysing data (including audio and image files) and texts, - undertaking a literature review or translation, - identifying research gaps, - formulating research aims, - developing hypotheses, - assisting with generating ideas or to develop one’s own thinking, - generating code and synthetic data, - undertaking transcription of interviews, meetings etc. to save time and effort rather than overcoming barriers (see exclusions below) - producing documents using other people’s work or from transcripts or recordings. Substantive use may exclude using GenAI for tasks such as assisting you with translation if you are a non-native speaker, transforming transcribed spoken language into written language if you face barriers to writing, formatting documents, or improving the standard of your English or of a foreign language. As with assessment, you should always follow the guidance of your tutors, supervisors, and of your department or faculty. Use of GenAI in research falls within the scope of research conduct and the permitted use of AI as outlined abov. Actions that are found to be in potential breach will be reviewed in line with the University's Code of practice and procedure on academic integrity in research. Your health and wellbeing Because of the way that GenAI tools work, they are not a replacement for human interaction and are not equipped to offer therapy or mental health support. You should be aware that GenAI tools lack emotional nuance and clinical awareness. They can sometimes give inaccurate and potentially dangerous advice. At times of heightened distress or mental health crisis, AI chatbots may reinforce harmful thoughts through feedback loops. The University’s Student Welfare and Support Services offer a range of support with welfare and wellbeing. This includes access to Togetherall, a free and anonymous online platform where for connecting with others about what’s going on in life - big or small. Togetherall also offers free courses, resources, and anonymous chats to support your wellbeing, 24 hours a day. The SWSS also provide a free counselling service and a wealth of resources on the Oxford Students website and MyOxford app. In addition, support and advice are available from your college, department, fellow students and the Students' Union. There are contacts for emergency (including out of hours) and non-emergency services for health, welfare and academic support. All student welfare services remain open throughout the vacations (except Bank Holiday Mondays and the Christmas closure period), with some adjusted opening hours (listed on each service's page) and vacation welfare support page. Using GenAI to support your studies Part of what a university education teaches is academic skills such as assimilating information, constructing an evidence-based argument, and expressing your thoughts in clear, coherent prose. AI tools cannot replace human critical thinking or the development of scholarly, evidence-based arguments and the subject knowledge that form the basis of your university education. You should always cross-check AI generated outputs against established sources to verify accuracy and identify erroneous information. You may make use of University-supported generative AI tools (e.g. ChatGPT Edu, Google Gemini, Notebook LM and Copilot Chat) to develop your academic skills and to support your studies. This should be done in consultation with your tutors, faculty, or department, and you should always follow their advice in relation to how they expect AI tools to be used (or not used) for different tasks. These tools are accessed via your University Single Sign-On (SSO) account. Your ongoing critical appraisal of GenAI outputs, by reviewing them critically for accuracy and relevance, will maximise their potential to support you in your studies. Academic writing and presentation skills Depending on your academic discipline, GenAI tools can be useful in developing your academic writing skills and providing initial feedback on them, translating between different styles, and critiquing your own writing. They cannot replace the need for you to develop such skills through tutorials or supervisions, and independent learning, however. Depending on your academic discipline, GenAI tools also may be used to support your academic reading, but there is a risk that they could undermine the development of critical academic skills (e.g. if you use a GenAI tool to summarise an article for you, rather than fully engaging with the literature or undertaking the task yourself). You should always remain alert to the limitations of AI-generated outputs. Here, again, the subject-specific guidance of your tutors, supervisors, and faculty or department is crucial, because appropriate use of AI to support academic reading varies across different academic disciplines. Appropriate use of GenAI tools to support your academic writing and presentation skills varies across academic disciplines. Always follow any advice and guidance of your tutors or supervisors, department/faculty, or college, on what is appropriate in your subject area. Supporting the learning process Generative AI tools may be useful in supporting your academic studies, but be sure to discuss AI outputs with academic staff to confirm your understanding and to help verify them against established sources, to ensure their accuracy. Appropriate use of GenAI tools to support the learning process varies across different academic disciplines. Always follow any advice and guidance of your tutors or supervisors, and of your department or faculty, and/or college, on what is appropriate in your subject area. Tips for using GenAI tools effectively The University provides you with access to secure, enterprise-level ChatGPT Edu, Google Gemini, Notebook LM and Copilot Chat tools. Different GenAI tools can be used for different purposes. Here are some examples of key uses for some of the secure tools the University supports: - ChatGPT Edu – Advanced content generation, summarising information and complex reasoning - Microsoft Copilot Chat – Web-grounded chat, summarising information, drafting content and web-based information retrieval - Google Gemini – AI assistance that is integrated with Google Workspace, or can be used as a standalone chat tool - Notebook LM – An AI assistant that can interact with and summarise lecture notes, papers and other uploaded sources to aid research and study. You may find it useful to try a few different GenAI tools and you should be aware that different tools will give different outputs to one another, from the same prompts. Within a single tool you may also get different outputs in response to the same prompt. It is important to be aware that: - You will get different responses using the same prompts from the same GenAI tool. AI outputs are not repeatable, and all tools can generate outputs that contain inaccuracies and fabrications. - You could spend a lot of time trying out different AI tools. Be careful to balance your exploration of GenAI with managing your time effectively. - GenAI tools may draw on data that can be months or years out of date and, whilst outputs seem plausible, they may contain errors and/or reflect biases from the original data the tool was trained on. For example, Western perspectives are overly represented. - GenAI tools do not replace the need for you to develop your own knowledge, skills, and critical awareness, as an independent learner. - Take care when inputting material into any third-party tools that are not provided by the University. These may not meet the University’s standards of information security and data protection. Never upload confidential, sensitive, or unpublished material into third-party AI tools. Help and technical support with GenAI tools If you need help or technical support with using University-supported GenAI tools: - Consider first seeking support from the company whose product you're using: - ChatGPT Edu: For access and activation queries, please use the OpenAI help portal. You can use the chat at the bottom of the page to ask questions and connect with support by clicking on the Message tab. If you are unable to resolve your issue through the help portal, then you should contact OpenAI support directly by email at [email protected]. - Microsoft Copilot: The Microsoft Support site can be searched to assist with queries on Copilot. - Google Gemini: Google's Gemini Apps Help page offers various pieces of advice and support for using Gemini. - NotebookLM: Google’s NotebookLM Help page covers help topics from getting started to troubleshooting NotebookLM. - If your query is about whether an outage is affecting your connection to a particular tool, try the relevant status pages: - OpenAI Status page for ChatGPT Edu - Microsoft Status page for Microsoft Copilot - Google Status page for Google Gemini and NotebookLM - For simple queries regarding University-supported GenAI tools and support, use the AI Competency Centre chatbot to be directed to relevant information. - Contact the University's IT Service Desk if you need more support - they can help you with ChatGPT Edu, Microsoft Copilot, or the GenAI tools in the University's Google workspace (Gemini and Notebook LM). If your query needs escalating, the IT Service Desk will involve our GenAI specialists at the AI Competency Centre or signpost you to tailored support from elsewhere in the University, as needed. Find out more To find out more about using GenAI tools at Oxford, please visit the Generative AI at Oxford webpage. This guidance is under continuous review and will be updated to reflect the evolving landscape of AI use across the University. Content last updated on 22 September 2025.</t>
         </is>
       </c>
+      <c r="D2" t="n">
+        <v>2045</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -490,7 +503,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AI guidance Guidance for University of Cambridge Staff on the Administrative Use of Generative AI This page provides guidance on the use of Generative Artificial Intelligence (GenAI) for administrative tasks in support of University activities, and links to sources of further information. - Scope - Structure and overview of this guidance - Benefits - Risks - Best practice: practical examples - Copilot: Useful Facts - Further reading on best practice with use of GenAI This guidance was published in February 2025 and is accurate as of that date. Due to the fast pace of change in this area, in particular with regard to the range of licensed GenAI tools being made available to staff and students, it will be reviewed and updated during autumn 2025. A summary of key points is also available here. Scope Please be aware this guidance only applies in limited circumstances, as described below. Scope of this guidance: technology This guidance exclusively concerns the use of GenAI. GenAI typically describes any type of AI which can be instructed to produce content. Large Language Models (LLMs), such as Copilot, OpenAI ChatGPT, Google Bard and Gemini, are part of this category of AI. They produce text-based outputs based on written or verbal instructions from human users. These are sometimes referred to as natural language text prompts. There are also GenAI tools such as DALL.E, Midjourney and Stable Diffusion that produce digital imagery based on written or verbal instructions. In addition to the standalone GenAI tools described above, GenAI is increasingly incorporated into software and systems to enhance their capabilities. This guidance applies to both use of standalone GenAI tools and GenAI features in software and systems. It does not apply to use of systems or software that may include GenAI features where those features are not being utilised. This guidance does not apply to other forms of AI that may be conceived, developed or utilised across the University. Nevertheless, some of the broad principles for good practice outlined below may be relevant in other contexts. Scope of this guidance: audience and context This guidance is aimed at members of staff (or equivalents such as casual workers, interns, volunteers or visiting staff) considering the use of GenAI for administrative tasks in support of University activities. This guidance applies to routine tasks such as the production of content for an email to a student or colleague. It also applies to more complex tasks such as the production of content for formal policies or strategic reports. Ultimately, staff are responsible for ensuring any use of GenAI is conducted reasonably, lawfully, and in conjunction with relevant University policies and procedures. Scope of this guidance: where this guidance does not apply This guidance does not apply to use of GenAI in other contexts. In particular, this guidance does not apply to: - Education - This guidance does not apply to any task or content creation undertaken in the direct provision of teaching, student learning and/or academic assessment. - It does not apply to the appropriate use of GenAI by students to support their learning. - It does not apply to inappropriate use of GenAI by students in regard to plagiarism or any other perceived form of academic misconduct. - It does not apply to programmes of study, courses or lectures where GenAI is the subject matter. - Research - This guidance does not apply to GenAI as a topic of research – it does not apply to research regarding any dimension of GenAI as a technology, its application, nor the impact of its application in any given scenario. - It does not apply to any research undertaken with the assistance of any form of GenAI. The ethics and appropriateness of its use in those circumstances will be assessed by other established means (e.g. research ethics processes). - Colleges and other non-University legal entities - This guidance does not apply to use of GenAI tools by College employees for any College business, or to the Students’ Union, student societies, or Cambridge University Press &amp; Assessment. Please see the ‘Further reading on best practice with use of GenAI’ section for other University resources on use of GenAI that may be relevant to the matters identified above. Structure and overview of this guidance Given the diverse range of work the University undertakes, it is not possible for the University to provide comprehensive instruction on circumstances in which it would or would not be appropriate to use GenAI tools. It is up to departments, faculties and individual members of staff to balance the benefits and risks of the use of GenAI, to make an informed decision about whether its use is appropriate or desirable – before it is initiated. In the limited circumstances where a formal risk assessment is required, the University Data Protection Impact Assessment (DPIA) and Information Security Risk Assessment (ISRA) processes remain the relevant risk assessments processes to follow. To help guide staff in their decision making we have provided the following: - a brief outline of some of the benefits of the use of GenAI - guidance on the risks associated with use of GenAI tools - practical examples of good and bad practice - useful facts about Copilot Regardless of the work being undertaken, it is recommended that staff avoid inputting confidential, sensitive or personal information into GenAI tools unless warranted and only in accordance with this guidance. Please see the UIS guidance on different data types: https://help.uis.cam.ac.uk/service/security/data-sec-classes. Where the use of GenAI will not encompass the use of confidential, sensitive, or personal information, the risk to the University is reduced. However, it is still important to consider whether its use constitutes the best available means of completing a task. Any use of AI must be appropriately transparent and accountable. If it is necessary and beneficial to use GenAI tools, it is recommended that wherever practicable the University’s licensed AI tools, Microsoft Copilot and Copilot for Microsoft 365 are utilised, regardless of the type of data that may be input. Use of other licenced GenAI tools is not prohibited, but such tools must be procured in accordance with any applicable procurement policy or process, including but not limited to the completion of any requisite risk assessments such as DPIAs and/or ISRAs. Any risk associated with their deployment rests with the relevant department. Any use of such GenAI tools should also be accordance with this guidance. Copilot is already available to staff. Microsoft Copilot is the basic licensed version and is available via a staff login and Copilot for Microsoft 365 is the more comprehensive version, which is available via an additional purchased licence. The public free version, available via a web browser, must not be used for University activities and purposes as it does not guarantee a sufficient level of information security or confidentiality. More information on Microsoft Copilot and Copilot for Microsoft 365 is available on the UIS website: https://help.uis.cam.ac.uk/service/collaboration/365/copilot. Please remember the Acceptable Use Policy (AUP) continues to apply, including its compliance monitoring and enforcement provisions, when using GenAI tools and staff are reminded of their obligation to abide by its terms. In all circumstances, staff are expected to exercise caution and use their judgement in their use of GenAI. Benefits Many potential benefits of using GenAI tools are already apparent, and the University encourages all its staff to make the best use of the information services made available to them. Here is a brief list of potential benefits in supporting University activities. Efficiency and productivity GenAI tools can quickly process a lot of information to produce a large amount of output, saving time that can be spent on other tasks, and boosting efficiency and productivity. Flexibility GenAI can create content in various formats, styles and languages, making it useful in a wide range of circumstances. For example, it could be used to generate drafts of meeting minutes, letters, press releases, social media posts, and other forms of documentation produced in the course of University business. That flexibility also allows the University to engage with different audiences across various platforms. In some circumstances, it may be appropriate and beneficial to use it to produce personalised content. Creativity GenAI can produce novel or unusual content from existing source material, making it a useful tool for the initial part of some creative tasks. For example, it could be used to draft materials that could form part of a marketing campaign. Understanding GenAI doesn’t just have to be used for content production and creation. It could be used to discover and summarise vast amounts of information in more digestible formats, and so it can be a valuable tool in the early stages of research undertaken to support administrative tasks. Risks There are, however, significant legal and reputational risks associated with use of GenAI tools, which can be broadly categorised as follows: - Bias, misinformation and inaccuracy - Data protection law non-compliance - Intellectual property and copyright law non-compliance - AI legislation non-compliance - Reputational damage and other risks This list is not exhaustive, given the overlapping nature of risk categories and the pace of AI development. Staff must consider relevant risks, and whether they are applicable to the circumstances in which they are considering use of GenAI, before any use of GenAI is initiated. Risk: Bias, misinformation and inaccuracy Much GenAI is trained to produce outputs based on information and patterns extracted from data in the public domain. Consequently, outputs will sometimes reflect the biases and prejudices of individuals and groups in society. GenAI can also be manipulated to deliberately produce biased or inaccurate outputs, presented as fact. Unlike human intelligence, AI does not have the capacity to apply judgement or understand context. It cannot apply moral or critical perspectives. Additionally, there is an inherent risk that the ongoing use of GenAI tools will create and sustain feedback loops, whereby GenAI tools will be trained on text outputs generated by other GenAI tools, further reinforcing existing biases and inaccuracies. In practical terms, that means some outputs will be inaccurate or unbalanced regardless of the phrasing of the text prompt, because the source material is inaccurate or unbalanced. Some output may also be inaccurate because the GenAI tool is ‘hallucinating’ – creating nonsensical or inaccurate outputs that are not directly attributable to the source material. For those reasons, it is important that any GenAI output is thoroughly evaluated by a human being before it is utilised for any purpose. This is especially important where there is the risk of an adverse impact on a group or individual, or the potential for infringement of a person’s rights (e.g. as defined under the Equality Act 2010, the Human Rights Act 1998 or any other relevant legislation). Risk mitigation(s): Ensure that all GenAI outputs are thoroughly evaluated by a human being before they are used. Ensure use of GenAI is acknowledged if it is used to make a significant and unrevised contribution to a substantive or impactful piece of work such as the production of content for formal policies or strategic reports. Risk: data protection law non-compliance GenAI tools and their use are subject to existing laws and regulations and any University policy relevant to their use. This includes data protection laws such as the UK GDPR, the Data Protection Act 2018 and the University Data Protection Policy. As with the use of other information tools and services, it is important to use licensed versions of tools paid for from a University budget and procured through any applicable procurement process. (Free, unlicensed information tools and services often rely upon intrusive data processing and/or selling as part of their business model.) The University’s standard licensed AI tools are Microsoft Copilot and Copilot for Microsoft 365, and this is the tool that should be used to process personal data, where necessary, for which the University is responsible. This ensures that technical, operational and legal safeguards are in place, which protect any personal data that the University controls or otherwise processes. By contrast, inputting data into a free or unlicensed GenAI tool could be considered equivalent to putting it into the public domain – signifying a potential personal data breach. Information input into GenAI tools is also often used to train those tools, which may not be a lawful use of personal data – especially if that data cannot be retrieved or deleted, for example from an AI neural network. Data input into the University’s licensed version of Microsoft Copilot and Copilot for Microsoft 365 is not used to train those tools. It is particularly important to be cautious about inputting sensitive personal information (special category data) such as medical information into GenAI tools. Processing of such information is subject to additional safeguards, and misuse could represent a serious breach of data protection law and/or a breach of confidentiality. Regardless of the type of information you wish to input into a GenAI, you must consider the task you are using it to support. Data must be collected, held and used for only that purpose – for example, as part of a governance process – and any use of AI must be compatible with that reason. With some exceptions (e.g. for academic research), it is not appropriate to use personal data that was collected for a different purpose to do something else with a GenAI tool. It is also important to be mindful of ‘automated decision making’. Automated decision making involves: - making a decision that will affect a person solely by automated means without any human involvement; or - profiling someone – automated processing of personal data to evaluate certain things about an individual that could be used as part of a decision-making process. A common example of automated decision making is a credit check conducted exclusively using AI to decide whether to provide someone with a personal loan. While the use of GenAI to produce text or digital imagery would not necessarily result in a decision being made about an individual, it is not inconceivable that the use of such technology could be used as part of an evaluation process. For example, to review an application for a parking permit to ensure the person applying meets the eligibility criteria. In such circumstances, it is imperative that a human being is ultimately involved in the decision-making process. If after careful consideration you decide to use a GenAI tool, you must tell the affected people that you’re going to do that. That doesn’t mean you must seek consent on a case-by-case basis, but it will mean that relevant privacy notices should be provided or updated. Risk mitigation(s): Be cautious about inputting personal data into GenAI tools, especially sensitive personal data, and only do so where warranted. Do not use free GenAI tools. Use the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. Deploy relevant privacy notices. Risk: intellectual property and copyright non-compliance It has been argued by some affected parties that the entire basis for training GenAI tools through publicly available data is a violation of intellectual property rights and copyright law. There are a series of ongoing and well-publicised copyright cases where high profile individuals and organisations have sued companies that own and operate GenAI. Bearing that in mind, it is important to consider the nature of the content being input into any GenAI tool and to consider whether the University has the right to input that information into that GenAI tool. It is also important that GenAI outputs are thoroughly checked by a human being and cited where appropriate. Risk mitigation(s): Consider whether it is appropriate to input material into GenAI tools. Cite outputs where appropriate. Use the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. Risk: AI legislation non-compliance In March 2024, the European Union (EU) introduced new laws that will require organisations using AI in the EU to employ a risk-based approach to their use of AI, especially with regard to the use of personal information. It will incrementally start to take effect from February 2025, and non-compliance with the legislation could result in penalties from European regulators. It will affect the University where it is processing EU citizens’ data using AI. Risk mitigation(s): Exercise caution and judgement regarding deployment of GenAI on EU citizens’ data. Document any use of GenAI tools in these circumstances. Risk: Reputational damage and other risks As outlined above, there are various legal risks posed by the use of GenAI, all of which could result in reputational damage to the University. There is also an environmental cost associated to use of GenAI: training GenAI tools requires vast amounts of power and indirectly generates enormous amounts of carbon, meaning there is a sustainability consideration to its use. In the development of some GenAI tools, outputs are checked and refined in a process known as Reinforcement Learning from Human Feedback (RLHF). That process includes human reviewers, often working in countries in the global south for very low wages, routinely viewing objectionable and distasteful materials, and has been reported to have a profoundly negative impact on the health and well-being of many of those workers. University staff will also be expected to provide human oversight of GenAI outputs. Whilst they would not ordinarily be exposed to objectionable nor distasteful materials in the course of administrative work, it is important to consider the risk to University staff wellbeing that could be posed by increased workloads and unrealistic expectations of what can be reasonably achieved using GenAI tools. Risk mitigation(s): Consider the wider impact on the University’s reputation before using GenAI. Consider any other relevant risks. Best practice: practical examples Here are a series of practical examples intended to show both best practice and scenarios in which the use of AI should be considered carefully. It remains important to bear in mind the general risks and benefits associated with use of GenAI in these different contexts. Example 1: Using GenAI for background research Capability: GenAI can be used as a research tool to help gather background information on a topic relating to something you are unfamiliar with. Example scenario: Using GenAI to provide an overview of a new piece of legislation that may affect your work at the University. Good practice: Using the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. Not inputting any personal or confidential information into Microsoft Copilot or Copilot for Microsoft 365, because it is not required to understand the new legislation. Bad practice: Using an unlicensed GenAI tool. Inputting confidential data into that unlicensed AI tool with the aim of further understanding the legislation, thus committing a personal data breach and/or breach of confidentiality. Example 2: Using GenAI to summarise information Capability: GenAI can be used to summarise information. Example scenario: Using GenAI to prepare a briefing on a University project for a meeting with a commercial partner. Good practice: Using the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. Treating the output as a draft and amending it as appropriate. Thoroughly checking the output to ensure it is factually accurate and unbiased, does not reveal anything confidential to the commercial partner and is reflective of the source material. Acknowledging GenAI has been used to help create the briefing if it has not been materially altered as part of the fact-checking or drafting process. Bad practice: Using an unlicensed GenAI tool. Treating the output as a final draft. Accepting the output as factually accurate and suitable for sharing with a third party and not bothering to check it before presenting it to the commercial partner. Failing to mention it has been created using a GenAI tool. Example 3: Using GenAI to draft a document Capability: GenAI has the ability to produce written outputs in various styles and formats. Example scenario: Using GenAI to create meeting minutes. Good practice: Considering whether use of GenAI is appropriate in these circumstances – this will depend on what the meeting is about. Considering whether the document is likely to contain sensitive information. If the document is likely to contain sensitive information, considering the type of sensitive information, and whether use of GenAI is warranted. If it is appropriate to use a GenAI tool, using the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365, and ensuring unauthorised AI note-taking bots are prevented from joining the meeting. Using the output as a draft and amending it as appropriate. Bad practice: Using an unlicensed GenAI tool. Inputting confidential or sensitive data into that unlicensed GenAI tool thus committing a personal data breach and/or breach of confidentiality. Failing to follow UIS advice on preventing unauthorised AI note-taking bots from joining your Teams meeting. Example 4: Using GenAI for numerical analysis Capability: GenAI can perform numerical analysis. Example scenario: Using GenAI to analyse the statistical results of a staff survey. Good practice: Considering whether the raw survey data contains personal or sensitive information. If it is appropriate to deploy a GenAI tool, using the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. Telling staff that AI will be used to analyse responses when they are choosing whether they wish to participate. Treating the output as a draft and verifying and amending it as appropriate. Bad practice: Using an unlicensed GenAI tool. Not telling staff that GenAI will be used to analyse their responses. Accepting the output as factually accurate and making an unquestioning decision based on the analysis. Failing to follow UIS advice on preventing unauthorised AI note-taking bots from joining your Teams meeting. Copilot: Useful Facts This section contains a few useful facts that may assist staff in using the University’s licensed version of Microsoft Copilot or Copilot for Microsoft 365. The version of Copilot accessible to most University MS365 users is called “Microsoft Copilot”. A more comprehensive version of Copilot is available called “Copilot for Microsoft 365”, and a licence for its use can be purchased by contacting UIS. This table compares the functionality available in Microsoft Copilot against the functionality available in Copilot for Microsoft 365. (Please be aware that GenAI tools are being constantly updated, so the information tabulated below may be out of date). | Functionality Questions | Microsoft Copilot | Copilot for Microsoft 365 | |---|---|---| | Is it available to University MS365 users? | Yes, through their standard login. | No, an additional licence must be purchased from UIS. | | Does it integrate with Microsoft Apps? | No. | Yes. | | Can it draft emails? | Yes, but text output must be copied into Outlook. | Yes, it will draft emails in Outlook. | | Can it draft documents? | Yes, but text must be copied into Word. | Yes, it will draft documents in Word. | | Can it be used with spreadsheets? | Yes, spreadsheets can be attached to chats. | Yes, but it will sometimes fail to produce outputs from Excel files with complex formatting | | Can it be used to create PowerPoint presentations? | No, but it can be used to create the content for a presentation via the chat function. | Yes. | | Can it summarise documents? | Yes, documents can be attached to chats. | Yes, documents can be attached to chats and it will summarise Microsoft documents in those apps. | | Will it summarise PDFs and other documents in standard formats? | Yes, via a chat. | Yes, via a chat. | | Is there a word limit for documents attached to a chat? | There is no known limit. | There is no known limit. | | What is the character limit for chat instructions? | 8,000 | 16,000 | | Is there a limit on the number of questions I can ask? | There is conversation limit of 30 questions, but you can start as many new chats as necessary. | There is conversation limit of 30 questions, but you can start as many new chats as necessary. | | What is the word limit on chat text outputs? | There is no known limit. | There is no known limit. | Here are some potentially useful tips for using Copilot: - When accessing Microsoft Copilot, you can check whether you are logged into your University MS365 account by viewing the top right-hand corner of your window – you will be able to see your initials (and your name if you click on the initials) if you are logged in. - When attaching documents, these will be automatically saved in a folder called ‘Microsoft Copilot Chat Files’ in your University MS365 account OneDrive. - Delete chat files that are no longer required. - Delete files uploaded into OneDrive as part of the chat process when no longer required. - There is more information regarding OneDrive on the UIS website: https://help.uis.cam.ac.uk/service/collaboration/365/onedrive. Further reading on best practice with use of GenAI University resources: - Applications: AI and undergraduate applications - Communications: OEAC staff please see the relevant pages of the OEAC website for further guidance on using GenAI in the production of content for communications. - Education: Blended Learning Service – AI and Education - UIS: Copilot - UIS: Guidance on information security (including policies and data classification) - UIS: LinkedIn Learning at the University of Cambridge (type in ‘GenAI’ when logged in) External resources: - ICO guidance resources on data protection and AI - An introduction to copyright law and practice in education, and the concerns arising in the context of GenerativeAI - Artificial intelligence (jiscinvolve.org) - Generative AI Framework for HM Government - Organisation for Economic Co-operation and Development (OECD) AI principles Authorship This guidance was composed without the use of AI.</t>
+          <t>AI guidance Guidance for University of Cambridge Staff on the Administrative Use of Generative AI This page provides guidance on the use of Generative Artificial Intelligence (GenAI) for administrative tasks in support of University activities, and links to sources of further information. - Scope - Structure and overview of this guidance - Benefits - Risks - Best practice: practical examples - Copilot, Gemini and NotebookLM: Useful Facts - Further reading on best practice with use of GenAI This guidance was first published in February 2025 and last updated in December 2025. It is accurate as of the latter date. Due to the fast pace of change in this area, in particular with regard to the range of licensed GenAI tools being made available to staff and students, it will be reviewed and updated again during summer 2026. A summary of key points is also available here. Scope Please be aware this guidance only applies in limited circumstances, as described below. Scope of this guidance: technology This guidance exclusively concerns the use of GenAI. GenAI typically describes any type of AI which can be instructed to produce content. Large Language Models (LLMs), such as Copilot, OpenAI ChatGPT, Google Gemini and Claude are part of this category of AI. Their primary function is to produce text-based outputs based on written or verbal instructions from human users. These are sometimes referred to as natural language text prompts. There are also GenAI tools such as DALL.E, Midjourney, Stable Diffusion, Adobe Firefly and Google Imagen that produce digital imagery based on written or verbal instructions. In addition to the standalone GenAI tools described above, GenAI is increasingly incorporated into software and systems to enhance their capabilities. This guidance applies to both use of standalone GenAI tools and GenAI features in software and systems. It does not apply to use of systems or software that may include GenAI features where those features are not being utilised. This guidance does not apply to other forms of AI that may be conceived, developed or utilised across the University. Nevertheless, some of the broad principles for good practice outlined below may be relevant in other contexts. Scope of this guidance: audience and context This guidance is aimed at members of staff (or equivalents such as casual workers, interns, volunteers or visiting staff) considering the use of GenAI for administrative tasks in support of University activities. This guidance applies to routine tasks such as the production of content for an email to a student or colleague. It also applies to more complex tasks such as the production of content for formal policies or strategic reports. Ultimately, staff are responsible for ensuring any use of GenAI is conducted reasonably, lawfully and in conjunction with relevant University policies and procedures. Scope of this guidance: where this guidance does not apply This guidance does not apply to use of GenAI in other contexts. In particular, this guidance does not apply to: - Education - This guidance does not apply to any task or content creation undertaken in the direct provision of teaching, student learning and/or academic assessment. - It does not apply to the appropriate use of GenAI by students to support their learning. - It does not apply to inappropriate use of GenAI by students in regard to plagiarism or any other perceived form of academic misconduct. - It does not apply to programmes of study, courses or lectures where GenAI is the subject matter. - Research - This guidance does not apply to GenAI as a topic of research – it does not apply to research regarding any dimension of GenAI as a technology, its application, nor the impact of its application in any given scenario. - It does not apply to any research undertaken with the assistance of any form of GenAI. The ethics and appropriateness of its use in those circumstances will be assessed by other established means (e.g. research ethics processes). - Colleges and other non-University legal entities - This guidance does not apply to use of GenAI tools by College employees for any College business, or to the Students’ Union, student societies, or Cambridge University Press &amp; Assessment. Please see the ‘Further reading on best practice with use of GenAI’ section for other University resources on use of GenAI that may be relevant to the matters identified above. Structure and overview of this guidance Given the diverse range of work the University undertakes, it is not possible for the University to provide comprehensive instruction on circumstances in which it would or would not be appropriate to use GenAI tools. It is up to departments, faculties and individual members of staff to balance the benefits and risks of the use of GenAI, to make an informed decision about whether its use is appropriate or desirable – before it is initiated. In the limited circumstances where a formal risk assessment is required, the University Data Protection Impact Assessment (DPIA) and Information Security Risk Assessment (ISRA) processes remain the relevant risk assessments processes to follow. To help guide staff in their decision making we have provided the following: - a brief outline of some of the benefits of the use of GenAI - guidance on the risks associated with use of GenAI tools - practical examples of good and bad practice - useful facts about Copilot, Gemini and NotebookLM Regardless of the work being undertaken, it is recommended that staff avoid inputting confidential, sensitive or personal information into GenAI tools unless warranted and only in accordance with this guidance. Please see the UIS guidance on different data types. Where the use of GenAI will not encompass the use of confidential, sensitive, or personal information, the risk to the University is reduced. However, it is still important to consider whether its use constitutes the best available means of completing a task. Any use of AI must be appropriately transparent and accountable. If it is necessary and beneficial to use GenAI tools, it is recommended that wherever practicable the University’s licensed GenAI tools, Copilot, Gemini and NotebookLM are utilised, regardless of the type of data that may be input. Use of other licenced GenAI tools is not prohibited, but such tools must be procured in accordance with any applicable procurement policy or process, including but not limited to the completion of any requisite risk assessments such as DPIAs and/or ISRAs. Any risk associated with their deployment rests with the relevant department. Any use of such GenAI tools should also be accordance with this guidance. Copilot, Gemini and NotebookLM are already available to staff. Microsoft 365 Copilot is the basic licensed version of Copilot and is available via a staff login, and Copilot for Microsoft 365 is the more comprehensive version, which is available via an additional purchased licence. More information on Microsoft 365 Copilot and Copilot for Microsoft 365 is available on the UIS website. Gemini and NotebookLM are available to all University members through Google Workspace. More information on Gemini is available here, and more information on NotebookLM is available here. The public, free versions of Copilot, Gemini and NotebookLM, available via a web browser, must not be used for University activities and purposes as they do not guarantee a sufficient level of information security or confidentiality. Please remember the Acceptable Use Policy (AUP) continues to apply, including its compliance monitoring and enforcement provisions, when using GenAI tools and staff are reminded of their obligation to abide by its terms. In all circumstances, staff are expected to exercise caution and use their judgement in their use of GenAI. Benefits Many potential benefits of using GenAI tools are already apparent, and the University encourages all its staff to make the best use of the information services made available to them. Here is a brief list of the potential benefits of using GenAI tools in support of University administrative activities. Efficiency and productivity GenAI tools can quickly process a lot of information to produce a large amount of output, saving time that can be spent on other tasks, thus boosting efficiency and productivity. Flexibility GenAI can create content in various formats, styles and languages, making it useful in a wide range of circumstances. For example, it could be used to generate drafts of meeting minutes, letters, press releases, social media posts, and other forms of documentation produced in the course of University business. That flexibility also allows the University to engage with different audiences across various platforms. In some circumstances, it may be appropriate and beneficial to use it to produce personalised content. Creativity GenAI can produce novel or unusual content from existing source material, making it a useful tool for the initial part of some creative tasks. For example, it could be used to draft materials that could form part of a marketing campaign. Understanding GenAI doesn’t just have to be used for content production and creation. It could be used to discover and summarise vast amounts of information in more digestible formats, and so it can be a valuable tool in the early stages of research undertaken to support administrative tasks. Risks There are, however, significant legal and reputational risks associated with use of GenAI tools, which can be broadly categorised as follows: - Bias, misinformation and inaccuracy - Data protection law non-compliance - Intellectual property and copyright law non-compliance - AI legislation non-compliance - Reputational damage and other risks This list is not exhaustive, given the overlapping nature of risk categories and the pace of AI development. Staff must consider relevant risks, and whether they are applicable to the circumstances in which they are considering use of GenAI, before any use of GenAI is initiated. Risk: Bias, misinformation and inaccuracy Much GenAI is trained to produce outputs based on information and patterns extracted from data in the public domain. Some of that data will be inaccurate because it is erroneous or obsolete, and some of it will be opinion. Consequently, outputs will sometimes be factually inaccurate or reflect the ignorance, biases or prejudices of individuals or groups in society. GenAI can also be manipulated to deliberately produce biased or inaccurate outputs, presented as fact. Unlike human intelligence, AI does not have the capacity to apply judgement or understand context. It cannot apply moral or critical perspectives. Additionally, there is an inherent risk that the ongoing use of GenAI tools will create and sustain feedback loops, whereby GenAI tools will be trained on text outputs generated by other GenAI tools, further reinforcing existing biases and inaccuracies. In practical terms, that means some outputs will be inaccurate or unbalanced regardless of the phrasing of the text prompt, because the source material is inaccurate or unbalanced. Some output may also be inaccurate because the GenAI tool is ‘hallucinating’ – creating nonsensical or inaccurate outputs that are not directly attributable to the source material. For those reasons, it is important that any GenAI output is thoroughly evaluated by a human being before it is utilised for any purpose. This is especially important where there is the risk of an adverse impact on a group or individual, or the potential for infringement of a person’s rights (e.g. as defined under the Equality Act 2010, the Human Rights Act 1998 or any other relevant legislation). Risk mitigation(s): Ensure that all GenAI outputs are thoroughly evaluated by a human being before they are used. Ensure use of GenAI is acknowledged if it is used to make a significant and unrevised contribution to a substantive or impactful piece of work such as the production of content for formal policies or strategic reports. Risk: data protection law non-compliance GenAI tools and their use are subject to existing laws and regulations and any University policy relevant to their use. This includes data protection laws such as the UK GDPR, the Data Protection Act 2018, the Data (Use and Access) Act 2025 and the University Data Protection Policy. As with the use of other information tools and services, it is important to use licensed versions of tools paid for from a University budget and procured through any applicable procurement process. (Free, unlicensed information tools and services often rely upon intrusive data processing and/or selling as part of their business model.) The University’s standard licensed GenAI tools are Copilot, Gemini and NotebookLM, and these are the tools that should be used to process personal data, where necessary, for which the University is responsible. This ensures that technical, operational and legal safeguards are in place, which protect any personal data that the University controls or otherwise processes. By contrast, inputting data into a free or unlicensed GenAI tool could be considered equivalent to putting it into the public domain – signifying a potential personal data breach. Information input into GenAI tools is also often used to train those tools, which may not be a lawful use of personal data – especially if that data cannot be retrieved or deleted, for example from an AI neural network. Data input into the University’s licensed versions of Copilot, Gemini and NotebookLM is not used to train those tools. It is particularly important to be cautious about inputting sensitive personal information (special category data) such as medical information into GenAI tools. Processing of such information is subject to additional safeguards, and misuse could represent a serious breach of data protection law and/or a breach of confidentiality. Regardless of the type of information you wish to input into a GenAI, you must consider the task you are using it to support. Data must be collected, held and used for only that purpose – for example, as part of a governance process – and any use of AI must be compatible with that reason. With some exceptions (e.g. for academic research), it is not appropriate to use personal data that was collected for a different purpose to do something else with a GenAI tool. It is also important to be mindful of ‘automated decision making’. Automated decision making involves: - making a decision that will affect a person solely by automated means without any human involvement; or - profiling someone – automated processing of personal data to evaluate certain things about an individual that could be used as part of a decision-making process. A common example of automated decision making is a credit check conducted exclusively using AI to decide whether to provide someone with a personal loan. While the use of GenAI to produce text or digital imagery would not necessarily result in a decision being made about an individual, it is not inconceivable that the use of such technology could be used as part of an evaluation process. For example, to review an application for a parking permit to ensure the person applying meets the eligibility criteria. In such circumstances, it is imperative that a human being is ultimately involved in the decision-making process. If after careful consideration you decide to use a GenAI tool, you must tell the affected people that you’re going to do that. That doesn’t mean you must seek consent on a case-by-case basis, but it will mean that relevant privacy notices should be provided or updated. Risk mitigation(s): Be cautious about inputting personal data into GenAI tools, especially sensitive personal data, and only do so where warranted. Do not use free GenAI tools. Use the University’s licensed versions of Copilot, Gemini or NotebookLM. Deploy relevant privacy notices. Risk: intellectual property and copyright non-compliance It has been argued by some affected parties that the entire basis for training GenAI tools through publicly available data is a violation of intellectual property rights and copyright law. There are a series of ongoing and well-publicised copyright cases where high profile individuals and organisations have sued companies that own and operate GenAI. Bearing that in mind, it is important to consider the nature of the content being input into any GenAI tool and whether the University has the right to input that information into that GenAI tool. It is also important that GenAI outputs are thoroughly checked by a human being and cited where appropriate. Risk mitigation(s): Consider whether it is appropriate to input material into GenAI tools. Cite outputs where appropriate. Use the University’s licensed versions of Copilot, Gemini or NotebookLM. Risk: AI legislation non-compliance In March 2024, the European Union (EU) introduced new laws that require organisations using AI in the EU to employ a risk-based approach to their use of AI, especially with regard to the use of personal information. It incrementally started to take effect from February 2025, and non-compliance with the legislation could result in penalties from European regulators. It affects the University where it is processing EU citizens’ data using AI. Risk mitigation(s): Exercise caution and judgement regarding deployment of GenAI to process EU citizens’ data. Document any use of GenAI tools in these circumstances. Risk: Reputational damage and other risks As outlined above, there are various legal risks posed by the use of GenAI, all of which could result in reputational damage to the University. There is also an environmental cost associated to use of GenAI: training GenAI tools requires vast amounts of power and indirectly generates enormous amounts of carbon, meaning there is a sustainability consideration to its use. In the development of some GenAI tools, outputs are checked and refined in a process known as Reinforcement Learning from Human Feedback (RLHF). That process includes human reviewers, often working in countries in the global south for very low wages, routinely viewing objectionable and distasteful materials, and has been reported to have a profoundly negative impact on the health and well-being of many of those workers. University staff will also be expected to provide human oversight of GenAI outputs. Whilst they would not ordinarily be exposed to objectionable nor distasteful materials in the course of administrative work, it is important to consider the risk to University staff wellbeing that could be posed by increased workloads and unrealistic expectations of what can be reasonably achieved using GenAI tools. Risk mitigation(s): Consider the wider impact on the University’s reputation before using GenAI. Consider any other relevant risks. Best practice: practical examples Here are a series of practical examples intended to show both best practice and scenarios in which the use of AI should be considered carefully. It remains important to bear in mind the general risks and benefits associated with use of GenAI in these different contexts. Example 1: Using GenAI for background research Capability: GenAI can be used as a research tool to help gather background information on a topic relating to something you are unfamiliar with. Example scenario: Using GenAI to provide an overview of a new piece of legislation that may affect your work at the University. Good practice: Using the University’s licensed versions of Copilot, Gemini or NotebookLM. Not inputting any personal or confidential information into Mthe University’s licensed versions of Copilot, Gemini or NotebookLM, because it is not required to understand the new legislation. Bad practice: Using an unlicensed GenAI tool. Inputting confidential data into that unlicensed AI tool with the aim of further understanding the legislation, thus committing a personal data breach and/or breach of confidentiality. Example 2: Using GenAI to summarise information Capability: GenAI can be used to summarise information. Example scenario: Using GenAI to prepare a briefing on a University project for a meeting with a commercial partner. Good practice: Using the University’s licensed versions of Copilot, Gemini or NotebookLM. Treating the output as a draft and amending it as appropriate. Thoroughly checking the output to ensure it is factually accurate and unbiased, does not reveal anything confidential to the commercial partner and is reflective of the source material. Acknowledging GenAI has been used to help create the briefing if it has not been materially altered as part of the fact-checking or drafting process. Bad practice: Using an unlicensed GenAI tool. Treating the output as a final draft. Accepting the output as factually accurate and suitable for sharing with a third party and not bothering to check it before presenting it to the commercial partner. Failing to mention it has been created using a GenAI tool. Example 3: Using GenAI to draft a document Capability: GenAI has the ability to produce written outputs in various styles and formats. Example scenario: Using GenAI to create meeting minutes. Good practice: Considering whether use of GenAI is appropriate in these circumstances – this will depend on what the meeting is about. Considering whether the document is likely to contain sensitive information. If the document is likely to contain sensitive information, considering the type of sensitive information, and whether use of GenAI is warranted. If it is appropriate to use a GenAI tool, uusing the University’s licensed versions of Copilot, Gemini or NotebookLM, and ensuring unauthorised AI note-taking bots are prevented from joining the meeting. Using the output as a draft and amending it as appropriate. Bad practice: Using an unlicensed GenAI tool. Inputting confidential or sensitive data into that unlicensed GenAI tool thus committing a personal data breach and/or breach of confidentiality. Failing to follow UIS advice on preventing unauthorised AI note-taking bots from joining your Teams meeting. Example 4: Using GenAI for numerical analysis Capability: GenAI can perform numerical analysis. Example scenario: Using GenAI to analyse the statistical results of a staff survey. Good practice: Considering whether the raw survey data contains personal or sensitive information. If it is appropriate to deploy a GenAI tool, using the University’s licensed versions of Copilot, Gemini or NotebookLM. Telling staff that AI will be used to analyse responses when they are choosing whether they wish to participate. Treating the output as a draft and verifying and amending it as appropriate. Bad practice: Using an unlicensed GenAI tool. Not telling staff that GenAI will be used to analyse their responses. Accepting the output as factually accurate and making an unquestioning decision based on the analysis. Copilot, Gemini and NotebookLM: Useful Facts This section contains a few useful facts that may assist staff in using the University’s licensed GenAI tools. Copilot Here are some tips for using Copilot: - The version of Copilot accessible to most University MS365 users is called “Microsoft 365 Copilot”. A more comprehensive version of Copilot is available called “Copilot for Microsoft 365”, and a licence for its use can be purchased by contacting UIS. - When accessing Microsoft 365 Copilot, you can check whether you are logged into your University MS365 account by viewing the top right-hand corner of your window – you will be able to see your initials (and your name if you click on the initials) if you are logged in. - When attaching documents, these will be automatically saved in a folder called ‘Microsoft Copilot Chat Files’ in your University MS365 account OneDrive. - Delete chat files that are no longer required. - Delete files uploaded into OneDrive as part of the chat process when no longer required. - There is more information regarding OneDrive on the UIS website. Gemini Here are some tips for using Gemini: - When accessing Google Gemini, you can check whether you are logged into your University account by viewing the top right-hand corner of your window – you will be able to see the University of Cambridge logo and one of your initials. - Standard users cannot delete conversations. These can only be deleted by UIS administrators. Consider whether using Copilot would be more appropriate in circumstances where you need or wish to delete any conversations with Gemini. NotebookLM Here are some tips for using NotebookLM: - When accessing Google NotebookLM, you can check whether you are logged into your University account by viewing the top right-hand corner of your window – you will be able to see one of your initials. - Delete notebooks that are no longer required. Further reading on best practice with use of GenAI University resources: - Admissions: AI and undergraduate applications - Communications: Generative AI tools guidelines - Education: Blended Learning Service – AI and Education - Education: Resources for use of AI in education and operations - UIS: Copilot - UIS: Google Gemini - UIS: Google NotebookLM - UIS: Guidance on information security (including policies and data classification) - UIS: LinkedIn Learning at the University of Cambridge (type in ‘GenAI’ when logged in) External resources: - ICO: Guidance and resources on data protection and AI - ISO: ISO - Artificial intelligence - JISC: An introduction to copyright law and practice in education, and the concerns arising in the context of GenerativeAI - GOV.UK: AI Playbook for the UK Government - National Cyber Security Centre: AI and cyber security: what you need to know - OECD: AI Principles Overview Authorship This guidance was composed without the use of AI.</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4109</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
         </is>
       </c>
     </row>
@@ -510,6 +536,19 @@
           <t>Guidance on how you might engage with Generative AI (GenAI) in your assessments effectively and ethically. GenAI is a technique in artificial intelligence in which outputs such as text, images, code, music, and video are generated by software. GenAI is potentially transformative as well as disruptive, and GenAI tools will feature in many academic and professional workplaces. Rather than seek to prohibit your use of them, we will support you in using them effectively, ethically and transparently. However, it may not always be appropriate to use GenAI. Whilst they are attractively powerful and easy to use, GenAI tools can provide misleading or incorrect information. They can also negatively impact your learning by reducing the need for critical engagement that is key to deep and meaningful learning. Additionally, you need to be aware of the difference between reasonable use of such tools, and at what point their use might be regarded as giving you an unfair advantage. Visit the Generative AI Hub For more details on how GenAI works, the ethical implications and limitations of the tools and the ways in which you can use them, please visit the Generative AI Hub. The Generative AI and Academic Skills Moodle course provides a more in-depth look at GenAI in an academic context. GenAI and academic integrity Academic misconduct is strictly prohibited, including the use of essay mills, homework help sites, plagiarism, collusion, falsification, impersonation or any other action which might give me an unfair advantage. An unfair advantage is: • when you hide something and aren't transparent about your approach. • when you take something directly from someone (or something) else and don't reference or acknowledge it. • when you don't follow the assessment guidance. It is not acceptable to use GenAI tools to write your entire assessment and present this as your own work. Words and ideas from GenAI tools are making use of other human authors' ideas without referencing them, which is considered by many to be a form of plagiarism. Using GenAI tools to check your grammar or spelling is usually appropriate if the tool is not rewriting a large proportion of your work. Similarly, tasks such as ideas generation or planning may be an appropriate use. For all assessments, your context and the nature of the assessment must be considered. Your teachers will give guidance on: • what ways (if at all) you are permitted to use GenAI. • which aspects of your work it is appropriate (or even expected) that you use GenAI for. If you are unsure about what constitutes acceptable use of GenAI in an assessment, ask for clarification from the module leader. If no explicit instructions are given, the default for assessments should be that you use GenAI in an assistive role while making sure that the final submission is still substantially your own work. Staff resources on how to guide students on the use of GenAI in assessments can be found on the Generative AI Hub. Category 2 describes in more detail how GenAI might be used in an assistive role. UCL does not use GenAI detectors when marking. Instead, if a marker has any concerns about your work, they may speak to you to get more information. You should not automatically assume this means that they suspect you of academic misconduct. Inappropriate use of GenAI is viewed as plagiarism. This is defined as the representation of other people’s work or ideas as your own without appropriate referencing or acknowledgement. This includes the use of GenAI tools that exceeds that permitted in the assessment brief. If teaching staff suspect that you are trying to pass off GenAI output as your own work then the regulations in the Academic Manual (9.2.5 a), 9.2.5 e) iii, and 9.2.6 c) may apply. You may be invited to an investigatory viva to probe the authorship of your work. How to acknowledge GenAI use in your work You should acknowledge GenAI use where it has been used to assist in the process of creating your work. The Library Skills pages share guidance on how and when to acknowledge GenAI in your work.</t>
         </is>
       </c>
+      <c r="D4" t="n">
+        <v>684</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -527,6 +566,19 @@
           <t>About Generative AI Generative AI tools automatically create content, including text, code, images, and more, based on user prompts. Examples include ChatGPT, Google Gemini, and Microsoft Copilot. Imperial has also launched the dAIsy platform. Text-focused tools are known as Large Language Models (LLMs) and use collections of existing data to predict outputs. They offer rapid content generation but can produce unreliable outputs, making them unsuitable for unverified academic use. Appropriate academic use of generative AI - Consider use of AI outputs as a starting point for research only and rely on academic sources such as databases and peer-reviewed sources. Developing critical thinking and evaluation skills is a key aspect of your education at Imperial. - If you use generative AI as a search tool, be sure to verify all information and cite any material you use for academic purposes. - Guard against AI “hallucinations” by fact-checking every statement before use. - Preserve your own voice in written work - uncritical AI use often yields generic, superficial text lacking true insight and will not demonstrate learning or substantial communication. - For support in developing your academic and scientific writing, consult Imperial’s Centre for Academic English guidance on GenAI and access the support they provide. Imperial guidance and support - Review your department’s current policy on using and disclosing generative AI in academic work. - Consult your Subject Librarian and library resources for advice on evaluating and selecting scholarly sources. - Refer to the guidance below as well as the library’s reference management pages for acknowledgement and referencing guidance. - Unless explicitly authorised, using AI to create assessed work may be treated as an offence such as contract cheating under Imperial’s Plagiarism, Academic Integrity &amp; Exam Offences regulations. - Familiarise yourself with Imperial’s Academic Misconduct Policy for rules on appropriate AI usage. Acknowledging and referencing use of generative AI tools Acknowledging A statement of acknowledgment shows the reader which AI tool you used and for what specific purpose. You should include a statement to acknowledge your use of generative AI tools for all assessed work, in accordance with guidelines from your department or course team. This statement should be written in complete sentences and include the following information: - Name and version of the generative AI tool e.g. Copilot, ChatGPT-5 - Publisher (name of company that provides the AI system) e.g. Microsoft, OpenAI - URL of the AI tool - Brief description (single sentence) of the way in which the tool was used (e.g. summarising notes, generating outlines) - Confirmation that the work is your own Example: I acknowledge the use of ChatGPT-5 (OpenAI, https://chatgpt.com) to generate an outline for background study. I confirm that no content generated by AI has been presented as my own work. Further requirements may be stipulated for a particular piece of assessed work where AI tools are allowed or required. This must be made clear to students when it is set. If unclear, please clarify with your module leader. Additional requirements may include expanded description in the ‘Acknowledgements’ or ‘Methods’ section, such as: - If relevant, the prompt(s) used to generate a response in the AI system. - The date the output was generated. - The output obtained (e.g. a ‘link to chat’ if ChatGPT, or a compilation of all output generated as an appendix). - How the output was changed for use or incorporation into a piece of work (e.g. a tracked-changes document or a descriptive paragraph). Referencing Referencing guidance is provided for Harvard and Vancouver referencing styles on the following pages: Your reference list and bibliography – Harvard Your reference list and bibliography – Vancouver</t>
         </is>
       </c>
+      <c r="D5" t="n">
+        <v>601</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -544,6 +596,19 @@
           <t>General guidance for all students on using generative AI tools in your studies. The University trusts you to act with integrity in your use of generative AI for your studies.It does not ban the use of generative AI, though its use is restricted for assessment. Some of your courses may also restrict its use in other ways. Always check your course level guidance.These top-level guidelines provide clarity on which uses of generative AI are strictly prohibited and constitute academic misconductThey also explain why you should be cautious about over-reliance on generative AI for your learning.This guidance is general and sets out the basics of the University’s position – it is essential that you also check the detailed information provided for each of your courses.Generative AI at EdinburghThe University recognises that developing skills in the responsible use of generative AI is important and will likely be significant for your future life and work. It also recognises that there are times when you may want – or be asked – to use it in your current studies. We want to ensure that you have the knowledge and skills to thrive in a changing world, and we recognise that generative AI can be used creatively, critically and with integrity.These guidelines are general to the whole University. It is important that you are aware that each course will have its own, more detailed, guidance. You should always check your course documentation on this, and speak to your Course Organiser if you are unsure.The University trusts you as students to act responsibly in relation to the use of generative AI. It also recognises that you need clarity on when its use breaches the University’s rules on academic misconduct. These guidelines provide you with this clarity. Unacceptable uses of generative AI for assessmentPassing off someone – or something’s – work as your own for an assessment is academic misconduct. This could be failing to cite a source you have used in piece of assessed work, getting someone else to complete an assessment for you, claiming authorship of machine-generated content or presenting machine-translated work as your own.If you submit a piece of work for assessment that is not your own original work you risk being investigated according to the university’s academic misconduct investigation procedures. This could have serious implications for you and your studies.The following uses of generative AI are not acceptable and constitute misconduct: if you use them you risk investigation and penalties.Presenting AI outputs as your own, original work.Use of an AI translator to convert assessments to English before submission: English is the language of teaching and assessment at Edinburgh – machine translation is treated as false authorship and is not acceptable.Submitting an assessment which includes elements of AI-generated text without acknowledgment.Submitting an assessment which includes AI-generated images, audio or video without acknowledgment.Submitting an assessment which includes AI-generated mathematical formulae or reasoning, or computer code, without acknowledgment.Citing AI-found sources without reading and verifying them.For more detailed information about the restrictions around using AI-supported online proofing tools, please see the University’s Guidance on Proofreading of Student Assessments. Using generative AI to support your learningWhile we have these clear restrictions around the use of generative AI in your assessed work, the University understands that there are ways in which you may wish to use it to support your studies. This might include using it to:brainstorm ideasget quick definitions of conceptsovercome writer’s block through dialoguecheck your grammarorganise or summarise informationre-format your referencesSome courses may encourage or even require you to use it in certain ways, while others may ask you not to use it at all. Again, it is important that you check your course-level guidance on this. Reasons to be cautious about your use of generative AIYou should be aware that there are risks and disadvantages associated with over-use of generative AI to support learning. Cognitive offloadingThere is growing research evidence that over-use of generative AI can negatively affect your learning. You may want to look at studies which raise concern over how ‘cognitive offloading’, ‘metacognitive laziness’ and reduction in capacity for critical thinking may be associated with over-reliance on this technology. If you routinely use generative AI for breaking down and summarising long texts, for example, you will not be developing your own critical skills in the analysis of complex documents. You will also not be practicing and learning how to bring together complex ideas using the power of your own intelligence. Similarly, if you are using it to regularly assist with mathematical reasoning or coding, you are undermining your own ability to learn and become expert at doing this yourself. To make the most of your time at university, embracing the hard work of learning is a better approach than looking for short-cuts. Bias and inaccuracyGenerative AI models are not ‘intelligent’ in the way that humans are intelligent. They have been trained on more text than a human could ever read, but have different capabilities and make different mistakes. While their output often appears convincing and reliable, their behaviour is strongly influenced by the data they are trained on, so they can perpetuate harmful biases, fabricate information and make errors. You will be held accountable for these errors and biases if you include them in assessed work. Higher education should help you develop advanced knowledge which is creative and rigorous, not generic and unreliable. It is best to use your time at university to develop high-level skills that are going to help you throughout life – original thought, engaging writing, critical use of evidence, creative risk-taking and innovation. Using the University’s own generative AI platform (ELM)All University of Edinburgh students have free access to ELM, which offers you a secure gateway to a range of generative AI models. The university encourages you to use ELM over other platforms such as GPT, DeepSeek, Grok etc for the following reasons:In ELM your data is secure – it will not be retained by third party services to train their models or for any other purpose.It is free to use for all staff and students, providing the same access for all and saving you money.ELM provides access to a range of language models including a locally-hosted instance of Llama. This has an optimized architecture that can achieve faster response times and reduced power consumption. You can also choose other models such as GPT within ELM if necessary for your task.Your lecturers do not have access to your chat history in ELM for the purposes of 'checking' your work - like your email account, it is private to you.You can access ELM and find out about training opportunities here. Acknowledging your use of AIIf you choose to use generative AI for aspects of an assessment, it is important to be transparent about how you have done so. You should include a brief acknowledgment at the end of your piece of work, for example:I used OpenAI o4 Mini via ELM to check grammar and spelling throughout my assignment. I also used the Create Image function in ChatGPT to generate the image on page 2.Again – check the detail in your course guidance if you are unsure what is required, as there may be specific things your Course Organiser would like you to cover in your acknowledgment. Citing your use of generative AIIf you use content generated by AI within your work, for example an AI-generated image or text from an AI chatbot, you will need to reference it. This means including an in-text citation or footnote in the body of your work, and a corresponding reference in your reference list. The Library’s guide to using generative AI gives very useful guidance on this. Environmental and social impact of generative AIMany in our community are concerned about the negative impacts of generative AI in areas such as:Energy and resource useExploitative labour practicesIntellectual propertyYou may wish to read more about these via the links above. While there are ongoing efforts to reduce the environmental impact of the datacentres that make AI models work, it is clear that use of generative AI has a higher impact than, for example, a simple web search. If you are concerned about this, consider using the locally-hosted instance of Llama in ELM (see above). It is more efficient in terms of resource use, and provides a more transparent alternative to OpenAI, meaning that it is easier for the university to measure and manage its power consumption.You might also try to limit use of generative AI to purposeful rather than casual use. Links to other sourcesPrinciplesEdinburgh Student Assembly principles on the use of generative AIRussell Group principles on generative AI use in education Further guidanceGenerative AI use for Postgraduate Research studentsLibrary guide to using generative AI in academic work TrainingUniversity of Edinburgh Digital Skills Programme Academic misconduct guidanceFurther guidance on academic misconduct (including plagiarism) and how to avoid itUniversity of Edinburgh Academic Misconduct Procedures Return to ELM main page This article was published on 2025-07-23</t>
         </is>
       </c>
+      <c r="D6" t="n">
+        <v>1486</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -561,6 +626,19 @@
           <t>University of Glasgow - MyGlasgow - not found Skip to main content Cookies We use cookies to improve user experience and allow for personalised advertising via third parties. You can find out more about cookies and how we use them on our privacy policy page . Analytics I'm happy with analytics data being recorded I do not want analytics data recorded Please choose your analytics preference Personalised advertising I’m happy to get personalised ads I do not want personalised ads Please choose your personalised ads preference save choices accept all privacy settings accept We use cookies Necessary cookies Necessary cookies enable core functionality. The website cannot function properly without these cookies, and can only be disabled by changing your browser preferences. Analytics cookies Analytical cookies help us improve our website. We use Google Analytics. All data is anonymised. Switch analytics ON OFF Clarity Clarity helps us to understand our users’ behaviour by visually representing their clicks, taps and scrolling. All data is anonymised. Switch clarity ON OFF Privacy policy close search Staff login Student login Staff a-z MyGlasgow MyGlasgow not found MyGlasgow Students MyGlasgow Staff IT Sport Not found The web page or resource you requested could not be found. Check that you have the right address, or: Go to MyGlasgow Students homepage Go to MyGlasgow Staff homepage Try searching MyGlasgow Search MyGlasgow search</t>
         </is>
       </c>
+      <c r="D7" t="n">
+        <v>224</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -578,6 +656,19 @@
           <t>Artificial Intelligence (AI) Guidance - Key Information for Students (1) Our approach to Artificial Intelligence (AI) Warwick Law School is committed to developing a holistic approach to AI in all aspects of our education. We seek to develop AI literacy among our students to instil good practice regarding the responsible use of AI as a tool to assist (but not replace) their learning and skills development. This includes promoting awareness about the ethical use of AI as well as about the concerns over the robustness and bias of many AI systems. We will monitor the use of AI by students to ensure that this is done responsibly and ethically. This includes monitoring the impact the use of AI has on development of essential academic skills by our students. Academic integrity must be ensured in all activities involving the use of AI. We are committed to understanding the implications of AI for our own subjects as well as the ethical issues raised in all aspects of AI and to ensurin that what we teach includes consideration of the legal and ethical challenges brought about by the use of AI. (2) Artificial Intelligence (AI) (a) AI Technologies Artificial Intelligence is an umbrella term covering a wide range of algorithmic and data-driven software systems. There are different types of algorithms (and combinations of different approaches) with varying capabilities, either of a deterministic or adaptive machine-learning type. AI performs a wide variety of tasks, not always clearly identified as “AI” in people’s minds (e.g., spell-checkers, auto-complete, recommendations on shopping websites or streaming services, etc). The Organisation for Economic Co-operation and Development (OECD) defines an AI system as “a machine-based system that, for explicit or implicit objectives, infers, from the input it receives, how to generate outputs such as predictions, content, recommendations, or decisions that can influence physical or virtual environments. Different AI systems vary in their levels of autonomy and adaptiveness after deployment”.[1] All AI systems have in common that they offer varying degrees of automation for particular tasks, often more efficiently and quicker than humans. A particular sub-category of AI is Generative AI Systems (“GenAI”). They can be useful for some academic tasks, but can also be misused in a way that violates our standards and expectations as to academic integrity. GenAI, such as ChatGPT or Claude, is based on deep-learning neutral networks utilising “transformer” technology. They are trained on vast amounts of data and produces outputs based on that data. The robustness and reliability of outputs can vary dramatically, and there are many caveats to the use of generative AI systems. (b) Limitations of GenAI Importantly, AI does not process information in the way humans do. It does not develop knowledge. It lacks common sense and the ability to locate information in a wider context/experience. Its outputs are generally based on the data on which it was trained, and, in the case of “self-learning” (adaptive) algorithms, data acquired during deployment; it therefore lacks the ability to produce truly original and creative outputs. It does not have the ability for critical thinking – one of the key academic skills we seek to instil and develop in our students. AI can be a very useful tool to help with certain tasks. It can uncover connections in data that might not be apparent to humans (although it is at risk of overfitting, or “hallucinating”, such connections) and can structure data better and faster than humans. Recent advances in the performance and capability of certain AI systems, particularly generative AI systems, have renewed interest in this technology, and have led to an explosion in academic, policy and legislative work. A lot of unsubstantiated or exaggerated claims are made about AI, and it is sometimes difficult to get a clear sense of what the technology is capable of and what its limitations are. There are also concerns about the quality of the data on which AI systems are trained, particularly regarding its robustness and accuracy, and biases. Furthermore, the degree of energy use and the resulting environmental impact of the infrastructure (e.g., data centres) required for some AI systems is starting to attract more attention and concern. (3) Permitted and prohibited uses of GenAI and other AI tools in the classroom (4) Academic Integrity With regard to academic integrity, our policy builds on the University’s Institutional Approach to Artificial Intelligence and Academic Integrity. Any changes to the University’s Institutional Approach, or any new University policies on the use of AI take precedence over this policy whenever there is a conflict between them. In accordance with both the University’s and the Law School’s academic integrity policy, the Law School prohibits copying/paraphrasing either whole outputs or elements of outputs generated by a GenAI system and submitted by students as their own work. Similarly, the use of AI to complete certain parts of an assessment, such as analysis or evaluation, is not permitted. However, even where the use of GenAI systems is not prohibited, the Law School discourages the use of such outputs even with correct and complete attribution. Assessments should be used by students to demonstrate their knowledge of the subject (i.e., what has been taught, including set readings) and their understanding and ability to utilise this in responding to specific questions. The use of GenAI in this process might make it more difficult for markers to establish how well a student has demonstrated this. The way in which such outputs are used as part of an assessment will be considered in grading the assessment against our marking criteria. The use of an AI system for any aspect of completing an assessment must be disclosed by a student. A failure to do so constitutes an academic misconduct. Such a disclosure must cover the following points: - Why was a GenAI system used (help in understanding the question; help in structuring work based on arguments developed; assist with initial summary of readings etc)? - Which GenAI system or systems was/were used (e.g., ChatGPT, Claude etc)? - How has the AI output been used in preparing the assessment? (as a research tool, to test arguments etc; see table below for acceptable uses). The way AI generated outputs are used by you in drafting your assessments will be taken into account when grading the assessment against the generic grade descriptors and assessment-specific marking criteria. (5) Permitted and prohibited uses of GenAI – Guidance to Students Unless expressly required for a specific assessment task, Warwick Law School does not encourage the use of GenAI tools for assessments. Students should be aware that GenAI tools can weaken the quality of your work – particularly if you rely on GenAI for accuracy, relevance and rigour. You should be particularly mindful of the tendency of GenAI tools to cite non-existent resources or information (“hallucinations”). GenAI may generate inaccurate or otherwise poorly constructed arguments. GenAI does not have the ability to demonstrate critical thinking, nor the ability to be genuinely creative. Most importantly, assessments are there for you to demonstrate to us (and to yourself!) how well you have understood what you have studied. Nevertheless, WLS acknowledges that some students may use GenAI technology when preparing for assessments and writing essays, and may want to gain experience of utilising it for their future legal careers. Below, we provide a clear rule and interpretative guidance on what would constitute tolerated and prohibited use of GenAI. This is always subject to specific instructions given for each assessment. Rule and Guidance The key overarching rule is: GenAI can act as a personal assistant for you (e.g. assistance in understanding key issues, help with research, proof-reading your work etc.). However, it must never be used to create the work, or certain parts of the work, for you. You must not submit any AI-generated output as your own work. The table below summarises what is acceptable and what is prohibited in a bit more detail. Note that any use of GenAI may be prohibited for specific assessment tasks. This might be the case e.g., where the assessment tests your key legal or academic skills.Here, your own unaided work would be essential. Always check the assessment instructions before you use any GenAI tool! | YOU CAN | YOU MUST NOT | o Example prompt:“Is the following question asking for a discussion on topic X?” o Careful here! Do not simply ask GenAI to prepare an outline for you. Do your preliminary research and have your points ready. Even slight variations in the prompt can produce vastly different results as can repeating the same prompt twice or more. o Example prompt: “Suggest an outline for the essay I am going to write on the topic X. I will argue for/against Y and the points I will make in my essay are A, B and C. My supporting evidence/examples are D and E.” or “What would be the best order to argue for/against Y with the points A, B and C, and examples D and E?” o Example prompt: “Check the tone and style of this essay and highlight the parts that need to be rewritten, but do not rewrite them!” ·Use GenAI as a search engine/database to find further sources. o Careful here! GenAI tools may sometimes generate sources that do not exist. Always remember to check that the source exists; that the reference/citation is accurate ( check books and journals though the library pages; check case databases for cases); verify that any quotations were taken from the indicated source etc. o Example prompt: “Provide some feedback on the consistency of the arguments made in the project, without rewriting it for me.” o Please remember that GenAI feedback may not reflect the assessment criteria. It’s important to refer to the module's assessment criteria to fully understand the expectations. | o Example prompt:“I need to write an essay, but I could not understand the question. Can you write me an essay on the following essay question: [the essay question].” o Example prompt: “I need to write an essay on the topic X, what should I argue, what should my stance be? Can you suggest some arguments I could use?” o You can only ask GenAI to provide guidance on the accuracy or validity of your arguments or improve the ideas you already have. Asking GenAI to generate ideas and arguments do not result in accurate or original supervised projects. Therefore, you must always double check what the GenAI tools suggest to you and never substitute them for your own voice. o Example prompt:“Provide some feedback on the following essay and rewrite the parts that need improvement.” or “Can you provide some feedback on the following essay?” (Careful here!GenAI tools usually tend to rewrite/revise the text you provide them, unless you clearly restrict them and/or prohibit them from rewriting the whole text in accordance with the feedback they provide. Therefore, even when you ask for feedback, you must ensure that it is you who makes the necessary changes depending on that feedback, not AI.) o Example prompt: “Check the tone and style of the following essay and make the necessary changes/improvements to make it sound more formal.” (You should only ask for suggestions or for some emphasis to be made on the parts that need improvement, you should never ask any GenAI tool to change the sentences you have written. Remember, it should entirely be your own work, GenAI should not and cannot be a contributing author!) |</t>
         </is>
       </c>
+      <c r="D8" t="n">
+        <v>1902</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -595,6 +686,19 @@
           <t>Using generative AI Understand where to use generative artificial intelligence (AI) appropriately for your studies and in preparation for your future. Go to: What is generative AI? | Generative AI and your studies | University of Nottingham policy | Further information Always check expectations for generative AI use and acknowledgement for any given module or assessment. What is generative AI? “Artificial intelligence, or AI, is technology that enables computers and machines to simulate human intelligence and problem-solving capabilities.” (IBM, 2024) Generative artificial intelligence is a form of AI technology that can produce text, images, and other media in response to user prompts. These tools (including ChatGPT and Microsoft Copilot) are not sentient - they only mimic intelligence, through algorithmic prediction and pattern recognition. Drawing on large quantities of data, these tools create outputs based on probability. It is important to remember that the responses provided by generative AI tools do not express meaning, understanding, or intentionality. As a result, responses generated by these tools cannot be relied upon to be accurate and always need to be fact-checked. Back to the top Generative AI and your studies The use of AI tools is becoming common practice across a variety of industries, which means that understanding how to use generative AI effectively and responsibly will likely be a key skill for employment. You might at times be asked to use AI within your studies, to help you develop skills relating to its effective, responsible, and professional use. For other assessments, use of generative AI may be prohibited, as the assessment is designed to develop your academic and transferable skills. Back to the top University of Nottingham policy Key points to remember Content created or significantly modified by generative AI, whether text, code, images, or video, should only be used if this is clearly stated to be essential or optional for an assessment task, and should always be fully evidenced and acknowledged. - Always consult your tutor or assessment documents on expectations for AI use - Always fact-check any information generated using AI - Always be transparent in acknowledging your use of generative AI, - Always keep records of your interactions with AI tools Back to the top Back to the top Continue your journey You may also be interested in: Further support Disability support service Language and communication skills</t>
         </is>
       </c>
+      <c r="D9" t="n">
+        <v>387</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -612,6 +716,19 @@
           <t>This is the current version of this document. You can provide feedback on this document to the document author - refer to the Status and Details on the document's navigation bar. Section 1 - Purpose (1) This Policy outlines the principles that support the responsible and ethical use of Artificial Intelligence (AI) at Macquarie University (the University), in alignment with the University’s purpose, values and strategic priorities. (2) This Policy ensures the consistent application of the eight principles that guide the responsible and ethical use of AI. Scope (3) This Policy applies to all Staff, Students and Affiliates of the University, encompassing all uses of Artificial Intelligence (AI) by these groups. Top of PageSection 2 - Policy (4) Artificial Intelligence (AI) has the potential to enhance teaching and learning, research, innovation and social impact at the University. However, AI also poses significant ethical, legal and social challenges that need to be addressed with care and responsibility. (5) The following eight principles outline the University’s expectations for the design and the responsible and ethical use of AI, which are informed by Australia’s AI Ethics Principles and the NSW Mandatory Ethical Principles for the use of AI: - Positive Impact: - AI should deliver positive results across research, education, and operations, supporting informed decision-making. Its use should align with the goal of delivering meaningful benefits compared to other available tools. - AI Literacy and Confidence: - The University will encourage AI literacy among Staff and Students, ensuring they can use AI tools responsibly and understand their broader implications in various contexts. - Academic and research integrity: - The University will build awareness among Students and Staff of their responsibilities around the use of AI tools. - The University will manage integrity-related risks posed by AI tools in accordance with the Academic Integrity Policy, the Assessment Policy and the Macquarie University Code for the Responsible Conduct of Research. - Fairness and Inclusivity: - AI tools and systems made available and authorised by the University for Students and Staff will be evaluated carefully before deployment to ensure that these do not unfairly discriminate against individuals or groups. - Diverse perspectives should be encouraged and included in AI development teams to ensure that systems are designed and deployed with a comprehensive understanding of potential impacts on different groups. - Engagement with Students, Staff and Affiliates should occur in order to understand needs and concerns relating to AI systems and to allow for feedback to be considered in the AI development process. - Privacy and Security: - The University will undertake regular assessments to ensure that the use of AI systems and tools does not compromise data security or intellectual property rights and complies with University policy, including the Privacy Policy, the Cyber Security Policy, the Data Breach Policy, the Intellectual Property Policy, and the AI Reference Architecture. - Accessibility and Equity: - The University will work to eliminate barriers and aim to ensure that appropriate AI systems and tools are available regardless of financial or personal circumstances. - Human Oversight and Responsibility: - The University is responsible for those AI tools and systems made available and authorised by the University to Staff, Students and Affiliates (Users). - For AI tools and systems supporting staff decision-making, the final decision-making authority resides with qualified staff who can validate or override AI outputs, particularly in high-risk contexts. - Users of AI systems and tools are responsible for any generated output used for work, research or study purposes. - The University will establish clear reporting processes for concerns about AI tools and systems provided by the University. - Users of AI tools and systems provided by the University must use these for their intended purpose and in accordance with the Acceptable Use of IT Resources Policy. - A risk assessment will be conducted by the Head of AI prior to the implementation of an AI system to identify potential risks and measures to mitigate these risks in accordance with the Risk Management Policy, and in compliance with the AI Reference Architecture. - Continuous Review and Improvement: - The University will regularly review its AI Policy (and any related procedures) and update as necessary to meet evolving needs and maintain ethical standards. (6) If a Student or Staff member is alleged to have used Generative AI in a manner that is inconsistent with the principles of this Policy, the University may investigate the allegation in accordance the relevant policy (i.e. Academic Integrity Policy, Staff Code of Conduct, Macquarie University Code for the Responsible Conduct of Research, Acceptable Use of IT Resources Policy). Top of PageSection 3 - Procedures (7) Nil. Top of PageSection 4 - Guidelines (8) Nil. Top of PageSection 5 - Definitions (9) The following definitions apply for the purpose of this Policy: - Affiliates refers to contractors, agents, honorary, clinical or adjunct appointees and consultants of the University. - AI has the meaning provided in the NSW AI Assurance Framework, being “intelligent technology, programs and the use of advanced computing Algorithms that can augment decision-making by identifying meaningful patterns in data”. - Deep Learning is a subset of machine learning that uses advanced neural networks to simulate human cognitive processes, enabling the handling of complex tasks. - Generative Artificial Intelligence (Gen AI) is subset of Deep Learning and a wide-ranging term that refers to any form of artificial intelligence capable of generating new content, such as text, images, video, audio or code (New South Wales Government’s Generative AI: Basic Guidance). - Machine Learning refers to systems that use advanced algorithms to learn from historical data and improve performance over time. - Staff means all persons employed by the University, including continuing, fixed term and casual Staff members. - Student means a person currently enrolled in a unit of study or program at the University.</t>
         </is>
       </c>
+      <c r="D10" t="n">
+        <v>967</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -629,6 +746,19 @@
           <t>Students will be equipped to use generative AI responsibly in their education and future careers under the sector-leading new assessment policy at the University of Sydney. From Semester 1 2025, the University will change its default to allow the use of AI for assessments, except for exams and in-semester tests or if teaching staff choose not to. From Semester 2, the University will move to a realistic and forward-looking ‘two-lane approach’ to assessments comprising: Students will be required to apply critical thinking and analysis to produce original work aided by appropriate learning tools, including acknowledging how they use AI. Professor Joanne Wright, Deputy Vice-Chancellor (Education), said the University of Sydney is leading the way in integrating modern AI technologies within education. “This is a substantial change to our teaching, assessment and program design, and it is absolutely necessary to ensure our graduates are equipped with the tools they need for the modern workforce. “Generative AI has already had a profound impact on workplaces and our graduates are expected to demonstrate skilled use of the relevant tools in job interviews. The changes we’re making to teaching and assessments ensures we are preparing students for their careers, without compromising their learning or the integrity of our world-class education.” Two academics from the University of Sydney were recently asked by TEQSA, the national quality assurance and regulatory agency, to show the risks and opportunities of AI in assessment. The resulting videos reveal just how easy it is for a novice to complete many traditional assessments, and equally how helpful AI can be to accelerate learning and enhance productivity. Professor Adam Bridgeman, Pro Vice-Chancellor (Educational Innovation), said universities have needed to adapt rapidly to the significant advancement in the capability of generative AI tools over the past two years. “It’s no secret that any take-home assessment can be completed to a high level by AI, and it’s not practical, enforceable or desirable to implement a blanket ban on these tools, or even to restrict their use. “We have worked closely with the regulator, educators and students to chart a way forward in a world where AI is ubiquitous and that satisfies the principles and purposes of higher education.” Training has been developed for staff to support the transition alongside workshops, resources and ongoing communications for students and staff. The changes are the latest in a range of University initiatives helping students and staff use generative AI equitably, effectively and ethically. These include a partnership with Microsoft to make the generative AI tool Copilot for Web available to students and staff for free, with regular training sessions. The University’s AI in Education Working Group of staff and students recently co-designed and launched a publicly available online guide AI in Education showing how generative AI can be used productively and responsibly in assessment and learning. The University has also developed an AI assistant for students called Cogniti, which allows teachers to create customised AI agents that can be steered with instructions and subject-specific information, answer students’ questions about content and syllabus, and provide instant personalised feedback, guidance and support, 24 hours a day. At Sydney, over 1000 Cogniti agents have been developed. Cogniti has won many awards and has been adopted by many other institutions in Australia and beyond. The University was named AI University of the Year in the 2024 Future Campus Awards, in recognition of its leadership in the field.</t>
         </is>
       </c>
+      <c r="D11" t="n">
+        <v>566</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -646,6 +776,19 @@
           <t>Using Artificial Intelligence (AI) in university Learn about our stance on Artificial Intelligence (AI) UNSW recognises there are ethical and responsible uses of AI and generative AI (GenAI) tools that can support student learning. AI can be a helpful tool for tasks, such as initial research, summarising information, data analysis and more. However, when it comes to completing independent research, coursework and assessments, it's important to ensure the work you produce is your own. The university adopts a firm approach to ensuring you complete the work that is expected and that this demonstrates you have met learning outcomes assigned within your courses. The degree to which you can use AI varies between faculties, programs and courses. Reach out to your course convenor, lecturer or tutor to understand the rules and expectations. Unsure about using AI in your work? When using AI in your assessment, a simple principle to remember is: If you are given permission and wish to use AI in the process of planning, designing, or writing your assessment, you should always clearly acknowledge this. Responsible use of Generative AI tools As an early adopter, UNSW supports and nurtures the ethical and responsible use of AI in research, learning, teaching, administration, and thought leadership. See our principles below on the ethical and responsible use of Artificial Intelligence at UNSW: - The use of AI systems at UNSW benefits UNSW, individuals, society, and the environment. - The use of AI systems at UNSW is equitable, and respectful of human rights, diversity, inclusivity, and accessibility. - AI systems and their lifecycle at UNSW are trustworthy and are used responsibly, safely, and reliably in accordance with their intended purpose. - The use of AI systems is transparent, and people understand when the AI system is engaging with or impacting them, the environment, and/or society. - AI systems and their lifecycle used at UNSW are identifiable, explainable, interpretable, accountable, and contestable. - AI systems and their lifecycle used at UNSW are secure and resilient. See also When using AI, remember to: - Check your course guidelines to see if the use of AI is permitted, including its usage as a translation tool. See the levels of AI assistance and what they entail - Maintain your academic integrity. Do not copy and paste AI-generated materials and claim them as your own. Learn how to reference AI in your assessments - Protect personal information. Do not include any personal or sensitive information in prompts, your own or other people's (i.e. addresses, name, emails, zID or intellectual property). For data privacy and protection, use Microsoft Copilot using your UNSW account - Verify accuracy of AI outputs. GenAI tools could produce invalid or unreliable information ('fabrications' or 'hallucinations'). Book an appointment with the Academic Skills team if you need guidance. Levels of AI assistance The Levels of AI Assistance framework is designed to help convenors communicate to students how much, or how little AI can be used in the process of planning, creating and producing an assignment. To ensure clarity in UNSW AI policy, and how to use AI responsibly in your assessments, we've created this resource for further guidance. Download the framework or read below. - This assessment is designed for you to complete without the use of any generative AI. You are not permitted to use any generative AI tools, software or service to search for or generate information or answers. - In completing this assessment, you are permitted to use standard editing and referencing functions in the software you use to complete your assessment (for example Microsoft Word, Mendeley, Zotero). You are not allowed to use any generative AI tools including prompts or features that generate text. Using functions that generate or paraphrase passages of text or other media, whether based on your own work or not, can be grounds for academic misconduct. - This category permits the use of generative AI as ‘inspiration’ for assessment. For example, generating initial ideas, structures, or outlines. Beyond that, the use of generative AI is prohibited. You are permitted to use generative AI tools, software or services to generate initial ideas, structures, or outlines only. After you've used generative AI for inspiration you must develop those ideas to produce your own work. - This category permits the use of generative AI as a 'coach'. Learning usually takes effort. In recognition of this, this category requires you to make a first attempt at the task yourself. Once this is done you can use generative AI to improve your submission. The focus is on your thoughts and creation with the AI helping you edit your work. The AI-based edit must be attributed, and this reinforces the responsible use of generative AI in a scholarly context. The degree of referencing or attribution may vary on the nature of the task – from general acknowledgement to full attribution of all editing suggestions. Your Convenor will specify the types of attribution required, as well as when generative AI tools can be used throughout the assessment. Keep copies of your drafts as your convenor may also request them as part of the submission If outputs of generative AI tools, software or services form part of your submission and are not appropriately attributed, your Convenor may ask you to explain your work. If you are unable to satisfactorily demonstrate your understanding of your submission and how you have done it you may be referred to UNSW Conduct &amp; Integrity Office for investigation for academic misconduct and possible penalties. - This assessment is designed for you to use generative AI as part of the assessed learning outcomes. Please refer to the assessment instructions for more details. This category expects a wide range of use of generative AI in assessment. Your convenor will specify what they want you to do with generative AI. This may include assessments where a first draft is generated by generative AI and you are asked to critique that draft; it may be an assessment where a particular generative AI tool is required to be used; or it may be an assessment where you have options to use or not use those tools. - This assessment would not likely require or benefit from the use of AI. However, if you do use it, it must be properly referenced. Frequently Asked Questions (FAQs) - Read your assessment instructions carefully to understand what level of AI use is permitted, and note that what is permitted will vary across different assessments. - At some points in your learning, it will be important to assess your understanding without the use of AI tools. - At other points, you may be assessed on how well you have learnt to use the tools. Your convenors will set the level of acceptable use of AI for each assessment based on course learning outcomes. - The unauthorised or unacknowledged use of AI in assessments is a form of cheating and is considered to be student misconduct at UNSW under the current Code of Conduct and Values. If you have been found to use AI in a manner that does not meet the course instructions, penalties may occur which would include a fail, a mark of zero for the course, suspension or permanent exclusion. - All academics marking assessments submitted through either Moodle Turnitin Assignment or Inspera now have access to Turnitin’s new AI detection tool. This provides academics with an estimated percentage of text that has similarities to AI-generated or AI-paraphrased text (text that was originally written by AI but then rewritten to avoid detection). The document will include highlights of the relevant passages that the detector has flagged. This is not always conclusive evidence that a student has inappropriately used generative AI, however, this will be a flag for a marker to further review a student’s submission. It’s important that students are aware of what tools use generative AI and may be inappropriate in an assessment. For example, Grammarly, Quillbot and translation tools such as Google Translate, DeepL and Baidu Translate are forms of generative AI. - When using AI tools, such as ChatGPT or Copilot, it's important to properly cite and credit use. Acknowledging the use of AI when you have used it helps ensure the honesty and integrity of your work. In cases where the use of AI has been prohibited, please respect this and be aware that where unauthorised use is detected, penalties may apply. - If you need help with your assessments, there are alternatives to unauthorised AI use. You can: - Seek support from your teacher if you’re under too much pressure or apply for Special Consideration if you’re eligible, or - Seek help from the Academic Skills Team by booking a consultation, attending a Study Hacks session, or exploring our toolkit to see our available resources. - Translation tools automatically convert text or speech from one language to another. Some popular tools include ChatGPT, Copilot, Google Translate and DeepL Translator. Acceptable use varies by course, so check assessment guidelines or consult teaching staff if you’re unsure. It is essential to create and express your own ideas in assessments. Misusing tools, such as copying outputs from ChatGPT and claiming them as your own, undermines your ability to demonstrate a genuine understanding of course material. Spelling and grammar checks, like those in Microsoft Word, are generally acceptable as they don’t alter the meaning of your work. However, verify suggested changes, as editing tools can unintentionally distort your understanding. Some programs, like Google Docs, include AI editing features that may generate or refine text. If AI tools such as ChatGPT or Grammarly are used where permitted, you must reference or acknowledge them. Keep draft versions of your work to show your process if concerns about validity arise. - UNSW acknowledges that these tools can sometimes support learning but warns that inappropriate use may hinder English language development. Many multilingual students note that translating writing into English can negatively affect learning and reduce originality. For example, dictating in one language and translating into English often results in AI-generated text that lacks nuance or fails to convey the intended meaning. Additionally, relying on translation tools may pose challenges if your work is flagged as AI-generated, requiring you to explain ideas that may not fully reflect your understanding. Always check assessment guidelines to confirm whether AI translation tools are permitted in your course. - If your Convenor has concerns that your submission contains passages of AI-generated text or media, you may be asked to have a conversation about your work. If you are unable to satisfactorily demonstrate your understanding of your submission, you may be referred to UNSW Conduct &amp; Integrity Office for investigation for academic misconduct and possible penalties. Have a question? If you have any questions about UNSW AI policy or referencing AI in university, we’re here to help.</t>
         </is>
       </c>
+      <c r="D12" t="n">
+        <v>1802</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -663,6 +806,19 @@
           <t>Page not found | Australian National University Skip to main content Page not found The requested page could not be found. We use cookies to improve your experience with ANU. For an optimal experience, we recommend enabling all cookies. The ANU Privacy Policy outlines how we handle your personal information - Read more Cookie settings Accept all Cookie Settings We recommend enabling all cookies to provide you with the optimal experience while visiting our website. Essential Cookies Always Active These cookies are required for basic site functionality and are always enabled. Analytics cookies are used to record anonymous site usage data. No personally identifiable data is collected. Marketing Cookies Marketing Cookies These cookies are set by a range of social media services that we have added to the site to enable you to share our content with your friends and networks. They are capable of tracking your browser across other sites and building up a profile of your interests. This may impact the content and messages you see on other websites you visit. If you do not allow these cookies you may not be able to use or see these sharing tools. Back Button Cookie List Search Icon Filter Icon Clear checkbox label label Apply Cancel Consent Leg.Interest checkbox label label checkbox label label checkbox label label Confirm my choices Your Privacy [`dialog closed`]</t>
         </is>
       </c>
+      <c r="D13" t="n">
+        <v>224</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -680,6 +836,19 @@
           <t>Page not found - my.UQ - University of Queensland Skip to menu Skip to content Skip to footer my.UQ Menu Page not found The requested page could not be found. We're sorry, but there is no web page that matches your entry. It is possible you typed the address incorrectly, or the page may no longer exist. You may wish to try another entry or choose from the links below, which we hope will help you find what you’re looking for. If you are certain that this URL is valid, please send us feedback about the broken link. You may wish to try one of the following links: my.UQ homepage UQ Search page UQ Homepage</t>
         </is>
       </c>
+      <c r="D14" t="n">
+        <v>115</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -694,7 +863,20 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>On this page AI Statement of Intent | Purpose | Scope | Principles | Policy statements | Roles and responsibilities | Definitions | Approval information | Version history | References AI Statement of Intent UTS is a recognised global leader in Artificial Intelligence (AI). Our thought leadership and innovation extend across: - The creation of new AI models, tools and technology through our research and research collaborations - The implementation of AI in real-world applications through our innovations and partnerships with business, civil society, and government - The education of our students to be skilful, responsible users of AI in their studies and future employment, and - Our work to ensure that ethical, legal and other societal impacts are considered in the development and use of AI. As a progressive organisation, UTS also evaluates and leverages AI models and tools in our business operations where it is appropriate to do so. 1. Purpose 1.1 The Artificial Intelligence Operations Policy (the policy) guides the use, procurement, development and management of artificial intelligence (AI) at UTS for the purposes of teaching, learning and operations. 2. Scope 2.1 This policy applies to staff and affiliates (hereafter staff) who are responsible for AI at UTS for teaching, learning and operational functions. 2.2 This policy applies to the: - development, approval, use and management of AI software, systems or platforms developed or created for use by UTS, and - approval, use and management of AI software, systems or platforms procured for use by UTS. 2.3 This policy does not apply to research projects and outputs (including university consulting). Information on the use of AI in research, as well as required research approvals and ethics clearances, is provided in the Research Policy and the Use of AI in Research Guidelines. 3. Principles 3.1 AI at UTS may be used for administrative and operational functions, teaching and learning activities and to improve user experiences as part of the delivery of the university’s object and functions (refer University of Technology Sydney Act 1989 (NSW)). 3.2 To ensure confidence in UTS processes, and alignment with the UTS 2030 strategy, AI must be ethical, reliable, transparent, secure and comply with applicable laws and regulations. 3.3 UTS acknowledges that: - there are legitimate concerns about the use and reliability of AI and will seek to identify the balance between opportunity for improvement and automation, while managing and mitigating risks to the university and its community at all times - algorithmic bias may result in erroneous or unjustified differential treatment which could have unintended or serious consequences for groups of individuals and/or for their human rights - the use of AI will be increasingly regulated and, as such, this policy and any associated procedure must be maintained to ensure compliance with current and emerging regulatory standards and government advice. 3.4 Use of AI systems must comply with the Privacy Policy, the Procurement Policy, the Information Security Policy and the Acceptable Use of Information Technology Resources Policy as appropriate. 4. Policy statements How is AI used at UTS? 4.1 At UTS, AI may be used to support teaching, learning and operational functions and activities, including but not limited to: - making operations more efficient (increasing consistency, speed, agility and scalability) - improving competitiveness to quickly adapt to changing conditions - improving speed and agility to identify issues, risks and opportunities or improve controls - protecting UTS physical and digital resources - verifying identity and highlighting potential cheating - providing feedback to students - identifying at-risk and high-achieving students (to improve learning outcomes and provide additional support) - engaging in student support activities - improving student and staff experiences and/or capabilities - recommending study pathways towards identified career goals - recommending optimal allocation of campus facilities, and - marketing activities including ranking prospects and personalisation. AI risks and opportunities 4.2 All AI systems exist on a spectrum of risk, ranging from low-risk (not automated, often non-operational, does not contain personal or sensitive data and does not have direct impacts on individuals) to high-risk automations (highly autonomous, normally operational AI systems with minimal controls that could impact individual and institutional safety and wellbeing). 4.3 Guided by the NSW Government’s AI Assessment Framework (the NSW framework) operational and non-operational AI will be assessed for risks and opportunities as outlined in the Artificial Intelligence Operations Procedure (the procedure) and the Risk Management Policy. 4.4 UTS will: - assess and manage the use of AI to understand and effectively manage these risks (refer the procedure), and - balance risks and opportunities to protect UTS and individuals and their human rights (refer also Risk Management Policy). AI endorsement, approval and oversight 4.5 Business owners must submit proposed AI systems to the Head of Data Analytics and Artificial Intelligence for feedback before commencement of any development or procurement activities as outlined in the procedure. 4.6 The Artificial Intelligence Operations Board (the board) will develop institutional knowledge and insights about the use, management and control of AI for the purposes of teaching, learning and operations at UTS. 4.7 The board’s terms of reference and membership are approved by the Chief Operating Officer (COO) and are available to staff (refer the procedure). The board will provide an annual report to the University Leadership Team. 4.8 The board is responsible for endorsing the use of AI as part of an identified business activity or solution before the procurement and/or development of AI systems. Where the board considers a system to be high risk, further advice (internal or external) may be sought before submission to the COO for endorsement. 4.9 Following the board’s or the COO’s endorsement of an AI system, the final approval for expenditure of funds will apply as follows: - For projects that require funding: refer to the financial delegations for project approval authority (refer Delegations). - For IT Capital Management Plan (ITCMP): follow standard ITCMP processes (available at ITCMP project governance and delivery framework (Staff Connect)). - For projects that result in the acquisition or procurement of an IT resource: refer to the Procurement Policy and the Acceptable Use of Information Technology Resources Policy for approval process and authority. 4.10 AI system owners must work with AI business owners in the ongoing management, governance and monitoring of AI in systems once procured or implemented, including liaising with information system stewards (refer Data Governance Policy and Transparency and reliability) or the Information Technology Unit as appropriate. Ethical principles for the use of AI 4.11 UTS follows the NSW Government’s Mandatory Ethical Principles for the Use of AI, summarised as follows: - Community benefit: AI should deliver the best outcome for human users, in this case, the UTS community, and provide key insights into decision-making. AI must be the most appropriate solution for a service delivery or a policy problem, considered against other analysis and policy tools. - Fairness: Use of AI will include safeguards to manage data bias or data quality risks. The best use of AI will depend on data quality and relevant data as well as careful data management to ensure potential data biases are identified and appropriately managed (refer also Data Governance Policy). - Privacy and security: AI will include the highest levels of assurance. The UTS community must have confidence that data is used safely and securely in a manner that is consistent with privacy, data sharing and information access requirements (refer also the Privacy Policy and the Records Management Policy). - Transparency: Review mechanisms will ensure that the UTS community can challenge and question AI-based outcomes and will have access to an efficient and transparent review mechanism if there are questions about the use of data or AI-informed outcomes (refer Policy breaches and complaints). - Accountability: While AI is recognised for analysing and looking for patterns in large quantities of data, undertaking high-volume routine process work, or making recommendations based on complex information, AI-based functions and decisions must always be subject to human review and intervention. AI system owners and business owners are responsible for the management of their AI systems. 4.12 The ethical principles for the use of AI are applied at each phase of the AI system lifecycle. The lifecycle stages include: - problem identification and requirements analysis - planning, design, data collection and modelling - development and validation (including training and testing stages) - deployment and implementation - monitoring, review and refinement (including when fixing any problems that occur) or destruction (removal of the system from use). Transparency and reliability 4.13 AI systems must only operate in accordance with their primary purpose or objective as outlined as part of the approval process. Where a change to the primary purpose is needed, this requires a separate risk assessment and endorsement. 4.14 Where AI is used by UTS to automate a function, process or decision that may impact staff, students or others, this must be specifically identified in the relevant privacy and/or AI use disclosure notice, which must include a review or enquiry mechanism. Privacy and records management 4.15 Where personal information is captured, used or stored by an AI system the business owner must complete a privacy impact assessment (refer Privacy hub: Privacy impact assessments (SharePoint)). This must be approved and managed in line with the Privacy Policy and information security classifications. 4.16 Use of biometric identification must be treated as processing sensitive personal information (refer Privacy Policy). 4.17 Data used to develop algorithms or AI systems, and any data generated, shared, managed and/or recorded as part of an AI system’s operation or algorithm, is considered corporate data and must be managed in line with the Data Governance Policy and the Privacy Policy. This requirement applies to the full system lifecycle and to the lifetime of the data (whichever is the longer). Policy breaches and complaints 4.18 Breaches of this policy or any associated procedures must be reported to the Chief Data Officer (CDO) and managed in line with the Code of Conduct and the relevant Enterprise agreement as appropriate. 4.19 Any data breaches or suspected data breaches will be managed in line with the Data Breach Policy. 4.20 Complaints in relation to the use or outcomes of UTS AI systems will be managed in line with the Staff Complaints Policy or the Student Complaints Policy. 5. Roles and responsibilities 5.1 Policy owner: The Chief Data Officer (CDO) is responsible for policy enforcement and compliance, ensuring that its principles and statements are observed. The CDO is also responsible for the approval of any associated university level procedure. 5.2 Policy contact: The Head of Data Analytics and Artificial Intelligence (Data Analytics and Insights Unit) is responsible for the day-to-day implementation of the policy and acts as a primary point of contact for advice on fulfilling its provisions. The Head of Data Analytics and Artificial Intelligence is also responsible for providing guidance and advice on the application of this policy and the procedure and for recommending appropriate training for staff who have responsibility for AI. 5.3 Implementation and governance roles: The Chief Operating Officer (COO) is responsible for the establishment of the Artificial Intelligence Operations Board as outlined in this policy and the procedure. The COO is responsible for endorsing high-risk AI systems before normal approval processes in line with this policy. The Deputy Vice-Chancellor (Research) is responsible for the management of all research activities, including guidance on AI in research (refer the Research Policy and the Use of AI in Research Guidelines). AI system owners and AI business owners are responsible for the approval, management and oversight of AI systems within their remit. 6. Definitions The following definitions apply for this policy and all associated procedures. These are in addition to the definitions outlined in Schedule 1, Student Rules. Definitions in the singular also include the plural meaning of the word. Algorithm means a series of specific directions or instructions built into computer software or systems to solve a defined problem or automate decision-making. Algorithms may use AI to produce improved outcomes. Algorithmic bias means an error or prejudice built into an algorithm (intentionally or unintentionally) that creates outcomes that are unfair, erroneous or favour one group of people over another and may impact an individual’s human rights. Artificial intelligence (AI) UTS uses the NSW Government’s AI Assessment Framework definition, which states that AI is ‘intelligent technology, programs and the use of advanced computing algorithms that can augment decision-making by identifying meaningful patterns in data’. AI is used to solve problems autonomously, and perform tasks to achieve defined objectives, in some cases without explicit human guidance. AI system (also system) means any software system, technology or program at UTS that uses AI as part of its decision-making processes, in part or in whole. AI systems include capabilities, analytics and algorithms on new or existing IT resources. AI system lifecycle means the time from inception through to review and renewal or destruction of an AI system. AI system owner means appropriate staff identified as responsible for the technical implementation of the AI system and its review and monitoring as outlined in the approved project. Where there are multiple AI system owners, a primary owner (normally the most senior staff member) must be identified. AI system owners must have a working relationship with any relevant information system steward (refer Data Governance Policy). Business owner (of AI systems) means staff with overall accountability for the AI system. Business owners have responsibility for establishing the business case for the system, implementing the system (including identifying users, user training and risk management), monitoring its activities (including reporting and review, ensuring benefits and outcomes are realised in line with the purpose), AI ethics and providing support to the AI system owner(s). Business owners may be self-identified (during an approval or initial scoping exercise) or appointed in line with their position description. Normally business owners will be a dean, director, senior manager or equivalent. Corporate data is defined in the Data Governance Policy. Information system steward is defined in the Data Governance Policy. IT resource is defined in the Acceptable Use of Information Technology Resources Policy. Non-operational AI system means AI systems that do not use a live environment for their source data, rather, provide analysis and insight from historical data. While, normally, non-operational AI represents a lower level of risk, the risk level needs to be carefully assessed, particularly where the outputs may be used to influence decision-making or action. Operational AI system means to either produce an act or decision, or to prompt a human to act. Normally these systems work in real time using a live environment for their source data. These systems generally present more risks than non-operational AI systems as they tend to have a real-world effect. However, not all operational AI systems are high risk (for example, digital information boards or apps that show the time of arrival of the next bus). Personal information (which includes health information for the purposes of this policy) is defined in the Privacy Policy. Research project is defined in the Research Policy. Research output is defined in the Research Policy. Approval information | Policy contact | Head of Data Analytics and Artificial Intelligence | |---|---| | Approval authority | Vice-Chancellor | | Review date | 2026 | | File number | UR23/685 | | Superseded documents | New policy | Version history | Version | Approved by | Approval date | Effective date | Sections modified | |---|---|---|---|---| | 1.0 | Vice-Chancellor | 18/05/2023 | 09/06/2023 | New policy. | | 1.1 | Vice-Chancellor | 24/05/2024 | 29/05/2024 | Updated to include the AI Statement of Intent. | | 1.2 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 20/06/2024 | 08/07/2024 | Updates to reflect the review of the Acceptable Use of Information Technology Resources Policy and the Information Security Policy. | | 1.3 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 24/04/2025 | 30/04/2025 | Update to refer to new Use of AI in Research Guidelines. | | 1.4 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 09/05/2025 | 04/06/2025 | Update to reflect new UTS 2030 strategy. |</t>
+          <t>On this page AI Statement of Intent | Purpose | Scope | Principles | Policy statements | Roles and responsibilities | Definitions | Approval information | Version history | References AI Statement of Intent UTS is a recognised global leader in Artificial Intelligence (AI). Our thought leadership and innovation extend across: - The creation of new AI models, tools and technology through our research and research collaborations - The implementation of AI in real-world applications through our innovations and partnerships with business, civil society, and government - The education of our students to be skilful, responsible users of AI in their studies and future employment, and - Our work to ensure that ethical, legal and other societal impacts are considered in the development and use of AI. As a progressive organisation, UTS also evaluates and leverages AI models and tools in our business operations where it is appropriate to do so. 1. Purpose 1.1 The Artificial Intelligence Operations Policy (the policy) guides the use, procurement, development and management of artificial intelligence (AI) at UTS for the purposes of teaching, learning and operations. 2. Scope 2.1 This policy applies to staff and affiliates (hereafter staff) who are responsible for AI at UTS for teaching, learning and operational functions. 2.2 This policy applies to the: - development, approval, use and management of AI software, systems or platforms developed or created for use by UTS, and - approval, use and management of AI software, systems or platforms procured for use by UTS. 2.3 This policy does not apply to research projects and outputs (including university consulting). Information on the use of AI in research, as well as required research approvals and ethics clearances, is provided in the Research Policy and the Use of AI in Research Guidelines. 3. Principles 3.1 AI at UTS may be used for administrative and operational functions, teaching and learning activities and to improve user experiences as part of the delivery of the university’s object and functions (refer University of Technology Sydney Act 1989 (NSW)). 3.2 To ensure confidence in UTS processes, and alignment with the UTS 2030 strategy, AI must be ethical, reliable, transparent, secure and comply with applicable laws and regulations. 3.3 UTS acknowledges that: - there are legitimate concerns about the use and reliability of AI and will seek to identify the balance between opportunity for improvement and automation, while managing and mitigating risks to the university and its community at all times - algorithmic bias may result in erroneous or unjustified differential treatment which could have unintended or serious consequences for groups of individuals and/or for their human rights - the use of AI will be increasingly regulated and, as such, this policy and any associated procedure must be maintained to ensure compliance with current and emerging regulatory standards and government advice. 3.4 Use of AI systems must comply with the Privacy Policy, the Procurement Policy, the Information Security Policy and the Acceptable Use of Information Technology Resources Policy as appropriate. 4. Policy statements How is AI used at UTS? 4.1 At UTS, AI may be used to support teaching, learning and operational functions and activities, including but not limited to: - making operations more efficient (increasing consistency, speed, agility and scalability) - improving competitiveness to quickly adapt to changing conditions - improving speed and agility to identify issues, risks and opportunities or improve controls - protecting UTS physical and digital resources - verifying identity and highlighting potential cheating - providing feedback to students - identifying at-risk and high-achieving students (to improve learning outcomes and provide additional support) - engaging in student support activities - improving student and staff experiences and/or capabilities - recommending study pathways towards identified career goals - recommending optimal allocation of campus facilities, and - marketing activities including ranking prospects and personalisation. AI risks and opportunities 4.2 All AI systems exist on a spectrum of risk, ranging from low-risk (not automated, often non-operational AI systems, do not contain personal or sensitive data and do not have direct impacts on individuals) to high-risk automations (highly autonomous, normally operational AI systems with minimal controls that could impact individual and institutional safety and wellbeing). 4.3 Guided by the NSW Government’s AI Assessment Framework (the NSW framework), UTS will: - assess operational and non-operational AI systems for risks and opportunities as outlined in the Artificial Intelligence Operations Procedure (the procedure) and the Risk Management Policy. - assess the use of AI to understand and effectively manage any risks through appropriate controls (refer the procedure), and - balance risks and opportunities to protect UTS and individuals and their human rights (refer also Risk Management Policy). 4.4 AI systems assessed as high-risk are unsanctioned and may be blocked or restricted. Unsanctioned AI systems must not be used on UTS devices or on personal devices that are used to undertake UTS activities (refer Acceptable Use of Information Technology Resources Policy and ThinkSecurely: High-risk GenAI monitoring on managed devices (SharePoint)). AI endorsement, approval and oversight 4.5 Business owners must submit proposed AI systems to the Head of Data Analytics and Artificial Intelligence for feedback before commencement of any development or procurement activities as outlined in the procedure. 4.6 The Artificial Intelligence Operations Board (the board) will develop institutional knowledge and insights about the use, management and control of AI for the purposes of teaching, learning and operations at UTS. 4.7 The board’s terms of reference and membership are approved by the Chief Operating Officer (COO) and are available to staff (refer the procedure). The board will provide an annual report to the University Leadership Team. 4.8 The board is responsible for endorsing the use of AI as part of an identified business activity or solution before the procurement and/or development of AI systems. Where the board considers a system to be high risk, further advice (internal or external) may be sought before submission to the COO for endorsement. 4.9 Following the board’s or the COO’s endorsement of an AI system, the final approval for expenditure of funds will apply as follows: - For projects that require funding: refer to the financial delegations for project approval authority (refer Delegations). - For IT Capital Management Plan (ITCMP): follow standard ITCMP processes (available at ITCMP project governance and delivery framework (Staff Connect)). - For projects that result in the acquisition or procurement of an IT resource: refer to the Procurement Policy and the Acceptable Use of Information Technology Resources Policy for approval process and authority. 4.10 AI system owners must work with AI business owners in the ongoing management, governance and monitoring of AI in systems once procured or implemented, including liaising with information system stewards (refer Data Governance Policy and Transparency and reliability) or the Information Technology Unit as appropriate. Ethical principles for the use of AI 4.11 UTS follows the NSW Government’s Mandatory Ethical Principles for the Use of AI, summarised as follows: - Community benefit: AI should deliver the best outcome for human users, in this case, the UTS community, and provide key insights into decision-making. AI must be the most appropriate solution for a service delivery or a policy problem, considered against other analysis and policy tools. - Fairness: Use of AI will include safeguards to manage data bias or data quality risks. The best use of AI will depend on data quality and relevant data as well as careful data management to ensure potential data biases are identified and appropriately managed (refer also Data Governance Policy). - Privacy and security: AI will include the highest levels of assurance. The UTS community must have confidence that data is used safely and securely in a manner that is consistent with privacy, data sharing and information access requirements (refer also the Privacy Policy and the Records Management Policy). - Transparency: Review mechanisms will ensure that the UTS community can challenge and question AI-based outcomes and will have access to an efficient and transparent review mechanism if there are questions about the use of data or AI-informed outcomes (refer Policy breaches and complaints). - Accountability: While AI is recognised for analysing and looking for patterns in large quantities of data, undertaking high-volume routine process work, or making recommendations based on complex information, AI-based functions and decisions must always be subject to human review and intervention. AI system owners and business owners are responsible for the management of their AI systems. 4.12 The ethical principles for the use of AI are applied at each phase of the AI system lifecycle. The lifecycle stages include: - problem identification and requirements analysis - planning, design, data collection and modelling - development and validation (including training and testing stages) - deployment and implementation - monitoring, review and refinement (including when fixing any problems that occur) or destruction (removal of the system from use). Transparency and reliability 4.13 AI systems must only operate in accordance with their primary purpose or objective as outlined as part of the approval process. Where a change to the primary purpose is needed, this requires a separate risk assessment and endorsement. 4.14 Where AI is used by UTS to automate a function, process or decision that may impact staff, students or others, this must be specifically identified in the relevant privacy and/or AI use disclosure notice, which must include a review or enquiry mechanism. Privacy and records management 4.15 Where personal information is captured, used or stored by an AI system the business owner must complete a privacy impact assessment (refer Privacy hub: Privacy impact assessments (SharePoint)). This must be approved and managed in line with the Privacy Policy and information security classifications. 4.16 Use of biometric identification must be treated as processing sensitive personal information (refer Privacy Policy). 4.17 Data used to develop algorithms or AI systems, and any data generated, shared, managed and/or recorded as part of an AI system’s operation or algorithm, is considered corporate data and must be managed in line with the Data Governance Policy and the Privacy Policy. This requirement applies to the full system lifecycle and to the lifetime of the data (whichever is the longer). Policy breaches and complaints 4.18 Breaches of this policy or any associated procedures must be reported to the Chief Data Officer (CDO) and managed in line with the Code of Conduct and the relevant Enterprise agreement as appropriate. 4.19 Any data breaches or suspected data breaches will be managed in line with the Data Breach Policy. 4.20 Complaints in relation to the use or outcomes of UTS AI systems will be managed in line with the Staff Complaints Policy or the Student Complaints Policy. 5. Roles and responsibilities 5.1 Policy owner: The Chief Data Officer (CDO) is responsible for policy enforcement and compliance, ensuring that its principles and statements are observed. The CDO is also responsible for the approval of any associated university level procedure. 5.2 Policy contact: The Head of Data Analytics and Artificial Intelligence (Data Analytics and Insights Unit) is responsible for the day-to-day implementation of the policy and acts as a primary point of contact for advice on fulfilling its provisions. The Head of Data Analytics and Artificial Intelligence is also responsible for providing guidance and advice on the application of this policy and the procedure and for recommending appropriate training for staff who have responsibility for AI. 5.3 Implementation and governance roles: The Chief Operating Officer (COO) is responsible for the establishment of the Artificial Intelligence Operations Board as outlined in this policy and the procedure. The COO is responsible for endorsing high-risk AI systems before normal approval processes in line with this policy. The Deputy Vice-Chancellor (Research) is responsible for the management of all research activities, including guidance on AI in research (refer the Research Policy and the Use of AI in Research Guidelines). AI system owners and AI business owners are responsible for the approval, management and oversight of AI systems within their remit. 6. Definitions The following definitions apply for this policy and all associated procedures. These are in addition to the definitions outlined in Schedule 1, Student Rules. Definitions in the singular also include the plural meaning of the word. Algorithm means a series of specific directions or instructions built into computer software or systems to solve a defined problem or automate decision-making. Algorithms may use AI to produce improved outcomes. Algorithmic bias means an error or prejudice built into an algorithm (intentionally or unintentionally) that creates outcomes that are unfair, erroneous or favour one group of people over another and may impact an individual’s human rights. Artificial intelligence (AI) UTS uses the NSW Government’s AI Assessment Framework definition, which states that AI is ‘intelligent technology, programs and the use of advanced computing algorithms that can augment decision-making by identifying meaningful patterns in data’. AI is used to solve problems autonomously, and perform tasks to achieve defined objectives, in some cases without explicit human guidance. AI system (also system) means any software system, technology, application or program at UTS that uses AI as part of its decision-making processes, in part or in whole. AI systems include capabilities, analytics and algorithms on new or existing IT resources. AI system lifecycle means the time from inception through to review and renewal or destruction of an AI system. AI system owner means appropriate staff identified as responsible for the technical implementation of the AI system and its review and monitoring as outlined in the approved project. Where there are multiple AI system owners, a primary owner (normally the most senior staff member) must be identified. AI system owners must have a working relationship with any relevant information system steward (refer Data Governance Policy). Business owner (of AI systems) means staff with overall accountability for the AI system. Business owners have responsibility for establishing the business case for the system, implementing the system (including identifying users, user training and risk management), monitoring its activities (including reporting and review, ensuring benefits and outcomes are realised in line with the purpose), AI ethics and providing support to the AI system owner(s). Business owners may be self-identified (during an approval or initial scoping exercise) or appointed in line with their position description. Normally business owners will be a dean, director, senior manager or equivalent. Corporate data is defined in the Data Governance Policy. Information system steward is defined in the Data Governance Policy. IT resource is defined in the Acceptable Use of Information Technology Resources Policy. Non-operational AI system means AI systems that do not use a live environment for their source data, rather, provide analysis and insight from historical data. While, normally, non-operational AI represents a lower level of risk, the risk level needs to be carefully assessed, particularly where the outputs may be used to influence decision-making or action. Operational AI system means to either produce an act or decision, or to prompt a human to act. Normally these systems work in real time using a live environment for their source data. These systems generally present more risks than non-operational AI systems as they tend to have a real-world effect. However, not all operational AI systems are high risk (for example, digital information boards or apps that show the time of arrival of the next bus). Personal information (which includes health information for the purposes of this policy) is defined in the Privacy Policy. Research project is defined in the Research Policy. Research output is defined in the Research Policy. Approval information | Policy contact | Head of Data Analytics and Artificial Intelligence | |---|---| | Approval authority | Vice-Chancellor | | Review date | 2026 | | File number | UR23/685 | | Superseded documents | New policy | Version history | Version | Approved by | Approval date | Effective date | Sections modified | |---|---|---|---|---| | 1.0 | Vice-Chancellor | 18/05/2023 | 09/06/2023 | New policy. | | 1.1 | Vice-Chancellor | 24/05/2024 | 29/05/2024 | Updated to include the AI Statement of Intent. | | 1.2 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 20/06/2024 | 08/07/2024 | Updates to reflect the review of the Acceptable Use of Information Technology Resources Policy and the Information Security Policy. | | 1.3 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 24/04/2025 | 30/04/2025 | Update to refer to new Use of AI in Research Guidelines. | | 1.4 | Deputy Director, Corporate Governance (Delegation 3.14.2) | 09/05/2025 | 04/06/2025 | Update to reflect new UTS 2030 strategy. | | 1.5 | Director, Governance Support Unit (Delegation 3.14.1) | 17/12/2025 | 22/12/2025 | Update to address use of high-risk GenAI. Minor update to definition of AI system. | References Acceptable Use of Information Technology Resources Policy Artificial Intelligence Operations Procedure NSW Government AI Assessment Framework NSW Government Mandatory Ethical Principles for the use of AI ThinkSecurely: High-risk GenAI monitoring on managed devices (SharePoint) Use of AI in Research Guidelines</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2795</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
         </is>
       </c>
     </row>
@@ -714,6 +896,19 @@
           <t>Key points: Gen AI isn’t going away, so learn to use it wisely and within the bounds of Curtin’s Gen AI guidelines. • Get permission before using Gen AI in your assessments • Declare any use of Gen AI • Use Curtin’s version of Grammarly for safe editing support • Double-check AI-generated content for accuracy • Never submit AI-written text as your own Generative AI tools like ChatGPT, Claude, or Google Gemini are everywhere. From writing help to meal plans, they’re reshaping how we learn and live. At Curtin, students are allowed to use Gen AI tools, but not without boundaries. Here’s how to navigate Gen AI tools at Curtin while keeping your academic integrity intact. Rule 1: You need permission Let’s start with the big one: if you want to use Gen AI to help with an assignment, you must get permission from your Unit Coordinator. That means before using AI to brainstorm ideas, generate outlines, get feedback on your writing or help with sentence structure or clarity, you need to check your unit’s specific rules or contact your tutor directly. Some units allow limited use of Gen AI, while others don’t allow it at all. Rule 2: If you use it, declare it If you get permission to use Gen AI, you also need to be transparent about how you used it. Curtin has provided a clear format for this: a declaration you include in your assignment submission that outlines what tools you used and how. You can find a declaration template and example on the Library website. If you use AI and don’t declare it? That could be seen as misconduct, even if you didn’t mean to cheat. Rule 3: Check your outputs for accuracy Gen AI tools are impressive, but they’re not perfect. They can ‘hallucinate’ false facts, give outdated advice or suggest biased responses. Always check anything it tells you against real sources, and don’t assume it’s right just because it sounds confident. You are responsible for all information submitted for assessments, so if the information from the Gen AI tool was incorrect and still used, this may affect your marks. What tools are available? All students have free access to Curtin’s version of Grammarly through Blackboard. This version has the generative AI features disabled, meaning it checks grammar and clarity but won’t rewrite your text or suggest full sentences. That makes it safe to use across all units. Microsoft Copilot, Adobe Express Premium and Microsoft Teams are other tools you can use at Curtin using your student log-in details. For more information, visit our website. Tools you should be cautious of While popular AI platforms like ChatGPT can be useful, don’t assume they’re always allowed. If you use them to generate parts of your assignment without permission or proper referencing, it’s likely to trigger Turnitin and raise red flags. When in doubt, ask Every unit at Curtin has different expectations. If you’re unsure whether GenAI use is okay in a particular assignment, don’t guess. Instead, ask your tutor or Unit Coordinator directly. Using Gen AI responsibly at Curtin is about being honest, informed and clear about your process. To learn more about using Gen AI at Curtin, familiarise yourself with the information available on our website.</t>
         </is>
       </c>
+      <c r="D16" t="n">
+        <v>542</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -728,7 +923,20 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ERROR: The request could not be satisfied 403 ERROR The request could not be satisfied. Request blocked. We can't connect to the server for this app or website at this time. There might be too much traffic or a configuration error. Try again later, or contact the app or website owner. If you provide content to customers through CloudFront, you can find steps to troubleshoot and help prevent this error by reviewing the CloudFront documentation. Generated by cloudfront (CloudFront) Request ID: hZs_xS4yJF8V9ACHH6f69YxrhQDybs2ZM5Qhc-Fob230l2WyR-otGg==</t>
+          <t>ERROR: The request could not be satisfied 403 ERROR The request could not be satisfied. Request blocked. We can't connect to the server for this app or website at this time. There might be too much traffic or a configuration error. Try again later, or contact the app or website owner. If you provide content to customers through CloudFront, you can find steps to troubleshoot and help prevent this error by reviewing the CloudFront documentation. Generated by cloudfront (CloudFront) Request ID: mQX9imsvjIEiWTe_SptReioqPDucxdIQwFzfUjlDYvNNX4nXjWKMxg==</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>82</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
         </is>
       </c>
     </row>
@@ -745,7 +953,20 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Using generative AI in teaching and learning Explore the new myCourses self-paced module: Generative AI for Teaching and Learning What is generative AI? Generative AI is a type of artificial intelligence that uses machine learning to create new types of media, including text, images, sound, and video. Many tools exist that use generative AI to create new content. Some examples include: Media | Example tools | |---|---| Text | Copilot (Secure version approved at McGill) | Images | Copilot (Secure version approved at McGill) Adobe Firefly, Midjourney, DALL-E3 (not approved for use at McGill) | Sound | Copilot (Secure version approved at McGill) Voiceify (not approved for use at McGill) | Video | D-ID (not approved for use at McGill) | A secure version of Microsoft Copilot has been approved at McGill. Copilot is an AI chatbot tool integrated into Microsoft Edge and accessible from other browsers. Read more about using Copilot at McGill. Generative AI tools are built upon large language models (LLM) that have been trained on enormous corpora of information and are designed to respond to input prompts with well-structured output. They are focused on predictive text (i.e., the most likely word to follow a previous word), as well as generated media based on patterns or styles in existing datasets. While the outputs can often demonstrate seemingly sophisticated language interaction, there may be situations where they provide inaccurate information in that interaction (e.g., fictional sources). These tools are constantly improving; however, it is important to examine any generative AI output with a critical lens. The McGill Library has a page on artificial intelligence with a section on AI Literacy that discusses the importance of critically approaching AI. Ethical use of generative AI The development of generative AI has brought many ethical considerations that must be addressed with its use. The 2018 Montreal Declaration for a Responsible Development of Artificial Intelligence and the 2021 UNESCO Recommendation on the Ethics of Artificial Intelligence provide a number of principles important to the adoption of these new technologies. Both documents offer an excellent framework for how organizations need to consider these new technologies. The emergence of generative AI is leading to a process of reflection on the evolution of the concept of academic integrity. For any questions related to disciplinary procedures, contact the Office of the Dean of Students. Learn more: AI in academia: The end of the essay? (Maple League of Universities - YouTube video) Infographic: Generative AI explained by AI (Visual Capitalist) Teaching AI literacy: How to begin (Inside Higher Education) What is generative AI? (McKinsey) How can generative AI be used in teaching and learning? In May 2023, the Senate Subcommittee on Teaching and Learning (STL) created a working group to address the use of generative AI at McGill. The working group drafted a report with key recommendations for the use of generative AI at McGill. The report also presents principles for the use of generative AI in teaching and learning. Many different strategies exist for using generative AI tools in course teaching. For example, instructors can use them to create sample texts for students to analyze; create images for presentations; design entire presentation materials; and generate sample practice questions. Strategies also exist for students to use generative AI tools to support their learning. For example, they can be used to brainstorm ideas; create images to support assignments such as presentations; and summarize documents. These resources offer more ideas for creating instructional materials and supporting student learning: How could AI be used for learning and teaching? and How AI can be used meaningfully by teachers and students in 2023. It is important to note that students need AI literacy skills to responsibly use generative AI tools. These potentially new literacy skills could include elements such as fact-checking and prompt engineering. Avoid AI detection tools AI detection tools are tools designed to identify content that is partially or wholly generated by AI. These tools (specifically regarding generated text) are unreliable and often inaccurate, a statement corroborated by OpenAI, the creators of ChatGPT. OpenAI states that their false positive rate is 9%, which is a similar rate found in other AI detection tools. A false positive is when the tool identifies text as being generated by AI when it was actually created by a student. False positive results misguide instructors and can create situations where students are wrongly accused of a violation that they did not commit, forcing them to defend work that is rightfully theirs. Such situations can result in a negative classroom climate and create unnecessary stress and anxiety for all involved. McGill therefore discourages the use of AI detection tools. Course outline statements There should be no default assumption as to the use of generative AI tools. Therefore, McGill recommends that instructors explain to students in their course outline what the appropriate use or non-use is of generative AI tools in the context of that course. The use or non-use of these tools should align with the learning outcomes associated with the course. For this reason, instructors will need to write their own context-appropriate course outline statements. Below are four external examples to draw on: Monash University policy and practice guidance around acceptable and responsible use of AI technologies: See the Actions box and the section entitled Specify conditions for the use of generative AI in assessment. University of Florida has an excellent AI resource page that shows concise examples of course outline statements and multiple categories of suggestions on how to either neutralize or capitalize on using AI in courses. University of Toronto syllabus language: This document provides suggestions for clarifying whether students can use generative AI tools; can use generative AI tools in certain instances; or cannot use them at all in the course. Update your course syllabus for ChatGPT (Medium): See the section entitled Before editing your syllabus and the one entitled Update your syllabus. If you allow students to use generative AI tools in your course, provide guidance in your course outline for how students should acknowledge the use. Monash University provides useful examples, as well as links to APA and MLA citation guidelines. See the section entitled How students acknowledge the use of generative AI. AI and assessment of student learning Generative AI tools can be used to support many different types of assessment. As with the planning of any assessment of student learning, it is important to be intentional about the strategy. In this case, be intentional about either designing AI into your assessments or designing AI out of your assessments. This reflective process will encourage you to think through your assessments and determine if the integration of AI is appropriate (or not) for allowing students to demonstrate their learning. Designing AI into an assessment could involve having students generate the assignment with an AI tool, then critique the output, and reflect on the process. Designing AI out of the assessment could involve in-class writing exercises, where students create and share their ideas with other students in class during class time. Either way, the decision should align with students’ achievement of the desired learning outcomes. Monash University provides excellent considerations for assessment design. Learn more: 6 Tenets of postplagiarism: Writing in the age of artificial intelligence (Teaching and Leadership) AI-generated content in the classroom: Considerations for course design (Illinois State University) Artificial Intelligence (UNESCO) Beyond Grading: Assessment in the age of AI (McGill, video, 50 minutes) Bloom’s taxonomy revisited with AI (Oregon State University) Bowen, J. A., &amp; Watson, C. E. (2024). Teaching with AI: A practical guide to a new era of human learning. Johns Hopkins University Press How do I Consider the Options for a Generative AI Course Policy? (Center for Teaching and Learning, University of Massachusetts Amherst) McGill Library guide on artificial intelligence (McGill Library) The Artificial Intelligence Assessment Scale (AIAS): A Framework for Ethical Integration of Generative AI in Educational Assessment. (2024). Journal of University Teaching and Learning Practice, 21(06). Resources: Have a question that was not answered in this article? Visit our FAQs. McGill University is on land which has served and continues to serve as a site of meeting and exchange amongst Indigenous peoples, including the Haudenosaunee and Anishinabeg nations. Teaching and Academic Programs acknowledges and thanks the diverse Indigenous peoples whose footsteps mark this territory on which peoples of the world now gather. This land acknowledgment is shared as a starting point to provide context for further learning and action. McLennan Library Building 3415 McTavish Street Suite MS-12 (ground level), Montreal, Quebec H3A 0C8 | mcgill.ca/tap</t>
+          <t>Using generative AI in teaching and learning Explore the new myCourses self-paced module: Generative AI for Teaching and Learning What is generative AI? Generative AI (gen AI) is a type of artificial intelligence that uses machine learning to create new types of media, including text, images, sound, and video. Many tools exist that use generative AI to create new content. Some examples include: Media | Example tools | |---|---| Text | Copilot (Secure version approved at McGill) | Images | Copilot (Secure version approved at McGill) Adobe Firefly, Midjourney, DALL-E3 (not approved for use at McGill) | Sound | Copilot (Secure version approved at McGill) Voiceify (not approved for use at McGill) | Video | D-ID (not approved for use at McGill) | A secure version of Microsoft Copilot has been approved at McGill. Copilot is an AI chatbot tool integrated into Microsoft Edge and accessible from other browsers. Read more about using Copilot at McGill. Generative AI tools are built upon large language models (LLM) that have been trained on enormous corpora of information and are designed to respond to input prompts with well-structured output. They are focused on predictive text (i.e., the most likely word to follow a previous word), as well as generated media based on patterns or styles in existing datasets. While the outputs can often demonstrate seemingly sophisticated language interaction, there may be situations where they provide inaccurate information in that interaction (e.g., fictional sources). These tools are constantly improving, however, it is important to examine any generative AI output with a critical lens. The McGill Library has a page on artificial intelligence with a section on AI Literacy that discusses the importance of critically approaching AI. Ethical use of generative AI The development of generative AI has brought many ethical considerations that must be addressed with its use. The 2018 Montreal Declaration for a Responsible Development of Artificial Intelligence and the 2021 UNESCO Recommendation on the Ethics of Artificial Intelligence provide a number of principles important to the adoption of these new technologies. Both documents offer an excellent framework for how organizations need to consider these new technologies. The emergence of generative AI is leading to a process of reflection on the evolution of the concept of academic integrity. For any questions related to disciplinary procedures, contact the Office of the Dean of Students. McGill instructors should follow the same disciplinary procedures as for any other instance where there are concerns about academic integrity. To note: the Code of Student Conduct was updated last month and it now includes specific reference to generative AI with respect to academic offenses (see Articles 25-b and 26-f). For further information, such as the quantity of cases McGill is dealing with, the Office of the Dean of Students might be able to provide information. Instructors might be able to mitigate such cases by providing students with guidance about whether and how gen AI use is permitted in their courses. McGill strongly recommends that all instructors include in their course outlines a statement about gen AI use. Learn more: AI in academia: The end of the essay? (Maple League of Universities - YouTube video) Infographic: Generative AI explained by AI (Visual Capitalist) Teaching AI literacy: How to begin (Inside Higher Education) What is generative AI? (McKinsey) How can generative AI be used in teaching and learning? In May 2023, the Senate Subcommittee on Teaching and Learning (STL) created a working group to address the use of generative AI at McGill. The working group drafted a report with key recommendations for the use of generative AI at McGill. The report also presents principles for the use of generative AI in teaching and learning. Many different strategies exist for using generative AI tools in course teaching. For example, instructors can use them to create sample texts for students to analyze, create images for presentations, design entire presentation materials, and generate sample practice questions. Strategies also exist for students to use generative AI tools to support their learning. For example, they can be used to brainstorm ideas, create images to support assignments such as presentations, and summarize documents. These resources offer more ideas for creating instructional materials and supporting student learning: How could AI be used for learning and teaching? and How AI can be used meaningfully by teachers and students in 2023. Assessment is one facet of course design. The course design approach we promote at McGill suggests beginning with learning outcomes – what knowledge/skills/values would we like students to leave a course with? From there, we can consider what types of assessments align with the desired outcomes. The advent of gen AI might mean rethinking what those learning outcomes are before considering how to redesign assessment. Rethinking learning outcomes – this is an important consideration with implications for higher ed/society. Specifically in online education, McGill promotes experiential learning activities that require students to apply skills, make decisions, and produce work similar to what they would encounter in professional practice. These activities may take the form of interactive simulations, scenario-based assessments, authentic tasks linked to real-world contexts, and reflective activities that help students connect their experiences with course concepts. In some cases, gen AI use is intentionally integrated into the learning activities and requires that any use of gen AI tools be properly cited. It is important to note that students need AI literacy skills to responsibly use generative AI tools. These potentially new literacy skills could include elements such as fact-checking and prompt engineering. All McGill instructors and students can explore the new myCourses self-paced module Generative AI for Teaching and Learning. Avoid AI detection tools AI detection tools are tools designed to identify content that is partially or wholly generated by AI. These tools (specifically regarding generated text) are unreliable and often inaccurate, a statement corroborated by OpenAI, the creators of ChatGPT. OpenAI states that their false positive rate is 9%, which is a similar rate found in other AI detection tools. A false positive is when the tool identifies text as being generated by AI when it was actually created by a student. False positive results misguide instructors and can create situations where students are wrongly accused of a violation that they did not commit, forcing them to defend work that is rightfully theirs. Such situations can result in a negative classroom climate and create unnecessary stress and anxiety for all involved. McGill therefore discourages the use of AI detection tools. Note: McGill also does not recommend online proctoring. Course outline statements There should be no default assumption as to the use of generative AI tools. Therefore, McGill recommends that instructors explain to students in their course outline what the appropriate use or non-use is of generative AI tools in the context of that course. The use or non-use of these tools should align with the learning outcomes associated with the course. For this reason, instructors will need to write their own context-appropriate course outline statements. Below are four external examples to draw on: Monash University policy and practice guidance around acceptable and responsible use of AI technologies: See the Actions box and the section entitled Specify conditions for the use of generative AI in assessment. University of Florida has an excellent AI resource page that shows concise examples of course outline statements and multiple categories of suggestions on how to either neutralize or capitalize on using AI in courses. University of Toronto syllabus language: This document provides suggestions for clarifying whether students can use generative AI tools; can use generative AI tools in certain instances; or cannot use them at all in the course. Update your course syllabus for ChatGPT (Medium): See the section entitled Before editing your syllabus and the one entitled Update your syllabus. If you allow students to use generative AI tools in your course, provide guidance in your course outline for how students should acknowledge the use. Monash University provides useful examples, as well as links to APA and MLA citation guidelines. See the section entitled How students acknowledge the use of generative AI. AI and assessment of student learning Generative AI tools can be used to support many different types of assessment. As with the planning of any assessment of student learning, it is important to be intentional about the strategy. In this case, be intentional about either designing AI into your assessments or designing AI out of your assessments. This reflective process will encourage you to think through your assessments and determine if the integration of AI is appropriate (or not) for allowing students to demonstrate their learning. Designing AI into an assessment could involve having students generate the assignment with an AI tool, then critique the output, and reflect on the process. Designing AI out of the assessment could involve in-class writing exercises, where students create and share their ideas with other students in class during class time. Either way, the decision should align with students’ achievement of the desired learning outcomes. Monash University provides excellent considerations for assessment design. Learn more: 6 Tenets of postplagiarism: Writing in the age of artificial intelligence (Teaching and Leadership) AI-generated content in the classroom: Considerations for course design (Illinois State University) Artificial Intelligence (UNESCO) Beyond Grading: Assessment in the age of AI (McGill, video, 50 minutes) Bloom’s taxonomy revisited with AI (Oregon State University) Bowen, J. A., &amp; Watson, C. E. (2024). Teaching with AI: A practical guide to a new era of human learning. Johns Hopkins University Press How do I Consider the Options for a Generative AI Course Policy? (Center for Teaching and Learning, University of Massachusetts Amherst) McGill Library guide on artificial intelligence (McGill Library) The Artificial Intelligence Assessment Scale (AIAS): A Framework for Ethical Integration of Generative AI in Educational Assessment. (2024). Journal of University Teaching and Learning Practice, 21(06). Resources: Generative AI for teaching and learning (myCourses module for instructors and students) Generative AI perspectives and practices from McGill instructors across disciplines (podcast series) (Re)designing assessments in the age of generative AI - slides (Re)designing assessment tasks in the age of generative AI - activity sheet Sharing experiences with generative AI in teaching and learning - slides Sharing experiences with generative AI (teaching and learning community) Teaching consultations (one-on-one meeting with a TAP staff member) Have a question that was not answered in this article? Visit our FAQs. McGill University is on land which has served and continues to serve as a site of meeting and exchange amongst Indigenous peoples, including the Haudenosaunee and Anishinabeg nations. Teaching and Academic Programs acknowledges and thanks the diverse Indigenous peoples whose footsteps mark this territory on which peoples of the world now gather. This land acknowledgment is shared as a starting point to provide context for further learning and action. McLennan Library Building 3415 McTavish Street Suite MS-12 (ground level), Montreal, Quebec H3A 0C8 | mcgill.ca/tap</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1805</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
         </is>
       </c>
     </row>
@@ -765,6 +986,19 @@
           <t>Policy on use of generative artificial intelligence (AI) in Major Research Papers (MRP) The MRP is an opportunity for the student to demonstrate knowledge and understanding of the research conducted on their topic, and show their ability to perform independent, graduate-level work. Researching and writing the MRP contribute to student learning, including the development and enrichment of critical thinking and critical analysis. For these reasons, it is important to understand when and how AI should and should not be used when developing and writing the MRP. Before using AI as part of writing an MRP, students should be aware that AI poses certain risks, including: • Academic integrity issues when AI-generated material is passed off as the student’s own work • Jeopardizing intellectual property of any materials or data that students input into AI – and many other free apps Jeopardizing confidentiality in the case of primary sources of data • • Environmental costs, including electricity consumption. While generative AI can be an effective tool to help with specific parts of the research process (see below), it is essential to consider whether it supports critical thinking and critical analysis and the building of skills in those domains (appropriate) or whether it offloads these skills to a generative AI tool (not appropriate).1 Before using AI generated output in your MRP, you must verify that it is accurate, avoids (unacknowledged) biases, and correctly acknowledges contributions from others. It is never acceptable to use AI generated text in your MRP. The following is a non-exhaustive list of permitted and prohibited uses.2 If you have questions, please ask your MRP supervisor and/or the professor responsible for the MA in Public and International Affairs. Permitted uses: Identifying preliminary sources • Brainstorming your topic or preliminary research questions • • Generating synonyms of keywords for database searches • Translating a text3 • (Re)formatting citations and references • Checking grammar, spelling and clarity Use with caution: • Clarifying concepts • Overcoming writer’s block • Assisting with data visualization • Summarizing source documents Prohibited uses: • Using verbatim or slightly modified AI-generated content to write any or all sections of the MRP • Creating a full bibliography, including the inclusion of fabricated references • Generating false data • Analyzing data instead of student-led verification and interpretation 1 Professor Jim Davies (Carleton University) shared this insight during the development of this policy. 2 These examples are inspired by the flyer developed by Majela Guzman, https://infograph.venngage.com/pl/LkF6MMgU3FA 3 Translating data or parts or the entirety of your MRP may result in losing intellectual property on this material. Policy on use of generative artificial intelligence (AI) in Major Research Papers (MRP) You must include a statement indicating how you used AI in your MRP research and writing. Any student suspected of prohibited use of AI will be referred to the disciplinary approach under Academic Regulation A-44. 4 https://www.uottawa.ca/about-us/leadership-governance/policies-regulations/a-4-academic-integrity-academic-misconduct</t>
         </is>
       </c>
+      <c r="D19" t="n">
+        <v>476</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -782,6 +1016,19 @@
           <t>Quick Links Artificial intelligence is everywhere and with it comes new opportunities and challenges. As these new platforms evolve so must the way instructors, TAs and students use them. Given the rapid pace of change and growth in artificial intelligence - this issue will be ongoing for the foreseeable future. The Associate Vice-President, Academic's website has more information about artificial intelligence in teaching and learning at University of Waterloo. At present, it's important for instructors to be explicit about whether artificial intelligence or tools like ChatGPT are allowed to be used to complete assignments, tests or exams, and if so, the extent to which it is allowed, and if it should be cited and how to cite it. A student who does not comply with the instructor's rules about the use of such tools will be subject to Policy 71 and an investigation into academic misconduct. *Note: Effective September 2025, AI detection functionality in Turnitin will no longer be available. We recommend that instructors focus on evidence of learning rather than focusing on finding misuse of artificial intelligence. Instructors, students and staff should use GenAI transparently. The Library has resources for citing the use of GenAI. Dr. Kari Weaver (UW Library) has also developed an Artificial Intelligence Disclosure (AID) Framework. Microsoft Copilot should be used through your UWaterloo account in order to protect the privacy and security of the data that you enter. Be sure not to share any personal, institutional or research data in a GenAI tool that saves and uses your prompt data!</t>
         </is>
       </c>
+      <c r="D20" t="n">
+        <v>255</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -799,6 +1046,19 @@
           <t>Guidelines: The Use of Generative Artificial Intelligence (AI) in Teaching and Learning at McMaster University – August, 2024 by McMaster University is licensed under a Creative Commons Attribution-NonCommercial 4.0 International License Introduction and Context In June 2023 McMaster launched an initial set of Provisional Guidelines on the Use of Generative AI in Teaching and Learning. These Provisional Guidelines were updated further in August 2024 and then used throughout the academic year. After a further year of teaching and learning with generative AI, these Provisional Guidelines require some revision. These revisions were informed by feedback from faculty, students and staff and were written and endorsed by the Expert Panel on AI in Teaching and Learning and the AI Advisory Committee. They are intended to guide both educators and students in understanding and interacting with generative AI in teaching and learning contexts. Staff may wish to consult the Provisional Guidelines on the Use of Generative AI in Operational Excellence. In this update we move from “Provisional” to “Guidelines” recognizing that the Guidelines are not a policy but do intersect with existing McMaster policies and that the Guidelines will need further updating. Questions, comments or suggestions about these Guidelines may be directed to the Vice-Provost, Teaching and Learning or to the Special Advisor to the Provost on Generative AI at macgenai@mcmaster.ca Learning requires active engagement: building mental models and habits of mind, then communicating, applying, evaluating, and reflecting on those mental models and habits of mind. Learning requires work – often slow and challenging work. Generative artificial intelligence offers a promise of efficiency and speed, a promise that can be at odds with the deliberate effort of learning. At McMaster, we suggest that generative artificial intelligence tools should be used for learning only when the educator judges that their use will aid in active, critical, and reflective engagement. In most disciplines, university-level learning focuses on process, rather than the end-product. In other words, it is more important that students learn the how (e.g. how to find a solution, how to evaluate sources, how to construct an argument, how to perform a lab task, etc.), as opposed to the what (i.e. specific content). Generative AI poses a significant risk to the process of learning by bypassing or obscuring the how. While generative AI poses these risks to learning, at McMaster we remain open to generative AI use for teaching and learning, as well as experimentation with new tools and techniques when they advance a course or program’s goals. Educators experimenting with generative AI for its benefits for learning will want to be clear on pedagogical goals and how generative AI will advance those goals. Beyond learning, generative AI introduces a range of concerns, including environmental impacts, disinformation, impacts on labour, questions of copyright and ownership, lack of transparency in model design and function, privacy and data collection and use. Educators and students can learn more about these issues and should discuss them in courses where appropriate. Educators can get support in talking with their students about generative AI through the MacPherson Institute, the Privacy Office, or through these resources. Generative artificial intelligence systems are trained to produce outputs that are plausible in each context. The models learn to associate inputs to outputs by processing massive amounts of text and image data from the open web and other sources. Despite their ability to produce human-like outputs, there is no proven correspondence between the way that human beings think and learn and the way that generative AI models learn, process, and generate text, images, sounds, and other media. Because of the way they process training data and produce their outputs, generative AI systems are prone to producing ‘hallucinations’ (false statements, impossible images, false citations and attributions and other errors). Likewise, these systems produce outputs that are biased by their training data; these biases are often subtle and thus hold the risk of being uncritically reproduced. There is no current solution for the hallucination and bias problems. As generative AI models produce output that cannot be guaranteed to be accurate and unbiased, university-educated domain experts will continue to be required, both to produce original work and to verify the accuracy of the work that generative models produce. McMaster must continue to train students in the core competencies of any domain of study, regardless of the ability of generative AI models to answer undergraduate-level questions in that domain. Deciding as a learner and educator whether, when, and how to use generative artificial intelligence requires careful thought and evaluation of the benefits and risks to learning. It is ever more essential for educators to carefully consider what skills they need students to learn – that is, what process of learning – for the course and program. Educational developers at the MacPherson Institute can support this planning. Guidelines on the Use of Generative AI in Teaching and Learning - 1. Undergraduate and graduate course outlines should include a statement on the acceptable and unacceptable use of generative artificial intelligence in the course, with attention to the use of generative artificial intelligence for studying/learning and/or assessment. For instance, students may or may not use generative AI tools for idea generation, structuring, editing assistance, translation, summarizing/paraphrasing information, etc. (refer to the Use of Translation and Editing Tools guide for information about how to use these tools responsibly in the context of academic integrity). - If no syllabus statement is included, students should ask the educator for clarification on expectations, and if generative AI use is permitted, receive written confirmation before using generative AI in the course. - Educators should review expectations on the use of generative AI with their students in class [see: sample slide deck]. - 2. Educators incorporating generative AI into courses should consider how the course and its goals align with those of the program and with program learning outcomes. Educators should consult with the Departmental chair for the program learning outcomes and any program or departmental norms and expectations related to the use of generative AI at the program level. Programs may wish to establish norms and expectations of generative AI use at the program level. Support for this work is available by contacting macgenai@mcmaster.ca - 3. Use of generative artificial intelligence by students in ways not described in the course outline may be cause for a violation of the academic integrity policy. Likewise, the submission for course credit of uncited or unacknowledged work not created by the student(s) who submitted it violates academic integrity (See McMaster Policy on Academic Integrity). Reach out to the Office of Academic Integrity with any questions on process or for support. Reach out to the MacPherson Institute at mi@mcmaster.ca for support with redesigning assessments. - 4. Automatic AI detection systems are not reliable and are therefore not recommended for separating student- from AI-produced work. Educators who suspect work may have been inappropriately generated by artificial intelligence should follow the academic integrity process. This conversation guide may be useful for talking with students. - 5. If using generative artificial intelligence in courses or for teaching and learning activities, educators and students should use institutionally supported tools that have a completed Privacy and Algorithmic Impact Assessment. McMaster has an enterprise license with Microsoft Copilot. Educators and students who use generative AI should use their McMaster single-sign on credentials to login to Microsoft’s Copilot. - 6. In selecting third-party technology tools educators must avoid those that sell student data to companies building large language models, as well as companies that use student data to train AI models or to improve services and products; educators should review user agreements and consult with the Office of Legal Services or the Privacy Office if unsure. - 7. Legal questions of intellectual property (such as copyright and privacy) continue to be evaluated by provincial and federal courts. Until such questions are resolved, employees should not use generative AI created content for proprietary work and all McMaster policies continue to remain in effect. - 8. Students in co-op and experiential learning environments that use generative AI as directed by or approved by the co-op/experiential learning employer should initiate a discussion with the course instructor on how to document and reflect on this use with respect to the course learning. - 9. Students and educators who use generative AI should complete this module to help them review and reflect on broader societal implications of the use of generative AI, including labour, copyright, bias, and environmental impact. - 10. Students and educators who use generative AI in any context within a course should cite or acknowledge its use drawing on McMaster Libraries’ LibGuide and follow any course specific instructions. - 11. Generative AI tools should not be used to provide grades (letter or numeric) for student work. Generative AI tools may be used to provide feedback on student work, provided the following conditions are met: - When generative AI tools are used to provide feedback of student work this use must be explicitly included in the course syllabus. - Students should have the ability to opt-out of AI generated feedback. - AI generated feedback must be checked for accuracy and bias before being returned to the student. - Documentation of the AI tool used for feedback is required. - Instructors, or teaching assistants when directed, are responsible for feedback, however it is produced, to ensure appropriateness and accuracy. If you would like to discuss options for feedback and evaluation, please reach out to the MacPherson Institute at mi@mcmaster.ca - 12. If instructors use generative AI in their teaching materials, they should explain in the course outline the extent to which generative AI has been, or will be, used and should clearly cite or label such uses in their course materials. Instructors should fact-check any generative AI produced materials and evaluate these materials for bias. - 13. Course instructors have three options for directing teaching assistant use of generative AI. These directions should be given to teaching assistants in writing. - Permitting teaching assistants to use generative AI for any aspect of teaching assistant work, with the exception of evaluations that include a numeric or letter grade (see #11). TAs must inform the instructor of the intended use of generative AI, and receive approval, before implementation. - Requiring teaching assistants to use generative AI for specified teaching tasks as outlined in the hours of work form and with training provided.?In the instance of required use: As directed by the course instructor explicitly in the hours of work form, teaching assistants will use generative AI for the specific teaching tasks. Teaching assistant may create role-based accounts for such use. Course instructors will provide teaching assistants with the necessary training to use generative AI for the specified teaching purpose(s) with this training included in the hours of work. Teaching assistants will evaluate all teaching materials/formative feedback developed with generative AI for accuracy before use with students. Any planned use of generative AI by teaching assistants will be shared with students in the course outline.? - Prohibiting teaching assistants from using generative AI for teaching tasks. Over the fall and winter of 2024 the AI Expert Panel on Teaching and Learning will continue to work. Some of the activities of the Expert Panel include: - Additional course outline language to differentiate uses of generative AI and recommendations for consideration in policies related to course outlines - Engaging educators and students in discussion about the use of generative AI for evaluating student work - Developing resources to support departmental chairs - Additional resources for educators to talk with students about generative AI - Suggested language for acknowledgement of generative AI use (in addition to language for citation) If you have suggestions for additional resources or discussions the AI Expert Panel on Teaching and Learning could support, please reach out to macgenai@mcmaster.ca Sample Syllabus Statements These sample syllabus statements may be included on a course syllabus to communicate with students the expectations around generative AI in a course. Instructors may adapt or modify these statements according to their individual teaching goals and course learning outcomes. Students are not permitted to use generative AI in this course. In alignment with McMaster academic integrity policy, it “shall be an offence knowingly to … submit academic work for assessment that was purchased or acquired from another source”. This includes work created by generative AI tools. Also state in the policy is the following, “Contract Cheating is the act of “outsourcing of student work to third parties” (Lancaster &amp; Clarke, 2016, p. 639) with or without payment.” Using Generative AI tools is a form of contract cheating. Charges of academic dishonesty will be brought forward to the Office of Academic Integrity. Example One Students may use generative AI in this course in accordance with the guidelines outlined for each assessment, and so long as the use of generative AI is referenced and cited following citation instructions given in the syllabus. Use of generative AI outside assessment guidelines or without citation will constitute academic dishonesty. It is the student’s responsibility to be clear on the limitations for use for each assessment and to be clear on the expectations for citation and reference and to do so appropriately. Example Two Students may use generative AI for [editing/translating/outlining/brainstorming/revising/etc] their work throughout the course so long as the use of generative AI is referenced and cited following citation instructions given in the syllabus. Use of generative AI outside the stated use of [editing/translating/outling/brainstorming/revising/etc] without citation will constitute academic dishonesty. It is the student’s responsibility to be clear on the limitations for use and to be clear on the expectations for citation and reference and to do so appropriately. Example Three Students may freely use generative AI in this course so long as the use of generative AI is referenced and cited following citation instructions given in the syllabus. Use of generative AI outside assessment guidelines or without citation will constitute academic dishonesty. It is the student’s responsibility to be clear on the expectations for citation and reference and to do so appropriately. Students may use generative AI throughout this course in whatever way enhances their learning; no special documentation or citation is required. Honour Pledges Honour pledges are formal, student-led commitments to uphold the principles of academic honesty and integrity. These pledges represent students’ personal assurance to maintain and respect academic standards, abstaining from any form of plagiarism, cheating, or other academic misconduct. They often form part of the assessment submission process, where students attach a pre-defined pledge to their work as a statement of authenticity. Several studies have investigated the use of honour codes and academic integrity and found them effective in reducing academic dishonesty. Instructors might consider developing honour pledges together with their students, or adapting this McMaster honour pledge to their purposes. “I understand and believe the main purpose of McMaster and of a university to be the pursuit of knowledge and scholarship. This pursuit requires my academic integrity; I do not take credit that I have not earned. I believe that academic dishonesty, in whatever form, is ultimately destructive to the values of McMaster, and unfair to those students who pursue their studies honestly. I pledge that I completed this assessment following the guidelines of McMaster’s academic integrity policy.”</t>
         </is>
       </c>
+      <c r="D21" t="n">
+        <v>2537</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -816,6 +1076,19 @@
           <t>As generative AI (GenAI) tools and platforms continue to expand and evolve, it is important to provide the UBC community with guidance and advice related to their opportunities as well as risks and challenges. Download: Principles and Guidelines for Generative Artificial Intelligence (GenAI) in Teaching and Learning GenAI tools are artificial intelligence systems that can generate content – such as texts, images, audio, and video – in response to prompts by a user, after being trained on an earlier set of data (from Glossary of GenAI terms). Some GenAI tools are accessed through standalone platforms (e.g., ChatGPT), while others may be embedded in other applications or platforms (e.g., Grammarly). GenAI has the potential to enrich teaching and learning activities, and some may also support inclusion and enhance accessibility, depending on how they are used. Learning how to responsibly use GenAI is important for all members of the UBC community given its growing presence in many academic and work environments. However, such tools can and have been used in ways that are harmful to individuals and communities, and careful attention must be paid to topics such as academic integrity, accessibility, equity, Indigenous data sovereignty, and privacy and intellectual property. The following principles and guidelines have been developed through discussions with a Generative AI in Teaching and Learning Advisory Committee during the 2023-2024 academic year, and through multiple consultations with various individuals and groups at UBC. They provide guidance on responsible and ethical use of GenAI in teaching and learning at UBC, balancing both opportunities and risks. These guidelines are designed to adhere to and support UBC’s strategic plans and commitments, and to align with existing UBC policies, procedures, and legal requirements (linked where relevant below). They also support and build upon the UBC Principles for Use of Generative AI. This is meant to be a living document, evolving as needed in a rapidly-changing landscape around GenAI in teaching and learning. For feedback or questions, please contact provost.vptl@ubc.ca. Principles The following broad principles around GenAI in teaching and learning at UBC serve as a foundation for the more specific guidelines that follow. Download: Principles For GenAI in Teaching &amp; Learning Alignment to Our Values and Priorities UBC strategic plans and commitments Use of GenAI in teaching and learning should be aligned with and support UBC strategic plans and commitments, including those related to decolonization and Indigenous human rights, equity, accessibility, sustainability, and wellness. Opportunities to enhance education GenAI can provide significant value in both teaching and learning activities through informed, responsible, and ethical use that mitigates risks and potential harms. Value for students’ future endeavours It is important for students to learn how to use GenAI effectively and responsibly, to prepare them for further work or studies when they leave UBC. Indigenous data sovereignty Use of GenAI should respect Indigenous data sovereignty and community protocols for use and sharing of Indigenous knowledges, intellectual properties, and data. Harm from false information about Indigenous communities, cultures, knowledges, histories, and contexts should be avoided. Academic integrity All uses of GenAI at UBC must uphold academic integrity and adhere to the academic misconduct regulations in the UBC Okanagan and Vancouver calendars. Building Capacity and Literacy GenAI literacy UBC will continue to provide opportunities to learn about capabilities and limitations of GenAI tools. Faculty, staff, and students should use those opportunities to develop basic GenAI literacy skills over time. Faculty and staff use of GenAI Faculty and staff may use GenAI in teaching and learning so long as this is within the bounds of legal, university, Faculty, or program-level policies and requirements, and the guidelines below. Student use of GenAI Students may use GenAI in work submitted for courses or other academic requirements only if expressly permitted within their courses or programs. They may choose to use GenAI to support their learning in other ways, within the bounds of legal and university policies and requirements, and the guidelines below. Considerations Accessibility Some GenAI tools can enhance accessibility for learners with a range of disabilities. It is important to also recognize, however, that there may be varying levels of accessibility to GenAI tools, whether related to cost, inaccessible infrastructure (such as websites or applications), or for other reasons. Those using GenAI in teaching and learning should ensure equitable access to the best of their ability. Intellectual property &amp; copyright Those using GenAI in teaching and learning should respect intellectual property rights in material they input into the tools, and in how they use outputs. Privacy &amp; confidentiality Use of GenAI in teaching and learning should protect privacy and confidentiality of personal and other sensitive information. Personal Responsibility Equity Biased training data and inputs can produce biased, discriminatory, inaccurate, or otherwise harmful outputs, with the potential to perpetuate systemic inequities. Those using GenAI in academic work should assess the risks and mitigate, to the best of their ability, the harmful effects of such bias. Human oversight and critical thinking All outputs of GenAI for teaching and learning purposes should undergo human review before sharing. Users should think critically about outputs from GenAI, including their potential for producing false or misleading information, especially if sources of information in the outputs cannot be identified and/or verified. Transparency Use of GenAI to produce text, images, videos, or other materials shared with others for teaching or learning purposes should be acknowledged by attributing the source of those materials. Responsibility Users of GenAI are accountable for the consequences of sharing the outputs generated with these tools, and have a responsibility to review them for inaccuracy and potential harm to the best of their ability. The university will provide resources to help individuals develop requisite skills.</t>
         </is>
       </c>
+      <c r="D22" t="n">
+        <v>941</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -833,6 +1106,19 @@
           <t>Page not found | Office of Teaching and Learning Page not found The requested page "/teaching-assessment-resources/teaching-context-ai/provisional-recommendations-use-generative-ai%20https://www.uregina.ca/policy/browse-policy/policy-ops-080-050.html" could not be found.</t>
         </is>
       </c>
+      <c r="D23" t="n">
+        <v>20</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -845,6 +1131,24 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Provisional Guidelines on the Use of Generative Artificial Intelligence (GenAI) in Teaching and Learning for Instructors at the University of Prince Edward Island – December 2023 Provisional Guidelines: The Use of Generative Artificial Intelligence (GenAI) in Teaching and Learning at the University of Prince Edward Island was adapted from Provisional Guidelines: The Use of Generative Artificial Intelligence (AI) in Teaching and Learning at McMaster University – June 2023 by McMaster University which is licensed under a Creative Commons Attribution-NonCommercial 4.0 International License. Preamble The Teaching and Learning Centre at UPEI has been engaging in conversations around the use of generative artificial intelligence and identified a need for institutional guidance for instructors prior to the start of the fall semester at the University of Prince Edward Island. The original version of these guidelines was developed by the Task Force on Generative AI in Teaching and Learning at McMaster University. The guidelines developed for UPEI were shared with a small group of instructors and administrators in August 2023 to adapt them to the UPEI context. We gratefully acknowledge the feedback these individuals provided. Over the fall 2023 semester the Generative Artificial Intelligence Taskforce (GAIT) was created and tasked with reviewing these guidelines as well as the exploration of challenges, risks and opportunities associated with Gen AI in teaching and learning at UPEI. These guidelines will continue to be updated as UPEI explores additional topics and as technology rapidly changes. Members of the Generative Artificial Intelligence Taskforce (GAIT) invite feedback and suggestions on these guidelines through this form. Feedback collected this semester on experiences, questions and concerns about using generative AI in teaching and learning will inform further updates as developments surrounding generative AI are dynamic. It is expected these guidelines will be updated again in time for spring course preparation. This current version was updated in December 2023. Potential policy changes implied by these guidelines will be addressed by the relevant governance bodies. Institutional policies take precedence over these recommendations. UPEI acknowledges the costs of generative AI arising from significant ethical issues related to academic integrity, labour, intellectual and artistic property rights in the data sets, and the environmental impacts of training large AI models (Lawton, 2023; Li, et al., 2023; Trust, n.d.). One goal of the Generative AI Task Force (GAIT) is to educate users regarding these costs and explore ways of mitigating their impact. 1 What is GenAI? Generative artificial intelligence uses models that learn the patterns and structure of their input training data and then generate new outputs (text, images, or other media) that have similar characteristics. Provisional Principles These overarching provisional principles have guided the development of these recommendations and will continue to be updated through conversations with our campus community. • Students want to learn, and instructors want to support their learning. • Participatory learning – learning which happens in relationships and community – continues to be a valuable and vital way for students to learn. • Assessments that require students to document the process of learning continue to be meaningful for student learning. • Generative AI poses risks, as well as opportunities. Individuals will have different reactions and different expectations for the technology. • Disciplinary differences and departmental cultures will vary around the use of generative AI. Provisional Guidelines 1. UPEI’s existing academic integrity regulations apply when using generative AI. Read Regulation 20 from the Undergraduate Academic Regulations on the UPEI website. For Graduate students it is Regulation 6 from the Graduate Academic Regulations. 2. Instructors have the freedom to choose whether or not to use generative AI tools for the teaching and learning processes, and to determine if generative AI will be used in course design, activities, and assessments. If an instructor chooses to implement generative AI, the decision should be based on course learning outcomes, instructors’ individual interests, and conventions and expectations of the discipline. As with any pedagogical tool or approach, instructors should weigh the benefits of incorporating generative AI into their courses against any risks inherent to the tool or approach. Instructors should also take into account the rapidly evolving nature of generative AI technology and reassess the opportunities and risks of any tool or approach on a regular basis. 3. Instructors with courses that incorporate generative AI should: • Build their own AI literacy. • Ensure the incorporation of generative AI will support core learning outcomes and offer meaningful learning. 2 • Describe or discuss with students the strengths, limitations, and ethical considerations of the technology, including factual inaccuracies and gaps, societal biases present in the training data, and the rationale for using generative AI in the course. • Recommendations for instructors to consider when incorporating generative AI into courses for student use. 4. 5. Individual instructors should clearly communicate to students if and to what extent generative AI is acceptable in the course as well as how it should be acknowledged or cited. It's recommended that instructors be very clear about their expectations regarding generative AI, and explicit when providing assignment instructions. To help reduce confusion, ensure these expectations are communicated in various ways, such as including them in course syllabi, on Moodle, instruction guidelines and repeated in class. Explain how different instructors can have different expectations for AI tools, and if use is permitted by one instructor, this does not mean AI tools will be permitted by others. Instructors should ensure that all students have a fair opportunity to gain access to the same set of features for any tools required in the course, which could mean choosing free tools or pursuing enterprise licensing. Any required subscriptions should be disclosed at the beginning of the course. Alternatives should be provided for Generative AI tools that are restricted to users 18+ (e.g., ChatGPT) and for situations where students have concerns about privacy or other terms and conditions. 6. Instructors who include assessments that incorporate generative AI should: • Consider including reflective components that invite students to comment on the use of/experience with generative AI in the assessment. • Explicitly review criteria and/or rubrics in ways that demonstrate how the use of generative AI is being assessed (see the TLC Instructional Resources Hub for examples). • Foster a learning environment that promotes academic integrity in all course learning activities. 7. Students may opt-out of assessments that require the use of generative AI in exceptional circumstances as approved by the course instructor. In these cases, students will not face academic penalty, but will be required to provide alternative and equivalent evidence of their learning as proposed to, and agreed to by, the course instructor. 8. Assessment alternatives that may be less susceptible to the use of generative AI include: oral exams, presentations followed by a Q and A, invigilated/in-class assessments, practical tests, assessments that incorporate class discussion/activities, and process-based work. 3 9. If instructors use generative AI in their course and teaching materials, they should explain in the course outline and/or materials the extent to which generative AI has been used. Instructors are responsible for the quality, ethics, and relevance of all of their course and teaching materials, including those produced by generative AI tools. Instructors using generative AI should take reasonable efforts (e.g., updating associated digital literacies) to mitigate adverse impacts to quality and ethical instruction. 10. Instructors incorporating generative AI should be aware of the privacy policies and user agreements of each generative AI tool and alert students to these policies. 11. Third-party tools designed to detect AI-generative text should not be used to check student work, as current evidence demonstrates that third-party AI-detection tools do not reliably work to detect text generated by artificial intelligence. 12. If you suspect student work may have violated the academic integrity policy, please review the steps to take and refer to the undergraduate and graduate calendars. You may want to use check out this educator resource on conducting a discovery interview with a student to understand the situation. 13. Consider risks before submitting student work to generative AI tools. Submitting a student’s work to AI tools is a breach of the student’s privacy and intellectual property rights and requires the consent of the student. More guidance on this is forthcoming. GAIT intends to continue dialogues with various units and Faculties across campuses, as well as between post-secondary institutions to refine and expand these guidelines as new information and technology emerges, and as we learn to work with these technologies. One example includes ongoing work to explore privacy impact assessments and security evaluations on recommended generative AI tools. GAIT recognizes that the Gen Ai landscape can change rapidly. These guidelines will be updated accordingly, and changes communicated with the campus community. The Teaching and Learning Centre (TLC) will continue to provide training and resources for instructors on how to use generative AI effectively. Instructors can email TLC@upei.ca for support or book an appointment with an Instructional Designer. Additional options for • Find responses to several FAQs around Gen AI the Instructional Resources Hub on the TLC website. • Refer to resources for faculty to talk with students about generative AI available through the Instructional Resources Hub on the TLC website. • See the TLC Newsletters delivered to your email inbox (also available on the TLC website). • Watch Campus Notices or check the TLC learning events calendar on the website for current • workshops. Request a 1-1 consultation and connect with members of the TLC team by emailing TLC@upei.ca. 4</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1566</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -857,6 +1161,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>403 Forbidden 403 Forbidden nginx</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Requests</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -869,6 +1191,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>The University supports the responsible use of generative AI (GenAI) when helpful to further its mission, the preservation, advancement, and dissemination of knowledge. These guidelines provide general advice for the UW community and can help you use GenAI responsibly by aligning with UW’s values and privacy principles. Additional GenAI resources based on use case: - Research: Review the Effective and Responsible Use of AI in Research page. - Teaching: Refer to guidance on integrating GenAI while maintaining academic standards. - Health care and medical research: Review UW Medicine’s GenAI guidelines. (Net ID required) Key Takeaways - Only UW-approved services and applications may be used with University data. The use of unapproved services, applications, and the unauthorized release of university data could result in violations of policy or law for which you or the University may be liable. UW-IT can review tools and use cases to help inform unit decisions about whether to approve a service or application. - All use of GenAI must comply with all relevant UW policies and standards. - Complimentary training, tool review, architectural guidance, and security assessments are available via the UW-IT AI website. - You are ultimately responsible and accountable for your use of GenAI and all outcomes derived from it. - UW’s Appropriate Use Policy and related security and privacy policies apply to the use of all technologies, including GenAI. - Students must adhere to policies and rules applicable to their course or project. Course instructors have the discretion to allow, prohibit, or put parameters around the use of GenAI. - You must review GenAI output before using or publishing it and are responsible for any harm caused by your use of GenAI. - GenAI may enhance, but does not replace, human judgment, particularly in decision-making affecting individuals or communities. - Avoid GenAI use that may reinforce inappropriate biases or create barriers for underrepresented groups. - Disclosing GenAI use is often advisable and may be mandatory; failure to do so may have serious consequences, particularly in published research or coursework. - Maintain detailed records of GenAI use, especially when personal data is involved. Document relevant processes in the TrustArc personal data inventory. - Ensure compliance with records protection and preservation laws, including Records Management Services AI Guidance. - Data intended for public consumption (classification Level 1: All Audiences) can be used with GenAI.. - Do not use data that is restricted (classification Level 2: Limited Audience through Level 4: Special Handling Requirements), unless appropriate security and privacy controls, including contractual protections when working with other parties are in place. - If you want to use GenAI for high-risk processes like hiring, admissions, or performance evaluations, contact uwprivacy@uw.edu for a privacy impact assessment. - UW-IT AI Resources - AI@UW - UW AI Community of Practice - UW AI Task Force, Town Halls, and AI Perspectives Speaker Series - UW Health Sciences Library AI Overview - Artificial Intelligence at the Allen School of Computer Science and Engineering - University of Washington Bothell &amp; Cascadia College AI Guide for Students - Internet2 NET+ AI Updates - EDUCAUSE Artificial Intelligence Library - Interim Guidelines for Purposeful and Responsible Use of Generative Artificial Intelligence (AI) in Washington State Government - Washington State Attorney General Artificial Intelligence Task Force and Report - City of Seattle Generative Artificial Intelligence Policy - City of Seattle Responsible Artificial Intelligence Program - City of Tacoma Generative Artificial Intelligence Guidelines Report suspected security and privacy incidents immediately: - Urgent issues: Call 206-221-5000. - Other incidents: Email uwprivacy@uw.edu. - General questions: Email help@uw.edu.</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>587</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -881,6 +1221,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Addressing the Limitations of Using Generative AI for Learning Within the academic technology ecosystem, generative AI is increasingly everywhere. The Office of Academic Technology (OAT) is the central authority for evaluating learning technologies on campus, including generative AI. OAT supports the responsible adoption of generative AI for academic use, including for teaching and learning. Responsible AI Use in Teaching and Learning UT Austin defines responsible use of AI in teaching and learning as using AI in ways that foster the achievement of learning outcomes. That means using generative AI in ways that advance what students should know, be able to do and the attitudes they should develop as a result of a learning experience. At the same time, responsible AI use on the Forty Acres means not using generative AI in ways that would negate or inhibit the realization of those outcomes. UT encourages faculty, students and staff to be both AI-Forward and AI-Responsible. On the forward side, UT Austin provides access to a variety of tools and resources that foster the adoption of AI to achieve learning outcomes. On the responsible side, it emphasizes the critical importance of AI literacy and awareness of “the Big 6” limitations of using AI for learning (see below). Engaging in AI Forward – AI Responsible Learning Part of responsible adoption involves creating opportunities for the Longhorn community to gain literacy on the benefits and limitations of generative AI use in education. This starts with having a clear definition of what generative AI is and what it is not. What is generative AI? Generative AI refers to models that generate or create new or original output (text, code, images, videos, music, etc.) using pre-existing data the model has been trained on. The purpose of generative AI is to create brand-new content. Synthetic content can lead to wonderful, creative output — and that same output is often rife with limitations. Being AI-forward requires being aware of and taking action to mitigate the limitations below. The Big 6: Six Key Limitations of Using AI for Learning 1.0 Privacy and Security UT Austin supports data that is publicly available or defined as Published University information. When learning with AI, protect yourself and others by only using trusted vendors who allow you to disable chat history or model training easily. All students, faculty and staff must always follow the University’s generative AI acceptable use policy, which notes that inputting confidential or controlled university data is not allowed unless there is a University contract in place that protects such data. 2.0 Hallucinations and Deception Hallucinations are common and occur when generative AI produces content that is untrue or factually inaccurate. For example, bots such as ChatGPT might report that you have only 37 rows of data in a data set when there are 72. AI can also be deceptive in a variety of ways, including agreeing with users’ input or opinions even when they are incorrect or problematic, wrapping feedback in convincing, authoritative language that makes it appear credible. Such interactions can implicitly discourage critical analysis and discernment, leading learners to have more confidence in their knowledge or skills than they should. Always use more traditional approaches to research to confirm and verify facts. 3.0 Misalignment Misalignment occurs when a user prompts generative AI applications to produce a specific output, and the AI ends up producing an unexpected or undesired result. For example, when asking a bot to give you the Excel formula for merging two missing cells, it may give you the formula for splitting two cells instead. Misalignment is particularly problematic with image generation but also occurs within synthetic or AI-generated text. Careful prompt engineering helps address misalignment in text-based AI, but you will not be able to avoid it completely. Humans should always evaluate the output of generative AI with critical thinking skills. 4.0 Bias Because humans train them, generative AI output has both explicit and implicit biases baked into it, including stereotypes. It won’t be possible to entirely avoid bias in generative AI, just as it is not possible to avoid it in the real world, but a few small tips can help you engage with greater awareness. Educate yourself on the nature of implicit bias. Be aware that because humans train the models, they will reproduce our biases. Be skeptical and avoid over reliance on the models for any project. When you observe output from AI that is clearly biased or laced with stereotypes, report it to the vendor of the app you are using. 5.0 Ethics Al models have several ethical considerations, including digesting intellectual property, spreading misinformation, and using gen Al to produce new works or results without contribution. Other ethical considerations relate to the labor used to generate the models, the environmental impacts of generative Al, and the business ethics of releasing Al models for revenue generation without a clear understanding of the impact on society. Similar to bias, it is essential to be aware of the ethical concerns of using Al so that you can engage in a transparent manner. 6.0 Cognitive Offloading Cognitive offloading is the process of humans using external tools to reduce the demand or “cognitive load” of completing tasks (Risko and Gilbert, 2016). Technologies such as generative AI chatbots can help increase productivity through cognitive offloading; however, if you do not employ those freed-up resources for other tasks, the overuse of generative AI could potentially “diminish specific cognitive skills” (León-Dominguez, 2024). Engaging in human activities such as actively critiquing and evaluating output from generative AI can help protect problem-solving and creative and critical thinking skills. Other things you can do to avoid the downsides of cognitive offloading include engaging in transformation of gen Al output to make it your own. For example, evaluate the output for hallucinations, misalignment, bias, or ethics and then transform that output to make it authentically yours with your original thoughts, opinions, knowledge; or work. Have you adopted AI Forward - AI Responsible practices? The Office of Academic Technology is interested in learning from you. Please share your examples with the OAT using the form linked below. If you have questions or comments about generative AI for learning, please email us at oat@utexas.edu. Share Your ExamplesFebruary 21, 2024</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1036</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -893,6 +1251,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Page not found - Artificial Intelligence (AI) at Purdue University Purdue Virtual Assistant Hi! I'm the Purdue Virtual Assistant. I can help answer your questions about IT Services. How can I help you? Skip to content 404 ERROR We’re sorry you were not able to find the page you were looking for. Search Search Major Tuition &amp; Costs Schedule a Visit Boilermakers’ Stories Apply</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>64</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -905,6 +1281,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CU Boulder Guidelines Implementation of AI is subject to all applicable CU Boulder policies, standards and guidelines. If you have any questions about how to assess the implications of AI for your use case, please email security@colorado.edu. As the uses and ramifications of AI as a technology tool continue to evolve and be better understood, so too are the effects it will have on data security in higher education. This page is intended to guide our community as you consider using AI on the CU Boulder campus. Below are some guidelines for limiting data security risk while using generative AI tools: - Use AI tools available and recommended for use on the CU Boulder campus found on the Office of Vice Chancellor for IT and Chief Information Officer website. If you have any questions about access to these tools, please email oithelp@colorado.edu. - AI tool use is only approved for data classified as Public (see CU's Data Classification Standard for more information). The standard CU Boulder IT security contractual provisions may not be in place by default. If you intend to share Confidential or Highly Confidential information with an AI-based service (or any service for that matter), the service needs to be reviewed for compliance with CU’s data security requirements via ICT Review. Information shared with Generative AI tools using default settings is not private and could expose proprietary or sensitive information to unauthorized parties. - Review AI tool output to verify integrity: the output should be accurate and not incomplete, incorrect, or biased. - AI-generated computer code should NOT be used for institutional IT systems and services unless it has been reviewed by a human for accuracy, security (ensuring no vulnerabilities are introduced), and efficiency. - Faculty, staff, and students using these tools must read and understand the AI tool vendor’s policies and become familiar with the limitations of use and how the vendor plans to store, process, or handle CU’s data. For example, if using ChatGPT, you will need to read and comply with OpenAI’s Policies because there are some limitations regarding how the product may be used. Additional Resources With any new technology, there are always risks when utilizing it. If you decide to utilize or explore AI tools, you will need to consider the potential positive and/or negative impacts it will have on the campus, your department, and your personal life. A great framework to help you determine whether an AI tool is reliable and/or truthful is the NIST AI Risk Management framework. Below is a high-level overview of the framework. | Valid &amp; Reliable | Trustworthy AI produces accurate results within expected timeframes. | |---|---| | Safe | Trustworthy AI produces results that conform to safety expectations for the environment in which the AI is used (e.g., healthcare, transportation, etc.). | | Fair &amp; Bias is Managed | Bias can manifest in many ways; standards and expectations for bias minimization should be defined prior to using AI. | | Secure &amp; Resilient | Security is judged according to the standard triad of confidentiality, integrity, and availability. Resilience is the degree to which the AI can withstand and recover from attack. | | Transparent &amp; Accountable | Transparency refers to the ability to understand information about the AI system itself, as well as understanding when one is working with AI-generated (rather than human-generated) information. Accountability is the shared responsibility of the creators/vendors of the AI as well as those who have chosen to implement AI for a particular purpose. | | Explainable &amp; Interpretable | These terms relate to the ability to explain how an output was generated, and how to understand the meaning of the output. | | Privacy Enhanced | This refers to privacy from both a legal and ethical standpoint. This may overlap with some of the previously listed attributes. | *Please Note: Appendix B of the NIST framework discusses risks unique to AI. It recommends you review these risks to understand how AI risk differentiates from other more familiar technological risks. To assist you in your consideration and implementation of these guidelines, reading material on the topic of AI concerns can be found on the following webpages:</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>695</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -917,6 +1311,24 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Working group aims to ensure trust in research Guidelines for the use of AI in science Science thrives on reproducibility, transparency, and accountability, and trust in research stems in particular from the fact that results are valid regardless of the institution where they were produced. Furthermore, the underlying data of a study must be published, and researchers must take responsibility for their publications. But what if AI is involved in the research? Experts have long used AI tools to design new molecules, evaluate complex data, and even generate research questions or prove a mathematical conjecture. AI is changing the face of research, and experts are debating whether the results can still be trusted. Recommendations published in the scientific journal PNAS Five principles should continue to ensure human responsibility in research, according to an interdisciplinary working group with members from politics, business, and academia published in the latest issue of the journal Proceedings of the National Academies of Sciences (PNAS). Urs Gasser, Professor for Public Policy, Governance and Innovative Technology at TUM, was one of the experts. The recommendations in brief: - Researchers should disclose the tools and algorithms they used and clearly identify the contributions of machines and humans. - Researchers remain responsible for the accuracy of the data and the conclusions they draw from it, even if they have used AI analysis tools. - AI-generated data must be labeled so that it cannot be confused with real-world data and observations. - Experts must ensure that their findings are scientifically sound and do no harm. For example, the risk of the AI being "biased" by the training data used must be kept to a minimum. - Finally, researchers, together with policymakers, civil society and business, should monitor the impact of AI and adapt methods and rules as necessary. "Signal effect for researchers" "Previous AI principles were primarily concerned with the development of AI. The principles that have now been developed focus on scientific applications and come at the right time. They have a signal effect for researchers across disciplines and sectors," explains Urs Gasser. The working group suggests that a new strategy council - based at the US National Academy of Sciences, Engineering and Medicine - should advise the scientific community. "I hope that science academies in other countries - especially here in Europe - will take this up to further intensify the discussion on the responsible use of AI in research," says Urs Gasser. - Blau, W. et al. PNAS 2024 Vol. 121 (22) e2407886121 Technical University of Munich Corporate Communications Center - Dr. Jeanne Rubner - jeanne.rubner @tum.de - +49 89 289 25283 - presse @tum.de - Teamwebsite Contacts to this article: Prof. Dr. Urs Gasser Technical Univeristy of Munich Chair of Public Policy, Governance and Innovative Technology School of Social Sciences and Technology (SOT) urs.gasser(at)tum.de</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>468</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -929,6 +1341,24 @@
           <t>Unknown</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Prof. Dr. Volker Markl Chair of Database Systems and Informa:on Management (DIMA) Technische Universität Berlin June 7, 2023 Policy Statement. 1. Effective immediately, as a general policy, we do not permit the use of ChatGPT or other large language models (LLMs) in DIMA for the preparation of research papers, technical reports, theses, PhD dissertations, or any other original work. 2. The use of LLMs shall be strictly prohibited, as it on the one hand might prevent a fair grading of student performance, and on the other hand present the very serious risk of plagiarism. Similar to copying code from Stack Overflow, there is a spectrum with respect to when plagiarism occurs. However, in the scientific world one should be particularly aware and be careful with respect to this. 3. Every DIMA member should be aware of this policy and also point this out to your students and mentees. For course/project reports and theses, we will require students to sign a form that they confirm that they did not use any LLM tools, such as ChatGPT for the writing of their theses. Of course, this also applies to research papers and PhD dissertations. 4. Please be mindful of this matter and bring any violations of this policy to my attention, so that DIMA will be an environment free of the risk of plagiarism. Use of AI Tools for Course Assignments, Theses, Research Papers, and PhD Dissertations</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>235</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -941,6 +1371,24 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Policy on the Use of Generative AI in Research Status December 2024 In addition to the presentation on this website, you can also download the AI policy as a PDF. With this policy, the University of Freiburg would like to raise awareness for the conscious use of generative AI in the research context and provide recommendations on how to use the corresponding tools. The Central Data Facility supports all researchers of the University of Freiburg with the implementation of university policies. Contents - Preface - Introduction/Background - Recommendations for Researchers at the University of Freiburg - Further Information - List of Contributors - Contact Persons - References Preface The application of generative artificial intelligence (genAI) in research offers many opportunities, but these must be weighed against risks. The University of Freiburg developed this policy in accordance with its mission statement and the structural and development plan “Shaping Digital Transformation” (2023, 1.), based on the “Living guidelines on the responsible use of generative AI in research” of the EU Commission” (2024, 2.) and the Guidelines of the German Research Foundation (2023, 3.) for dealing with generative models for text and image generation. This document is based on the issues discussed during the event “ChatGPT – AI Tools in Research” (2023, 4.). A responsible and informed approach to genAI aims to prevent misuse and to ensure a sensible use of AI in all research processes. With this policy, we aim to raise awareness for a conscious use of genAI in research contexts and provide recommendations for the use of corresponding tools. Guidelines for the use of AI-based tools in study and teaching, as well as in administration, are currently in development. This policy must be understood as a snapshot since the development of AI is currently difficult to assess and changes will likely become necessary. Therefore, this document will be updated regularly. Introduction/Background What is “generative artificial intelligence”? The term “generative AI” describes AI systems that can autonomously create novel content in response to prompts. These systems learn from data received during their training phase and use this information to generate outputs. The basis for this are so-called Large Language Models (LLMs), which are created using very large datasets and highly complex calculations. Opportunities and Risks of AI The use of genAI in text and data processing provides the ability to quickly and conveniently create texts, images, videos, and code. Chatbots based on generative language models, such as ChatGPT or You.com, excel at generating texts with a wide range of applications from literature reviews to generating programming code or debugging it. AI-based annotation of audio/video recordings or simultaneous translations are already widely used. Extracting data from (multiple) publications and summarizing them is very easy and quick with LLMs. As a translation tool, LLMs potentially provide equal opportunities for researchers who are less proficient in the language used. However, risks exist as genAI is not neutral and may contain (derogatory) discrimination based on training data (so-called “biases”) or provide plausible but incorrect answers that do not correspond to facts (so-called “hallucinations”). This can promote the creation and dissemination of misinformation. Moreover, scientific misconduct, such as failing to disclose the use of genAI, poses a risk of misuse, as does the potential infringement of intellectual property. The linguistic quality of the generated results is often so good that the outcomes are hardly distinguishable from those created by humans. Additional risks for research may arise from the lack of transparency of tools, fees for accessing services, the use of unknown input data, or the concentration on a few providers. Recommendations for Researchers at the University of Freiburg Transparency Researchers should disclose which AI systems they have used and clearly label their contributions. Responsibility and Accountability Researchers remain responsible for the accuracy of the generated data, texts, and results, even if they are AI-generated or AI-based. Labelling and Documentation It must be indicated whether data and the results derived from them are AI-generated. The origin and use of the utilized methods, AI systems, and data sources must be fully documented, ideally in a way that the results can be reproduced. Yet, for solutions that are only accessible via API (Application Programming Interface) (such as ChatGPT), reproducibility is not always guaranteed, as the service changes over time, and the stochastic nature of LLMs can lead to differing outputs. Avoiding Bias Researchers must ensure that their results are scientifically grounded and must consider and, if necessary, avoid potential harm scenarios. The use of genAI also carries the risk of biases that can lead to discriminatory decisions. In relation to the training data used, systematic bias that stems from societal conditions, where certain prejudices are inherent in the data, must be avoided. Bias during the data collection or data annotation process, or in the choice of algorithm or system design, should be minimized. Authorship in Publications Related to AI The Committee on Publication Ethics (2023, 5.) states clearly that AI systems cannot be authors in scientific publications, among other reasons because they are not legal persons. The use of AI tools must be transparently listed in the methods section of publications. Only natural persons can appear as authors in scientific publications. They must ensure that the use of generative models does not infringe on anyone else’s intellectual property and that no scientific misconduct, such as plagiarism, occurs. Reference is made here to the regulations of the Albert Ludwig University for ensuring academic integrity (2022, 6.). The potential for generating texts, e.g., as templates for modifications by authors, can be used as long as this is documented and the authors take responsibility for the content, results (such as codes), and references. In publications, the rights of publishers or copyright holders must be respected, e.g., when data is provided to commercial vendors. It is critically important to assess whether the sharing of data can be free of charge if it involves a commercial provider. DFG Application Process, Review The use of generative models in applications to funding by the DFG is evaluated by the DFG itself as neither positive nor negative. However, when preparing reviews, the DFG (2023, 3.) prohibits the use of generative models with regard to the confidentiality of the review process. Documents submitted for review are confidential and must not be used as input for generative models. See also the section “Authorship in Publications Related to AI” in this policy. Promoting and Supporting the Responsible Use of genAI The responsible use and further development of generative AI should consider the limits of the technology, its environmental impact, and its societal effects. Based on liberal democratic values, discrimination must be avoided in the development and use of genAI, diversity and fairness must be ensured, and harm to persons, lives, and the environment must be averted. Last but not least, considerations about energy consumption by the use of AI systems, which require significant computational resources particularly for training, should be taken into account (see examples here). Orientation on Ethical Issues Researchers should consider ethical principles when using genAI. They must be aware of the risk of abuse even when using or developing AI tools. This includes abuse scenarios for unlawful military use or use for criminal activities (Dual Use Research of Concern). In doubtful cases, especially in instances with a high risk of abuse, researchers should consult the Committee for Responsibility in Research (Kommission für Verantwortung in der Forschung, KVF), which can discuss such issues in an interdisciplinary setting and advise researchers. See also here: Information on Good Research Practice at the University of Freiburg. Compliance with Legal Requirements Compliance with data protection regulations and the protection of intellectual property rights through responsible and appropriate handling of personal data must be guaranteed. In addition, regulations on export control law must be adhered to when publishing or conducting research across borders, and relevant medical device regulations must be observed if applicable. Further Information AI Tools at the University of Freiburg (intranet access required) The University of Freiburg provides its members with GDPR-compliant access to genAI, see here. The page also contains examples of energy consumption related to genAI. Research and Innovation in the EU Regarding AI The Commission and the countries of the European Research Area and stakeholders have jointly presented a number of guidelines to support the European research community in the responsible use of generative artificial intelligence (AI) (2.). EU AI Act The “EU Artificial Intelligence Act” (EU AI Act, 2024, 7.) addresses the rapid technological development of all AI systems and incorporates this into its legal framework. The EU AI Act aims to create reliable conditions for the research and application of AI. International Conference on Machine Learning Five principles are intended to further secure human responsibility in research, as now called for by an interdisciplinary working group with members from politics, industry, and science in the Proceedings of the National Academies of Sciences (PNAS) (2024, 8.). List of Contributors - Prof. Dr. Stefan Rensing, Vice Rector for Research and Innovation - Prof. Dr. Stefan Günther, Chief Information Officer - Prof. Dr. Frank Hutter, Professorship for Machine Learning - Prof. Dr. Silja Vöneky, Professorship for Public Law, International Law, Legal Ethics and Comparative Law, and Chair of the Committee for Responsibility in Research - Dr. Marc Herbstritt, Chief Information Security Officer - Klaus Scharpf, Data Protection Officer As a basis for the section “Recommendations for Researchers at the University of Freiburg,” individual text blocks were generated on July 9, 2024, by ChatGPT (GPT-4o) Comments from Senate members were integrated into this version following the resolution on December 18, 2024. Contact Persons References - Jahresbericht der Universität Freiburg 2023, S. 7 https://uni-freiburg.de/wp-content/uploads/Jahresbericht_der_Universitaet_Freiburg_2023.pdf (aufgerufen am 5.11.2024) - Living guidelines on the responsible use of generative AI in research (März 2024) https://research-and-innovation.ec.europa.eu/document/2b6cf7e5-36ac-41cb-aab5-0d32050143dc_en (aufgerufen am 5.11.2024) - Stellungnahme des Präsidiums der Deutschen Forschungsgemeinschaft (DFG) zum Einfluss generativer Modelle für die Text- und Bilderstellung auf die Wissenschaften und das Förderhandeln der DFG (September 2023) https://www.dfg.de/resource/blob/289674/ff57cf46c5ca109cb18533b21fba49bd/230921-stellungnahme-praesidium-ki-ai-data.pdf (aufgerufen am 5.11.2024). - ChatGPT – KI-Tools in der Forschung (Oktober 2023) https://videoportal.uni-freiburg.de/video/chatgpt-ki-tools-in-der-forschung-englisch-untertitelt/b08e66cd4ec53fba503a7f4028825d1b (aufgerufen am 5.11.2024) - Committee on Publication Ethics (COPE) (2023) https://publicationethics.org/guidance/cope-position/authorship-and-ai-tools (aufgerufen am 5.11.2024) - Ordnung der Albert-Ludwigs-Universität zur Sicherung der Redlichkeit in der Wissenschaft, Amtliche Bekanntmachungen Jahrgang 53, Nr. 31, S. 148ff (1. Juni 2022) https://uni-freiburg.de/wp-content/uploads/Uni-Freiburg-Ordnung-Redlichkeit-in-der-Wissenschaft-1.pdf (aufgerufen am 5.11.2024) - KI-Gesetz der Europäischen Kommission (2024) https://www.europarl.europa.eu/topics/de/article/20230601STO93804/ki-gesetz-erste-regulierung-der-kunstlichen-intelligenz (aufgerufen am 5.11.2024) - Blau, Wolfgang. et al. (2024), Protecting scientific integrity in an age of generative AI, Vol. 121 (22) e2407886121, PNAS.</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1735</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -953,6 +1401,24 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Status: 29 January 2025 The use of AI in your studies offers many opportunities. Generative AI, a sub-area of machine learning, can create content such as texts and images. This can have far-reaching changes for academic work. If used correctly, generative AI can enrich your studies. However, its use should always be understood as a support and complement and not as a substitute for independent learning, reflection and argumentation. This handout is intended to help you understand generative AI better and use it in a more reflective way. Due to the rapid pace of development, the website will be updated regularly. Only the German version of this page is legally valid. Guidelines for students 1. Be informed about the rules The teacher should decide and communicate in the first two weeks of lectures whether and to what extent AI applications may be used in the course of an examination. If no specifications are made, you can currently assume that its use is permitted as long as it has not been expressly prohibited. However, if in doubt, please ask! 2. Use generative AI responsibly 3. What AI can help with Finding ideas, researching topics and literature: AI can provide inspiration and spark creativity. AI can help to research topics, explore fields of research and find literature. Structure and time management: AI can help to structure your own learning process, organise a piece of work or plan a project. Repetition and understanding: AI can help to summarise content or explain difficult concepts. You can use generative AI to ask questions of a text. However, please note: AI also makes mistakes. Support with writing: AI can help you get into writing, find ideas for structuring texts and improve your ability to express yourself. AI can help to check for grammar and spelling mistakes and make stylistic refinements. However, make sure that the linguistic correction does not change the meaning and check the adjustments made by AI! Consistency check: AI can help you to critically check your own text, e.g. for consistent use of terms and argumentative consistency. However, independent discussion and reflection remain essential. Arguments must be developed independently and information critically scrutinised. You alone are responsible for the content and style of your text. 4. Improve your ability to use AI sensibly Prompt learning: Experiment with different questions and instructions to achieve the best possible results. Expand your skills: Use workshops, online courses or tutorials to further your training in the application of generative AI. Here you will find further information and counselling services. 5. Take a critical approach to AI Quality control: Always check the information provided by AI for accuracy. Language models often provide inaccurate or even invented sources. Check whether the sources mentioned even exist and are useful for your argumentation. Work independently with the sources. Learn to assess the value of AI-generated answers: AI-generated answers are often very well formulated and appear linguistically convincing. But they are not always factually correct or scientifically sound. The programmes are designed to give an incomplete or incorrect answer rather than no answer at all. Always check what you are being offered by AI! Practise independent thinking: Use AI results as inspiration and support, but think for yourself. Formulate your own arguments. Empower your own thoughts. 6. Observe ethical and academic integrity Comply with data protection: Do not upload any sensitive or confidential information to AI tools. Risk of unintentional plagiarism: The direct and unchecked use of AI-generated texts can lead to unintentional plagiarism. Check the generated texts carefully and do not adopt excessive amounts of text. Document and reflect on how you have worked with AI and which text passages are characterised by it. Follow the teacher´ s instructions. Cultivate a scientific ethos: The fact that unauthorised AI use may not be detected or that plagiarism or other attempts at deception may not be proven does not absolve you from working in a scientifically honest manner. Scientific research is a matter of honesty and integrity. Basically, you are responsible for the scientific quality of your text. You confirm this with your declaration of academic integrity (sample declaration of academic integrity in docx format). 7. Contribute to overcoming inequalities in studying Promoting equal opportunities in studies: AI can help you to personalise learning processes and balance out inequalities in your studies. However, students with more experience in using digital tools or with better research skills could benefit more from AI. Therefore, take advantage of courses and exchanges with fellow students to learn from their experience. Through exchange and practice, you can help to ensure that everyone benefits from AI and that existing differences in prior knowledge or digital skills are not reinforced. Regulations at the University of Erfurt on the use of generative AI for examinations On 4 December 2024, the Senate of the University of Erfurt adopted the recommendations for teachers on dealing with generative AI in teaching and examinations. In essence, it recommends active engagement with and a critical approach to generative AI in teaching and examinations. There is no and cannot be a regulation that applies to the entire university as to whether AI tools can be used for examinations. The specific design of examinations is generally at the discretion of the lecturers/examiners. They should generally communicate examination formats and examination conditions in the first two weeks of lectures. The teacher decides - whether and which AI applications are permitted in the course of an examination, - what restrictions exist - and how permitted use is to be documented and reflected upon. The University of Erfurt provides a template for a declaration of academic integrity and for a declaration of consent (template)regarding the authorised resources. Both declarations can and should be adapted by the lecturer to the respective examination. In the specific requirements for the examination, teachers who authorise the use of AI can request a critical analysis (in the form of a reflection of approx. 1 page). The examination paper should then contain a section in which you as a student state which tools you have used and reflect on how the use of AI has changed the content, structure and linguistic aspects of your examination paper. Can I use AI tools in written work (seminar papers, bachelor's, master's and master's theses)? Whether and which aids, including AI tools, you are allowed to use, how you should document and, if necessary, reflect on this and which assessment standards apply to the examination should be determined by the teacher in the first two weeks of the lecture. The declaration of consent (template) can be used for this purpose. With your declaration of academic integrity you as a student expressly declare that you have written your text independently and in accordance with academic standards, have only used authorised resources and have labelled them in accordance with the specifications. You are responsible for the content and quality of your text. Important: Observe the examination regulations! Students who demonstrably do not adhere to the specifications and use AI tools without authorisation or do not/insufficiently label them may be accused of cheating or using unauthorised aids and will receive a failing grade (5.0). A second attempt to cheat in the degree programme can lead to the loss of the right to take the examination. Can I use AI tools for written/electronic (remote) exams? Whether and which aids, including AI tools, you are allowed to use during an exam is determined by the teacher. Teachers can prohibit all aids, including the use of generative AI, during written and electronic (remote) examinations. If the use of AI tools is expressly permitted, clear guidelines must be set and compliance must be ensured by means of control mechanisms. Important: Observe the examination regulations. Students who demonstrably do not adhere to the specifications and use AI tools without authorisation and/or do not or insufficiently label them may be accused of cheating or using unauthorised aids and will receive a failing grade (5.0). A second attempt to cheat in the degree programme can lead to the loss of the right to take the examination Is my lecturer allowed to conduct oral examinations as a supplement to the written work? Since summer 2024, the framework examination regulations of the University of Erfurt allow a supplementary oral examination to the defence of the written thesis. This checks the extent to which students have actually understood the topic and explored it independently. This examination relates to the same examination content as the written paper. "In all modules [...] the module examination "h) Written paper 70% in conjunction with oral/practical examination 30%" is also part of the defence of the written paper. It is also permitted as an additional module examination for the defence of the written paper. If one of the two partial examinations is assessed with 5.0, the combined examination is deemed to have been assessed as insufficient."[1] Whether this examination format is used will be determined by the examiners in the first two weeks of lectures. A subsequent addition of an oral defence to a purely written examination is not permitted. [1] § Section 9 (6) and (9) B-RPO-2019, Section 10 (6) and (9) M-RPO-2019, Section 10 (6) and (9) MEd-RPO-2019, Section 6 (6) and (9) Theol-PO-KaTh-2021, Section 7 (8) Theol-PO-KaTh-2009</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1541</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -965,6 +1431,24 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>This guide provides orientation for all students, staff, and external parties at the University of Jena regarding the responsible use of generative artificial intelligence (AI) as a tool in professional life as well as in studies, teaching, and research. In order to use AI tools safely as an aid to support one's own work, users should also be aware of the risks. You can also find the handout as a PDF document in the HanFRIEDThis link requires a loginde administration manual. - What do we mean by generative artificial intelligence? By “generative AI” we mean computer models capable of autonomously generating new content—such as images, texts, or music—based on human or machine input, after learning patterns and structures from a training dataset. - Under what requirements is it possible to work at the university? AI-based tools have immense potential to increase the efficiency and effectiveness of our work. Where generative AI can be used profitably and without risk, its use should be permitted. To guide and raise awareness for responsible, reflective, and legally compliant use, key points are compiled in the chapter "What must be considered when using generative AI tools?". We must always bear in mind that although a text-generating AI may produce well-formulated texts based on statistical probabilities, it does not actually recognise their meaning or evaluate their coherence or factual accuracy. Examples of the use of AI tools Creative work - Generating new ideas - Supporting the development of one's own ideas Research - Discovering new sources or issues on specific topics - Summarising sources to gain an initial overview Writing process (e.g. letters, emails, minutes, publications, proposals) - Assistance with phrasing and sentence structure - Feedback on grammar, style, and structure to improve one’s own texts - Overcoming writer’s block (AI as a sparring partner) Text analysis of materials, literature synthesis or data preparation - Summarising or merging your own documents or texts - Analysing texts or examining them for specific characteristics - Supporting data preparation processes, e.g. for transcriptions Translations - Translating sentences or sections for practice or understanding - Translating emails or other correspondence for communication purposes Teaching materials and exam tasks - Generating ideas, examples or templates for new examination tasks - Supporting the design of teaching materials - Supporting the customisation of materials Targeted use of an AI tool in teaching - Training in the use of AI, e.g. for writing prompts - Digital assistants for learning and exam preparation Image material - Generating images, e.g. for internal presentations, reports or talks Assessments and evaluations - Supporting the preparation of evaluations (e.g. criteria selection and phrasing) - Assistance with phrasing Administrative tasks - Assistance with phrasing, summaries, or correspondence Examples against the use of AI tools - Processing of personal data (unless the data protection requirements can be met) - Unverified adoption of a complete concept or its elaboration by AI - Unverified adoption of a summary or analysis in a report or publication - Complete and unverified use of translations (e.g. in exams or reports) (note: use for language learning after consultation with the lecturer) - Use in examinations without being named as an aid and without the examiner's permission (note: the decision to use AI in examinations is made by the examiner) - Use of an AI tool as an aid in a course without prior consultation with the lecturer - Assessment of examinations (term paper or other examinations) or assessment of another person's performance - Evaluation of applicants or other personnel-related decisions - Preparation of an employment reference or employee appraisal - Analysis of employee data (e.g. absences, sick leave, holidays) - Evaluation of applications or assessments General information on the use of AI in specific areas In study and teaching, the guidelines for the preparation of academic work de apply. The writing of an academic piece of work or completion of exams must reflect the student’s own work. Use of AI in this context may only occur as a supporting tool and only with the examiner's agreement. Lecturers are required to design examinations in such a way that they adequately reflect the intended learning objective and are meaningful. If AI use is to be excluded, this is best achieved through a suitable assessment format. Guidance is available via the University’s pages on digital assessments and the support services of Servicestelle LehreLernen. In academic work, the “Principles of Good Scientific Practice” must also be upheld when using generative AI. In particular, reference is made to the DFG statement on the Influence of Generative Models of Text and Image Creation on Science and the HumanitiesExternal link and the statutes for safeguarding good research practice at the University of Jena. Researchers must remain aware of their responsibility for the integrity of any content created with or by AI. The ERA Forum’s guideExternal link is also recommended. Access and accounts Use of AI tools often requires registration with an email address. In professional contexts, institutional email addresses and contact details should be used. For team or API access, the University Computing Centre (URZ) can provide accounts for functional purposesExternal link. If you use your work e-mail address, it is possible that the external provider will create a user profile based on the name contained therein and link it to the person. The „IT-Zentrum der Thüringer Hochschulen“ enables anonymous use of ChatGPT via a web portal. No personal data of the employees is transmitted to OpenAI, only the chat is sent to ChatGPT. Staff can access it via https://ai-chatbot.hs-itz.deExternal link after selecting University Jena as institution and logging in with their URZ account. On 10 June 2025, the HAWKI HS-ITZ service was updated to the HAWKI2 version. The new version can be tested under: https://ai-chatbot.tu-ilmenau.de/hawki2/External link. We would also like to draw attention to the Chat AI tool (https://chat-ai.academiccloud.de/External link) from AcademicCloud, which is provided by the Gesellschaft für wissenschaftliche Datenverarbeitung mbH Göttingen (GWDG). University members can register with this service using their university email address and use various AI models for a chat. Another option for free access (including ChatGPT) is provided by KI-Campus: https://www.unidigital.news/kostenfreier-zugang-vom-ki-campus-zu-chatgpt-und-offenen-sprachmodellen-ueber-hawki-gwdg/External link. - Procurement To obtain commercial AI tools, please contact the URZ software service via the service portalExternal link. - Billing The following procedure is established for the use of OpenAI products (ChatGPT Plus and API): The costs are charged by collective booking to the PSP element specified in the service portal. The costs are averaged across all users in the respective billing period in order to distribute exchange rate fluctuations and foreign currency fees fairly. The URZ must receive the billing information from the OpenAI web portal in order to be able to carry out billing. The exact procedure differs depending on the type of product used. - ChatGPT Plus ChatGPT Plus users will be charged a subscription of $20.00 per month plus transaction costs (exchange rate fluctuations and foreign currency fees of approximately $4.00). All users are obliged to download the billing documents provided by OpenAI in the web portal for their account on a monthly basis and make them available to the URZ (via the service portal in the same process in which access was requested). - ChatGPT API When using the API, the costs are variable depending on the actual usage. An estimate of the expected monthly or annual costs is helpful for financial accounting. In each API access (organisation), several members can be authorised (‘team’). To give the URZ access to the billing information, softwarebeschaffung@uni-jena.de must be added as a user and authorised as an owner. What must be considered when using generative AI tools? - 1. Check tool settings before use. Data or information that is processed in the context of work-related activities should not be included in the training of an AI. This applies in particular to work protected by copyright, e.g. academic assignments by students, and personal data. Please check the settings in the AI tool before using it. There is usually an option to refuse use for training purposes. If this is not the case, we advise against using the tool in a university context. If possible, the input history and, if available, the memory function should also be deselected in the settings. - 2. Be cautious with personal, sensitive, or confidential information. When entering data into an AI tool, please ensure that no data relating to a person or sensitive university information is entered or uploaded. This also applies to copyright-protected works and documents declared as confidential as well as information that may allow conclusions to be drawn about individuals via indirect channels. It is advisable to anonymise personal data before entering it (e.g. use a synonym instead of a name). When entering your own personal details in AI tools, it should also be borne in mind that user profiles with personal information may be created and made available to third parties. - 3. Do not use AI for decision-making. Generative AI tools should not be used as the basis or even the final decision for personal decisions (see Art. 22 General Data Protection Regulation). For example, AI should not be used for the selection of applicants, the assessment of students' examination results or third-party funding applications by researchers. The processing of data in an AI on the purposes of which certain personal aspects are ‘evaluated’ is not permitted. Please always bear in mind that AI does not recognise the meaning, significance or implications of the outcome it creates. - 4. Careful and conscientious checking of the results. The result of generative AI should be treated with caution and evaluated carefully. The information generated by the system may be incorrect and correlations may not be represented correctly (phenomenon of confabulation). Users should also check the accuracy of references. Discrimination and inequality in the AI-generated work should also be checked so that certain groups are not disadvantaged and existing social injustices are not reinforced, as AI can create or reinforce distortions or bias. Users are ultimately responsible for critically scrutinising the generated content and ensuring that it is correct and ethically acceptable. It is also important to ensure that protected works or parts thereof are not reproduced. The rights of the author continue to exist, even if the AI has generated the result. - 5. Making the use of AI transparent. Be open about the use of generative AI. Its use should be clearly labelled and its use and underlying purposes openly communicated. It is also advisable to keep documentation on the use, for example when working on larger texts. In addition, the AI tool should also be named as the source for AI-generated images. For example, in the multimedia area of our content management system for image documents, the value ‘AI-generated’ can also be selected in the ‘Author’ field. Overall, we recommend that the use of generative AI in the university context be carefully considered and critically reflected upon, considering ethical, social and educational considerations to ensure that it supports the objectives of the university's activities. These recommendations are regularly updated and adapted to current developments and legal practice.</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1842</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -977,6 +1461,24 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>The Guideline on the use of generative AI tools in teaching and research can be found here on the website in full as a text to read or as a PDF to download. This text outlines the university's position regarding generative AI tools. The download section is organized thematically and sorted by subpages. Download Dear University Members and Staff, Talk is everywhere about ChatGPT and other generative AI (GenAI) tools. The University of Tübingen believes it is its duty to address this debate so as to help shape developments and produce guidelines. To this end, the President’s Office has set up the Generative AI work group, consisting of members from every faculty, central administration and relevant institutions. The role of the work group will be to advise the President’s Office on the use of GenAI at the University of Tübingen. Its members take a critical yet optimistic attitude to the potential of GenAI. Together, the President’s Office and the work group have discussed principles, which will continue to be developed. Their aim is to achieve the critical, reflexive, transparent and responsible use of GenAI. The current status of the discussion is given below. As a forward-looking and progressive university, the University of Tübingen recognizes the transformative potential of GenAI. This potential currently encompasses many areas of society and is changing both university and non-university work environments. GenAI is already becoming incorporated in various professions at rapid speed. There will no longer be a world without AI. In future, many University of Tübingen students will work in professions where the use of GenAI will be an everyday part of work processes. Likewise, GenAI will increasingly change the day-to-day work of researchers in various disciplines, as well as that of administrative staff. The University of Tübingen sees this as a major challenge, but also a substantial opportunity. After all, the University can be the place where critical, reflexive, transparent and responsible ways of working with GenAI are negotiated, developed, and transmitted. For instance, it contributes to shaping social change in the context of AI in a way that is both sensitive to problems and at the same time constructive. The potential for GenAI in the field of text and data processing is extremely diverse. For the University of Tübingen it extends over every relevant area: GenAI has the potential to change how students learn and operate in a data-saturated scientific world. It can enable new didactic approaches in digital teaching, open up new ways for researchers to work with texts or images, contribute to the expansion of science communication and last but not least provide support at an administrative level. The variety of possibilities makes it especially difficult to determine potential, or to develop rules on how to proceed. What is clear is that – whether in studies, teaching, research or science communication – the potential of GenAI varies, and sweeping assessments have little to offer. At present the University is in an exploratory phase, where it has to investigate, test and discuss critically the potential in all of these fields. Given the speed of technical development and the technological hype, we need to evaluate the potential of GenAI realistically, in order to define a framework in which it can be used by a forward-looking university. Besides its wide potential, GenAI also has many problematic implications. These include the fact that there are still many unresolved copyright and data protection issues. Generated texts can produce erroneous, ambiguous or misleading results and ‘hallucinate’ sources. GenAI can reproduce any bias recorded in the system’s training data. Social, cultural and scientific prejudices can be incorporated in the system and the generated texts. Developers can sometimes deliberately manipulate the generated texts. In addition, extensive use of GenAI has a substantial ecological footprint, in particular through electricity consumption, CO2 emissions, consumption of minerals and water. Furthermore, different payment models for stronger and weaker AI systems can further increase economic inequalities (e.g. between students with different incomes). Therefore, a key objective of the University of Tübingen is to test the potential of GenAI and apply it productively in various areas of the University, while bearing in mind these problematic implications. This includes developing both basic and subject-specific study programs as well as the legal framework, e.g. for application in examinations. The University will also benefit from a critical discourse on the potential and the limits of GenAI in relation to research, science communication and administration. Achieving these objectives will demand a lot of work and attention. However, it is already clear that key guiding principles will be indispensable. Firstly, members of the University must tackle GenAI in a critical and reflexive way. Many of the problems with GenAI (including at a social level) arise from a naive attitude. A critical and reflexive attitude demands not only the development of a sophisticated awareness of the problems, but also the ability to realistically assess the potential and limitations of GenAI. Secondly, use of GenAI should be organized transparently. If GenAI is used (whether for research, studies, administration or science communication), the procedure must be documented and made visible/transparent in the relevant format. Thirdly, all members of the University are exhorted to use GenAI responsibly in line with good scientific practice. Among other things this means that when working with GenAI it is the individual responsibility of the authors to ensure that their texts do not contain any plagiarism and all sources are critically examined. It also means that each user must assume responsibility for how and to what end the data provided by AI systems are processed. The way in which these principles are applied must by their nature be applied differently depending on the field of work and culture of the discipline. Departments and institutions are called on to formulate and provide their own guidelines. The Generative AI work group and the President’s Office are currently working on basic solutions in order to respond to urgent procedural questions concerning examinations. These will form the basis for future development in the faculties and institutions. If we can provide the fundamental conditions for critical, reflexive, transparent and responsible use, GenAI can offer potential to enhance work processes both within the University and beyond. What precisely these enhancements will consist of and how a critical process of evaluation can assess them with regard to their problematic implications will be the subject of ongoing discussion at the University of Tübingen in coming years.</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1070</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -987,6 +1489,24 @@
       <c r="B36" t="inlineStr">
         <is>
           <t>Germany</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Der Einsatz generativer KI (GKI) wie ChatGPT hat das Potenzial, akademische Arbeits- und Bildungsprozesse umfänglich und nachhaltig zu verändern. Sie kann personalisiertes Lernen ermöglichen, die Lehre unterstützen und Forschung fördern. Aus diesem Grund befürwortet die Goethe-Universität grundsätzlich die Erprobung und Anwendung von GKI in Studium und Lehre. Bei der Nutzung von GKI sind jedoch sowohl ethische, rechtliche und natürlich auch didaktische Aspekte zu berücksichtigen, weshalb mit einer speziell zu dem Thema eingerichteten, interdisziplinären Arbeitsgruppe unterschiedlicher Statusgruppen zielgruppenspezifische Handlungsempfehlungen erarbeitet wurden, die Ihnen, ausgehend von dieser allgemeinen Einführung zum Thema GKI, zur Verfügung stehen. Mit sorgfältiger Planung und Vorbereitung sowie einem klaren Handlungsrahmen kann generative KI ein wertvolles Werkzeug in der Hochschullehre sein. Allgemeine Empfehlungen und Hinweise Bitte beachten Sie die folgenden grundsätzlichen Hinweise im Umgang mit Tools der generativen Künstlichen Intelligenz (GKI) und den nachfolgenden Handreichungen: Kritische Reflektion: Reflektieren Sie die Ergebnisse der KI grundsätzlich kritisch, da es sich bei generativen KIs um statistische Modelle handelt, die häufig vorkommende Aussagen und Einstellungen aus vorab verarbeiteten Trainingsdaten reproduzieren. Sind z.B. Biases in den Trainingsdaten enthalten (z.B. einseitige oder verzerrte Darstellungen), so werden diese auch in den generierten Ergebnissen reproduziert. Je nach Fachgebiet und Fragestellung können die Ergebnisse sehr nützlich und korrekt oder aber falsch und irreführend sein. Geistiges Eigentum: Bitte beachten Sie, dass generative KIs Inhalte erstellen können, die auf bestehenden Daten basieren und entsprechend geistiges Eigentum eine wichtige Rolle spielt. So können z.B. in den Trainingsdaten der KI urheberrechtlich geschützte Inhalte vorhanden sein, wodurch generierte Inhalte problematisch sein könnten. Auch Daten, die man z.B. zur Überprüfung an eine KI gibt, können urheberrechtlich geschützt sein. Stellen Sie sicher, dass die Informationen, die Sie eingeben, und die Ergebnisse, die Sie erhalten, keine Urheberrechtsverletzungen darstellen. Zum jetzigen Stand können KI-Programme selbst keine Urheberschaft innehaben. Je nachdem wie stark die Einflussnahme derdie Nutzerin an dem generierten Text war, ist entweder ersie derdie Urheber*in oder das Ergebnis ist nach dem Urheberrecht gemeinfrei. Persönliche Daten: Geben Sie keine persönlichen oder sensiblen Informationen ein, wenn Sie KI-Tools nutzen. In den meisten Fällen liegt der Sitz der Betreiber der Tools aktuell noch in den Vereinigten Staaten und es lässt sich nicht kontrollieren, was mit den eingegebenen Daten passiert (Schrems II-Urteil des EuGHs). Selbst mit einer Einwilligung der betroffenen Personen lassen sich Rechte wie den Abruf aller erfassten Daten oder deren Löschung nicht oder nur sehr eingeschränkt wahrnehmen. Dies ist mit der Datenschutz-Grundverordnung (DS-GVO) nicht vereinbar. Aktualität: Vieles rund um KI-Technologien befindet sich im Moment noch in einer Aushandlungsphase. Daher können sich die Möglichkeiten, Risiken und rechtlichen Rahmenbedingungen jederzeit ändern. Wir bemühen uns, die Informationen auf dieser Seite auf dem neuesten Stand zu halten, können jedoch keine Garantie für die Aktualität geben. Korrekturen und Hinweise nehmen wir gerne entgegen. Was ist generative Künstliche Intelligenz (GKI)? Der Begriff “Generative KI” beschreibt KI-Systeme, die in der Lage sind, auf Anfrage neuartige Inhalte selbstständig zu erstellen. Diese Systeme lernen aus Daten, die sie während ihrer Trainingsphase erhalten haben, und nutzen dieses Wissen, um Ausgaben z.B. in Textform zu erzeugen. Neben der Textgenerierung gibt es auch andere Beispiele für generative KI wie Bildgenerierung, Musikkomposition und die Erzeugung von Programmcode zur Entwicklung von Anwendungen. Language Models (LM) oder Sprachmodelle sind eine Unterklasse der generativen KI. Diese Modelle lernen die Wahrscheinlichkeit von Sequenzen von Wörtern in einer bestimmten Sprache. Large Language Models (LLM) sind sehr große Sprachmodelle, die auf enormen Mengen von Textdaten trainiert wurden. Dadurch sind sie in der Lage, menschenähnliche Texte zu generieren, und können für eine Vielzahl von Aufgaben eingesetzt werden. Mit dem richtigen Training können sie Aufgaben wie maschinelles Übersetzen, Frage-Antwort-Systeme, Textzusammenfassung und mehr bewältigen. So beeindruckend die Ergebnisse sind, die mit LLMs erzielt werden können, sollten sie nicht mit Wissensdatenbanken verwechselt werden. Die Texte, die beim Trainieren der Modelle verarbeitet werden, sind im Endprodukt nicht mehr wörtlich enthalten. Man darf sich Programme wie ChatGPT deshalb nicht als Suchmaschinen vorstellen, die in Textkorpora nach relevanten Stellen suchen und Antworten durch Copy &amp; Paste zusammenstellen. Stattdessen handelt es sich um rein statistische Modelle, die Aussagen und Einstellungen reproduzieren, die häufig in ihren Trainingsdaten vorkommen. Weiterführende Informationen Friedrich Wolf – Über, mit und von KI lernen? – Ein pädagogischer Rundgang (Video, 1:26 h) Welche Anwendungen und Dienste gibt es? Da sich die verfügbaren Tools aktuell sehr schnell weiterentwickeln, versuchen wir hier einen Überblick über bestehende Tool-Kategorien zu geben, die im weiteren Verlauf der Handreichung immer wieder aufgegriffen werden. | Kategorie | Beschreibung der Kategorie | |---|---| | Literaturrecherche | Tools dieser Kategorie bieten eine Vielzahl von Funktionen zur Unterstützung der Literaturrecherche in der Hochschullehre. Sie ermöglichen es den Studierenden, wissenschaftliche Literatur effizient zu finden, zu organisieren und relevante Artikel oder Autor*innen zu identifizieren. Mithilfe dieser Tools können Studierende Literaturdatenbanken durchsuchen, Literaturlisten erstellen oder sich einen Überblick über aktuelle Forschungsergebnisse zu bestimmten Themen verschaffen. Durch die Integration in Literaturverwaltungsprogramme wie Citavi oder Zotero können gefundene Artikel auch direkt in die persönliche Bibliothek importiert werden. Ein Beispiel für ein Tool dieser Kategorie ist Researchrabbit*. Die Universitätsbibliothek bietet eine Übersicht verschiedener Tools für die Literaturrecherche. | | Textproduktion | Tools dieser Kategorie unterstützen Studierende aktiv bei der Schreibpraxis in der Hochschullehre. Mit Funktionen wie KI-Autovervollständigung, automatische Zitation, Formatierung nach verschiedenen Schreibstilen und Plagiatsprüfung assistieren sie beim Verfassen von wissenschaftlichen Arbeiten. Diese Tools können den Schreibprozess beschleunigen, indem sie beim Formulieren komplexer Sätze oder beim Finden passender Referenzen helfen. Sie ermöglichen Studierenden, ihre Schreibkompetenzen weiterzuentwickeln und wissenschaftliche Standards einzuhalten. Ein Beispiel für ein Tool dieser Kategorie ist JenniAI*. | | Textverständnis | Tools dieser Kategorie unterstützen das Textverständnis von Studierenden, indem sie ihnen ermöglichen, Texte interaktiv zu erkunden und besser zu verstehen. Durch das Markieren von Begriffen, Passagen oder wichtigen Informationen in einem Text und der anschließenden Nutzung eines integrierten Chatbots können Studierende Erklärungen, Definitionen oder zusätzliche Informationen erhalten. Diese Tools können auch Fragen beantworten oder weiterführende Quellen empfehlen, um das Verständnis eines bestimmten Textes zu vertiefen. Diese Tools sind besonders nützlich, wenn Studierende komplexe wissenschaftliche Texte lesen und analysieren müssen. Sie können dazu beitragen, dass Studierende bedeutungsvolle Verbindungen und Zusammenhänge in einem Text erkennen und das Verständnis vertiefen. Durch die Interaktion mit einem Chatbot erhalten Studierende individuelle Unterstützung und können ihr Textverständnis weiterentwickeln. Ein Beispiel für ein solches Tool ist Explainpaper*. | | Plagiatserkennung | Tools dieser Kategorie sind speziell darauf ausgerichtet, Plagiate in wissenschaftlichen Arbeiten aufzudecken. Sie ermöglichen Dozierenden und Studierenden, alle eingereichten Texte auf potenzielle Ähnlichkeiten mit anderen Quellen oder bereits veröffentlichten Arbeiten zu überprüfen. Diese Tools durchsuchen umfangreiche Datenbanken und nutzen fortschrittliche Algorithmen, um verdächtige Übereinstimmungen zu identifizieren. Sie helfen dabei, die Integrität der akademischen Arbeit zu wahren und Studierende zu ermutigen, eigenständig zu arbeiten und ihre eigenen Ideen zu entwickeln. Ein Beispiel für ein Tool dieser Kategorie ist Turnitin*. | | Bildgenerierung | Tools dieser Kategorie nutzen Deep-Learning-Algorithmen, um aus Texteingaben Bilder zu generieren oder bestehende Bilder zu verändern. Sie ermöglichen es Studierenden, mithilfe von Beschreibungen oder Anweisungen hochqualitative, visuelle Inhalte zu erstellen. Diese Tools sind besonders nützlich für die Erstellung von Bildern oder Diagrammen für Präsentationen, Poster, Webseiten oder Berichte. Ein Einsatz solcher Tools kann Zeit und Ressourcen bei der Materialerstellung sparen sowie Studierende oder Lehrende, welche nicht über ausgeprägte künstlerische Fähigkeiten oder umfangreiche Designkenntnisse und Software verfügen, dazu befähigen, visuell ansprechendes Material zu erstellen. Ein Beispiel für ein Tool dieser Kategorie ist DreamStudio* welches das StableDiffusion Modell zur Bildgenerierung verwendet. | | Präsentationserstellung | Tools dieser Kategorie ermöglichen es Studierenden und Lehrenden, auf einfache Weise ansprechende Präsentationen zu erstellen. Sie basieren auf Texteingaben, die bereitgestellt werden müssen, und generieren daraus automatisch Folien mit relevanten Inhalten. Diese Tools bieten verschiedene Designvorlagen, Animationsmöglichkeiten und die Möglichkeit, multimediale Elemente wie Bilder oder Videos einzufügen. Sie erleichtern die Erstellung von visuell ansprechenden Präsentationen und sparen Zeit. Studierende und Lehrende müssen sich weniger mit dem Gestalten der Folien beschäftigen, sondern können sich mehr auf den Inhalt ihrer Präsentationen konzentrieren. Diese Tools ermöglichen es, professionell aussehende Präsentationen zu erstellen und ihre Informationen auf eine zugängliche und ansprechende Weise zu präsentieren. Ein Beispiel für ein Tool dieser Kategorie ist SlidesAI*. | Bestehende Sammlungen und Datenbanken zu KI-Tools - Sammlung von Tools mit dem Fokus auf Textverarbeitung: VK:KIWA - Umfassende Toolliste zu verschiedensten Kategorien: AI Tools Directory - Datenbank mit über 50 Kategorien und 3000 Tools: AI Tools Update - Umfangreiche Datenbank und Community zu KI-Tools: FUTUREPEDIA - Datenbank zu KI-Tools: Future Tools - Umfangreiche Sammlung von KI-Tools mit Erklärvideos: Miroboard von Jan Foelsing - sehr umfassende und aktuelle KI-Sammlung: The Generative AI Landscape - KI-Tools nach Erscheinungsdatum sortiert: There’s An AI For That Nutzung von generativer KI in Studium und Lehre Ergänzend zu dieser allgemeinen Einführung zum Thema generativer KI (inkl. Toolkategorien und -sammlung) gibt es zwei weitere Handlungsempfehlungen speziell für Lehrenden und Studierende. - Einsatz von KI in der Lehre (Zielgruppe Lehrende) - Einsatz von KI im Studium (Zielgruppe Studierende) Weitere Unterstützungsangebote zu dem Thema KI in der Lehre an der Goethe-Universität sind: - „Über, mit und von KI lernen? – Ein pädagogischer Rundgang“ (studiumdigitale) - „Einsatzmöglichkeiten von KI-Tools in der Lehre“ (studiumdigitale) - „Was machen wir mit KI und was macht KI mit uns? Ethische Aspekte im Umgang mit KI-Tools in der Hochschullehre“ (studiumdigitale) - „KI-Anwendungen wie ChatGPT in Lehre und Prüfungen“ (IKH) - „KI-gestütztes Schreiben vermitteln“ (IKH &amp; Schreibzentrum) - Online Lehrlabor „ChatGPT als Herausforderung und Chance. Was macht die KI mit dem Schreiben?„ (Schreibzentrum) - Tipps zur Nutzung von KI-Schreibtools in der Lehre (Schreibzentrum) - Impulsreihe im Rahmen des Verbundprojekts HessenHub Frequently Asked Questions (FAQ) Kontakt Die Handreichungen wurden von der AG: Generative KI mit dem Fokus auf Studium und Lehre erstellt. Hinweise und Feedback nehmen wir gerne über folgende Adresse entgegen: ag-gki@studiumdigitale.uni-frankfurt.de</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1590</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Trafilatura</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final cleanup: config alignment, logger removal, color updates, README, requirements,project structure added
</commit_message>
<xml_diff>
--- a/data/raw_extracted_data.xlsx
+++ b/data/raw_extracted_data.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -533,11 +533,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Guidance on how you might engage with Generative AI (GenAI) in your assessments effectively and ethically. GenAI is a technique in artificial intelligence in which outputs such as text, images, code, music, and video are generated by software. GenAI is potentially transformative as well as disruptive, and GenAI tools will feature in many academic and professional workplaces. Rather than seek to prohibit your use of them, we will support you in using them effectively, ethically and transparently. However, it may not always be appropriate to use GenAI. Whilst they are attractively powerful and easy to use, GenAI tools can provide misleading or incorrect information. They can also negatively impact your learning by reducing the need for critical engagement that is key to deep and meaningful learning. Additionally, you need to be aware of the difference between reasonable use of such tools, and at what point their use might be regarded as giving you an unfair advantage. Visit the Generative AI Hub For more details on how GenAI works, the ethical implications and limitations of the tools and the ways in which you can use them, please visit the Generative AI Hub. The Generative AI and Academic Skills Moodle course provides a more in-depth look at GenAI in an academic context. GenAI and academic integrity Academic misconduct is strictly prohibited, including the use of essay mills, homework help sites, plagiarism, collusion, falsification, impersonation or any other action which might give me an unfair advantage. An unfair advantage is: • when you hide something and aren't transparent about your approach. • when you take something directly from someone (or something) else and don't reference or acknowledge it. • when you don't follow the assessment guidance. It is not acceptable to use GenAI tools to write your entire assessment and present this as your own work. Words and ideas from GenAI tools are making use of other human authors' ideas without referencing them, which is considered by many to be a form of plagiarism. Using GenAI tools to check your grammar or spelling is usually appropriate if the tool is not rewriting a large proportion of your work. Similarly, tasks such as ideas generation or planning may be an appropriate use. For all assessments, your context and the nature of the assessment must be considered. Your teachers will give guidance on: • what ways (if at all) you are permitted to use GenAI. • which aspects of your work it is appropriate (or even expected) that you use GenAI for. If you are unsure about what constitutes acceptable use of GenAI in an assessment, ask for clarification from the module leader. If no explicit instructions are given, the default for assessments should be that you use GenAI in an assistive role while making sure that the final submission is still substantially your own work. Staff resources on how to guide students on the use of GenAI in assessments can be found on the Generative AI Hub. Category 2 describes in more detail how GenAI might be used in an assistive role. UCL does not use GenAI detectors when marking. Instead, if a marker has any concerns about your work, they may speak to you to get more information. You should not automatically assume this means that they suspect you of academic misconduct. Inappropriate use of GenAI is viewed as plagiarism. This is defined as the representation of other people’s work or ideas as your own without appropriate referencing or acknowledgement. This includes the use of GenAI tools that exceeds that permitted in the assessment brief. If teaching staff suspect that you are trying to pass off GenAI output as your own work then the regulations in the Academic Manual (9.2.5 a), 9.2.5 e) iii, and 9.2.6 c) may apply. You may be invited to an investigatory viva to probe the authorship of your work. How to acknowledge GenAI use in your work You should acknowledge GenAI use where it has been used to assist in the process of creating your work. The Library Skills pages share guidance on how and when to acknowledge GenAI in your work.</t>
+          <t>Engaging with Generative AI in your education and assessment Guidance on how you might engage with Generative AI (GenAI) in your assessments effectively and ethically. GenAI is a technique in artificial intelligence in which outputs such as text, images, code, music, and video are generated by software. GenAI is potentially transformative as well as disruptive, and GenAI tools will feature in many academic and professional workplaces. Rather than seek to prohibit your use of them, we will support you in using them effectively, ethically and transparently. However, it may not always be appropriate to use GenAI. Whilst they are attractively powerful and easy to use, GenAI tools can provide misleading or incorrect information. They can also negatively impact your learning by reducing the need for critical engagement that is key to deep and meaningful learning. Additionally, you need to be aware of the difference between reasonable use of such tools, and at what point their use might be regarded as giving you an unfair advantage. Key resources - For more details on how GenAI works, the ethical implications and limitations of the tools and the ways in which you can use them, please visit the Generative AI Hub. - The Generative AI and Academic Skills Moodle course provides a more in-depth look at GenAI in an academic context. - You should acknowledge GenAI use where it has been used to assist in the process of creating your work. The Library Skills pages share guidance on how and when to acknowledge GenAI in your work. GenAI and academic integrity Academic misconduct is strictly prohibited, including the use of essay mills, homework help sites, plagiarism, collusion, falsification, impersonation or any other action which might give me an unfair advantage. An unfair advantage is: - when you hide something and aren’t transparent about your approach. - when you take something directly from someone (or something) else and don’t reference or acknowledge it. - when you don’t follow the assessment guidance. It is not acceptable to use GenAI tools to write your entire assessment and present this as your own work. Words and ideas from GenAI tools are making use of other human authors’ ideas without referencing them, which is considered by many to be a form of plagiarism. Using GenAI tools to check your grammar or spelling is usually appropriate if the tool is not rewriting a large proportion of your work. Similarly, tasks such as ideas generation or planning may be an appropriate use. For all assessments, your context and the nature of the assessment must be considered. Your teachers will give guidance on: - what ways (if at all) you are permitted to use GenAI. - which aspects of your work it is appropriate (or even expected) that you use GenAI for. If you are unsure about what constitutes acceptable use of GenAI in an assessment, ask for clarification from the module leader. If no explicit instructions are given, the default for assessments should be that you use GenAI in an assistive role while making sure that the final submission is still substantially your own work. Staff resources on how to guide students on the use of GenAI in assessments can be found on the Generative AI Hub. Category 2 describes in more detail how GenAI might be used in an assistive role. UCL does not use GenAI detectors when marking. Instead, if a marker has any concerns about your work, they may speak to you to get more information. You should not automatically assume this means that they suspect you of academic misconduct. Inappropriate use of GenAI is viewed as plagiarism. This is defined as the representation of other people’s work or ideas as your own without appropriate referencing or acknowledgement. This includes the use of GenAI tools that exceeds that permitted in the assessment brief. If teaching staff suspect that you are trying to pass off GenAI output as your own work then the regulations in the Academic Manual (9.2.5 a), 9.2.5 e) iii, and 9.2.6 c) may apply. You may be invited to an investigatory viva to probe the authorship of your work.</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -593,11 +593,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>General guidance for all students on using generative AI tools in your studies. The University trusts you to act with integrity in your use of generative AI for your studies.It does not ban the use of generative AI, though its use is restricted for assessment. Some of your courses may also restrict its use in other ways. Always check your course level guidance.These top-level guidelines provide clarity on which uses of generative AI are strictly prohibited and constitute academic misconductThey also explain why you should be cautious about over-reliance on generative AI for your learning.This guidance is general and sets out the basics of the University’s position – it is essential that you also check the detailed information provided for each of your courses.Generative AI at EdinburghThe University recognises that developing skills in the responsible use of generative AI is important and will likely be significant for your future life and work. It also recognises that there are times when you may want – or be asked – to use it in your current studies. We want to ensure that you have the knowledge and skills to thrive in a changing world, and we recognise that generative AI can be used creatively, critically and with integrity.These guidelines are general to the whole University. It is important that you are aware that each course will have its own, more detailed, guidance. You should always check your course documentation on this, and speak to your Course Organiser if you are unsure.The University trusts you as students to act responsibly in relation to the use of generative AI. It also recognises that you need clarity on when its use breaches the University’s rules on academic misconduct. These guidelines provide you with this clarity. Unacceptable uses of generative AI for assessmentPassing off someone – or something’s – work as your own for an assessment is academic misconduct. This could be failing to cite a source you have used in piece of assessed work, getting someone else to complete an assessment for you, claiming authorship of machine-generated content or presenting machine-translated work as your own.If you submit a piece of work for assessment that is not your own original work you risk being investigated according to the university’s academic misconduct investigation procedures. This could have serious implications for you and your studies.The following uses of generative AI are not acceptable and constitute misconduct: if you use them you risk investigation and penalties.Presenting AI outputs as your own, original work.Use of an AI translator to convert assessments to English before submission: English is the language of teaching and assessment at Edinburgh – machine translation is treated as false authorship and is not acceptable.Submitting an assessment which includes elements of AI-generated text without acknowledgment.Submitting an assessment which includes AI-generated images, audio or video without acknowledgment.Submitting an assessment which includes AI-generated mathematical formulae or reasoning, or computer code, without acknowledgment.Citing AI-found sources without reading and verifying them.For more detailed information about the restrictions around using AI-supported online proofing tools, please see the University’s Guidance on Proofreading of Student Assessments. Using generative AI to support your learningWhile we have these clear restrictions around the use of generative AI in your assessed work, the University understands that there are ways in which you may wish to use it to support your studies. This might include using it to:brainstorm ideasget quick definitions of conceptsovercome writer’s block through dialoguecheck your grammarorganise or summarise informationre-format your referencesSome courses may encourage or even require you to use it in certain ways, while others may ask you not to use it at all. Again, it is important that you check your course-level guidance on this. Reasons to be cautious about your use of generative AIYou should be aware that there are risks and disadvantages associated with over-use of generative AI to support learning. Cognitive offloadingThere is growing research evidence that over-use of generative AI can negatively affect your learning. You may want to look at studies which raise concern over how ‘cognitive offloading’, ‘metacognitive laziness’ and reduction in capacity for critical thinking may be associated with over-reliance on this technology. If you routinely use generative AI for breaking down and summarising long texts, for example, you will not be developing your own critical skills in the analysis of complex documents. You will also not be practicing and learning how to bring together complex ideas using the power of your own intelligence. Similarly, if you are using it to regularly assist with mathematical reasoning or coding, you are undermining your own ability to learn and become expert at doing this yourself. To make the most of your time at university, embracing the hard work of learning is a better approach than looking for short-cuts. Bias and inaccuracyGenerative AI models are not ‘intelligent’ in the way that humans are intelligent. They have been trained on more text than a human could ever read, but have different capabilities and make different mistakes. While their output often appears convincing and reliable, their behaviour is strongly influenced by the data they are trained on, so they can perpetuate harmful biases, fabricate information and make errors. You will be held accountable for these errors and biases if you include them in assessed work. Higher education should help you develop advanced knowledge which is creative and rigorous, not generic and unreliable. It is best to use your time at university to develop high-level skills that are going to help you throughout life – original thought, engaging writing, critical use of evidence, creative risk-taking and innovation. Using the University’s own generative AI platform (ELM)All University of Edinburgh students have free access to ELM, which offers you a secure gateway to a range of generative AI models. The university encourages you to use ELM over other platforms such as GPT, DeepSeek, Grok etc for the following reasons:In ELM your data is secure – it will not be retained by third party services to train their models or for any other purpose.It is free to use for all staff and students, providing the same access for all and saving you money.ELM provides access to a range of language models including a locally-hosted instance of Llama. This has an optimized architecture that can achieve faster response times and reduced power consumption. You can also choose other models such as GPT within ELM if necessary for your task.Your lecturers do not have access to your chat history in ELM for the purposes of 'checking' your work - like your email account, it is private to you.You can access ELM and find out about training opportunities here. Acknowledging your use of AIIf you choose to use generative AI for aspects of an assessment, it is important to be transparent about how you have done so. You should include a brief acknowledgment at the end of your piece of work, for example:I used OpenAI o4 Mini via ELM to check grammar and spelling throughout my assignment. I also used the Create Image function in ChatGPT to generate the image on page 2.Again – check the detail in your course guidance if you are unsure what is required, as there may be specific things your Course Organiser would like you to cover in your acknowledgment. Citing your use of generative AIIf you use content generated by AI within your work, for example an AI-generated image or text from an AI chatbot, you will need to reference it. This means including an in-text citation or footnote in the body of your work, and a corresponding reference in your reference list. The Library’s guide to using generative AI gives very useful guidance on this. Environmental and social impact of generative AIMany in our community are concerned about the negative impacts of generative AI in areas such as:Energy and resource useExploitative labour practicesIntellectual propertyYou may wish to read more about these via the links above. While there are ongoing efforts to reduce the environmental impact of the datacentres that make AI models work, it is clear that use of generative AI has a higher impact than, for example, a simple web search. If you are concerned about this, consider using the locally-hosted instance of Llama in ELM (see above). It is more efficient in terms of resource use, and provides a more transparent alternative to OpenAI, meaning that it is easier for the university to measure and manage its power consumption.You might also try to limit use of generative AI to purposeful rather than casual use. Links to other sourcesPrinciplesEdinburgh Student Assembly principles on the use of generative AIRussell Group principles on generative AI use in education Further guidanceGenerative AI use for Postgraduate Research studentsLibrary guide to using generative AI in academic work TrainingUniversity of Edinburgh Digital Skills Programme Academic misconduct guidanceFurther guidance on academic misconduct (including plagiarism) and how to avoid itUniversity of Edinburgh Academic Misconduct Procedures Return to ELM main page This article was published on 2025-07-23</t>
+          <t>General guidance for all students on using generative AI tools in your studies. Revision March 2026 These guidelines provide you with guidance on acceptable and unacceptable uses of both generative and agentic AI in your studies.The University trusts you to act with integrity in your use of AI in your learning.To make the most of your time at university, embracing the hard work of learning is a better approach than looking for AI-enabled short-cuts.The University does not ban the use of AI, though its use will be restricted for much of your assessed work.Where necessary, some of your courses may also restrict its use in other ways. You must always check your course level guidance.These top-level guidelines provide you with clarity on which uses of generative and agentic AI are strictly prohibited and constitute academic misconduct.They also explain why you should be cautious about over-reliance on AI for your learning.This guidance is general and applies to the whole University – it is essential that you also check the detailed information provided by each of your courses.Generative AIThe University recognises that developing skills in the responsible use of generative AI is important and will likely be significant for your future life and work. It also recognises that there are times when you may want – or be asked – to use it in your current studies. We want to ensure that you have the knowledge and skills to thrive in a changing world, and we recognise that generative AI can be used creatively, critically and with integrity.These guidelines are general to the whole University. It is important that you are aware that each course will have its own, more detailed, guidance. You should always check your course documentation on this, and speak to your Course Organiser if you are unsure.The University trusts you as students to act responsibly in relation to the use of generative AI. It also recognises that you need clarity on when its use breaches the University’s rules on academic misconduct. These guidelines provide you with this clarity.Agentic AIAI agents and AI browsers are forms of AI that are able to operate autonomously in complex environments. Agentic AI tools do not require human prompts or continuous oversight and are able to perform self-directed tasks. For example, customer service agents are able to work autonomously across multiple channels and information sources to rapidly answer customer questions and make recommendations.Using an AI agent within Learn or any other University learning or assessment platform which requires you to log in is not permitted. Sharing your login details with an agent or agentic browser is a breach of the University Computing Acceptable Use Policy. This will result in your access to University digital services being removed and disciplinary action being taken against you.Unacceptable uses of generative AI for assessmentPassing off someone – or something’s – work as your own for an assessment is academic misconduct. This could be failing to cite a source you have used in a piece of assessed work, getting someone or something else (such as an AI agent) to complete your work for you, claiming authorship of machine-generated content or presenting machine-translated work as your own.If you submit a piece of work for assessment that is not your own original work you risk being investigated according to the university’s academic misconduct investigation procedures. This could have serious implications for you and your studies. Those on professionally accredited programmes may be referred for fitness to practice concerns if found to engage in academic misconduct.The following uses of generative and agentic AI are not acceptable and constitute misconduct: if you use them you risk investigation and penalties.Presenting AI outputs as your own, original work.Using an AI translator to convert assessed work to English before submission: English is the language of teaching and assessment at Edinburgh – machine translation is treated as false authorship and is not acceptable.Submitting an assessment which includes elements of AI-generated text without acknowledgment.Submitting an assessment which includes AI-generated images, audio or video without acknowledgment.Submitting an assessment which includes AI-generated mathematical formulae or reasoning, or computer code, without acknowledgment.Citing and referencing AI-found sources without reading and verifying them.Using an AI agent or AI browser to complete any type of work – assessed or not – within your virtual learning environment.For more detailed information about the restrictions around using AI-supported online proofing tools, please see the University’s Guidance on Proofreading of Student Assessments (pdf). Use of live translation apps in classThe University’s Accessible and Inclusive Learning Policy allows you to make audio recordings of classes but does not allow you to share and distribute these recordings with a third party. AI-based translation apps retain and process recordings in a way that is not allowed in this policy. They can also negatively effect the group dynamic in tutorials and seminars. As a result, you must not use third-party AI-based translation apps in class.You may however use translation services outside the classroom to help clarify and enhance your understanding of lecture, lab or seminar notes where necessary. You should only use the University’s generative AI service – ELM – to do this as it has in-built privacy protections. You can access ELM and find out about training opportunities here.Using generative AI to support your learningWhile we have these clear restrictions around the use of AI in your assessed work, the University understands that there are ways in which you may wish to use it to support your studies.This might include using it to:brainstorm ideasget quick definitions of conceptsovercome writer’s block through dialoguecheck your grammarorganise or summarise informationre-format your referencesSome courses may encourage or even require you to use it in certain ways, while others may ask you not to use it at all. Again, it is really important that you check your course-level guidance on this.Reasons to be cautious about your use of generative AIYou should be aware that there are risks and disadvantages associated with over-use of generative AI to support learning.Cognitive offloadingThere is growing research evidence that over-use of generative AI can negatively affect your learning. You may want to look at studies which raise concern over how ‘cognitive offloading’, ‘metacognitive laziness’ and reduction in capacity for critical thinking may be associated with over-reliance on this technology.If you routinely use generative AI for breaking down and summarising long texts, for example, you will not be developing your own critical skills in the analysis of complex documents. You will also not be practicing and learning how to bring together complex ideas using the power of your own intelligence. Similarly, if you are using it to regularly assist with mathematical reasoning or coding, you are undermining your own ability to learn and become expert at doing this yourself. To make the most of your time at university, embracing the hard work of learning is a better approach than looking for short-cuts.Bias and inaccuracyGenerative AI models are not ‘intelligent’ in the way that humans are intelligent. They have been trained on more text than a human could ever read, but have different capabilities and make different mistakes. While their output often appears convincing and reliable, their behaviour is strongly influenced by the data they are trained on, so they can perpetuate harmful biases, fabricate information and make errors. You will be held accountable for these errors and biases if you include them in assessed work.Higher education should help you develop advanced knowledge which is creative and rigorous, not generic and unreliable. It is best to use your time at university to develop high-level skills that are going to help you throughout life – original thought, engaging writing, critical use of evidence, creative risk-taking and innovation.Using the University’s own generative AI platform (ELM)All University of Edinburgh students have free access to ELM (Edinburgh access to Language Models), which offers you a secure gateway to a range of generative AI models.The university encourages you to use ELM over other platforms such as GPT, DeepSeek, Grok etc for the following reasons:In ELM your data is secure – it will not be retained by third party services to train their models or for any other purpose.It is free to use for all staff and students, providing the same access for all and saving you money.ELM provides access to a range of language models including a locally-hosted instance of Llama. This has an optimized architecture that can achieve faster response times and reduced power consumption. You can also choose other models such as GPT within ELM if necessary for your task.You can access ELM and find out about training opportunities here.Acknowledging your use of AIIf you choose to use generative AI for permitted aspects of an assessment, it is important to be transparent about how you have done so. You should include a brief acknowledgment at the end of your piece of work, for example:I used GPT 5 via ELM to check grammar and spelling throughout my assignment.I also used Midjourney to generate the image on page 2.Again – check the detail in your course guidance if you are unsure what is required, as there may be specific things your Course Organiser would like you to cover in your acknowledgment.Citing your use of generative AIIf you use content generated by AI within your work, for example an AI-generated image or text from an AI chatbot, you will need to reference it. This means including an in-text citation or footnote in the body of your work, and a corresponding reference in your reference list.The Library’s guide to using generative AI gives very useful guidance on this. Environmental and social impact of generative AIMany in our community are concerned about the negative impacts of generative AI in areas such as:Energy and resource useExploitative labour practicesIntellectual propertyYou may wish to read more about these via the links above.While there are ongoing efforts to reduce the environmental impact of the datacentres that make AI models work, it is clear that use of generative AI has a higher impact than, for example, a simple web search. If you are concerned about this, consider using the locally-hosted instance of Llama in ELM (see above). It is more efficient in terms of resource use, and provides a more transparent alternative to OpenAI, meaning that it is easier for the university to measure, manage and offset its power consumption.You might also try to limit use of generative AI to purposeful rather than casual use.Links to other sourcesPrinciplesEdinburgh University Students Assembly on AI – principles Further guidanceGenerative AI use for Postgraduate Research studentsLibrary guide to using generative AI in academic workResearchAI for Teaching Innovation projectHigher Education Policy Institute Student Generative AI Survey 2025TrainingUniversity of Edinburgh Digital Skills ProgrammeAcademic misconduct guidanceFurther guidance on academic misconduct (including plagiarism) and how to avoid itUniversity of Edinburgh Academic Misconduct Procedures Return to ELM main page This article was published on 2025-07-23</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1486</v>
+        <v>1802</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -606,7 +606,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -623,11 +623,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>University of Glasgow - MyGlasgow - not found Skip to main content Cookies We use cookies to improve user experience and allow for personalised advertising via third parties. You can find out more about cookies and how we use them on our privacy policy page . Analytics I'm happy with analytics data being recorded I do not want analytics data recorded Please choose your analytics preference Personalised advertising I’m happy to get personalised ads I do not want personalised ads Please choose your personalised ads preference save choices accept all privacy settings accept We use cookies Necessary cookies Necessary cookies enable core functionality. The website cannot function properly without these cookies, and can only be disabled by changing your browser preferences. Analytics cookies Analytical cookies help us improve our website. We use Google Analytics. All data is anonymised. Switch analytics ON OFF Clarity Clarity helps us to understand our users’ behaviour by visually representing their clicks, taps and scrolling. All data is anonymised. Switch clarity ON OFF Privacy policy close search Staff login Student login Staff a-z MyGlasgow MyGlasgow not found MyGlasgow Students MyGlasgow Staff IT Sport Not found The web page or resource you requested could not be found. Check that you have the right address, or: Go to MyGlasgow Students homepage Go to MyGlasgow Staff homepage Try searching MyGlasgow Search MyGlasgow search</t>
+          <t>University of Glasgow - MyGlasgow - not found Skip to main content Cookies We use cookies to improve user experience and allow for personalised advertising via third parties. You can find out more about cookies and how we use them on our privacy policy page . Analytics I'm happy with analytics data being recorded I do not want analytics data recorded Please choose your analytics preference Personalised advertising I’m happy to get personalised ads I do not want personalised ads Please choose your personalised ads preference save choices accept all privacy settings accept We use cookies Necessary cookies Necessary cookies enable core functionality. The website cannot function properly without these cookies, and can only be disabled by changing your browser preferences. Analytics cookies Analytical cookies help us improve our website. We use Google Analytics. All data is anonymised. Switch analytics ON OFF Clarity Clarity helps us to understand our users’ behaviour by visually representing their clicks, taps and scrolling. All data is anonymised. Switch clarity ON OFF Privacy policy close search Staff login Student login Staff a-z MyGlasgow MyGlasgow not found MyGlasgow Students MyGlasgow Staff Animal Welfare IT Sport Not found The web page or resource you requested could not be found. Check that you have the right address, or: Go to MyGlasgow Students homepage Go to MyGlasgow Staff homepage Try searching MyGlasgow Search MyGlasgow search</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -636,7 +636,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Using generative AI Understand where to use generative artificial intelligence (AI) appropriately for your studies and in preparation for your future. Go to: What is generative AI? | Generative AI and your studies | University of Nottingham policy | Further information Always check expectations for generative AI use and acknowledgement for any given module or assessment. What is generative AI? “Artificial intelligence, or AI, is technology that enables computers and machines to simulate human intelligence and problem-solving capabilities.” (IBM, 2024) Generative artificial intelligence is a form of AI technology that can produce text, images, and other media in response to user prompts. These tools (including ChatGPT and Microsoft Copilot) are not sentient - they only mimic intelligence, through algorithmic prediction and pattern recognition. Drawing on large quantities of data, these tools create outputs based on probability. It is important to remember that the responses provided by generative AI tools do not express meaning, understanding, or intentionality. As a result, responses generated by these tools cannot be relied upon to be accurate and always need to be fact-checked. Back to the top Generative AI and your studies The use of AI tools is becoming common practice across a variety of industries, which means that understanding how to use generative AI effectively and responsibly will likely be a key skill for employment. You might at times be asked to use AI within your studies, to help you develop skills relating to its effective, responsible, and professional use. For other assessments, use of generative AI may be prohibited, as the assessment is designed to develop your academic and transferable skills. Back to the top University of Nottingham policy Key points to remember Content created or significantly modified by generative AI, whether text, code, images, or video, should only be used if this is clearly stated to be essential or optional for an assessment task, and should always be fully evidenced and acknowledged. - Always consult your tutor or assessment documents on expectations for AI use - Always fact-check any information generated using AI - Always be transparent in acknowledging your use of generative AI, - Always keep records of your interactions with AI tools Back to the top Back to the top Continue your journey You may also be interested in: Further support Disability support service Language and communication skills</t>
+          <t>Using generative AI Understand where to use generative artificial intelligence (AI) appropriately for your studies and in preparation for your future. Go to: What is generative AI? | Generative AI and your studies | University of Nottingham policy | Further information Always check expectations for generative AI use and acknowledgement for any given module or assessment. What is generative AI? “Artificial intelligence, or AI, is technology that enables computers and machines to simulate human intelligence and problem-solving capabilities.” (IBM, 2024) Generative artificial intelligence is a form of AI technology that can produce text, images, and other media in response to user prompts. These tools (including ChatGPT and Microsoft Copilot) are not sentient - they only mimic intelligence, through algorithmic prediction and pattern recognition. Drawing on large quantities of data, these tools create outputs based on probability. It is important to remember that the responses provided by generative AI tools do not express meaning, understanding, or intentionality. As a result, responses generated by these tools cannot be relied upon to be accurate and always need to be fact-checked. Back to the top Generative AI and your studies The use of AI tools is becoming common practice across a variety of industries, which means that understanding how to use generative AI effectively and responsibly will likely be a key skill for employment. You might at times be asked to use AI within your studies, to help you develop skills relating to its effective, responsible, and professional use. For other assessments, use of generative AI may be prohibited, as the assessment is designed to develop your academic and transferable skills. Back to the top University of Nottingham approach Key points to remember Content created or significantly modified by generative AI, whether text, code, images, or video, should only be used if this is clearly stated to be essential or optional for an assessment task, and should always be fully evidenced and acknowledged. - Always consult your tutor or assessment documents on expectations for AI use - Always fact-check any information generated using AI - Always be transparent in acknowledging your use of generative AI, - Always keep records of your interactions with AI tools Back to the top Back to the top Continue your journey You may also be interested in: Further support Disability support service Language and communication skills</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -696,7 +696,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ERROR: The request could not be satisfied 403 ERROR The request could not be satisfied. Request blocked. We can't connect to the server for this app or website at this time. There might be too much traffic or a configuration error. Try again later, or contact the app or website owner. If you provide content to customers through CloudFront, you can find steps to troubleshoot and help prevent this error by reviewing the CloudFront documentation. Generated by cloudfront (CloudFront) Request ID: t2-yWNkESFrwS1kYo-F1lhIoOXMaMcGscuLDIpqEzsqxyAhxX3K5pQ==</t>
+          <t>ERROR: The request could not be satisfied 403 ERROR The request could not be satisfied. Request blocked. We can't connect to the server for this app or website at this time. There might be too much traffic or a configuration error. Try again later, or contact the app or website owner. If you provide content to customers through CloudFront, you can find steps to troubleshoot and help prevent this error by reviewing the CloudFront documentation. Generated by cloudfront (CloudFront) Request ID: TdBswHUJAjAV1a5QIKlMeCkrlK2e1wGk5X-OUVCkHVV1ySNFcsRdFw==</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -936,7 +936,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -953,11 +953,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Using generative AI in teaching and learning Explore the new myCourses self-paced module: Generative AI for Teaching and Learning What is generative AI? Generative AI (gen AI) is a type of artificial intelligence that uses machine learning to create new types of media, including text, images, sound, and video. Many tools exist that use generative AI to create new content. Some examples include: Media | Example tools | |---|---| Text | Copilot (Secure version approved at McGill) | Images | Copilot (Secure version approved at McGill) Adobe Firefly, Midjourney, DALL-E3 (not approved for use at McGill) | Sound | Copilot (Secure version approved at McGill) Voiceify (not approved for use at McGill) | Video | D-ID (not approved for use at McGill) | A secure version of Microsoft Copilot has been approved at McGill. Copilot is an AI chatbot tool integrated into Microsoft Edge and accessible from other browsers. Read more about using Copilot at McGill. Generative AI tools are built upon large language models (LLM) that have been trained on enormous corpora of information and are designed to respond to input prompts with well-structured output. They are focused on predictive text (i.e., the most likely word to follow a previous word), as well as generated media based on patterns or styles in existing datasets. While the outputs can often demonstrate seemingly sophisticated language interaction, there may be situations where they provide inaccurate information in that interaction (e.g., fictional sources). These tools are constantly improving, however, it is important to examine any generative AI output with a critical lens. The McGill Library has a page on artificial intelligence with a section on AI Literacy that discusses the importance of critically approaching AI. Ethical use of generative AI The development of generative AI has brought many ethical considerations that must be addressed with its use. The 2018 Montreal Declaration for a Responsible Development of Artificial Intelligence and the 2021 UNESCO Recommendation on the Ethics of Artificial Intelligence provide a number of principles important to the adoption of these new technologies. Both documents offer an excellent framework for how organizations need to consider these new technologies. The emergence of generative AI is leading to a process of reflection on the evolution of the concept of academic integrity. For any questions related to disciplinary procedures, contact the Office of the Dean of Students. McGill instructors should follow the same disciplinary procedures as for any other instance where there are concerns about academic integrity. To note: the Code of Student Conduct was updated last month and it now includes specific reference to generative AI with respect to academic offenses (see Articles 25-b and 26-f). For further information, such as the quantity of cases McGill is dealing with, the Office of the Dean of Students might be able to provide information. Instructors might be able to mitigate such cases by providing students with guidance about whether and how gen AI use is permitted in their courses. McGill strongly recommends that all instructors include in their course outlines a statement about gen AI use. Learn more: AI in academia: The end of the essay? (Maple League of Universities - YouTube video) Infographic: Generative AI explained by AI (Visual Capitalist) Teaching AI literacy: How to begin (Inside Higher Education) What is generative AI? (McKinsey) How can generative AI be used in teaching and learning? In May 2023, the Senate Subcommittee on Teaching and Learning (STL) created a working group to address the use of generative AI at McGill. The working group drafted a report with key recommendations for the use of generative AI at McGill. The report also presents principles for the use of generative AI in teaching and learning. Many different strategies exist for using generative AI tools in course teaching. For example, instructors can use them to create sample texts for students to analyze, create images for presentations, design entire presentation materials, and generate sample practice questions. Strategies also exist for students to use generative AI tools to support their learning. For example, they can be used to brainstorm ideas, create images to support assignments such as presentations, and summarize documents. These resources offer more ideas for creating instructional materials and supporting student learning: How could AI be used for learning and teaching? and How AI can be used meaningfully by teachers and students in 2023. Assessment is one facet of course design. The course design approach we promote at McGill suggests beginning with learning outcomes – what knowledge/skills/values would we like students to leave a course with? From there, we can consider what types of assessments align with the desired outcomes. The advent of gen AI might mean rethinking what those learning outcomes are before considering how to redesign assessment. Rethinking learning outcomes – this is an important consideration with implications for higher ed/society. Specifically in online education, McGill promotes experiential learning activities that require students to apply skills, make decisions, and produce work similar to what they would encounter in professional practice. These activities may take the form of interactive simulations, scenario-based assessments, authentic tasks linked to real-world contexts, and reflective activities that help students connect their experiences with course concepts. In some cases, gen AI use is intentionally integrated into the learning activities and requires that any use of gen AI tools be properly cited. It is important to note that students need AI literacy skills to responsibly use generative AI tools. These potentially new literacy skills could include elements such as fact-checking and prompt engineering. All McGill instructors and students can explore the new myCourses self-paced module Generative AI for Teaching and Learning. Avoid AI detection tools AI detection tools are tools designed to identify content that is partially or wholly generated by AI. These tools (specifically regarding generated text) are unreliable and often inaccurate, a statement corroborated by OpenAI, the creators of ChatGPT. OpenAI states that their false positive rate is 9%, which is a similar rate found in other AI detection tools. A false positive is when the tool identifies text as being generated by AI when it was actually created by a student. False positive results misguide instructors and can create situations where students are wrongly accused of a violation that they did not commit, forcing them to defend work that is rightfully theirs. Such situations can result in a negative classroom climate and create unnecessary stress and anxiety for all involved. McGill therefore discourages the use of AI detection tools. Note: McGill also does not recommend online proctoring. Course outline statements There should be no default assumption as to the use of generative AI tools. Therefore, McGill recommends that instructors explain to students in their course outline what the appropriate use or non-use is of generative AI tools in the context of that course. The use or non-use of these tools should align with the learning outcomes associated with the course. For this reason, instructors will need to write their own context-appropriate course outline statements. Below are four external examples to draw on: Monash University policy and practice guidance around acceptable and responsible use of AI technologies: See the Actions box and the section entitled Specify conditions for the use of generative AI in assessment. University of Florida has an excellent AI resource page that shows concise examples of course outline statements and multiple categories of suggestions on how to either neutralize or capitalize on using AI in courses. University of Toronto syllabus language: This document provides suggestions for clarifying whether students can use generative AI tools; can use generative AI tools in certain instances; or cannot use them at all in the course. Update your course syllabus for ChatGPT (Medium): See the section entitled Before editing your syllabus and the one entitled Update your syllabus. If you allow students to use generative AI tools in your course, provide guidance in your course outline for how students should acknowledge the use. Monash University provides useful examples, as well as links to APA and MLA citation guidelines. See the section entitled How students acknowledge the use of generative AI. AI and assessment of student learning Generative AI tools can be used to support many different types of assessment. As with the planning of any assessment of student learning, it is important to be intentional about the strategy. In this case, be intentional about either designing AI into your assessments or designing AI out of your assessments. This reflective process will encourage you to think through your assessments and determine if the integration of AI is appropriate (or not) for allowing students to demonstrate their learning. Designing AI into an assessment could involve having students generate the assignment with an AI tool, then critique the output, and reflect on the process. Designing AI out of the assessment could involve in-class writing exercises, where students create and share their ideas with other students in class during class time. Either way, the decision should align with students’ achievement of the desired learning outcomes. Monash University provides excellent considerations for assessment design. Learn more: 6 Tenets of postplagiarism: Writing in the age of artificial intelligence (Teaching and Leadership) AI-generated content in the classroom: Considerations for course design (Illinois State University) Artificial Intelligence (UNESCO) Beyond Grading: Assessment in the age of AI (McGill, video, 50 minutes) Bloom’s taxonomy revisited with AI (Oregon State University) Bowen, J. A., &amp; Watson, C. E. (2024). Teaching with AI: A practical guide to a new era of human learning. Johns Hopkins University Press How do I Consider the Options for a Generative AI Course Policy? (Center for Teaching and Learning, University of Massachusetts Amherst) McGill Library guide on artificial intelligence (McGill Library) The Artificial Intelligence Assessment Scale (AIAS): A Framework for Ethical Integration of Generative AI in Educational Assessment. (2024). Journal of University Teaching and Learning Practice, 21(06). Resources: Generative AI for teaching and learning (myCourses module for instructors and students) Generative AI perspectives and practices from McGill instructors across disciplines (podcast series) (Re)designing assessments in the age of generative AI - slides (Re)designing assessment tasks in the age of generative AI - activity sheet Sharing experiences with generative AI in teaching and learning - slides Sharing experiences with generative AI (teaching and learning community) Teaching consultations (one-on-one meeting with a TAP staff member) Have a question that was not answered in this article? Visit our FAQs. McGill University is on land which has served and continues to serve as a site of meeting and exchange amongst Indigenous peoples, including the Haudenosaunee and Anishinabeg nations. Teaching and Academic Programs acknowledges and thanks the diverse Indigenous peoples whose footsteps mark this territory on which peoples of the world now gather. This land acknowledgment is shared as a starting point to provide context for further learning and action. McLennan Library Building 3415 McTavish Street Suite MS-12 (ground level), Montreal, Quebec H3A 0C8 | mcgill.ca/tap</t>
+          <t>Using generative AI in teaching and learning See examples of how McGill instructors have incorporated statements on the use of generative AI in their course outlines. Explore the new myCourses self-paced module: Generative AI for Teaching and Learning What is generative AI? Generative AI (gen AI) is a type of artificial intelligence that uses machine learning to create new types of media, including text, images, sound, and video. Many tools exist that use generative AI to create new content. Some examples include: Media | Example tools | |---|---| Text | Copilot (Secure version approved at McGill) | Images | Copilot (Secure version approved at McGill) Adobe Firefly, Midjourney, DALL-E3 (not approved for use at McGill) | Sound | Copilot (Secure version approved at McGill) Voiceify (not approved for use at McGill) | Video | D-ID (not approved for use at McGill) | A secure version of Microsoft Copilot has been approved at McGill. Copilot is an AI chatbot tool integrated into Microsoft Edge and accessible from other browsers. Read more about using Copilot at McGill. Generative AI tools are built upon large language models (LLM) that have been trained on enormous corpora of information and are designed to respond to input prompts with well-structured output. They are focused on predictive text (i.e., the most likely word to follow a previous word), as well as generated media based on patterns or styles in existing datasets. While the outputs can often demonstrate seemingly sophisticated language interaction, there may be situations where they provide inaccurate information in that interaction (e.g., fictional sources). These tools are constantly improving, however, it is important to examine any generative AI output with a critical lens. The McGill Library has a page on artificial intelligence with a section on AI Literacy that discusses the importance of critically approaching AI. Ethical use of generative AI The development of generative AI has brought many ethical considerations that must be addressed with its use. The 2018 Montreal Declaration for a Responsible Development of Artificial Intelligence and the 2021 UNESCO Recommendation on the Ethics of Artificial Intelligence provide a number of principles important to the adoption of these new technologies. Both documents offer an excellent framework for how organizations need to consider these new technologies. The emergence of generative AI is leading to a process of reflection on the evolution of the concept of academic integrity. For any questions related to disciplinary procedures, contact the Office of the Dean of Students. McGill instructors should follow the same disciplinary procedures as for any other instance where there are concerns about academic integrity. To note: the Code of Student Conduct was updated last month and it now includes specific reference to generative AI with respect to academic offenses (see Articles 25-b and 26-f). For further information, such as the quantity of cases McGill is dealing with, the Office of the Dean of Students might be able to provide information. Instructors might be able to mitigate such cases by providing students with guidance about whether and how gen AI use is permitted in their courses. McGill strongly recommends that all instructors include in their course outlines a statement about gen AI use. Learn more: AI in academia: The end of the essay? (Maple League of Universities - YouTube video) Infographic: Generative AI explained by AI (Visual Capitalist) Teaching AI literacy: How to begin (Inside Higher Education) What is generative AI? (McKinsey) How can generative AI be used in teaching and learning? In May 2023, the Senate Subcommittee on Teaching and Learning (STL) created a working group to address the use of generative AI at McGill. The working group drafted a report with key recommendations for the use of generative AI at McGill. The report also presents principles for the use of generative AI in teaching and learning. Many different strategies exist for using generative AI tools in course teaching. For example, instructors can use them to create sample texts for students to analyze, create images for presentations, design entire presentation materials, and generate sample practice questions. Strategies also exist for students to use generative AI tools to support their learning. For example, they can be used to brainstorm ideas, create images to support assignments such as presentations, and summarize documents. These resources offer more ideas for creating instructional materials and supporting student learning: How could AI be used for learning and teaching? and How AI can be used meaningfully by teachers and students in 2023. Assessment is one facet of course design. The course design approach we promote at McGill suggests beginning with learning outcomes – what knowledge/skills/values would we like students to leave a course with? From there, we can consider what types of assessments align with the desired outcomes. The advent of gen AI might mean rethinking what those learning outcomes are before considering how to redesign assessment. Rethinking learning outcomes – this is an important consideration with implications for higher ed/society. Specifically in online education, McGill promotes experiential learning activities that require students to apply skills, make decisions, and produce work similar to what they would encounter in professional practice. These activities may take the form of interactive simulations, scenario-based assessments, authentic tasks linked to real-world contexts, and reflective activities that help students connect their experiences with course concepts. In some cases, gen AI use is intentionally integrated into the learning activities and requires that any use of gen AI tools be properly cited. It is important to note that students need AI literacy skills to responsibly use generative AI tools. These potentially new literacy skills could include elements such as fact-checking and prompt engineering. All McGill instructors and students can explore the new myCourses self-paced module Generative AI for Teaching and Learning. Avoid AI detection tools AI detection tools are tools designed to identify content that is partially or wholly generated by AI. These tools (specifically regarding generated text) are unreliable and often inaccurate, a statement corroborated by OpenAI, the creators of ChatGPT. OpenAI states that their false positive rate is 9%, which is a similar rate found in other AI detection tools. A false positive is when the tool identifies text as being generated by AI when it was actually created by a student. False positive results misguide instructors and can create situations where students are wrongly accused of a violation that they did not commit, forcing them to defend work that is rightfully theirs. Such situations can result in a negative classroom climate and create unnecessary stress and anxiety for all involved. McGill therefore discourages the use of AI detection tools. Note: McGill also does not recommend online proctoring. Course outline statements There should be no default assumption as to the use of generative AI tools. Therefore, McGill recommends that instructors explain to students in their course outline what the appropriate use or non-use is of generative AI tools in the context of that course. The use or non-use of these tools should align with the learning outcomes associated with the course. For this reason, instructors will need to write their own context-appropriate course outline statements. Below are four external examples to draw on: Monash University policy and practice guidance around acceptable and responsible use of AI technologies: See the Actions box and the section entitled Specify conditions for the use of generative AI in assessment. University of Florida has an excellent AI resource page that shows concise examples of course outline statements and multiple categories of suggestions on how to either neutralize or capitalize on using AI in courses. University of Toronto syllabus language: This document provides suggestions for clarifying whether students can use generative AI tools; can use generative AI tools in certain instances; or cannot use them at all in the course. Update your course syllabus for ChatGPT (Medium): See the section entitled Before editing your syllabus and the one entitled Update your syllabus. If you allow students to use generative AI tools in your course, provide guidance in your course outline for how students should acknowledge the use. Monash University provides useful examples, as well as links to APA and MLA citation guidelines. See the section entitled How students acknowledge the use of generative AI. Course outline statements from McGill instructors The following examples demonstrate how some McGill instructors have communicated their expectations, requirements, and/or limitations regarding the use of generative AI by students within specific courses. These statements have been reproduced with instructor permission. AI and assessment of student learning Generative AI tools can be used to support many different types of assessment. As with the planning of any assessment of student learning, it is important to be intentional about the strategy. In this case, be intentional about either designing AI into your assessments or designing AI out of your assessments. This reflective process will encourage you to think through your assessments and determine if the integration of AI is appropriate (or not) for allowing students to demonstrate their learning. Designing AI into an assessment could involve having students generate the assignment with an AI tool, then critique the output, and reflect on the process. Designing AI out of the assessment could involve in-class writing exercises, where students create and share their ideas with other students in class during class time. Either way, the decision should align with students’ achievement of the desired learning outcomes. Monash University provides excellent considerations for assessment design. Learn more: 6 Tenets of postplagiarism: Writing in the age of artificial intelligence (Teaching and Leadership) AI-generated content in the classroom: Considerations for course design (Illinois State University) Artificial Intelligence (UNESCO) Beyond Grading: Assessment in the age of AI (McGill, video, 50 minutes) Bloom’s taxonomy revisited with AI (Oregon State University) Bowen, J. A., &amp; Watson, C. E. (2024). Teaching with AI: A practical guide to a new era of human learning. Johns Hopkins University Press How do I Consider the Options for a Generative AI Course Policy? (Center for Teaching and Learning, University of Massachusetts Amherst) McGill Library guide on artificial intelligence (McGill Library) The Artificial Intelligence Assessment Scale (AIAS): A Framework for Ethical Integration of Generative AI in Educational Assessment. (2024). Journal of University Teaching and Learning Practice, 21(06). Resources: Generative AI for teaching and learning (myCourses module for instructors and students) Generative AI perspectives and practices from McGill instructors across disciplines (podcast series) (Re)designing assessments in the age of generative AI - slides (Re)designing assessment tasks in the age of generative AI - activity sheet Sharing experiences with generative AI in teaching and learning - slides Sharing experiences with generative AI (teaching and learning community) Teaching consultations (one-on-one meeting with a TAP staff member) Have a question that was not answered in this article? Visit our FAQs. McGill University is on land which has served and continues to serve as a site of meeting and exchange amongst Indigenous peoples, including the Haudenosaunee and Anishinabeg nations. Teaching and Academic Programs acknowledges and thanks the diverse Indigenous peoples whose footsteps mark this territory on which peoples of the world now gather. This land acknowledgment is shared as a starting point to provide context for further learning and action. McLennan Library Building 3415 McTavish Street Suite MS-12 (ground level), Montreal, Quebec H3A 0C8 | mcgill.ca/tap</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1805</v>
+        <v>1864</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -966,7 +966,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1223,11 +1223,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Addressing the Limitations of Using Generative AI for Learning Within the academic technology ecosystem, generative AI is increasingly everywhere. The Office of Academic Technology (OAT) is the central authority for evaluating learning technologies on campus, including generative AI. OAT supports the responsible adoption of generative AI for academic use, including for teaching and learning. Responsible AI Use in Teaching and Learning UT Austin defines responsible use of AI in teaching and learning as using AI in ways that foster the achievement of learning outcomes. That means using generative AI in ways that advance what students should know, be able to do and the attitudes they should develop as a result of a learning experience. At the same time, responsible AI use on the Forty Acres means not using generative AI in ways that would negate or inhibit the realization of those outcomes. UT encourages faculty, students and staff to be both AI-Forward and AI-Responsible. On the forward side, UT Austin provides access to a variety of tools and resources that foster the adoption of AI to achieve learning outcomes. On the responsible side, it emphasizes the critical importance of AI literacy and awareness of “the Big 6” limitations of using AI for learning (see below). Engaging in AI Forward – AI Responsible Learning Part of responsible adoption involves creating opportunities for the Longhorn community to gain literacy on the benefits and limitations of generative AI use in education. This starts with having a clear definition of what generative AI is and what it is not. What is generative AI? Generative AI refers to models that generate or create new or original output (text, code, images, videos, music, etc.) using pre-existing data the model has been trained on. The purpose of generative AI is to create brand-new content. Synthetic content can lead to wonderful, creative output — and that same output is often rife with limitations. Being AI-forward requires being aware of and taking action to mitigate the limitations below. The Big 6: Six Key Limitations of Using AI for Learning 1.0 Privacy and Security UT Austin supports data that is publicly available or defined as Published University information. When learning with AI, protect yourself and others by only using trusted vendors who allow you to disable chat history or model training easily. All students, faculty and staff must always follow the University’s generative AI acceptable use policy, which notes that inputting confidential or controlled university data is not allowed unless there is a University contract in place that protects such data. 2.0 Hallucinations and Deception Hallucinations are common and occur when generative AI produces content that is untrue or factually inaccurate. For example, bots such as ChatGPT might report that you have only 37 rows of data in a data set when there are 72. AI can also be deceptive in a variety of ways, including agreeing with users’ input or opinions even when they are incorrect or problematic, wrapping feedback in convincing, authoritative language that makes it appear credible. Such interactions can implicitly discourage critical analysis and discernment, leading learners to have more confidence in their knowledge or skills than they should. Always use more traditional approaches to research to confirm and verify facts. 3.0 Misalignment Misalignment occurs when a user prompts generative AI applications to produce a specific output, and the AI ends up producing an unexpected or undesired result. For example, when asking a bot to give you the Excel formula for merging two missing cells, it may give you the formula for splitting two cells instead. Misalignment is particularly problematic with image generation but also occurs within synthetic or AI-generated text. Careful prompt engineering helps address misalignment in text-based AI, but you will not be able to avoid it completely. Humans should always evaluate the output of generative AI with critical thinking skills. 4.0 Bias Because humans train them, generative AI output has both explicit and implicit biases baked into it, including stereotypes. It won’t be possible to entirely avoid bias in generative AI, just as it is not possible to avoid it in the real world, but a few small tips can help you engage with greater awareness. Educate yourself on the nature of implicit bias. Be aware that because humans train the models, they will reproduce our biases. Be skeptical and avoid over reliance on the models for any project. When you observe output from AI that is clearly biased or laced with stereotypes, report it to the vendor of the app you are using. 5.0 Ethics Al models have several ethical considerations, including digesting intellectual property, spreading misinformation, and using gen Al to produce new works or results without contribution. Other ethical considerations relate to the labor used to generate the models, the environmental impacts of generative Al, and the business ethics of releasing Al models for revenue generation without a clear understanding of the impact on society. Similar to bias, it is essential to be aware of the ethical concerns of using Al so that you can engage in a transparent manner. 6.0 Cognitive Offloading Cognitive offloading is the process of humans using external tools to reduce the demand or “cognitive load” of completing tasks (Risko and Gilbert, 2016). Technologies such as generative AI chatbots can help increase productivity through cognitive offloading; however, if you do not employ those freed-up resources for other tasks, the overuse of generative AI could potentially “diminish specific cognitive skills” (León-Dominguez, 2024). Engaging in human activities such as actively critiquing and evaluating output from generative AI can help protect problem-solving and creative and critical thinking skills. Other things you can do to avoid the downsides of cognitive offloading include engaging in transformation of gen Al output to make it your own. For example, evaluate the output for hallucinations, misalignment, bias, or ethics and then transform that output to make it authentically yours with your original thoughts, opinions, knowledge; or work. Have you adopted AI Forward - AI Responsible practices? The Office of Academic Technology is interested in learning from you. Please share your examples with the OAT using the form linked below. If you have questions or comments about generative AI for learning, please email us at oat@utexas.edu. Share Your ExamplesFebruary 21, 2024</t>
+          <t>Addressing the Limitations of Using Generative AI for Learning Within the academic technology ecosystem, generative AI is increasingly everywhere. The Office of Academic Technology (OAT) is the central authority for evaluating learning technologies on campus, including generative AI. OAT supports the responsible adoption of generative AI for academic use, including for teaching and learning. Responsible AI Use in Teaching and Learning UT Austin defines responsible use of AI in teaching and learning as using AI in ways that foster the achievement of learning outcomes. That means using generative AI in ways that advance what students should know, be able to do and the attitudes they should develop as a result of a learning experience. At the same time, responsible AI use on the Forty Acres means not using generative AI in ways that would negate or inhibit the realization of those outcomes. UT encourages faculty, students and staff to be both AI-Forward and AI-Responsible. On the forward side, UT Austin provides access to a variety of tools and resources that foster the adoption of AI to achieve learning outcomes. On the responsible side, it emphasizes the critical importance of AI literacy and awareness of “the Big 6” limitations of using AI for learning (see below). Engaging in AI Forward – AI Responsible Learning Part of responsible adoption involves creating opportunities for the Longhorn community to gain literacy on the benefits and limitations of generative AI use in education. This starts with having a clear definition of what generative AI is and what it is not. What is generative AI? Generative AI refers to models that generate or create new or original output (text, code, images, videos, music, etc.) using pre-existing data the model has been trained on. The purpose of generative AI is to create brand-new content. Synthetic content can lead to wonderful, creative output — and that same output is often rife with limitations. Being AI-forward requires being aware of and taking action to mitigate the limitations below. The Big 6: Six Key Limitations of Using AI for Learning 1.0 Privacy and Security UT Austin supports data that is publicly available or defined as Published University information. When learning with AI, protect yourself and others by only using trusted vendors who allow you to disable chat history or model training easily. All students, faculty and staff must always follow the University’s generative AI acceptable use policy, which notes that inputting confidential or controlled university data is not allowed unless there is a University contract in place that protects such data. 2.0 Hallucinations and Deception Hallucinations are common and occur when generative AI produces content that is untrue or factually inaccurate. For example, bots such as ChatGPT might report that you have only 37 rows of data in a data set when there are 72. AI can also be deceptive in a variety of ways, including agreeing with users’ input or opinions even when they are incorrect or problematic, wrapping feedback in convincing, authoritative language that makes it appear credible. Such interactions can implicitly discourage critical analysis and discernment, leading learners to have more confidence in their knowledge or skills than they should. Always use more traditional approaches to research to confirm and verify facts. 3.0 Misalignment Misalignment occurs when a user prompts generative AI applications to produce a specific output, and the AI ends up producing an unexpected or undesired result. For example, when asking a bot to give you the Excel formula for merging two missing cells, it may give you the formula for splitting two cells instead. Misalignment is particularly problematic with image generation but also occurs within synthetic or AI-generated text. Careful prompt engineering helps address misalignment in text-based AI, but you will not be able to avoid it completely. Humans should always evaluate the output of generative AI with critical thinking skills. 4.0 Bias Because humans train them, generative AI output has both explicit and implicit biases baked into it, including stereotypes. It won’t be possible to entirely avoid bias in generative AI, just as it is not possible to avoid it in the real world, but a few small tips can help you engage with greater awareness. Educate yourself on the nature of implicit bias. Be aware that because humans train the models, they will reproduce our biases. Be skeptical and avoid over reliance on the models for any project. When you observe output from AI that is clearly biased or laced with stereotypes, report it to the vendor of the app you are using. 5.0 Ethics Al models have several ethical considerations, including digesting intellectual property, spreading misinformation, and using gen Al to produce new works or results without contribution. Other ethical considerations relate to the labor used to generate the models, the environmental impacts of generative Al, and the business ethics of releasing Al models for revenue generation without a clear understanding of the impact on society. Similar to bias, it is essential to be aware of the ethical concerns of using Al so that you can engage in a transparent manner. 6.0 Cognitive Offloading Cognitive offloading is the process of humans using external tools to reduce the demand or “cognitive load” of completing tasks (Risko and Gilbert, 2016). Technologies such as generative AI chatbots can help increase productivity through cognitive offloading; however, if you do not employ those freed-up resources for other tasks, the overuse of generative AI could potentially “diminish specific cognitive skills” (León-Dominguez, 2024). Engaging in human activities such as actively critiquing and evaluating output from generative AI can help protect problem-solving and creative and critical thinking skills. Other things you can do to avoid the downsides of cognitive offloading include engaging in transformation of gen Al output to make it your own. For example, evaluate the output for hallucinations, misalignment, bias, or ethics and then transform that output to make it authentically yours with your original thoughts, opinions, knowledge; or work. Share your stories Have you adopted AI Forward – AI Responsible practices? The Office of Academic Technology is interested in learning from you. Please share your examples with the OAT using the form linked below. If you have questions or comments about generative AI for learning, please email us at oat@utexas.edu. Limitations of Using AI for Learning last updated February 21, 2024</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1036</v>
+        <v>1045</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1253,11 +1253,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Page not found - Artificial Intelligence (AI) at Purdue University Purdue Virtual Assistant Hi! I'm the Purdue Virtual Assistant. I can help answer your questions about IT Services. How can I help you? Skip to content 404 ERROR We’re sorry you were not able to find the page you were looking for. Search Search Major Tuition &amp; Costs Schedule a Visit Boilermakers’ Stories Apply</t>
+          <t>Page not found - Artificial Intelligence (AI) at Purdue University Skip to content 404 ERROR We’re sorry you were not able to find the page you were looking for. Search Search Major Tuition &amp; Costs Schedule a Visit Boilermakers’ Stories Apply</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: dependency updates and portability improvements
- sentence-transformers 2.7.0 → 5.3.0 (BERTopic StaticEmbedding fix)
- Add lxml_html_clean (trafilatura compatibility)
- Add setup.py for cross-machine import portability
- Fix Unmapped Frame palette in framing_interpret.py
- Update README with setup instructions
</commit_message>
<xml_diff>
--- a/data/raw_extracted_data.xlsx
+++ b/data/raw_extracted_data.xlsx
@@ -473,11 +473,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Guidance on safe and responsible use of Gen AI tools The aim of this guidance is to help you use GenAI tools safely and responsibly, so you feel confident about exploring different ways of using this technology to support your learning. Generative Artificial Intelligence (GenAI) is a fast-evolving technology and, during your time at Oxford, the University wants to enable and support the safe and productive use of these tools that will be important in your future. Ethical use GenAI tools must be used responsibly and ethically, in accordance with the academic standards of rigour and integrity that are expected of you as a student at Oxford. You should always use AI tools with integrity, honesty, and transparency, and maintain a critical approach to using any output generated by these tools. This document contains some useful tips for using GenAI to support your studies at Oxford. You should always follow the advice and guidance of your tutors and/or supervisors, and consult your department or faculty in relation to ethical use. Assessment For each specific assessment you will be given prior written notice of whether or not the use of AI is permitted. You are fully responsible for the accuracy, originality, and quality of work you submit for assessment, and you must follow the rules on AI use for each specific assessment you are taking. You must make a formal declaration of any permitted AI-use in the format prescribed by your assessment setter. Any unauthorised use of AI in work submitted for assessment constitutes cheating and plagiarism under University rules, penalties for which include failing the relevant assessment and, in appropriate cases, expulsion. Any use of AI in work submitted for assessment is unauthorised unless you are specifically told differently in writing, in advance of the assessment, in instructions from your faculty’s or department for the specific assessment in question. Even if a type of AI use has been authorised for a previous assessment, or for formative work, it is your responsibility to ensure that you comply with the rules on AI use for the specific assessment you are taking, in the knowledge that all types of AI use are unauthorised unless specifically listed in assessment instructions. Cases of suspected unauthorised use of AI in assessment are covered by the University’s student conduct regulations. You should make yourself familiar with these regulations, as any actions that are found potentially to be in breach of them will be reviewed in line with the University’s Code of Discipline and Academic Disciplinary procedure. You should always follow the guidance of your tutors and/or supervisors, and of your department or faculty. Use in research All research undertaken by academic staff and students, including by postgraduate students, must meet the expectations in the Policy for using Generative AI in Research: guidelines for researchers and professional staff. Substantive use of GenAI should be declared whenever a stand-alone AI tool is used (such as ChatGPT Edu), but not where GenAI functionality is embedded within existing software. Substantive use of GenAI by students who are conducting research as part of a graduate research programme is defined as: - interpreting and analysing data (including audio and image files) and texts, - undertaking a literature review or translation, - identifying research gaps, - formulating research aims, - developing hypotheses, - assisting with generating ideas or to develop one’s own thinking, - generating code and synthetic data, - undertaking transcription of interviews, meetings etc. to save time and effort rather than overcoming barriers (see exclusions below) - producing documents using other people’s work or from transcripts or recordings. Substantive use may exclude using GenAI for tasks such as assisting you with translation if you are a non-native speaker, transforming transcribed spoken language into written language if you face barriers to writing, formatting documents, or improving the standard of your English or of a foreign language. As with assessment, you should always follow the guidance of your tutors, supervisors, and of your department or faculty. Use of GenAI in research falls within the scope of research conduct and the permitted use of AI as outlined abov. Actions that are found to be in potential breach will be reviewed in line with the University's Code of practice and procedure on academic integrity in research. Your health and wellbeing Because of the way that GenAI tools work, they are not a replacement for human interaction and are not equipped to offer therapy or mental health support. You should be aware that GenAI tools lack emotional nuance and clinical awareness. They can sometimes give inaccurate and potentially dangerous advice. At times of heightened distress or mental health crisis, AI chatbots may reinforce harmful thoughts through feedback loops. The University’s Student Welfare and Support Services offer a range of support with welfare and wellbeing. This includes access to Togetherall, a free and anonymous online platform where for connecting with others about what’s going on in life - big or small. Togetherall also offers free courses, resources, and anonymous chats to support your wellbeing, 24 hours a day. The SWSS also provide a free counselling service and a wealth of resources on the Oxford Students website and MyOxford app. In addition, support and advice are available from your college, department, fellow students and the Students' Union. There are contacts for emergency (including out of hours) and non-emergency services for health, welfare and academic support. All student welfare services remain open throughout the vacations (except Bank Holiday Mondays and the Christmas closure period), with some adjusted opening hours (listed on each service's page) and vacation welfare support page. Using GenAI to support your studies Part of what a university education teaches is academic skills such as assimilating information, constructing an evidence-based argument, and expressing your thoughts in clear, coherent prose. AI tools cannot replace human critical thinking or the development of scholarly, evidence-based arguments and the subject knowledge that form the basis of your university education. You should always cross-check AI generated outputs against established sources to verify accuracy and identify erroneous information. You may make use of University-supported generative AI tools (e.g. ChatGPT Edu, Google Gemini, Notebook LM and Copilot Chat) to develop your academic skills and to support your studies. This should be done in consultation with your tutors, faculty, or department, and you should always follow their advice in relation to how they expect AI tools to be used (or not used) for different tasks. These tools are accessed via your University Single Sign-On (SSO) account. Your ongoing critical appraisal of GenAI outputs, by reviewing them critically for accuracy and relevance, will maximise their potential to support you in your studies. Academic writing and presentation skills Depending on your academic discipline, GenAI tools can be useful in developing your academic writing skills and providing initial feedback on them, translating between different styles, and critiquing your own writing. They cannot replace the need for you to develop such skills through tutorials or supervisions, and independent learning, however. Depending on your academic discipline, GenAI tools also may be used to support your academic reading, but there is a risk that they could undermine the development of critical academic skills (e.g. if you use a GenAI tool to summarise an article for you, rather than fully engaging with the literature or undertaking the task yourself). You should always remain alert to the limitations of AI-generated outputs. Here, again, the subject-specific guidance of your tutors, supervisors, and faculty or department is crucial, because appropriate use of AI to support academic reading varies across different academic disciplines. Appropriate use of GenAI tools to support your academic writing and presentation skills varies across academic disciplines. Always follow any advice and guidance of your tutors or supervisors, department/faculty, or college, on what is appropriate in your subject area. Supporting the learning process Generative AI tools may be useful in supporting your academic studies, but be sure to discuss AI outputs with academic staff to confirm your understanding and to help verify them against established sources, to ensure their accuracy. Appropriate use of GenAI tools to support the learning process varies across different academic disciplines. Always follow any advice and guidance of your tutors or supervisors, and of your department or faculty, and/or college, on what is appropriate in your subject area. Tips for using GenAI tools effectively The University provides you with access to secure, enterprise-level ChatGPT Edu, Google Gemini, Notebook LM and Copilot Chat tools. Different GenAI tools can be used for different purposes. Here are some examples of key uses for some of the secure tools the University supports: - ChatGPT Edu – Advanced content generation, summarising information and complex reasoning - Microsoft Copilot Chat – Web-grounded chat, summarising information, drafting content and web-based information retrieval - Google Gemini – AI assistance that is integrated with Google Workspace, or can be used as a standalone chat tool - Notebook LM – An AI assistant that can interact with and summarise lecture notes, papers and other uploaded sources to aid research and study. You may find it useful to try a few different GenAI tools and you should be aware that different tools will give different outputs to one another, from the same prompts. Within a single tool you may also get different outputs in response to the same prompt. It is important to be aware that: - You will get different responses using the same prompts from the same GenAI tool. AI outputs are not repeatable, and all tools can generate outputs that contain inaccuracies and fabrications. - You could spend a lot of time trying out different AI tools. Be careful to balance your exploration of GenAI with managing your time effectively. - GenAI tools may draw on data that can be months or years out of date and, whilst outputs seem plausible, they may contain errors and/or reflect biases from the original data the tool was trained on. For example, Western perspectives are overly represented. - GenAI tools do not replace the need for you to develop your own knowledge, skills, and critical awareness, as an independent learner. - Take care when inputting material into any third-party tools that are not provided by the University. These may not meet the University’s standards of information security and data protection. Never upload confidential, sensitive, or unpublished material into third-party AI tools. Help and technical support with GenAI tools If you need help or technical support with using University-supported GenAI tools: - Consider first seeking support from the company whose product you're using: - ChatGPT Edu: For access and activation queries, please use the OpenAI help portal. You can use the chat at the bottom of the page to ask questions and connect with support by clicking on the Message tab. If you are unable to resolve your issue through the help portal, then you should contact OpenAI support directly by email at [email protected]. - Microsoft Copilot: The Microsoft Support site can be searched to assist with queries on Copilot. - Google Gemini: Google's Gemini Apps Help page offers various pieces of advice and support for using Gemini. - NotebookLM: Google’s NotebookLM Help page covers help topics from getting started to troubleshooting NotebookLM. - If your query is about whether an outage is affecting your connection to a particular tool, try the relevant status pages: - OpenAI Status page for ChatGPT Edu - Microsoft Status page for Microsoft Copilot - Google Status page for Google Gemini and NotebookLM - For simple queries regarding University-supported GenAI tools and support, use the AI Competency Centre chatbot to be directed to relevant information. - Contact the University's IT Service Desk if you need more support - they can help you with ChatGPT Edu, Microsoft Copilot, or the GenAI tools in the University's Google workspace (Gemini and Notebook LM). If your query needs escalating, the IT Service Desk will involve our GenAI specialists at the AI Competency Centre or signpost you to tailored support from elsewhere in the University, as needed. Find out more To find out more about using GenAI tools at Oxford, please visit the Generative AI at Oxford webpage. This guidance is under continuous review and will be updated to reflect the evolving landscape of AI use across the University. Content last updated on 22 September 2025.</t>
+          <t>Guidance on safe and responsible use of Gen AI tools The aim of this guidance is to help you use GenAI tools safely and responsibly, so you feel confident about exploring different ways of using this technology to support your learning. Generative Artificial Intelligence (GenAI) is a fast-evolving technology and, during your time at Oxford, the University wants to enable and support the safe and productive use of these tools that will be important in your future. Ethical use GenAI tools must be used responsibly and ethically, in accordance with the academic standards of rigour and integrity that are expected of you as a student at Oxford. You should always use AI tools with integrity, honesty, and transparency, and maintain a critical approach to using any output generated by these tools. This document contains some useful tips for using GenAI to support your studies at Oxford. You should always follow the advice and guidance of your tutors and/or supervisors, and consult your department or faculty in relation to ethical use. Assessment For each specific assessment you will be given prior written notice of whether or not the use of AI is permitted. You are fully responsible for the accuracy, originality, and quality of work you submit for assessment, and you must follow the rules on AI use for each specific assessment you are taking. You must make a formal declaration of any permitted AI-use in the format prescribed by your assessment setter. Any unauthorised use of AI in work submitted for assessment constitutes cheating and plagiarism under University rules, penalties for which include failing the relevant assessment and, in appropriate cases, expulsion. Any use of AI in work submitted for assessment is unauthorised unless you are specifically told differently in writing, in advance of the assessment, in instructions from your faculty’s or department for the specific assessment in question. Even if a type of AI use has been authorised for a previous assessment, or for formative work, it is your responsibility to ensure that you comply with the rules on AI use for the specific assessment you are taking, in the knowledge that all types of AI use are unauthorised unless specifically listed in assessment instructions. Cases of suspected unauthorised use of AI in assessment are covered by the University’s student conduct regulations. You should make yourself familiar with these regulations, as any actions that are found potentially to be in breach of them will be reviewed in line with the University’s Code of Discipline and Academic Disciplinary procedure. You should always follow the guidance of your tutors and/or supervisors, and of your department or faculty. Use in research All research undertaken by academic staff and students, including by postgraduate students, must meet the expectations in the Policy for using Generative AI in Research: guidelines for researchers and professional staff. Substantive use of GenAI should be declared whenever a stand-alone AI tool is used (such as ChatGPT Edu), but not where GenAI functionality is embedded within existing software. Substantive use of GenAI by students who are conducting research as part of a graduate research programme is defined as: - interpreting and analysing data (including audio and image files) and texts, - undertaking a literature review or translation, - identifying research gaps, - formulating research aims, - developing hypotheses, - assisting with generating ideas or to develop one’s own thinking, - generating code and synthetic data, - undertaking transcription of interviews, meetings etc. to save time and effort rather than overcoming barriers (see exclusions below) - producing documents using other people’s work or from transcripts or recordings. Substantive use may exclude using GenAI for tasks such as assisting you with translation if you are a non-native speaker, transforming transcribed spoken language into written language if you face barriers to writing, formatting documents, or improving the standard of your English or of a foreign language. As with assessment, you should always follow the guidance of your tutors, supervisors, and of your department or faculty. Use of GenAI in research falls within the scope of research conduct and the permitted use of AI as outlined abov. Actions that are found to be in potential breach will be reviewed in line with the University's Code of practice and procedure on academic integrity in research. Your health and wellbeing Because of the way that GenAI tools work, they are not a replacement for human interaction and are not equipped to offer therapy or mental health support. You should be aware that GenAI tools lack emotional nuance and clinical awareness. They can sometimes give inaccurate and potentially dangerous advice. At times of heightened distress or mental health crisis, AI chatbots may reinforce harmful thoughts through feedback loops. The University’s Student Welfare and Support Services offer a range of support with welfare and wellbeing. This includes access to Togetherall, a free and anonymous online platform where for connecting with others about what’s going on in life - big or small. Togetherall also offers free courses, resources, and anonymous chats to support your wellbeing, 24 hours a day. The SWSS also provide a free counselling service and a wealth of resources on the Oxford Students website and MyOxford app. In addition, support and advice are available from your college, department, fellow students and the Students' Union. There are contacts for emergency (including out of hours) and non-emergency services for health, welfare and academic support. All student welfare services remain open throughout the vacations (except Bank Holiday Mondays and the Christmas closure period), with some adjusted opening hours (listed on each service's page) and vacation welfare support page. Using GenAI to support your studies Part of what a university education teaches is academic skills such as assimilating information, constructing an evidence-based argument, and expressing your thoughts in clear, coherent prose. AI tools cannot replace human critical thinking or the development of scholarly, evidence-based arguments and the subject knowledge that form the basis of your university education. You should always cross-check AI generated outputs against established sources to verify accuracy and identify erroneous information. You may make use of University-supported generative AI tools (e.g. ChatGPT Edu, Google Gemini, Notebook LM and Copilot Chat) to develop your academic skills and to support your studies. This should be done in consultation with your tutors, faculty, or department, and you should always follow their advice in relation to how they expect AI tools to be used (or not used) for different tasks. These tools are accessed via your University Single Sign-On (SSO) account. Your ongoing critical appraisal of GenAI outputs, by reviewing them critically for accuracy and relevance, will maximise their potential to support you in your studies. Academic writing and presentation skills Depending on your academic discipline, GenAI tools can be useful in developing your academic writing skills and providing initial feedback on them, translating between different styles, and critiquing your own writing. They cannot replace the need for you to develop such skills through tutorials or supervisions, and independent learning, however. Depending on your academic discipline, GenAI tools also may be used to support your academic reading, but there is a risk that they could undermine the development of critical academic skills (e.g. if you use a GenAI tool to summarise an article for you, rather than fully engaging with the literature or undertaking the task yourself). You should always remain alert to the limitations of AI-generated outputs. Here, again, the subject-specific guidance of your tutors, supervisors, and faculty or department is crucial, because appropriate use of AI to support academic reading varies across different academic disciplines. Appropriate use of GenAI tools to support your academic writing and presentation skills varies across academic disciplines. Always follow any advice and guidance of your tutors or supervisors, department/faculty, or college, on what is appropriate in your subject area. Supporting the learning process Generative AI tools may be useful in supporting your academic studies, but be sure to discuss AI outputs with academic staff to confirm your understanding and to help verify them against established sources, to ensure their accuracy. Appropriate use of GenAI tools to support the learning process varies across different academic disciplines. Always follow any advice and guidance of your tutors or supervisors, and of your department or faculty, and/or college, on what is appropriate in your subject area. Use in careers The development of AI tools is moving at an incredibly fast pace and, in some cases, introducing significant changes to the way we live our personal and professional lives. Therefore, being aware of how the use of AI can intersect with the job application and assessment process is important. Whilst employers look for tech-literate graduates, they often have different perspectives on the use of AI in their application or assessment processes. To find out more information explore the guidance from Oxford University Careers Service. Tips for using GenAI tools effectively The University provides you with access to secure, enterprise-level ChatGPT Edu, Google Gemini, Notebook LM and Copilot Chat tools. Different GenAI tools can be used for different purposes. Here are some examples of key uses for some of the secure tools the University supports: - ChatGPT Edu – Advanced content generation, summarising information and complex reasoning - Microsoft Copilot Chat – Web-grounded chat, summarising information, drafting content and web-based information retrieval - Google Gemini – AI assistance that is integrated with Google Workspace, or can be used as a standalone chat tool - Notebook LM – An AI assistant that can interact with and summarise lecture notes, papers and other uploaded sources to aid research and study. You may find it useful to try a few different GenAI tools and you should be aware that different tools will give different outputs to one another, from the same prompts. Within a single tool you may also get different outputs in response to the same prompt. It is important to be aware that: - You will get different responses using the same prompts from the same GenAI tool. AI outputs are not repeatable, and all tools can generate outputs that contain inaccuracies and fabrications. - You could spend a lot of time trying out different AI tools. Be careful to balance your exploration of GenAI with managing your time effectively. - GenAI tools may draw on data that can be months or years out of date and, whilst outputs seem plausible, they may contain errors and/or reflect biases from the original data the tool was trained on. For example, Western perspectives are overly represented. - GenAI tools do not replace the need for you to develop your own knowledge, skills, and critical awareness, as an independent learner. - Take care when inputting material into any third-party tools that are not provided by the University. These may not meet the University’s standards of information security and data protection. Never upload confidential, sensitive, or unpublished material into third-party AI tools. Help and technical support with GenAI tools If you need help or technical support with using University-supported GenAI tools: - Consider first seeking support from the company whose product you're using: - ChatGPT Edu: For access and activation queries, please use the OpenAI help portal. You can use the chat at the bottom of the page to ask questions and connect with support by clicking on the Message tab. If you are unable to resolve your issue through the help portal, then you should contact OpenAI support directly by email at [email protected]. - Microsoft Copilot: The Microsoft Support site can be searched to assist with queries on Copilot. - Google Gemini: Google's Gemini Apps Help page offers various pieces of advice and support for using Gemini. - NotebookLM: Google’s NotebookLM Help page covers help topics from getting started to troubleshooting NotebookLM. - If your query is about whether an outage is affecting your connection to a particular tool, try the relevant status pages: - OpenAI Status page for ChatGPT Edu - Microsoft Status page for Microsoft Copilot - Google Status page for Google Gemini and NotebookLM - For simple queries regarding University-supported GenAI tools and support, use the AI Competency Centre chatbot to be directed to relevant information. - Contact the University's IT Service Desk if you need more support - they can help you with ChatGPT Edu, Microsoft Copilot, or the GenAI tools in the University's Google workspace (Gemini and Notebook LM). If your query needs escalating, the IT Service Desk will involve our GenAI specialists at the AI Competency Centre or signpost you to tailored support from elsewhere in the University, as needed. Find out more To find out more about using GenAI tools at Oxford, please visit the Generative AI at Oxford webpage. This guidance is under continuous review and will be updated to reflect the evolving landscape of AI use across the University. Content last updated on 22 September 2025.</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2045</v>
+        <v>2132</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -486,7 +486,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ERROR: The request could not be satisfied 403 ERROR The request could not be satisfied. Request blocked. We can't connect to the server for this app or website at this time. There might be too much traffic or a configuration error. Try again later, or contact the app or website owner. If you provide content to customers through CloudFront, you can find steps to troubleshoot and help prevent this error by reviewing the CloudFront documentation. Generated by cloudfront (CloudFront) Request ID: TdBswHUJAjAV1a5QIKlMeCkrlK2e1wGk5X-OUVCkHVV1ySNFcsRdFw==</t>
+          <t>ERROR: The request could not be satisfied 403 ERROR The request could not be satisfied. Request blocked. We can't connect to the server for this app or website at this time. There might be too much traffic or a configuration error. Try again later, or contact the app or website owner. If you provide content to customers through CloudFront, you can find steps to troubleshoot and help prevent this error by reviewing the CloudFront documentation. Generated by cloudfront (CloudFront) Request ID: LpHcOPd1AzBVm1_ESxzBgQeTYAW8TmLqUx4xdZCjjKxZOKxa6mBSbw==</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -936,7 +936,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -966,7 +966,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1073,11 +1073,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>As generative AI (GenAI) tools and platforms continue to expand and evolve, it is important to provide the UBC community with guidance and advice related to their opportunities as well as risks and challenges. Download: Principles and Guidelines for Generative Artificial Intelligence (GenAI) in Teaching and Learning GenAI tools are artificial intelligence systems that can generate content – such as texts, images, audio, and video – in response to prompts by a user, after being trained on an earlier set of data (from Glossary of GenAI terms). Some GenAI tools are accessed through standalone platforms (e.g., ChatGPT), while others may be embedded in other applications or platforms (e.g., Grammarly). GenAI has the potential to enrich teaching and learning activities, and some may also support inclusion and enhance accessibility, depending on how they are used. Learning how to responsibly use GenAI is important for all members of the UBC community given its growing presence in many academic and work environments. However, such tools can and have been used in ways that are harmful to individuals and communities, and careful attention must be paid to topics such as academic integrity, accessibility, equity, Indigenous data sovereignty, and privacy and intellectual property. The following principles and guidelines have been developed through discussions with a Generative AI in Teaching and Learning Advisory Committee during the 2023-2024 academic year, and through multiple consultations with various individuals and groups at UBC. They provide guidance on responsible and ethical use of GenAI in teaching and learning at UBC, balancing both opportunities and risks. These guidelines are designed to adhere to and support UBC’s strategic plans and commitments, and to align with existing UBC policies, procedures, and legal requirements (linked where relevant below). They also support and build upon the UBC Principles for Use of Generative AI. This is meant to be a living document, evolving as needed in a rapidly-changing landscape around GenAI in teaching and learning. For feedback or questions, please contact provost.vptl@ubc.ca. Principles The following broad principles around GenAI in teaching and learning at UBC serve as a foundation for the more specific guidelines that follow. Download: Principles For GenAI in Teaching &amp; Learning Alignment to Our Values and Priorities UBC strategic plans and commitments Use of GenAI in teaching and learning should be aligned with and support UBC strategic plans and commitments, including those related to decolonization and Indigenous human rights, equity, accessibility, sustainability, and wellness. Opportunities to enhance education GenAI can provide significant value in both teaching and learning activities through informed, responsible, and ethical use that mitigates risks and potential harms. Value for students’ future endeavours It is important for students to learn how to use GenAI effectively and responsibly, to prepare them for further work or studies when they leave UBC. Indigenous data sovereignty Use of GenAI should respect Indigenous data sovereignty and community protocols for use and sharing of Indigenous knowledges, intellectual properties, and data. Harm from false information about Indigenous communities, cultures, knowledges, histories, and contexts should be avoided. Academic integrity All uses of GenAI at UBC must uphold academic integrity and adhere to the academic misconduct regulations in the UBC Okanagan and Vancouver calendars. Building Capacity and Literacy GenAI literacy UBC will continue to provide opportunities to learn about capabilities and limitations of GenAI tools. Faculty, staff, and students should use those opportunities to develop basic GenAI literacy skills over time. Faculty and staff use of GenAI Faculty and staff may use GenAI in teaching and learning so long as this is within the bounds of legal, university, Faculty, or program-level policies and requirements, and the guidelines below. Student use of GenAI Students may use GenAI in work submitted for courses or other academic requirements only if expressly permitted within their courses or programs. They may choose to use GenAI to support their learning in other ways, within the bounds of legal and university policies and requirements, and the guidelines below. Considerations Accessibility Some GenAI tools can enhance accessibility for learners with a range of disabilities. It is important to also recognize, however, that there may be varying levels of accessibility to GenAI tools, whether related to cost, inaccessible infrastructure (such as websites or applications), or for other reasons. Those using GenAI in teaching and learning should ensure equitable access to the best of their ability. Intellectual property &amp; copyright Those using GenAI in teaching and learning should respect intellectual property rights in material they input into the tools, and in how they use outputs. Privacy &amp; confidentiality Use of GenAI in teaching and learning should protect privacy and confidentiality of personal and other sensitive information. Personal Responsibility Equity Biased training data and inputs can produce biased, discriminatory, inaccurate, or otherwise harmful outputs, with the potential to perpetuate systemic inequities. Those using GenAI in academic work should assess the risks and mitigate, to the best of their ability, the harmful effects of such bias. Human oversight and critical thinking All outputs of GenAI for teaching and learning purposes should undergo human review before sharing. Users should think critically about outputs from GenAI, including their potential for producing false or misleading information, especially if sources of information in the outputs cannot be identified and/or verified. Transparency Use of GenAI to produce text, images, videos, or other materials shared with others for teaching or learning purposes should be acknowledged by attributing the source of those materials. Responsibility Users of GenAI are accountable for the consequences of sharing the outputs generated with these tools, and have a responsibility to review them for inaccuracy and potential harm to the best of their ability. The university will provide resources to help individuals develop requisite skills.</t>
+          <t>As generative AI (GenAI) tools and platforms continue to expand and evolve, it is important to provide the UBC community with guidance and advice related to their opportunities as well as risks and challenges. Download: Principles and Guidelines for Generative Artificial Intelligence (GenAI) in Teaching and Learning GenAI tools are artificial intelligence systems that can generate content – such as texts, images, audio, and video – in response to prompts by a user, after being trained on an earlier set of data (from Glossary of GenAI terms). Some GenAI tools are accessed through standalone platforms (e.g., ChatGPT), while others may be embedded in other applications or platforms (e.g., Grammarly). GenAI has the potential to enrich teaching and learning activities, and some may also support inclusion and enhance accessibility, depending on how they are used. Learning how to responsibly use GenAI is important for all members of the UBC community given its growing presence in many academic and work environments. However, such tools can and have been used in ways that are harmful to individuals and communities, and careful attention must be paid to topics such as academic integrity, accessibility, equity, Indigenous data sovereignty, and privacy and intellectual property. The following principles and guidelines have been developed through discussions with a Generative AI in Teaching and Learning Advisory Committee during the 2023-2024 academic year, and through multiple consultations with various individuals and groups at UBC. They provide guidance on responsible and ethical use of GenAI in teaching and learning at UBC, balancing both opportunities and risks. These guidelines are designed to adhere to and support UBC’s strategic plans and commitments, and to align with existing UBC policies, procedures, and legal requirements (linked where relevant below). They also support and build upon the UBC Principles for Use of Generative AI. This is meant to be a living document, evolving as needed in a rapidly-changing landscape around GenAI in teaching and learning. For feedback or questions, please contact provost.vptl@ubc.ca. Principles The following broad principles around GenAI in teaching and learning at UBC serve as a foundation for the more specific guidelines that follow. - UBC strategic plans and commitments: Use of GenAI in teaching and learning should be aligned with and support UBC strategic plans and commitments, including those related to decolonization and Indigenous human rights, equity, accessibility, sustainability, and wellness. - Opportunities to enhance education: GenAI can provide significant value in both teaching and learning activities through informed, responsible, and ethical use that mitigates risks and potential harms. - Value for students’ future endeavours: It is important for students to learn how to use GenAI effectively and responsibly, to prepare them for further work or studies when they leave UBC. - GenAI literacy: UBC will continue to provide opportunities to learn about capabilities and limitations of GenAI tools. Faculty, staff, and students should use those opportunities to develop basic GenAI literacy skills over time. - Faculty and staff use of GenAI: Faculty and staff may use GenAI in teaching and learning so long as this is within the bounds of legal, university, Faculty, or program-level policies and requirements, and the guidelines below. - Student use of GenAI: Students are encouraged to explore GenAI tools to support their personal learning and academic development. For assessed work (assignments, exams, projects, theses, etc.), students may only use GenAI if expressly permitted by their instructor, supervisor, or program. Instructors set the conditions for GenAI use in submitted assessed academic work, including when and how its use must be acknowledged. - Academic integrity: All uses of GenAI at UBC must uphold academic integrity and adhere to the academic misconduct regulations in the UBC Okanagan and Vancouver calendars. - Indigenous data sovereignty: Use of GenAI should respect Indigenous data sovereignty and community protocols for use and sharing of Indigenous knowledges, intellectual properties, and data. Harm from false information about Indigenous communities, cultures, knowledges, histories, and contexts should be avoided. - Equity: Biased training data and inputs can produce biased, discriminatory, inaccurate, or otherwise harmful outputs, with the potential to perpetuate systemic inequities. Those using GenAI in academic work should assess the risks and mitigate, to the best of their ability, the harmful effects of such bias. - Accessibility: Some GenAI tools can enhance accessibility for learners with a range of disabilities. It is important to also recognize, however, that there may be varying levels of accessibility to GenAI tools, whether related to cost, inaccessible infrastructure (such as websites or applications), or for other reasons. Those using GenAI in teaching and learning should ensure equitable access to the best of their ability. - Intellectual property &amp; copyright: Those using GenAI in teaching and learning should respect intellectual property rights in material they input into the tools, and in how they use outputs. - Privacy &amp; confidentiality: Use of GenAI in teaching and learning should protect privacy and confidentiality of personal and other sensitive information. - Human oversight and critical thinking: All outputs of GenAI for teaching and learning purposes should undergo human review before sharing. Users should think critically about outputs from GenAI, including their potential for producing false or misleading information, especially if sources of information in the outputs cannot be identified and/or verified. - Transparency: Use of GenAI to produce text, images, videos, or other materials shared with others for teaching or learning purposes should be acknowledged by attributing the source of those materials. - Responsibility: Users of GenAI are accountable for the consequences of sharing the outputs generated with these tools, and have a responsibility to review them for inaccuracy and potential harm to the best of their ability. The university will continue to develop resources to help individuals develop requisite skills.</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>941</v>
+        <v>946</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1163,20 +1163,20 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>The Sedona Conference Journal Volume 26 Forthcoming 2025 Navigating AI in the Judiciary: New Guidelines for Judges and Their Chambers Hon. Herbert B. Dixon Jr., Hon. Allison H. Goddard, Maura R. Grossman, Hon. Xavier Rodriguez, Hon. Scott U. Schlegel &amp; Hon. Samuel A. Thumma February 2025 Recommended Citation: Hon. Herbert B. Dixon Jr. et al., Navigating AI in the Judiciary: New Guidelines for Judges and Their Chambers, 26 SEDONA CONF. J. 1 (forthcoming 2025), https://thesedonaconference.org/sites/default/files/publications/Navigating% 20AI%20in%20the%20Judiciary_PDF_021925.pdf. Copyright 2025, The Sedona Conference For this and additional publications see: https://thesedonaconference.org/publications. THE SEDONA CONFERENCE JOURNAL 2/24/2025 11:17 AM NAVIGATING AI IN THE JUDICIARY: NEW GUIDELINES FOR JUDGES AND THEIR CHAMBERS Hon. Herbert B. Dixon, Jr., Hon. Allison H. Goddard, Prof. Maura R. Grossman, Hon. Xavier Rodriguez, Hon. Scott U. Schlegel, and Hon. Samuel A. Thumma Five judges and a lawyer/computer science professor walked into a bar . . . well, not exactly. But they did collaborate as members of the Working Group on AI and the Courts as part of the ABA’s Task Force on Law and Artificial Intelligence to develop the following guidelines for responsible use of AI by judicial officers. The guidelines reflect the consensus view of these Working Group members only, and not the views of the ABA, its Law and AI Task Force, The Sedona Conference, or any other organizations with which the authors may be affiliated. The authors include: • Dr. Maura R. Grossman, a Research Professor in the Cheriton School of Computer Science at the University of Waterloo and an Adjunct Profes- sor at Osgoode Hall Law School of York Univer- sity, who serves as a special master in both U.S. state and federal court; • Hon. Herbert B. Dixon, Jr., Senior Judge of the Superior Court of the District of Columbia; • Hon. Allison H. Goddard, U.S. Magistrate Judge of the U.S. District Court for the Southern Dis- trict of California; • Hon. Xavier Rodriguez, U.S. District Judge of the U.S. District Court for the Western District of Texas; NAVIGATING AI IN THE JUDICIARY: NEW GUIDELINES 2/24/2025 11:59 AM 2 THE SEDONA CONFERENCE JOURNAL [Vol. 26 • Hon. Scott U. Schlegel, Judge of the Louisiana Fifth Circuit Court of Appeal; and • Hon. Samuel A. Thumma, Judge of the Arizona Court of Appeal, Division One. We hope you will find these guidelines useful in your work as judges. They provide a framework for how you can use AI and Generative AI responsibly as judicial officers. THE SEDONA CONFERENCE JOURNAL 2/24/2025 11:17 AM 2025] NAVIGATING AI IN THE JUDICIARY 3 Guidelines for U.S. Judicial Officers Regarding the Responsible Use of Artificial Intelligence These Guidelines are intended to provide general, non-tech- nical advice about the use of artificial intelligence (AI) and gen- erative artificial intelligence (GenAI) by judicial officers and those with whom they work in state and federal courts in the United States. As used here, AI describes computer systems that perform tasks normally requiring human intelligence, often us- ing machine-learning techniques for classification or prediction. GenAI is a subset of AI that, in response to a prompt (i.e., query), generates new content, which can include text, images, sound, or video. While the primary impetus and focus of these Guide- lines is GenAI, many of the use cases that are described below may involve either AI or GenAI, or both. These Guidelines are neither intended to be exhaustive nor the final word on this sub- ject. I. FUNDAMENTAL PRINCIPLES An independent, competent, impartial, and ethical judiciary is indispensable to justice in our society. This foundational prin- ciple recognizes that judicial authority is vested solely in judicial officers, not in AI systems. While technological advances offer new tools to assist the judiciary, judicial officers must remain faithful to their core obligations of maintaining professional competence, upholding the rule of law, promoting justice, and adhering to applicable Canons of Judicial Conduct. In this rapidly evolving landscape, judicial officers and those with whom they work must ensure that any use of AI strength- ens rather than compromises the independence, integrity, and impartiality of the judiciary. Judicial officers must maintain im- partiality and an open mind to ensure public confidence in the justice system. The use of AI or GenAI tools must enhance, not diminish, this essential obligation. NAVIGATING AI IN THE JUDICIARY: NEW GUIDELINES 2/24/2025 11:59 AM 4 THE SEDONA CONFERENCE JOURNAL [Vol. 26 Although AI and GenAI can serve as valuable aids in per- forming certain judicial functions, judges remain solely respon- sible for their decisions and must maintain proficiency in under- standing and appropriately using these tools. This includes recognizing that when judicial officers obtain information, anal- ysis, or advice from AI or GenAI tools, they risk relying on ex- trajudicial information and influences that the parties have not had an opportunity to address or rebut. The promise of GenAI to increase productivity and advance the administration of justice must be balanced against these core principles. An overreliance on AI or GenAI undermines the es- sential human judgment that lies at the heart of judicial deci- sion-making. As technology continues to advance, judicial offic- ers must remain vigilant in ensuring that AI serves as a tool to enhance, not replace, their fundamental judicial responsibilities. Judicial officers and those with whom they work should be aware that GenAI tools do not generate responses like tradi- tional search engines. GenAI tools generate content using com- plex algorithms, based on the prompt they receive and the data on which the GenAI tool was trained. The response may not be the most correct or accurate answer. Further, GenAI tools do not engage in the traditional reasoning process used by judicial of- ficers. And, GenAI does not exercise judgment or discretion, which are two core components of judicial decision-making. Us- ers of GenAI tools should be cognizant of such limitations. Users must exercise vigilance to avoid becoming “anchored” to the AI’s response, sometimes called “automation bias,” where humans trust AI responses as correct without validating their results. Similarly, users of AI need to account for confirmation bias, where a human accepts the AI results because they appear to be consistent with the beliefs and opinions the user already has. Users also need to be aware that, under local rules, they THE SEDONA CONFERENCE JOURNAL 2/24/2025 11:17 AM 2025] NAVIGATING AI IN THE JUDICIARY 5 may be obligated to disclose the use of AI or GenAI tools, con- sistent with their obligation to avoid ex parte communication. Ultimately, judicial officers are responsible for any orders, opinions, or other materials which are produced in their name. Accordingly, any such work product must always be verified for accuracy when AI or GenAI is used. II. JUDICIAL OFFICERS SHOULD REMAIN COGNIZANT OF THE CAPABILITIES AND LIMITATIONS OF AI AND GENAI GenAI tools may use prompts and information provided to them to further train their model, and their developers may sell or otherwise disclose information to third parties. Accordingly, confidential or personally identifiable information (PII), health data, or other privileged or confidential information should not be used in any prompts or queries unless the user is reasonably confident that the GenAI tool being employed ensures that in- formation will be treated in a privileged or confidential manner. For all GenAI tools, users should pay attention to the tools’ set- tings, considering whether there may be good reason to retain, or to disable or delete, the prompt history after each session. Particularly when used as an aid to determine pretrial re- lease decisions, consequences following a criminal conviction, and other significant events, how the AI or GenAI tool has been trained and tested for validity, reliability, and potential bias is critically important. Users of AI or GenAI tools for these forego- ing purposes should exercise great caution. Other limitations or concerns include: • The quality of a GenAI response will often de- pend on the quality of the prompt provided. Even responses to the same prompt can vary on different occasions. • GenAI tools may be trained on information gathered from the Internet generally, or NAVIGATING AI IN THE JUDICIARY: NEW GUIDELINES 2/24/2025 11:59 AM 6 THE SEDONA CONFERENCE JOURNAL [Vol. 26 proprietary databases, and are not always trained on non-copyrighted or authoritative le- gal sources. • The terms of service for any GenAI tool used should always be reviewed for confidentiality, privacy, and security considerations. GenAI tools may provide incorrect or misleading infor- mation (commonly referred to as “hallucinations”). Accord- ingly, the accuracy of any responses must always be verified by a human. III. POTENTIAL JUDICIAL USES FOR AI OR GENAI Subject to the considerations set forth above: • AI and GenAI tools may be used to conduct le- gal research, provided that the tool was trained on a comprehensive collection of reputable le- gal authorities and the user bears in mind that GenAI tools can make errors; • GenAI tools may be used to assist in drafting routine administrative orders; • GenAI tools may be used to search and sum- marize depositions, exhibits, briefs, motions, and pleadings; • GenAI tools may be used to create timelines of relevant events; • AI and GenAI tools may be used for editing, proofreading, or checking spelling and gram- mar in draft opinions; • GenAI tools may be used to assist in determin- ing whether filings submitted by the parties have misstated the law or omitted relevant le- gal authority; THE SEDONA CONFERENCE JOURNAL 2/24/2025 11:17 AM 2025] NAVIGATING AI IN THE JUDICIARY 7 • GenAI tools may be used to generate standard court notices and communications; • AI and GenAI tools may be used for court scheduling and calendar management; • AI and GenAI tools may be used for time and workload studies; • GenAI tools may be used to create unoffi- cial/preliminary, real-time transcriptions; • GenAI tools may be used for unofficial/prelim- inary translation of foreign-language docu- ments; • AI tools may be used to analyze court opera- tional data, routine administrative workflows, and to identify efficiency improvements; • AI tools may be used for document organiza- tion and management; • AI and Gen AI tools may be used to enhance court accessibility services, including assisting self-represented litigants. IV. IMPLEMENTATION These Guidelines should be reviewed and updated regularly to reflect technological advances, emerging best practices in AI and GenAI usage within the judiciary, and improvements in AI and GenAI validity and reliability. As of February 2025, no known GenAI tools have fully resolved the hallucination prob- lem, i.e., the tendency to generate plausible-sounding but false or inaccurate information. While some tools perform better than others, human verification of all AI and GenAI outputs remains essential for all judicial use cases.</t>
+          <t>%PDF-1.7 %���� 284 0 obj &lt; &gt;stream h�222W0P���w,-��/�p.J�LW�S��/JO���w.JM,���sI,I�p�22025022144�42�50W70P��j��L.�/�O+Y��_����_�S063����OA5����0��P��R��J�avv�:� endstream endobj 285 0 obj &lt; &gt;stream h��Yko[7�+�c�E &gt;gH�0��u�E��&amp;Φ� ~Pc�#�� Y���� �T?;I�X42y� Μ93dCv�B���_R@��P�!���C*�݂�g����Jrp�\��]�\"?H��.a� �?;\^]�ϯ��O���Ű�|\ ��Q�׃w�e��lN�������b�]n����^�-����'�N׿-����xyy��@��0���{~x�������v�V���_�\,�&gt;l�2;\��OC ������ ���j������S�κ�|��� �/���O�9?�o�����l�/!��.�8v�![~�_,f��&lt;�����v�vs��^_�W6��v�ؾ�0�y����[ӻ.krnv���/�?[�A]n�f����P��k�P�e��ܮ7�_�#&amp;)�����&lt;"Uu}���W�YLcǇ'� �_�/g;��A ����y��7�˹ A� ��ލn�Q0T�:�2�����z�z�T�@Ũ��A�X_M�v�/�v��B�e�G[OCh ������� ]b�4�&lt;)۞�`����}L &amp;�%�C0&lt;�4�F� bb�%�����+e�ل�+��Le���Z �ڻ�������!�w��o kz �6�B�����Ǌ&lt;��i�˙R�+%Ó2��RWh�jJ�b3d ��}�^ 8�s�|(�! �}* rfh�p��k ��P ����S!М� �8��? �@�汇�]O���J����C7�i�ϕ2��ﺬޏ9� : Ї���9�E��2���YC��[�y��sb��m!��b�� $��x.� ����IMp!�Q'$&gt;2 �B� Б�I�$(�� u̬H��4��28�GZ���S6J���@��o)���������&lt;Q�5�R3�tsC�� �@����(D��$� ���`�o��X� D �y� �Q�cr���uD�`��S��$V'����69Z���^��z��Km 2mR�B���� Q�����z��Ch��\��:w-J����T�c:2Y �7��a��֞\=�����$ء���_�':XA'��(��I�` �����|P*(A���rMj �O�%�� ��%����K�%8O*ijc �Sb���S)S{ ����8��([�7W"��{d[&amp;�D�DA�b��o�&amp;3�ɇ'��4���d�1ej�#&lt;״Ͻ�I�E3� E�ˡ �F=�8�Tm��ĮH�1�J�B;��;^����`�MF뵌�ӻ���t$��rv#-Y�R��Y7t�ə�� AY�8��c��v��&lt;�J���t�Qkq#Zh7�ͼ/����1[�U���^h-�QK�(�}'K�ф���CK� �(S�U)�X��J8&gt;v�8�Pe����pUA�$�)��&lt;2P� 5 N  ��L��#pFa��3 p,ʨ�� �1d"�c@�^���V��&amp;$?c0� �Be��&amp; �~=,*���V}���X��(,-�e���\�0��~�Vsm����I*�I�g���u�v sfvw=H)\C���c���$��3�PaK�:�����-K��[d��u�Ne#;QaVM ����� ؖ.�����6�HwA �|$�c_fE ������E5bՈ}���n�� 6` �b���K.���ݨ�`����1�*��Ƀ�)��u��=��)�n�ɡ��Xr�} �ؒ��Ԣ��� ��SJ�ѐ��ƨqJ � QS��Gj��@�@$I?)�� S9�_��E&gt;� �.��7�Ʌ�c&lt;��L������) �A �#�t� �-`ښ�D4����L����k�b��yY�L &lt;� ��0[B�j�K&amp;���a� (T�" �ATE�dq!ӎU�ހ�V`3z��� h���D��22��V�i̶yb� �C����B̯R�b_m� B�Ik�0 f�m�H�N 8��ܲ�T1��8Ŷ��$&lt; fx�sUj��2��c��R%L8�a�P��͘� f&gt;T��J�&lt;ّ�̿����x���\��w�z@��B�F��S�v-�L[�%v���/��&gt;�pD6&gt;@�1�@�ܻf&amp;�����[�y'(&lt;7pM,݃ŶEE����p$E2ڌ }cT�jO4�A��FΒ �Q�t�i a8�~�]3t[LP #J2��0*" ΀ We� =`z�:/Ť:����d�D�L�m�Z��l c�d��ߌ6`F̣_�&gt;洦���F2 �ebv5J�G;���M�eZ%s�x�6���B�&amp;&amp;�&amp;�ڟ&lt;����[�� �����l�*� �+�fn�*�� ўx��̌l9\j�i�l,���d!��p��+��0��}$o} ���B'�|�V�n��Z2t�Mm*މ��-��}�����}���c%c ��{e � �|�ި��}��6��W[���4����z�&gt;]����+O_�_P�h�f'뷫%-p��2�ǔ�^�{�� WL����� ���O\��׫� ������|}~�� �~� ���'.��O\ʰ�������j��&gt;Zn��/&gt;�7����R;�O�i���l&gt;.L��&amp;J�M��N� ��V�W�Ǭ��7oHw��A��kd{iݽ�=�V�״j��7Qs ^O� v�Ӱ�3/��6�y�����e�a�w��Bxw�%�#��s�� �wyG�;��!�v}7��j_�x˱7 n G� m�U?��/y�4�&gt;���K�� �h?!����FZ�&gt;2�!:| ����+x{��Sh�H�JH?�~��G�4�����m���aT���M������M��y�Mf���Dg��=��)o���i%��O1E�p���o�j�����w��O� endstream endobj 286 0 obj &lt; &gt;stream h�222S0P���w�/�+Q����L)�626�)BH(e �L!�9��SF`%��!������vv�� endstream endobj 287 0 obj &lt; &gt;stream hެX]o��+|l_, �yQH�[4��ng�# GM|�X�c_4���G����*-�dH���p8���*�w*�2?�gQQ��I�R�G�:2Y�"�����U�� ��) Z��!�E���K\R��Z��HJ5$���(Z�u�Tt��T�C&amp;͆j����Ϋ&gt;� |z��s S�Ť&gt;g� |.a �&lt; �t(K������� ��0�#��� �[jeJ?�F�&lt;�*��ph�RK8�4sX �Qk� ,�X,��T�0���`�p ;�x�L� ��x2�#�A`N�L0�$�CIْx�J4&lt;�4)�d�`w��F��T��pá�ۄ��Z�e 3�G��7��`��0�6_�22`���X�M��s�F��ʕ &lt;��c2 l2A��&lt;���I+g%k�� ���Y����(0;�C`��+B�y�C`�r`nLu`��1�}.��90'�&amp;|ɻ����S� �hF#1*�D8F%gRo�xO�[6.��Ux 6짟�O|�Ju^�M��rs��*&gt;d�'_��6��'lbq^/�ߧ+&gt;�&lt;��iU��z;k&amp;�����i'8K����ʔ%B K�R�,�H-�4�b�Q*Ez�2���s"e&lt;�Y?y�{�G��E��E�~#�^�w2_�R���,�Tf(�Ňz�}�K}�&gt; �UՆ����x9���Yۇ�|-�E}����W?OW���� 쭊/��Dz�Κ��2�k5�iGN�����M���z�b���ٺ���u��Y���b~S��8g����ndd{�8[�W��U��}p�S{R��nl��h7F\�7 �Iŷ%,}Q�G�������@m��vt49x�I�/�V� o�"�H� 9�&amp; i]�/��:9�:R&amp;�P}�:��J̾J! ؛C0�u�CKrf���$9$������i���f #���BV �b�&gt;+|V���Y��g�϶YM�\��R$M� "K!�� � �� � �� � �� � �� � �� Jo�զ�P��z�����T�[ܳʗ�����#��� ���|y/Ŋ�3Sy�)oY?�i�&amp;�fz�~�Y["��b^�� � ��������Mr��3@֯ʽ� �|.01���=..�׋Jh��e*w`� 2È��`ɣ?�(���x`&lt; ���M��� �@�Ph�,���v�*01ތ����Q�˯���\�i���e��&lt;}��r��Ϊ&amp;��,��� E�3.�#����(�ܺ�R `�4��[ mL��̋���I-��z� ��C������}�Q����13�?��\��P�ёt&amp;�,/�_��� �h�Өy�У���G����z&gt;J��|�FL�`o���E��܀+�ŷ�S���n�Y=��(6w�cuS/��z�g�Y5�׷ŗ��淸5-o��O���+L��m{3�ͧ� ��d޹&amp;mӈ�|�#���,32į�q�W�W���ҪV[\�f�e�QN�� �W�v�ͷ׋�7����=������3��cz!{�� ��^� =&gt;��=��GO̠4@O���C9L9$��OSCC4�^�&gt;M z�&amp;׋٧����]�Y t/k�H󽑧o⏛�=M����mOV�md����k���'=v~S����/����/�3.`x� u�+��U1�sE~�s� ��^�߁�\�߁�\�߁� ���StοQ=ނ � � �cz!���Kt?c���_���B��ڕ��s�J���U� �� �. �dz1����C4�^����_�h ��}�$ �M��Oӫ� ����N��:�N��]_ꔓ����(oԥE�K�o=W��η�w�;ߒށ�|{z��j8�� -�&lt;^�Q�3�?��o�U�&gt;� ��W{����m���� 0~{V� endstream endobj 288 0 obj &lt; &gt;stream h�26S0P06W0�T�62���� �4�f`� LZ�IKkc����_������`� RY���ZQ� \�X�����`hg`��P endstream endobj 289 0 obj &lt; &gt;stream h��Wmo�8�+����_Ǝ#�V�RZ��ݩ􎓢|HK�F�AzZ���8qHy;�]!׎=3~��x�U�q�"&amp;�f��� ��� $��bBِ0( � ��i=d�J��b �^��ES�I�C�����dRIɴ��4Ӏ�Q �Ҙ��I��;b�+͌`Jڈ�- ��+����B��A�ж3�X)�f"���Z��������[�t�]���DyS��.�d�lB�ɺ���'y��E�$�V&amp;Q1): ���0~4��HK:�x 2��s�%J �I Ҏ��h Ƅ����w�=њ�JRob�n�I�/_���%+**���O�Y����M�����k�4�j�����|�N�����G�F�5&amp;$� 5�8�� c��&amp;~O�Y0��no�3]�U^�߰U�U�W�"qr�zk�&lt;�g��|�����C��F)�&amp;U���'��T �:_U�:���}��������5䍯 }��� ���\��9W��jyG�� =�(&lt;9|�����Y�u.��\'�\v�$�w ]R9 �l�7�~D����e뼘ϐ y�� �/x�SE���R�5�J�űr�?��[q��/� ���R� �7zm��ǻ UbW��J�_���_�w�Rˑ�r���|��?�bt��bDxA��Ma�O�.B�b endstream endobj 290 0 obj &lt; &gt;stream hެW�n1 ������hE�6H�S�C���81�8��;��Z[n�(�3$%��982��S ���{9$v3I�z4d�bd�����hɕ}G�A=���� )��D�3�L1�'J �)% ��þ�5�6@��rY�YV�U1�� x���(f�`=�3���W�s��+c� 0���I(:�z��F��4]Q3 H�Qp=�����P�ՉǗ�'� �����eV �-L�� ;�g&amp;q ,8H��r��0��S�!� �S̱��9���I2��'�E�pN�b!$ .V�"�n��tg%- ]u�7� ��bu��]Ұwy���t�]t��׋���������buz ����뗷���y�x�}\��u_�b�����n��d�����7f˛8.+�ܨ/ţ$���Cb��O��+ ��o������NU�Lܹ���æ��1���$Z��D�yJ�;��J�ʡq��r�G�Ct�?�K-�&lt;���lK�n��ct�����������1n��o,YH�6��F�m�m��������}-g����Ɩ�7�&lt;�I�d���N\��b�c.f�#���E��Iy��Bf�Zz�k�)S����u�����^�4܊�v&amp;.��U_D���8FX���N�Ӑ}�/�U�X�=��E�Q/��-�z��b&amp;���w��XC�XI=� n%�s����9� s 2���J�?Y) &gt;stream h�̔�J�@�_e��ݝ� H�V�I(Mn�H��xIJ�����&amp;KUh � r����d&gt;~� � 8��V:C�� 4m�L��4#S)@ȥ��[vW�M�� k�h����mPb��2�J����6�K�EݲE����a�o(;z���q�oٓ}/Ϟ�ʖr�&gt;[��ٷ��(�Gʏd�Ϝr ΋"�.�T���F��2f3�j�*�a�V��������u����&lt;��* �;��(_:���s�)�7?�Ũ  � K��� .6�V�XƲm���Y����{���y�ٖu�����!@�"e�M���`3����!,�X�˜��/��OL*��g� u$������Ɉ�0B�� �&lt;A)��)�9��\�I�b��d�oL'i�����Q0b�`��-�F��12&amp;�*~������d'Jɸ��s�^ң��:��9O�ʣȜ��%�ퟬ� endstream endobj 292 0 obj &lt; &gt;stream h� �� �@D�z �$MH!*'���h��9�]��"��L1�7M�w��{8`����=�� _��e����j�72 )��Y �]ӵ��p�Ub�'\"�&amp;�*��(&amp;,V5,r�d�����C����R- endstream endobj 2 0 obj &lt; &gt;stream H���KO�0���w#��?�B m���YT,2mZ�"t:����qS( B��|m��;��e�^/�y ��,��b�X.`��� X��W�oS�(�E���X���^?Wpvv&gt; �M8p0B�M$lK��*r�� Vsίcb�-��b�~�2��$p�=�̑�O�v �l��H�f�՘x� ��.�Q;�h��������M6�����Fȹ�`J}��P�RA� �Z4��}c��Y��; �}�Q��y׸Ȧ�s$�C×�۞�^���$m/�=�H�1� {�?�����UoZ�0�mZ8��UA �Zwh%��y�j���}���KDG]�o����$l_��#*7e$���t�׻U]����A ��?J�|�H4p�͎��a]E �gߎn �7E��iWE���������`&lt;�g~ٴv�����֭��(e�azdB�J��iI�Z/��G�O��S��g � 0 �84 endstream endobj 3 0 obj &lt; &gt;stream H���MK1���s� 3��$ު��-Ң�O~ &lt;���-�fA����$Of�Y����L�&lt;%dQYH�B�Go��F�!��f*Ӈ蒸_B�&amp; &gt;j�~��: �� ��a ���#U���D�r6?~m"*i�z#G�#�T��K�Ss#'���t �ӼnTޣ}k^�� )=���J:ȝ�\W�4ݗ�7��jcc&lt;�(\��4V!��A&amp;������.�}#��Dt�z��B �U{���(�׷�fL��B�� 7�J�n�ǧm k��=�^W�-w���v)��� K�a���%�Y��Gۙ 6t% ����#�4�+� endstream endobj 4 0 obj &lt; &gt;stream H��SMo�@��+��Ff� ,)��Ɖ⪵�Z���ap�N?~}gwqKrH�\����7o��@�C��&lt;� A �H-{��Gk[ ���pa�Pg֧ (�Ql�㘃� �(���=�`O�}�oO��P��~ʎ�f#9F��s�]�ӛP��r!G�L����"�xINb@�; E$�|4U�-Ա&lt;���K� 4��4�� �P � �� �PU�/��| ����%%\^��rvV:�K֟�o&amp; ��j4���8 �4Ԁ6��V��D�-y�Z��=�&amp;�Ϫ��m�=�U��J]�0,�\�M' 3��ђ�4Q�:���ZW�� #���NT�D�d�]tC{� 2�)9��ԋ�4[�Ds0��N=�Ym��r�o�1�~�/��!�U�W5{��z�z(��T��Xvу�L�4� C���LK�t{�qV�!~0�mUC}$ǆ���{�=��W1�.F-�w�u�d r�?�����{T� Run fc �H �d$f�� E�Cm�WkT�N�P�V:v��n��Q7�&gt;�ʕ�c���&lt;;� ��&amp;:A[n2�^7  �AP endstream endobj 5 0 obj &lt; &gt;stream H��SMo�0 ��W�h �GI�PH���n�P���kW��m��HINmo�A�H?�# c�[| ~��eB�\K�7���k|4&gt;��@�"�R�Ź`f\�/ 4 &gt;stream H��TMo�0 ��W�( ��O�9��6l�e�� � �XnܺJf7+�_?��b ,[� ��GI�+���w��%&lt;�*�x���h��;nٍf �N8�u�Ҽ���u �)�-�)Z�GFf��(���e�&amp;5�d�� 犋n? .��EBPo%`�v�q�5 0���9�(�r�GG�0��J ,&amp;����`�8� �h� �uG�@c�������/}�BU��BX�����}3`��:W����-��$�1a���a0W ���T9+� �4[���@�5VǺ���p.~eP-�������g%��,�:w�RS跂v�\�}�� ������g } �7MR�h���4��Q^�q�_td[9��{Y/�.ǀS���5G&lt;�J��aWɞ�b�I�o�tw��������y����T��� M �&gt;�&gt;����a����C�by����n��Ҁ����m����[�,��'T�J�� �I ��A��w6�"��;���q��w1���bq�:�w`�o�E�O���8) endstream endobj 7 0 obj &lt; &gt;stream H��S�o�0~篸G{�1``�"���6-��P�!�&amp;/8�*#]J&amp;����6mU-i �wߏ;Vo� .�`RU "�6yβ �$��֤��H}�A �fO�ȁ� �;j�a�5��{{ ? t�e��V���H���SpY_���g���V��$2f\�����/%�&amp;���`:�|V�O � ��t�(?�!���bnP�Eqθ��'Lx"�x���Fi��ǚT ��Rpm��mlDG z endstream endobj 8 0 obj &lt; &gt;stream H��Tێ�@ }�W�1S5C&amp;�!X��EUEPU�UH��lBC�m���'!H��./Ɍ���&gt;���&lt; �BX]0Ka��k�Wlқϼf�V� \�Tc&amp;�^�v�;�C�"��}�q��+��;�t� n��MXN� �~^��ȳg�NK���c45�#��˰�_9� (S��;ȍadt��4GC���}�:�tD����ds�a�� � �/:O�(U]�&gt;s �QpV����^�G�&lt;{H��,�J��'r��&gt;Z�:���m�UQ1َ���B��P�V��J��lM^�8�8O`C��I�f�&amp;�nƩ���[��杈~���l�3?�9����8�"on-�3}���p����睊��B'te�L}�������]��r-�I�K�P� ��t(֊�i�s3�lȠ�1���z�Ӽ���i)y�TsS�&lt;+D��G�1=Q�d��S���� ������!q�P]]�N�t��}̈����� +)���h�v�銏4L��#��[��iT�OOd_e��5�����q{��}jz�L͙������km�9ZQ�����}e�X��� ΋��U �u��3}�Y�-���ק����t�G�+�8*V endstream endobj 9 0 obj &lt; &gt;stream H��TMO�@�ﯘ#c�cAX�M�M�у�MMcH m����� �RMc����yof �1q�@&gt;���PedzpbsyNh�[N��Y�|AfF��Fh����V� C0&amp;V���-G` � ��}�Y�)�� i3�RBu%@�e� ;d� KT�FO�]eH MP����g~F�Y���hz$q���e��NW+g-��ZK�� t��{Z@�gߥ���0' ����D+��`(Ҏ�����L���"���8,������lF�'�7e!WN��'4]��g3����&gt;|,�B((�(��B-�' ߗ:��%�f&amp;�:�Q�\4��_h���g���b] (F]�+�I�d�Qc|yR#�em����� �����f��0��?b�e���Qq�5���������/U?��ҿ�? �d�@ endstream endobj 23 0 obj &lt; &gt;stream x��z \Tם�����y� �&lt;��y1 0� 3�y\`ATPQAE@Ѡ���E ��H�F�&amp;�&amp;�vöӦ��6!m �ͿI��$&amp;ۤi�ݘ��&amp;Mlm�X� ��� �mw���w���?���&lt;~��y���w~�BH2F �k\���ۇB�� �v����]��~������ G��^OH6m��w�����!�O�ro�ٳ���'� �Zֽ��뷞�e��Tԍ�� ����rf�����ҩuX~����w}g{�q �� B��v���U�������;� �c ��5X��ֹu�q��V_$ĺ��wg&lt;� `}�ؾoǆ��[�!ل(�#�ZY��k�v��횲�V9Ã�����UՏ���9�5Ť| ��)� ���oQ1e��7�l�I�B��2�W�6r�qE��O�#�8.��4]' K�,˼ ����T� P:`(��X�U��%B � I����~q#�w�?I�A���� pV7����RBˎ�?92Q�3���7I�T'Ri�g��%�T,�� ��=~iv%o��vq2;���&gt;���Y�'v�Y�� ���C��t�0���t��S/3$� �Ө0Y8�Ṿ�+��$����2�I!���� �[��rD&gt;���1����}�+�|�2��~B��l$"�e4�%&lt;�&lt;�i��˲�[�^�i+�O�,/F�2L7~ʟ ��H��j�]i3��ŔB������Ѣ��w��dl �~��r�&amp;�R��*x'~?��:MJ�q�y�-l!k�ߑE�G��j%M�2i��I~H������v�Ab��4��/�ȿ�� ������O1��"��d}��'�LC"�sC������ ���"P1����Y�,|&gt; ����g�?0��E�NRO�C�1�0݋$��b,�K�Rݤ�J�K�?�Ť���d0O��YGߓ����O!�ϒ#�qr�� Y%�$C�wK"�k�z��s���-������C]i�� c�R�{m)q�U ��H �K��n_G�Ex?^NZ�&amp;�Kv�����Է�k����7�/MoI_�(�X��k�ط �Ο��v�]}� }�O�])�%b_x���޿� 8�J|�W y�7?��߾�����_��|CI�����P ePV�@� �B���y��u�kK�E��`~�?wN�/7'ۛ�q:��6k��l2����&amp;9I�R*䜌eh H 暖�f�R�!Ժ#n�C�]|e�_ :�ӝj��h"�&gt;��6���1� 2� ��ڣ����Y Q���Ͻ��K�^��tk_��ַb!���� ��X����.Aۄ|�5��HS�H� S[�l� di���ŉ�,����&gt;FH�� s\ �ڱZKMD �1R�s��FWJ�@ʄl NC�9e�_�� `X��A���R� �&gt;ڵ� �ڄ�����&gt;^I��1�^ڒ¬4�1���]�A9'��)U�Ua{��AmH�6Z:Fy�N�]T��?ҁw7 kR?���_���*��fr�� ����ul�N��8��. �6�%�:|�.wW����9���nl M���� ut;D�F�Hԑ#��ƲضcwD�� ��� "�� �:EM�1����4*�����l��_X��y�C, s疴\_�cT��&gt; u�h(,��ZԗF?��DEt:��u���m��a�P{Չj@E���������t7w�K�nv �l��y��,��#�9"��N�c�U-�nw�r$1 .3���:���'v �����'��N^���8��o��,�?��wFZ�Y� V��Ě�Hk�3�ㆥ-5�zܝkb����i2�3��l��(Ap�w������ц2��D�+g+`���^��ڎ��Z��v�c�s"&gt;���к����� ��k�*���*h;��5'��v��嵎���;^�v� )�3�M�� t��� k���S��:j�9��@��˅�/oA@���'E�e(�*B�n�D7-�^ �jZ���Z2�E!N��2�L�d ��%-��������CEt�5fj �Ś����� nTJò���s8ŭs������xM m�Z9�J�9��K�`�a���G6�u;.��O`kZ.X�Z ��?�ꖹ��j)�V���"���D�?ٮ���*����� �콕�����{�|o{oo/w����K�Wz�='z({Oeρ Z�c��c���d��`���x��+��v`e���V�����6�'�=���o�o��r`��yjˋ[.ma�l3Z�l;�#���`�i3F�M��z7��M�M�����ލ'6����FV�Ѿ�q#���_�F�`��鍛��n��������n��l8�Mo�&gt;�=��+w��X�{�&amp;`���e� p?z��~�P�~�� �D@��t�K�b��SH4+��,X�/&lt;��� ��4^uJg����֩�&lt;4~�b �`?_b��w��� ݁t�4o��i�����~��Hw!5��qw��Cw3��� :G��tp�DjG��F�$ �� ��`x� ?���¤j -�Ԅԁԇ�- ���r+.�V�"��H�F�#qD�� ɏT�Ԏ�"�r�!�r�!�r;��=�r�l4� ���6���~l� k���G܇#�����p�}Xӈq;R/��H,JهR���}��&amp;Oj� &lt;�?����'e�,{T��?�-�\1 H��t��2�x���+���U؍�w���(|7Ne7Ne7Ne7Ne7�$w� x������l�* ZQ���"�K0��P�@(D �+H,����砏_���&lt;��b󐟇+��V�!$ �&amp;W��������3 g.�a:���:s� �y ���� �ߠ���׫LX�5R ���8�p�N�@�r �q ��똳W ���U��j��WO\eH���H��Ԅ$å4�R�x#����@�'�O���hzb艓Op� �|83/��]�p~(��3�� ���Ƙv�x���{�{l;�7�1�܇ �� ���m �q���A�0 A��J�쵇�=u��k���Ă��&gt;~Ċo�i�� ~(d �A)�`�?�����睘�ǟ/�d��&lt;&gt;�%vl�? Dn��!1�H$��G20Q�.������ :��3���Ύ��ǲ������Q�o )�� +�ߊ��Aߜ0������߆rx�)�Sw �C�����ȡA t��f�p&amp;f���&amp;���"��e�G|�_ ���D� B:~�؏ ε ;���H��Б|��H~~�?�rc�ڰ�EC�AW`Є �A�o� ��@����l�&amp;ק��i\��L�&amp;Þ�k&amp;��d�01��g2�4�3 &amp;�%�u��Eui1摆�� H,�R�u� �X�o� �Ci'�ɦIZ��0yq���I6 q:&amp;�&amp;�&amp;ON���wL@ � �g+�FU�C!+P *~�,h�hS��d�B�R�8�ZF{�(��@���;�v�a� �&gt;������� ����7���|�����������F��vu��J�,�" ��*5�_kh+�'���$� � ZS���''�8 �#� ��N� fRy}�n��S+ ��p�NJ�������R�Cp-v�ҁ1��8zm��(�h�� ���44W ���j!�k���K���AP4�n�|+r�8��s O�f�Y�Z�2���u��:��~{�/]�}���V!(fN����ag���ܵK��p�!�� V�a,;+*�F;��hG�z ��w�Ap.CB_ilp0*X�[ǻN�_��V��C�&gt;���i4#f׿�&lt;3�]��wNg�w��ӕf� ױK*L7�.�ܙXӮ~�mq�Y��]��D�K"�� ���%��� S�� ,�nʖ6���B� �b� jw5�O��R�uKJ�J����9R�Q�9���!F���&gt;��W|�UQA���Q�&amp;��f�� v�K�mm2� C&gt;�n�����&lt;�q�6v!Ƅ�21��藈�1�b��"���q�߈��zB&amp;���� C�����=RK�����,�� �U2����ҿm����=����D���#-7ԿB� �ş� YEة���0������ϧ�VƿC %w��9�mϑS(��� �A�r/i'� �#�'���,���&amp;�d/��|��a���^r��#~RBr�D_���3$@n"E�)�O�u�4YȤ��r�Ax�l��'��y-ŧG?D�H�TCB3�nw}��� �W�9I.ⳅ�En��I X�a\��f�92D&gt;�+݄�2�q��?Jn#�T�=Ln�ג5d=�:�RI&amp;���"v��7Q�T y����� �ԓ���g����� ���d&gt;w�22���*��p�z�0u� �WDm�#mć��Dp��po��$������:�p_ �'��`]��D�/`�ZKv�!n ��N�� ����#}1�~�}�J#i�w0^C�"*p�.�����s]�6r �.aFȃ�2 �RA��� ;�y G=��m"�9#���^ew�+�v��?�_� �W�Ũյd#j���&lt;&amp;�Ĺ�� �-��[l*�ʼF��-�j�Yf���{��MF��(F�E�E�M���n�A z�n��mRv��O,x`������3uK������w��i�"��hx�h��gm�Z�EUcn�9kfc�/;�q͒;����4ˢ,���mi��|�e���N�X�&gt;� t�� N��[� ����K� k]R$�)R�P,٥�\�:m��l�bJ���(��6m��0`)0ԙ� �ɺl� �֒��T��~�ʚS��j�sr��:����iv��m�R/�/B{����!���WC�ѷ�~ z7D�C'BTc��SP�),txt�,� �s 8υ� ��U�f��|�Hd�S�B�U&amp;�mU��lUCk�p�&gt;D+j�:GM=`��Á:� =�p*=ǩ�II !��BѴ���j�ڨ�RӘ�*���x�}ؕY$��)���"�v���CjF�..*(P��3�s����� �.�5�].�_M��Q}�h 5ǌ���91?=Jb~ ��zY{��t\�� �۶O�i�Rt���W�_�ĒΘ��m)��)t,y�y�� �&gt;-�|r���61�mێ� ���p�'J���G��k��|3�����2���:]&lt;�|�{�B���ag0���J)wL��c2����P����Z��w�휷�����!��A�L ��v�oDQQa��vrɔAo�惓N�d�S�Zt�ڰ����/'�����6D��7���SI��W&amp;y�8E��fx&amp;.�z\.����ܽ�����nC�R.���b���; �����ʔV�'�S�T�^�2R ���� !s�5�i�5�3@��w8�[���L�!�w&lt;9��`� �J��͝�_W�_�PVZ�r^�8�[(�+��PqZ:�� �VAiYiq�AUe�jn]i�6�ŕ�ʸ�!^�v�z��.и@�+&amp;~�Fpp 9U�ܳ�k �!Bi�m! ������ ���-�8� ����+9e����1-��C F���*����R��G����"J|�Jd-;��� i�SB��D�����s�j��^�4�DĔ��I |Z�� ;��(�gB�WЩ�Ũ��,/����ѠO�� �@2�vyEC� � J( ER�KCɖ�Yy�ΐVX��4T,�X���O^z�x{�}M�c}#�V�VCE${�����"���l�e�]+��ӑ�-'��|r����⧯��R9Z�+�3#C���V��������ifh*�x��ִ�'i��OX��ߴlW)�w������߳ "b�$ &amp;��Y�jwdf�y��f���PL�&gt;��ٍvj��f�� x�� ����)�l0S��`�XhUx"�1�G��� G�� ��� &gt;�WM�Ҿ�������;�{I5 _ˏi ��g �{��t��`�2�J=o�x�D��y%loid��y�e I3ka2�N�mC��m��o�i/k/���W7�ާEe�m���Gͅ�����:�Kl�}~`Z�%mm �Ǒ�]����23CA�I�qno�W|]Tt K����cBm��� ��̯�U������[Go�_���L�Q��+����M���;��{`�G�&lt;.�)�Ba���W8�Tj�q����u��&gt;�Wv6�z��~ݜ���:���K����^��feTh�AF˽ U�1�����Ư�n�7x��?f�/����P燻Y���=Q�( �ޤ��E��+ �·[�6p4@e���gs��19�� �:���eu�r�~�,�&lt;[y�q��ќק�77�k.&lt;�? �w��̠h�C+�Л�s�/4� �����F���A���47 ���H��SϘs�#~eS�����ޜ� � ���;9�r(Y�1�R�9-9�ɿ�×� �Y��xH�����E���W�[�ʜ��|� �� Nk� /oa�m��u�c��CW0Z\&gt;ZZ +���RF�壪�*����.�mX k�-D����"�f��ߺ.�&lt;��:���Q�&gt;�f,O�h{��'qIpM�7�Fh{���b;��I K�׶ͺ43��bi�)��F�~���ہ �!��; S��eӾ�'Რ�R��y���_A����[��� ^��OS栌Q��}��Q,)�-��xr��X�Կn��1�P�.=�`���������� �\���Uͳfr��k{Ѭ����T�Z��o5�dP3� #N��M��̫3�3LH��z2��|�Rg�峪տ� ��� }3ä �_������S+���pB _tg &lt;��g��Y�k6�$�+����'���Ȓ�U4�(IoI��2J3(�ٔV���D�oRJ�*Ś2/��U P�P��`��8�(�� 1��h�ٴɌʒ�L2�&amp;�"Z2�5�V� �N�j�2�6[Fr���ezmŶ�6Zf3�(E� �V�&amp;� ��m67��e�B\��iɦQC�2����QZ �c�Yd�/x�S�%ܞ��n�"M�ɧ�pm[(a1B� |m��R)�"�N�AD��Dd��]&amp;/���*_X�U�۶��)���. #�X��, 1� P%�LҖej�0�2��/S����i���F�=��?������|�K��P ��F[��� �T!�e�b�P˫�S����-O�� Z_��z3�Հ�� }A�JJ�.�Ϋ�켼�����}����j8l�~�,�[�+��suE�y���T�XДEj�BՌD!�#T �O�'A�BqK4��F#�D�5�t�b)WdWT����r����rP��� ��A[�(��i� ��C_9ʁ�_,��#��ED��(RP0 P4V��z+(E�R�W��Q����5���P�hq,+ԡϳ`tQ�Ět�QG��/]�޻h�vR��ۢi�*�v&amp;.�4���KjM��� ��-�ŏ����ش��t�lGC�~�Y���� O�c�te�&amp;Q�()q��F�CQ_�/јoQ�5��� :X��Hzf-�x�I�I�^�ul��U�*#xJ� �Ft��h�V���� �rpn�.,n\�XA�Q�ց`x �)&gt;dKN�r��] V�q����AUuh*�k�ܩ�S���F^��J� lfY�K�/;�si���]��{^�L��M��4���S���l�]�.�R)���/����w~v�9�IOW�E�H/����5�ۈ�Z���:���[� ��� ��}��@՜ޕN�CQ����7������5ݛW'�:���+�IuW��ҟ�T�/��*U�&amp;Ĥ�ٟ+��JaO�h�V ��B5*�F�*U=��,Ț3h��� ��Jbbw�y��;�n�(�ęYd���2�U��wT�N�;�k*ʫ*V�W�2�Q�3f����i\3���^����,�zsN�I�97�v�њXTtݣ��)[̜:j�����M#H�Ԡ_r������q�}ұ��M�� �d���͜�۷��I@����-�� ���P� �+ �79�����q�g0�w ��hk�)��Z����mN?�o�Ϸw �\�w��o�X��^�zO˽#U����Ә\*��'Sl�P��,-�R]���zX�XS���f�w��K�ܹ��;o�YG֜�e���# e���$0Ħ!�"������[���,�2A�.rS2��K�9&lt;�t��i�y}^Y6]Q���'������;XX�/,,CH�Г;n�f���pM�&amp;��A�Y�כ��4 Pz&lt;~� �����֔�-�Tey�����3�u�ݏ�}�_ ՛ %�SEc~ �� n�l� {TT���r+��t�zŒt��j�r�D/-��Ο�i�����#4������-��ǚt��mû����]_:g?'�zS3@!m�;�V - Т�1�hq�ԧP�H8���aU��������j�����ދhp��A���§�~�6� l�B��7{�C��ʌ�gJ�� |n���5�?�bEzQ�f��2D�ܟ?�6q_�76�����{ν#�fdi��4zK�۶dK��k ?"� d��&gt;��b�F�.���3��&lt;�瓟�z]���:�\�ε�u��= It����Œ��j�F�j�d�&amp;C7i�1b&gt;�1*.�����bmv��Bѫ�1љ���Th�ZlFh�N{�Nϧ������*Ib 2 1��6� e/p��m�cʢ3ԗ$:C�mlۉ3��9bg'δ1ebO�L rt\�tb5&gt;F`�� �n 0zL��(OU��%bM:Ҹ� ����U�p삉��SW�t�=կ�qf=��� �t��ݛ�f�Ҧg�|��Ϸ�s�7������kZ|���˿���= W O�ʐ�8�p��w�?pl/��C!.���a�BKDE���)�� �=� ��) :sF'E6="ХG�r���Ƴ�1��Bn� �ђ� � �'�z~����D z,��h���`�l��R�O$"FBV憂]D�ߔ �.qO Y��S��mE�|�w�"�L� &lt;�!2�aQj!-O\�O�]���~�d����7 W����M�ٗ�&gt;�?�n�)�z��pz�q����E�BfܡE�0�K��~P, X�}��-��AR$��B���I�`�UӰ&lt; i �k� �jKs��xv�4�ܒ�� ����ί��N���y^��"�I�I��� ��!���A��Н\��q9� !p�I0���P�N��r�N��܂���r&amp;��\��Xt�����+�����b���q�� ��s��n�E�a�a֑9:����H5sn��f'Q�˅���2 x�j�t����\� �1�����8���f�T4}R�� � Ģ ���E �ɇ�.گuA�%3��v�� dF ͤ�� �Z�� B��&amp;MXH6,�Eg�~%�t��O�p)�A'�����&gt;���m����M��Ne�v�wp%�W|�i߫-�.1��*�b��������*b�O�r� �1��_ ��{�g��/e4��;�M��ۻ���X*��9pK���Jo�hY�l$ۼ�| ��˾��-N� :'f��� ��50)���0�h��0�&amp;MnZ�N��UI��2� �ݡ�\����wtOv��69q��7�j��.�~��s�Y�f5���B���rz�d��n�5F�/*��Ѳ�������&amp;r��D�� Y�1+ ��� b�\x~���DTk��@T07�; i���c����l\�Kٔ��/A /�G#yUH��E��Ga8 �`���E���4�J��`:�`�y��.&gt;]:˃ȇ� ����7� �"��t� �w�&amp;d#L8�#�Na7����Za��_`y,��M����8��u(�����v��x����H��I̊O!j50�H.E�@�KEI)�R��DZ+�� �"��T�J��&lt;[����;�� �R���~4M�w�t[Em����pΨ�������� &gt;Ӭ�j,f��Ō�m�ļ)K�� �xm�6#� ׬�v�a�3�M�N9u���NH׶�=r��� P�^��/J��O��z�U�U���x��g�~K��|�����c*V�n�E�ٔ����=K�� ��]���� m���l�gݖ��G�� ��I;����ݵCo�sy2;o� �Ω L����iCu���}l����^�����?��̲L^&gt;x���ҟBϵ�UV�:�6U����F� &amp; �v�&amp; 9V86:p&lt;��A FH�Ft��,��l8�n�f]vkvg���ъ�Q�b�l���B8��b���=�kε��b����F�����H6i��S�Mv^�ސ� �d�K��M&amp;j���*���P�������Zdن���q:�xȠ���hB �� ��6�\)�F� ��Q�G�� ;��9&gt;��F� 9Sìq=���-�'�&gt;:=�}����!k�SmG'��柍���������~�| M!x.i�t��+��w�IÆ뾼�� ^]ȴZv�b2������uS�n�}����Ma���=�6Ef&gt;�h����&gt;���a`�!L���������]` � ��X�/������� �?��S*S�z������Ã��+�7�����#����VC��h���~=��:�S[��� B�!����lF~��ˠV�����E��6c�Gɪ2ݜ$G3���2�(����dd�䪜)�d�C���(�'F&gt; �A�vL�{�ǕÚq$ L8 ��#��a���Z �˭���e��ڳ��4� +o�� �9����+����;ۇ�&gt;%}������V � L�=�l�أ�v�Q����=wN�{f�goͱ��S��q��uضf��z�x� �3�=�YoYOO�lì�^���8��ԭ2�]֌�q� ����T��On2�=D�P�.�Z�ڞ425 Us��9xC������v��\�v?����� �NB���k�~�,�Q�+��*�r}�D�ǄM/m[seϢdoW�-'��y"�$ t|��?���t��a�2�O������֞�`���2^�%w ���՗��^Z�f�޿����Q��G���� �5Y0f��*$��oҚ�ؔkB �� �37��ð1�+�:��:�1�'���r���.�tG=F� +D� +��؉k�Sc�}A��9��牤�� �Y��=�[l&amp;x��i�i҄EӐ�B@��wޭ���w�w���v[Yt(��y�7����!V���~%�38%�ƭ�۪��/��pu����54(6NhY��O k��W�ԁ��Ě9,��F�WՆ��� �=-T/�2�}Ì&gt;z�|C�ҥ�-\wٟ�\#Չ�O�n��5�_��^���V��� �#�G�%i^������ĐZ��^B�`�W��/5�����ڥbW�kIז.V��u���dש.c�| �r�&lt;�� m|�����F�?�SJ�\1��|&amp;]R�rư6L$ ��V �(�Z&gt;��B��Ѧ�n���v��nW��WȤ�� ��Z�DBq%J{�W:�DI�s=N�{/k��E%G��x9v( ���0�4���$����ET]� ��AM��[[)&gt;��� lB� t�Й_���wdĺt,�iQ�tj���yd� n�ݲ�&gt;����µW~A��9�s*f D���X&amp;����8��F������t�i4�VG��ѪD��d��+�A'�����ZT�����,��"����t'�zF# r�n� ��3&lt;���m #�݋��E�mw���-�- 8`�7o ���5C�rf \���_�LA&gt;���U�c�-�\$ݹw��H`������ů09��Y��6�`C�, +�ot&gt;׉����5ت����'�� ���z:��л��b�,�-F� I�1L1��Xʇ�1����i-�[՝1��+���n��j�����E����;���� �Q��� 0&gt;2�}�8Z��z�z�5Hn��Ky����)����]4w@4QT�����lM��%F�ǉ0���"�D��p�*�dk�݄�&amp;C�8J��n��L�a@�G����p�fj0��|��!������H�ݶ�3z�Kn�@|���Y���"d� 5z�� �xhYp�f��+�#� m�4�X�����?a�� ǀ����Ӄ�q݅�"bTj�����D� @������隉��s֣t�� ll�^p���� ����7t�6�7�� �j�s����'�~���v�e7ݐZ�u�g6,�﫷���H�� �ɞ%�������u#[��p%b��~�-���]����=[�vކڮ���.+��� ��O�]�  �yd��v�DGM]��%�c�6��tR��t��{蒘����tRVu&amp;�͊����Vv֒��&lt;�Q����K��7�w b���Pj�nr/Մ�����g ut�|���C�Dw����E��i����u&gt;w&gt;���S1o�m�L]���j+恻[Jh�_�Xj��&lt;}���ǽ&amp;+��~ W$�N(�,$�Q1|�13�L�H���� uÐ+3p� U�&amp;&amp;���"���/��+�2C�S��l�d���pAp���'+�-J��?c������۩S�R�mχ�s ̧�)�{� t$u&lt;�Vd?�"w�H�x�t�]!}$�#�q鴄Gl" H��n�&gt;��4� ��Jҏ%�R�XB���^�u�&lt;��T֕Je��'UHeKgS �֦���HM� N�J'�6R�B�X^�}� c6 ��jᗵX�U��K��P�֪�oՈ{"|G9ky� s�k��Vs'5�J,������*{n��?���#,5���s�P*U�����]D�h�^OG���ơX�0!�I]�S�f�N=�B�����s¥��h�'�M����d�R�:v\0��z�`���k�E�ֵ�4�I�����"[�X��[�o����XiP��c�W�~l *���i1Y8�8G�H ��&amp;&amp;C�\�l���K��0�X��xH���`3#�2�����6"��^��䂏1�"�{6��X�'ZCV붲2K�~F��pɕ O����I��� P�A����C��(���I[�-J����t����&gt;����}�A��~ `��|��C2��h3�3�;[}���m�  �{ԇ�+|���y J��e@6��e �d���q�D��d�W2�XY֚[U9�Uԯ�`�?��#(��_����U6���{���702��qD�FJ���Y4 �T3�l�E8�pS��-p� sK�f+8�g��'�kj ��@Ϭ-�͌�^Sߛ�7��)��t�+��j�Ɏ���5:F���cc�����@����mUr5D�f��e��r�|� %�������'��-uX%�R�Xޏ���;a)��5����L�kx�����1��H�@8�����P�Q������F��?���z��+�&amp;�N(  v��wo r� ���������ъL�3�*�4������k L`�r0�C� ʈ7������������f�C~����������刼C\�e���� '�p��!�L�t#�6�� �|:���K��`�{a���'����o��渙��A��X�Z�) X,�r�c�m�����3�F 1�1�M1��ru �W�7Ə����� j�-�!56;�rl~ M� �MTʮJ�&lt;Կ�#Q%�~���?��;��:懟�����.��.xk����0� S5U���_�������U�.�?�r�t]�B;\.dr��:��f��5�Հe&lt;�rM��`@�J��_�_uFѲr������ JL�V�C��j���Z_�*����TN�A,/)o)�Q~�|�l �����2�Fl�eĔ�2�� z!"���D��Jn_\V-.C��uQ��D3X�����r(�eu�D��� eQgS�ڴ��m�V��`zl=� �=�����Y�j1rv��� ,� �yL����t��� r3��c�C��m�u&lt;�f��k����?�l'茤^��'��j��&gt;��l�.�����.+��R�9����� �Œ��O��x��1���{C-,8���Ҳ����.�������{/��8;�Z�iKj~SVF�_�Ũ�3�� ��=��2�)�� ��b%�.�� |fQ���&gt;h����z? �n]�0`k�� T�WG�@��4�u5(; Y?�h���=�A�.v�߸ O��V�-~��9&lt;��W��9���~�f����~יVzY��qs, �V�: v��G~�6'5� �_��}�WS'/j �68� �Ɠ�&lt; ��T����Hd�Tp�J�{��{��R�7�T/AW��&gt;��ȅ���#������������ȅ1����E��R� �R�[ ���t����*�������W����X��"�)�h�p�|m����b#���ҩLRc��$�1-�~�lU�q�7 �1�y��� �L �`�1~�E+��2L1���|�������7��A[ ����L[����8E��̂��x-IM)E Rt4a.=Q��ͦ��|�HƸ.�� �l�� �ՙ�����&lt; 9��:��(� 3����驹˹g�!E���߶m��F�SĠ]�qr=*���5׮��¸�ҷ����ǩ-צm~)"4q N�V���1_d�l�=��P \N��n TXߠ��dJ.�n1��Ӓ��??�n~�x`p��S����ZӶ)� ����Z� �x��q�^3�2��=x�50V&amp;Ȅ�0�_3���*�M���t�L�M�L�灗�5bz|0Q�(ٌ� � ��*� ���� ������%���Ȍc�!��\,��l %[�g}7oUw#��@��'��4�� �`�^�LF��� ~�m|� ��v۬�YK��Ж�-���y�a��9�O�ke�5�[g����;l�Ǐ���Fh��t��x��3t�Q� uՏ[R�c�-!N���@¿���Ԇ�����W��1{[e��G�+���_3�Z��ۿ��L��g�?���O�N�O۞���} tוe��X Q�Q�A�$@$b%�7") (RE�� �$%���$fǌ�t[i;���i+q"�Iwǚ��INr"�mgi�-gf:vz��9�8�d {&amp;���mA���N�=猖*�W�P ������{ S��l�d�"�TFE;����'� a�,�$ WYX�]��Ҙ)F_��4b���# ����)Z � E�fh�B: Y�D�Q�1pZ� �B��l��ͼ����&lt;Mu�G���7�w�R��:Xs���5���T ^� /�ߌ�h��_��x�Uw��v��@��5�Zv�꒨\2����ՁQDZ.��� �� ����\j�w��A b}n_�w�'��;��k�&amp;z�?mm�gZ�����k�J���/`g�L�f ���l�G�� ��E1-3�HM/�마,�2�J��(8$D�����Dѹiݾ�ͨ'z%���3'�s�����/��Xtw{��mr�`��� /,%:��q+P�{O �)��C#��up��� ���T��^�՚c���|T��,0L[f���μVc� E2�v��%�|9~��A�� �����i��.4�������a�nP�۬�N]c0JLZ ��,���9t�Ǜ���CS!�� c�%µP��,�:� |�P=��&amp;R4x�Ì�5���^3�u�@t�&lt;����u ��Ouߪ{�N�[�U�����ɨR�8S�*�2%�*�TZի�7U��u���!�*��I�w7���w|��&gt;�F�j0 ��Ȁ��C�?� ^ ����o�L&amp;�"3[�H^=I�dSLV�D�ӡ= !�6r�e-6+��ߛ��&gt;Ea�X� ��[|]�EȺ-.�D+�+ ]M �V��9&lt;����ML`�V*��j��|&gt;o '%��MC+�&lt;��I��T�*$ϻ� J�u�����E���_u�t� ����v�I�� 1Ǻ ��Z8���ɱ�Qi��&gt;�`�����E��d$��v��K ��]Mv�#Ο! �Oz�W3͵�v�-�x�! ��j��z�o_�{�u�f��[zS�vx� &amp;�G��/�Pm����_����;�A-�pD���V���^8�7���&gt;Z݋�0�� ���7j~���f�� kz� )��@т)k����(+�M`��?���� �W�[bQV�����J �uu��Q�����f�i#�0U*�0rs �nSId�:_�7p&gt;��0����+ �d$����+F�w`8`��pp܊1l4�Km� ��hK��GE�T �+*� ����1u^M��g�|0m��F+~��/�*�z%�f�f�8�#�jSg{��do�-9� � a���0&amp;���p�ʂe�)� )��x���f�'1���\��^��Ny��̱�^������,b�N���Q&lt;��� &lt;ϙ�Fs�̬��H,��[ȒL�$[ٲ9Z��/_7�uf��h��m��m�H����Z�5���/n��u�Xrչ�Dݿ��V���"A��D�E�Sd�lݽ�f&gt; ~�F�wV�3�)%r}{F 粫��ӻ���` �&lt;��]*}턓����_h�8C��6�=4�U� ��r��c����������]�l�G*׾��{$��Ov� �0���Μ��Z3���d��V�)6��o��T.���i�����TG+�������ԁF�Ǿ`=g����}�{ �� ~VR�; $k��h=��x��l���Ҫ*�-x��׼2�(%�����W������ȥ(�GU�J�;�6�}���3��͕�6�,q�=���m�s��1��_�)�o���l �`��~��m fӪ; ��x�j�Yx����6^�W-�W�+o�����$·�T(�[�� �3!N2݂�"D����3������楍L���hK� n �iK�(�"O�D���1Z��d�H�FlzB�ք��L��ن��L��2��d���b(��Slh��+� ���c� ��� �u澡�+�&lt;:�r�ߘ� ���Z�v�o_c��Qy��_��&gt; ����`R;�^E�� *'_�ӻ?��Ze�Kj��;����m*��'��H�VF� �5�Ғ xDM�y�bp1 �((Ԡ��@'����:c*�������U�.TO�n�K]�d� � �0���2�� � rLD�@9/8/;�'䜯9�Հ�r5`v�SN�X�) �������?��1�s��7�8 5|_�)��q�Ьҭ���� J�Q�t��0���:�O�Q&amp;S �⯷X(� ��w{�WS�P�yL�W;$�Y��b�K�v9�V}�U{������E��l$����X����� "�[Q,�^�B��Z7�����4D5�[�k�̇�e�A{�LU�B�����h�E��6# ēG��-�z*t�������?��UJfS������647ڽ�#(9�t��t�rL{r&lt;�qa�*k��đ�6��8;���[�b�A�� S��r���⺇����] ���F�X�}���фn)���Y7��ʏ �%�����q��of Ex.�ר��G%�,�}�44�p� ^g��5�`*)g���6�&lt;�AJ���,ksc ����aG42���g��b�"�k�f�eM�zg҉�#0�zD+S q�]�&gt;DK(�β�~�򨌐�~� ���f�p����C4�#�����$��t �N�x�ޓr� ˘;8��9��� A��� ��RPs����"�h��RHl@ � ������$vp��τj��� $��kS���!P�R��u ��6�řU� f�� �W̴��C�%��2"$���잼L�K����;�p� ј �|�C/{��V��X���Q�4pt��E���Щ��5�����2�O�����y��x�P�E����ı��,�zů���E��F��׿�Q4 ��jP�l����k���".�gM� �] �� ��1W��r�pMj���-�\�����}�?�� :�S�U߱�����X�^s{��P�əx�ߢrK�\�= �~���NM� YB&amp;��=�0�6zl:g����h�Y��`�_21F���� R=�Фz�2�n�L� ������&lt;= ������/J���G���Wi�/Yb� �: �;I������� �[@� %Us���� 4�g�T*�Ğ���\4,{�{�{�l�O%�hٔy�v�)�=�7��FsJA6ge0�gϊLa��/`��#�8:5zq���(�G��6j0��9���a��H�͘ɴ�G S�=�Q�`�/S$����-��@F�=Jg͗ͯ�e �'���_�/��� �~��\C��2 �D��Zhkk�E��3�zȐ� �q�5Ιhf6��Y�\��̼�a2��\�Y �v��~@���[c�����.���v�5=' �F�&amp;:��X��9d ��æjph�y� ���`�{����7����!�A����Ώe?���v�)�n?�&lt;�n�|�|����[��8~��8\(_.�ʗ�7����k�W�h��\�ˤ_�⩤h��z�7� 5A?��30Vlr0�#]���xk ��I�$?�(��9�ꤤ���#k�є"{�O�L1=�څ��&gt;O i�4�'U��#��l/ic��� z� �I F��)-ꋣ�(�GKP���� ��Cz�Y�� �� Ǻ�����JU ���/;�% |s r��%ߔ�� �:o��%+z�Q�w�9$�]zGR/4� ��U/T���= ��j��?��_�#%¯H�f���6���TP����`0It�V��A��]�!p�C���C���+p�oF�"�WiS##ux�7 9 E����;�� �7���(����"�V�\Ů���R��J�۬y���Mj�)��]� .�b}�0���]��*Պ?kkk�R'/T����إ�Ns��W ^k� ~�k��_ B�(m���[x] Y__'��W�ڪ}� B� |iR��.� m��K�VP�%���G6V^��_,:-��6�R!�D�G��b�I(ݬG��QB��"�����P��^�B����ZLԀ�}���RՂ�W'$N,��#�F2���7���� �3&gt;� UnO���\�Jd�E��ڳ��h1��`��i��1��}��s�Q��;_|�&lt;���4f���Z� Ei1�_ԣC{����7�K,� hx�^"�J-��gn8 6��ų w)�r{8[�&lt;��_?� �� ��C�Ӛ�3�z�;h�ܐS]y�����j��I� 9t��Dd���+�/m�[ ԃ��S�IR㐤H�䆡���l2�It$�ZE�3�D����z�����i�y�:��;�� '������b�PS,r�� �]x��?c�n2p�y���(_S��_��Ԋ ��T�pV#�Y̵Q�?�ґ0vt$�����9��nq���]�������x�#I%&lt;�h��XH,'d*��c? �꯲&lt;+�[��,�;LּcU��^M�� ��������dw0 6�l��H,�5[��U&gt;���刾+���v�I �d���������nj�����-�3b�=��B�����ذ1�_���H_3����- ��-��泑��+vEPU� ��wZ+�l���R��I�v-ٻ���ks�U\r����A.,��Me �z ]-� �F�h:�}{b�gbb\�3����Йfk��z��ڒk�����z��c߉b�!��˲Ǣ�㯶� rν3���u'F��#�P8� W�^��MP&lt;^��&gt;�4����W�|���O�� ���#`\2]ӯ��~�p_3|�`˖va������н�T�f����vZi5A� �=�d@�[) 4���� x���Q������$� ��Ʈ��3�|�j��F�Q[[���l�&lt;�x�^�I�c�H$] ���|�F�^������5�#��u v5W�F�P�n`�`i�/�4ˤ��4�y� �6�n�#���y�-=M��R� C 7ߘ N�I*�IGӅ�Bz9�m�%��D���W�aL7���yV�  :���f]]�K&gt;���"��ۂ-��%� ��X�0&gt;�ɋ�vg&gt;�Z��j)�������K&amp;��[��~V3�EJ��h���&amp;�H�u-�l&amp;���I��=�w�J���� �ʪ���B1��JlCV�LMS� ��;�+G4�a=� �IU��&lt;%ѸƮ!��4_����ß�3`�L��wOͨ ��'&gt;�����Ւ���Cl62y�l� �* �74����gt�s�|�55�ͱI�B \tz�f��t�#���)�o_��X��E�d��g��0vWw�#���L�5s�b[C&gt;�Ncx2L�� ^�C@L%��L;��0� r����b�������7�i� ���] C�&amp;쥵k���,��^ �����G+ڭ���)8B�����k��Ca Ap�����ޟ�6��$�X1��7ngmv�� ��f|B_O{;ߖ������|� �g�y^��Y�P�Yق�L"�iFv젆g��/ K�å��z�7�}�`�O&amp;��L�V��Yk��An'�!L�A��ޮ�5+4�~�7���0�/��L�gs�/��g���������AHΓ0�'� ���r�B�r�Q |(Q�o����'��6����B�B�rV�@x4��������f�^�ښX ��KM|S{�`�竭g�9b+ s ��x&lt;�dSx4��d�hf��9�U+� #���HQ&amp;QU�UE�� [�j����`�:^�qqup݈E�]7gb;��{ ��[��]�N�b�%� ����j�}�6�����5��K��Ē��$���~m7�V���K?�,޶ � �$ H�'��ހ����C��z�5��"��qm)�b�� �D���Y�hj�s��Z�6.�PCK ��|�_g��E������ 9�hn������� ��Vc v� +VNz��˳�z2ұ~���9ӻ?��&gt;}$���כc3�c}�(�a/wʇb'+7�*㐜�o�sYþ Y��/���W ����M�]@3n� xm��h\x�D�,a�%d�0J �NK~�L����Y8C�g �Nf��F�H9X�L�� �Q� �I� SQPD�������� ���+s�|��� O�&lt;���=��7X6��tpO��r0ɖ��ʂ/iH�=��nU�+&lt;&gt;���9ά�Y�U?i������&amp;o4j|��+J m��'�� ��W(X���V����~�������a��|S-��ۢ��Ū1Z����ܥ�&amp;) �_T-2&amp;{&gt;�y &gt;�(�yIG���jO�)ɶ��Uv�=�����Hف�����1���AG��1zl�c�ܡ����Tc`j��� � m��պ�ss3��� 8t�@СU~�!�K��*�j5U��RGK��� mNV�'IɄ�'��7��Gt6)���㪯�Q_���U����q�~�0). �*�=�� �TH��%�ˮ��ߝ&amp;~=���S�" _��ӛk�Cb極u =������2���Jt��A�� 2BE�[&lt;�W��?T�ų�"xPow�J�`, [z�L �rJH�Ts��[G� �@�S���KQ�ɪc��c\�g����"熻����_�������_��}�3� ��O��}��@�)����Y� �w��J�i���E?�T��.�+���U~�(�l���1t?vH�#�;�ܮ&lt;�ֻ����؎*8�Wν�t�c�������h&amp;T�Z�F�꿴=� h��*�v�r��p���/$A�Qٗl�� {�=�/�S�&lt;���~I�4��Q��};�5R�'�'߅S˻a�M�Snc�8b�1�e��-� #�B,�����P����c�:z�{x�0}���-�u�$����\ ���y��f�g�h�� ��j`� �S�do��#M��yfL�]π��A���`j0=�00��5���������ྒྷ '�I�I�? �I�I�d���I��$7������&amp;��x��e &amp;bx41==799���_��;ȫ��SGG�۽� l܍���Im��#-�?R���l����Ks���9���Ç �k� =z�8���������.F��E�b�[� ��"�*���[i��� ���ao��M�� �"}ӊ��@q��N�е%�X�E��� ����loK��ݨ~؊�y �#N�V��T/�w���������/� �' �V��U�l�n4��{� ���sU��Z���y_�gi��:��]�0(��:�:� �to��9���f�E��gV���la�|ho�cŻ ��_�X��pɟ�j�9&gt;#�.�[j��B+�GT�����Մ}bj�؄D��Ct���ӯLK�I׃�v¡�0^��D������Y��� �ZP��`F:-�@X�+�� �B�A����}��\��!��jT&lt;���A��ڀ�D�����'ϔ�%�͕2�49 ��X'�#��߱XS�N�:_�)&lt;6ۉ�Nw磝7:%�I�s���IP%�IZ5l �U��x�Pi����k%���R�֟ž��aڔ���Ѳ �h�Ri%7l��S��&amp;�K�=��=��n�n���L�%L�­ �9��봳5p�ؚ�ZQS����bwT��Cm����}$W���,�w��I�t4ʐX��p����n�pI9^V�L��`^F� E���ᙕ��70���I�]pӔ[���1����P��C�)���Y3��P�B�v�3=fj�e��niI&amp; WB� ���\��֪��Z�?��~�⒎���6��2dc��v����s�7;hD�!i�YZE&lt;i��[I�{nS�iﴶ�e���9B��^�za:T�9��S�c{�~�C���tFHĝ*���ɧ���l�W"���*:\n�wl�^S�WoAd���B��]���R������FL"&lt;'�1X�_�U0�m ]a��}���vN6�\l�.[b��� ��!�=�Rs�B�"��痺?� ��~�ad�Í ��j�70�{�钇&gt;��] �� �=����}~c ��3��&gt;��g"�|�+ �y��L��*�����*?|n e�9�)S&amp;��ʞ��Sgq#���x���{�?T ���X�I(����yS��x��w{&gt; /~a1%b�����KF���.@�!KAQ#�`r��6��y �m�m�#iz� L���&gt;�;6w����_���B�� ;w�9)�&lt;�����,�� ���G�o-K� ��2@ՃBq�!3i��t��_^�=�kB6~6�����9A@3��� 3 �|��ͳ3�Ό�&lt;8scF�D3�3G$�'�z��� ��d&amp;`c FU�L�b2K���R~I�� P����Uhbii�|�X.��8�T��|"y� ���B����2I_.c�&amp;�N���q�]�=�h�:�gti.�!B��:D�oPҎ.�ң�ro��� ��X\y�u�C:9/_t]�A��^�`�%x�ƔK�O����%��o�v���Q&amp;B�1&amp;ŉS� ����KH �����Ѕ]]!&gt;$�'hU I��&gt;Cuz���LĘ�D2�Ƚ�L��`�T�d������ĉ�T�L��@��{,2�����8u�`�~�qQ�A�ў}h�Y�b�my��e�ZOm:�li��/��XG��b��6�g6��A�̱ʛ �@C� ��P����6�� �̥0̍6Ü� KW�t���3zz��:��g�U��o����w\e�¾�� !�$��&amp;��c.�&lt;�ͮ�&amp;�j+ έ;ſ�j���"�[� o���� 7{���'��zǵf���j��͝V��5�{iBZ���4[�v[]�N����j ��Kۗ@�q]Y֫*�PI�X �Bb!�F�X� ��$�E�$R4 �E�Z�X���8rg���v&lt;=T�J&amp;�-'��M�H� ��"��ݙd�N��:��3�;�,h��A��lg�i ,}��,��������0��-�Z�.��J-׹e)���`G�: ۭ%�/�������}u���w���M����T��h����w�D3���G}�;E���}�n �o�4����OO�9!�V�g0P�_=엤!̿�%��27��+���n ���  !�pLZ-56�jph-(P��}���?� C����� :��}9��'v���RSE���_�= ͱ/}�L!�61E��o��f+@? ���kӯN�9-�V�*I�$#��ύPX{�|�^����0�bP�O�����ľa���mTO��}�]���5�[� ܵkyj �R6����3vp��������{�d `�`�&gt;`�E���Q����}dـ \�oll�e4,�(�vQ��J@/H8(S {*��rE�i�jn��� pJ�~� �Ws�� 0 �5�U��b` �*mb�2���gI1��`B ��@�yD_�M� jD�����E al��Wf��(�/� �'��IuE;�2�mm�X�+Z�yj����^��z��J ����`P9D]��.�W�P��%L��i6K���@�� A����V������'�?��0�� sQk���vb`w?�xa�S�+ù�R�Vq�)NPQ�ojɔ_߭ �7f�,^��f� ���.������v8� u�LS �T�ІB���*�d����0Z[k��X 0j)��e5������G���u闖�N��_P��`�Ho �v+���.��.�d�u/�]8��Da�@!?[L�n��&lt;�����5��:i�ʗ� !��F����bb-v� ��d����9���6���`qO�\D0x�id]�k#��LA��W���_ �|�G��tS�Ӎ���qtDS��`�����:��?��Tʜl�i#�R*�|�V���2����ї"�����_�Cs�����} ��,�cn\ȿ��ժ��*����*ǺmO/����W՘j�z��_��Ę�w�6�:�O_�OJ:A��;���~X��t%D*a�Ahzp�A�ڃ`~�ڃo&gt;HI�}����˕p�8\&gt;�S3���i�&lt;1�K7����fu�=E��]^:~� �����O ;vB�\Vr�����4ο}�dμp �O�&gt;5{�z�|���3�@ X�2�8��:}z�a5 ��,C�� $����X����Xu�=�,#�:��� ªk �R�&lt;3Ő�.0O14�sL����T�K�:X��ڽ��b�1�B͑z����~���5�w��"�.p���55�#p�}�J�a��/Β�i/Hc���*�k��+�1��l�&gt;덝�͆��h*�� ����D�Rp&amp;�1�1&lt;���pgv$;����?L�d�A�`� f'����q|r&amp;��M���)v||:çӊ�\7)��Ύe�� �+��t $��WF������HG�\v$�-`aV?CX�Z��~ip��x���� � @��u^Dŧ�\X@�y4Z�=��%���+Tᅅ%�鬯?0�v{&lt;���]�3���x�؎�W���w�Ԛ� �G������ 6U�1U@�)4#�GT��� �տ@�� ���b(� �l�s7e� �������R�:��.��U���6������ �q�[3�H���Ώ\JX���9�rˤ� �ۮ̭�ܮ�&lt;|���4!�S��%&lt;#| �wo3#|9�zɌ�r�0}��;��w3y:�������ӿ���{D�˒Q8R���ݞ�� d�P���W��*�f�J��|c�\!*Z��Eޜ!�I+���mxK�"d�_��"j�J0�\Q^�"���`)Y� $-Y��v����p�wBդ�UT�Ju��2� � 428l��2�� &amp;� �2���Y����JJ��a}�J���RVoZ�42Y�$��k�\@��M���&amp;h� �d&amp;Z�@�A�,g�G ���;T6 &gt;�Vx�x&lt;&gt; � �*�`�h�T��j���*�P�^U�G��� Y�_�� a�w���,�� ��Z�Uђ�E�=��1������*��K��D'���N��tY5֊��Ʊ/� i��D6��6B�ZO���������?ܐ�&amp;(t=K�%� �"_���]t%��` �'�� � _ .s{�d��\�B YS�WX����h0Z)�^i4��6�V�9��3*P��O"�q��@�D�FH!��7e�%� V��zؠL��e���4����V9D���g�G�Փ/H�9H�Z���D��N��� ��mz�ͦ����]z[������'�4K`��^&amp;�:���X�� k;Hvǎ��P� A(��e�T���~����j��TssOY������8��dAړ�!�8�� ��ǉ(=8%�Qz�ٕX\��{��خX&lt;�݌���96;���)� �_��|��!�䣃C���� �XF�+Ã��;��;�N�tj���D��Hb5�RJ}��� J��̛L #T��J�Qh��h�: 6�*�, �[���` ��8 1񄰑T���Qbu{�� ո�,�IS��RCL�C&amp;�� �6���-���~�҄�W��7"��-I�%9�jAtJ�sUoJDXW�[��(#�W ����]����_K,rrax�q)Ŝq�� �ik������:$�/2�� ]Շ�2���� �*��U���V�`�+����_O ���W8��c}�_ }���̀�e8h ]M̃��m��U|�����!� -�t �#v� �IZ�M ��n?�w_�~������Z���N�3 R~" ��0끈P&amp;� �8h(�߿���㝞N&lt;� �� ���8-��Gp�ڃfC3,�+08E-�P[�����\u�AǙ9UU��ť=9 p�@ ܉�����HOJI��R���]���!��eP��)�س ��Ә͜�,㒜9Ds@svt�����9d��AB�2��.JA�\�p(r1��`��2 ��87���R����������� EE���Ri4ش4�|E�i5��jZ��ܳnY;����nWo��m�X{��7?l���I��΂ � Ēi0)NZ%�A�d0�!��!Hj�n�L����T�3�w��¦� �&gt;&amp;�H����(b9u������+֒�v�7��%o�G$Q���礜�� ��;qHPX��7ܸ�6�߼�.��\� �|�p�$��̃����A�� ����l�� ~h�ߙ�2�j����~㚑\4�ѨS����y3��� ���� ʏ�c �����h"(&lt;����&amp;�-�(�F x���â�Ƶ�4�Nj��t���废�H9�;�{NGUP�=xOV� � � ;$;v$�4ɧ�|ҝ�5��bg[�� ���F��R6X�(��&lt;2���jh���'�~�g@ yP�� �P���W2 M&amp;��g�d"�`GO$("�L &amp;�,�Hu2 ��t���������Ӭ�� ��~�JE;�+��&amp;3���E=$?���ᘢ ������|��jl�V���i��)��)X�gu�{�2d[��]��{ �px�pޖ�m&amp;�� �Y*5���Ml1�����Mf��U: e}������U:��J(��uI�YJ,�t: �9������X.8C��\yC��ԜG}�.W&gt;*�;k��ŏ=�g��$�~�Z�(y;/�c����C�?�z&gt;}p�T������b4�߮�_��ٗ_��t�T#mQ��!��seM����Nb/q� �o� ���ɵ��N�yR��x��g�� �T�V��j` ���� г ���~������)~�@1wfnm����M ;&gt;F-2�� ]�\�:J�,;_��`ؽ��l ��)`���ɣ_;J2G�G�R*�(&amp;�S� �Dp ����ŕ�)����ѩ���S!b���k���LL.L�M^��((�JO�k��%�&amp;ʵZ8�'�Z��ۘ#�� �^K%�x�,�Z ҏ��r���\/=)�4�V~e+z���a�倕rNa.�j�32��*Λ �7O��&amp;�3I���</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1771</v>
+        <v>12172</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>PDF</t>
+          <t>Requests</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1253,11 +1253,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Page not found - Artificial Intelligence (AI) at Purdue University Skip to content 404 ERROR We’re sorry you were not able to find the page you were looking for. Search Search Major Tuition &amp; Costs Schedule a Visit Boilermakers’ Stories Apply</t>
+          <t>Page not found - Artificial Intelligence (AI) at Purdue University Purdue Virtual Assistant Hi! I'm the Purdue Virtual Assistant. I can help answer your questions about IT Services. How can I help you? Skip to content 404 ERROR We’re sorry you were not able to find the page you were looking for. Search Search Major Tuition &amp; Costs Schedule a Visit Boilermakers’ Stories Apply</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>

</xml_diff>